<commit_message>
[v0.4.0-20261001T040433Z][TM-004] Register detailed cases and identity vectors
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R273bfaa83b6049a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rbc6ef8bb2639460e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R040b0abcea5b431b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R6440d552f63d4ee6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Raf16677dbd7a4485"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rc1d784c2090d4389"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rf593c1d785cd445b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R6b7a1e7c3e3044e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R4341405b107e4236"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R1d84b9095f3648d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R2b6cc7a070834b86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Re3106a0d2e2d4b80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R6a57cec12e994a8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rf6cef35fabc24ddd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R870d1980669b4311"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rb0e4008c77844b04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rbc5331d93c774516"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rc90f2e9dd79b4bb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R277b58ca05794dbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rd0996dd94d3c45f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R887b18a934b54a2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Red3b7ea71774408d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -731,8 +731,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="TMTable5" displayName="TMTable5" ref="A4:K39" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:K39"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="TMTable5" displayName="TMTable5" ref="A4:K47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:K47"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="任务编号"/>
     <x:tableColumn id="2" name="层级"/>
@@ -751,8 +751,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:M113" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:M113"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:M133" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:M133"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="功能编号"/>
     <x:tableColumn id="2" name="用例编号"/>
@@ -794,8 +794,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="TMTable8" displayName="TMTable8" ref="A4:M6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:M6"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="TMTable8" displayName="TMTable8" ref="A4:M7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:M7"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="发布编号"/>
     <x:tableColumn id="2" name="版本"/>
@@ -1091,8 +1091,8 @@
         <x:v>已登记用例</x:v>
       </x:c>
       <x:c r="B8" s="11" t="n">
-        <x:f>COUNTA('05测试用例'!B5:B113)</x:f>
-        <x:v>109</x:v>
+        <x:f>COUNTA('05测试用例'!B5:B133)</x:f>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>包含细化用例及未来概要场景</x:v>
@@ -1115,7 +1115,7 @@
         <x:v>细化产品用例</x:v>
       </x:c>
       <x:c r="B10" s="11" t="n">
-        <x:v>67</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
         <x:v>逐条结果按运行批次记录；变体在独立结果Excel列出</x:v>
@@ -1148,7 +1148,7 @@
         <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="B13" s="10" t="n">
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C13" s="4" t="str">
         <x:v>在05测试用例筛选此状态</x:v>
@@ -1245,7 +1245,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f032e25c44a498a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb58c15311bf44e1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1953,7 +1953,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf83fc05e890d4999"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R442989d133f3481a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2102,7 +2102,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95753fc0b9574ea2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4227ee48b2e4820"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2497,7 +2497,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc10d539c148d4de5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R416a3d7305724974"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3416,7 +3416,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6b51f9b912f4f1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fa85358b3444e5f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3592,10 +3592,10 @@
         <x:v>0.4.0</x:v>
       </x:c>
       <x:c r="H8" s="9" t="str">
-        <x:v>规划中</x:v>
+        <x:v>开发中</x:v>
       </x:c>
       <x:c r="I8" s="9" t="str">
-        <x:v>docs/product/README.md:21</x:v>
+        <x:v>releases/v0.4.0-20261001T040433Z/02-breakdown.md</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -4126,7 +4126,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R511cbb049ee44e39"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9554a7b42354ae4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5193,260 +5193,564 @@
         <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:56</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="32" customHeight="1">
+    <x:row r="33" ht="72" customHeight="1">
       <x:c r="A33" s="4" t="str">
-        <x:v>TASK-TM001-PLAN</x:v>
+        <x:v>TASK-TM004-SOURCE</x:v>
       </x:c>
       <x:c r="B33" s="4" t="str">
-        <x:v>历史分组</x:v>
+        <x:v>具体任务</x:v>
       </x:c>
       <x:c r="C33" s="4" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="D33" s="4" t="str">
+        <x:v>REQ-TM004</x:v>
+      </x:c>
+      <x:c r="E33" s="4" t="str">
+        <x:v>AC-TM004-001
+AC-TM004-002
+AC-TM004-003
+AC-TM004-004</x:v>
+      </x:c>
+      <x:c r="F33" s="4" t="str">
+        <x:v>TM-002授权句柄、项目目录</x:v>
+      </x:c>
+      <x:c r="G33" s="4" t="str">
+        <x:v>只遍历授权根下已确认的主/子日志；失权停扫、重授补扫；越界拒绝；预览与采集分别判定</x:v>
+      </x:c>
+      <x:c r="H33" s="4" t="str">
+        <x:v>TM-002授权接口及可续扫合同</x:v>
+      </x:c>
+      <x:c r="I33" s="4" t="str">
         <x:v>不适用</x:v>
       </x:c>
-      <x:c r="D33" s="4" t="str">
-        <x:v>REQ-TM001</x:v>
-      </x:c>
-      <x:c r="E33" s="4" t="str">
+      <x:c r="J33" s="4" t="str">
+        <x:v>baseline_pending</x:v>
+      </x:c>
+      <x:c r="K33" s="4" t="str">
+        <x:v>releases/v0.4.0-20261001T040433Z/02-breakdown.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="72" customHeight="1">
+      <x:c r="A34" s="9" t="str">
+        <x:v>TASK-TM004-PARSER</x:v>
+      </x:c>
+      <x:c r="B34" s="9" t="str">
+        <x:v>具体任务</x:v>
+      </x:c>
+      <x:c r="C34" s="9" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="D34" s="9" t="str">
+        <x:v>REQ-TM004</x:v>
+      </x:c>
+      <x:c r="E34" s="9" t="str">
+        <x:v>AC-TM004-001
+AC-TM004-002
+AC-TM004-003
+AC-TM004-004</x:v>
+      </x:c>
+      <x:c r="F34" s="9" t="str">
+        <x:v>版本来源明确的完整原始行</x:v>
+      </x:c>
+      <x:c r="G34" s="9" t="str">
+        <x:v>抽取usage、模型、UTC时间、主/子标志及来源标识；不保留正文</x:v>
+      </x:c>
+      <x:c r="H34" s="9" t="str">
+        <x:v>raw样本、TM-003事件合同</x:v>
+      </x:c>
+      <x:c r="I34" s="9" t="str">
         <x:v>不适用</x:v>
       </x:c>
-      <x:c r="F33" s="4" t="str">
+      <x:c r="J34" s="9" t="str">
+        <x:v>baseline_pending</x:v>
+      </x:c>
+      <x:c r="K34" s="9" t="str">
+        <x:v>releases/v0.4.0-20261001T040433Z/02-breakdown.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="72" customHeight="1">
+      <x:c r="A35" s="4" t="str">
+        <x:v>TASK-TM004-LINEAGE</x:v>
+      </x:c>
+      <x:c r="B35" s="4" t="str">
+        <x:v>具体任务</x:v>
+      </x:c>
+      <x:c r="C35" s="4" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="D35" s="4" t="str">
+        <x:v>REQ-TM004</x:v>
+      </x:c>
+      <x:c r="E35" s="4" t="str">
+        <x:v>AC-TM004-001
+AC-TM004-002
+AC-TM004-003
+AC-TM004-004</x:v>
+      </x:c>
+      <x:c r="F35" s="4" t="str">
+        <x:v>父子与fork来源证据</x:v>
+      </x:c>
+      <x:c r="G35" s="4" t="str">
+        <x:v>证实父子关系时正确归属；证实继承历史时跨会话去重；歧义诊断且不污染可信量</x:v>
+      </x:c>
+      <x:c r="H35" s="4" t="str">
+        <x:v>raw父子/fork样本、PARSER</x:v>
+      </x:c>
+      <x:c r="I35" s="4" t="str">
         <x:v>不适用</x:v>
       </x:c>
-      <x:c r="G33" s="4" t="str">
-        <x:v>六文档、完整追踪、SOP 修正、基线通过</x:v>
-      </x:c>
-      <x:c r="H33" s="4" t="str">
-        <x:v>需求</x:v>
-      </x:c>
-      <x:c r="I33" s="4" t="str">
-        <x:v>TEST-TM001-GOVERNANCE</x:v>
-      </x:c>
-      <x:c r="J33" s="4" t="str">
-        <x:v>historical_group_not_minimal_task</x:v>
-      </x:c>
-      <x:c r="K33" s="4" t="str">
-        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="42" customHeight="1">
-      <x:c r="A34" s="9" t="str">
-        <x:v>TASK-TM001-SERVER</x:v>
-      </x:c>
-      <x:c r="B34" s="9" t="str">
-        <x:v>历史分组</x:v>
-      </x:c>
-      <x:c r="C34" s="9" t="str">
-        <x:v>不适用</x:v>
-      </x:c>
-      <x:c r="D34" s="9" t="str">
-        <x:v>REQ-TM001</x:v>
-      </x:c>
-      <x:c r="E34" s="9" t="str">
-        <x:v>不适用</x:v>
-      </x:c>
-      <x:c r="F34" s="9" t="str">
-        <x:v>不适用</x:v>
-      </x:c>
-      <x:c r="G34" s="9" t="str">
-        <x:v>FastAPI/SQLAlchemy/Alembic 工程、真实认证/权限/审计 API；随机可撤销 token 固定30天到期、不滑动，改密/重置/停用撤销旧会话</x:v>
-      </x:c>
-      <x:c r="H34" s="9" t="str">
-        <x:v>计划、数据/测试</x:v>
-      </x:c>
-      <x:c r="I34" s="9" t="str">
-        <x:v>E2E-TM001-001、E2E-TM001-002、E2E-TM001-003</x:v>
-      </x:c>
-      <x:c r="J34" s="9" t="str">
-        <x:v>historical_group_not_minimal_task</x:v>
-      </x:c>
-      <x:c r="K34" s="9" t="str">
-        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="42" customHeight="1">
-      <x:c r="A35" s="4" t="str">
-        <x:v>TASK-TM001-DATA</x:v>
-      </x:c>
-      <x:c r="B35" s="4" t="str">
-        <x:v>历史分组</x:v>
-      </x:c>
-      <x:c r="C35" s="4" t="str">
-        <x:v>不适用</x:v>
-      </x:c>
-      <x:c r="D35" s="4" t="str">
-        <x:v>REQ-TM001</x:v>
-      </x:c>
-      <x:c r="E35" s="4" t="str">
-        <x:v>不适用</x:v>
-      </x:c>
-      <x:c r="F35" s="4" t="str">
-        <x:v>不适用</x:v>
-      </x:c>
-      <x:c r="G35" s="4" t="str">
-        <x:v>独立测试/生产 SQLite 文件、可执行造数 SQL、生产首建管理员、回归账号/独立预期及安全重置；已有生产密码不可被重建覆盖</x:v>
-      </x:c>
-      <x:c r="H35" s="4" t="str">
-        <x:v>计划、工程骨架</x:v>
-      </x:c>
-      <x:c r="I35" s="4" t="str">
-        <x:v>TEST-TM001-SERVER、E2E-TM001-001、E2E-TM001-005</x:v>
-      </x:c>
       <x:c r="J35" s="4" t="str">
-        <x:v>historical_group_not_minimal_task</x:v>
+        <x:v>baseline_pending</x:v>
       </x:c>
       <x:c r="K35" s="4" t="str">
-        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:11</x:v>
+        <x:v>releases/v0.4.0-20261001T040433Z/02-breakdown.md</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="72" customHeight="1">
       <x:c r="A36" s="9" t="str">
+        <x:v>TASK-TM004-INCREMENTAL</x:v>
+      </x:c>
+      <x:c r="B36" s="9" t="str">
+        <x:v>具体任务</x:v>
+      </x:c>
+      <x:c r="C36" s="9" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="D36" s="9" t="str">
+        <x:v>REQ-TM004</x:v>
+      </x:c>
+      <x:c r="E36" s="9" t="str">
+        <x:v>AC-TM004-001
+AC-TM004-002
+AC-TM004-003
+AC-TM004-004</x:v>
+      </x:c>
+      <x:c r="F36" s="9" t="str">
+        <x:v>追加、半行、重复片段、跨来源ID、重启</x:v>
+      </x:c>
+      <x:c r="G36" s="9" t="str">
+        <x:v>持久游标、唯一键及事务；完整行才提交；跨来源不误去重；重扫幂等</x:v>
+      </x:c>
+      <x:c r="H36" s="9" t="str">
+        <x:v>TM-003 SQLite身份合同、PARSER</x:v>
+      </x:c>
+      <x:c r="I36" s="9" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="J36" s="9" t="str">
+        <x:v>baseline_pending</x:v>
+      </x:c>
+      <x:c r="K36" s="9" t="str">
+        <x:v>releases/v0.4.0-20261001T040433Z/02-breakdown.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="72" customHeight="1">
+      <x:c r="A37" s="4" t="str">
+        <x:v>TASK-TM004-DIAGNOSTIC</x:v>
+      </x:c>
+      <x:c r="B37" s="4" t="str">
+        <x:v>具体任务</x:v>
+      </x:c>
+      <x:c r="C37" s="4" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="D37" s="4" t="str">
+        <x:v>REQ-TM004</x:v>
+      </x:c>
+      <x:c r="E37" s="4" t="str">
+        <x:v>AC-TM004-001
+AC-TM004-002
+AC-TM004-003
+AC-TM004-004</x:v>
+      </x:c>
+      <x:c r="F37" s="4" t="str">
+        <x:v>缺usage、未知格式、读取失败</x:v>
+      </x:c>
+      <x:c r="G37" s="4" t="str">
+        <x:v>UI区分可信零、未知、缺失、无授权；诊断不泄露正文或完整路径</x:v>
+      </x:c>
+      <x:c r="H37" s="4" t="str">
+        <x:v>TM-003诊断接口、PARSER</x:v>
+      </x:c>
+      <x:c r="I37" s="4" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="J37" s="4" t="str">
+        <x:v>baseline_pending</x:v>
+      </x:c>
+      <x:c r="K37" s="4" t="str">
+        <x:v>releases/v0.4.0-20261001T040433Z/02-breakdown.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="72" customHeight="1">
+      <x:c r="A38" s="9" t="str">
+        <x:v>TASK-TM004-DATA</x:v>
+      </x:c>
+      <x:c r="B38" s="9" t="str">
+        <x:v>具体任务</x:v>
+      </x:c>
+      <x:c r="C38" s="9" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="D38" s="9" t="str">
+        <x:v>REQ-TM004</x:v>
+      </x:c>
+      <x:c r="E38" s="9" t="str">
+        <x:v>AC-TM004-001
+AC-TM004-002
+AC-TM004-003
+AC-TM004-004</x:v>
+      </x:c>
+      <x:c r="F38" s="9" t="str">
+        <x:v>隔离Claude Code 2.1.126原生投影与合成反例</x:v>
+      </x:c>
+      <x:c r="G38" s="9" t="str">
+        <x:v>版本化fixture生成、追加/半行/撤权程序、独立expected及SQLite只读检查</x:v>
+      </x:c>
+      <x:c r="H38" s="9" t="str">
+        <x:v>raw来源、TM-002/003数据合同</x:v>
+      </x:c>
+      <x:c r="I38" s="9" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="J38" s="9" t="str">
+        <x:v>baseline_pending</x:v>
+      </x:c>
+      <x:c r="K38" s="9" t="str">
+        <x:v>releases/v0.4.0-20261001T040433Z/02-breakdown.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="72" customHeight="1">
+      <x:c r="A39" s="4" t="str">
+        <x:v>TASK-TM004-E2E</x:v>
+      </x:c>
+      <x:c r="B39" s="4" t="str">
+        <x:v>具体任务</x:v>
+      </x:c>
+      <x:c r="C39" s="4" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="D39" s="4" t="str">
+        <x:v>REQ-TM004</x:v>
+      </x:c>
+      <x:c r="E39" s="4" t="str">
+        <x:v>AC-TM004-001
+AC-TM004-002
+AC-TM004-003
+AC-TM004-004</x:v>
+      </x:c>
+      <x:c r="F39" s="4" t="str">
+        <x:v>最终安装App、真实服务、隔离SQLite</x:v>
+      </x:c>
+      <x:c r="G39" s="4" t="str">
+        <x:v>全部细TC绑定固定Playwright Electron测试；逐步原始记录及历史功能全量回归</x:v>
+      </x:c>
+      <x:c r="H39" s="4" t="str">
+        <x:v>SOURCE→DATA、TM-001包执行器</x:v>
+      </x:c>
+      <x:c r="I39" s="4" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="J39" s="4" t="str">
+        <x:v>baseline_pending</x:v>
+      </x:c>
+      <x:c r="K39" s="4" t="str">
+        <x:v>releases/v0.4.0-20261001T040433Z/02-breakdown.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="72" customHeight="1">
+      <x:c r="A40" s="9" t="str">
+        <x:v>TASK-TM004-RELEASE</x:v>
+      </x:c>
+      <x:c r="B40" s="9" t="str">
+        <x:v>具体任务</x:v>
+      </x:c>
+      <x:c r="C40" s="9" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="D40" s="9" t="str">
+        <x:v>REQ-TM004</x:v>
+      </x:c>
+      <x:c r="E40" s="9" t="str">
+        <x:v>AC-TM004-001
+AC-TM004-002
+AC-TM004-003
+AC-TM004-004</x:v>
+      </x:c>
+      <x:c r="F40" s="9" t="str">
+        <x:v>完整候选</x:v>
+      </x:c>
+      <x:c r="G40" s="9" t="str">
+        <x:v>文档、矩阵、总表、Changelog同步；DMG安装门禁；交总控集成</x:v>
+      </x:c>
+      <x:c r="H40" s="9" t="str">
+        <x:v>E2E与此前版本全回归</x:v>
+      </x:c>
+      <x:c r="I40" s="9" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="J40" s="9" t="str">
+        <x:v>baseline_pending</x:v>
+      </x:c>
+      <x:c r="K40" s="9" t="str">
+        <x:v>releases/v0.4.0-20261001T040433Z/02-breakdown.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="32" customHeight="1">
+      <x:c r="A41" s="4" t="str">
+        <x:v>TASK-TM001-PLAN</x:v>
+      </x:c>
+      <x:c r="B41" s="4" t="str">
+        <x:v>历史分组</x:v>
+      </x:c>
+      <x:c r="C41" s="4" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="D41" s="4" t="str">
+        <x:v>REQ-TM001</x:v>
+      </x:c>
+      <x:c r="E41" s="4" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="F41" s="4" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="G41" s="4" t="str">
+        <x:v>六文档、完整追踪、SOP 修正、基线通过</x:v>
+      </x:c>
+      <x:c r="H41" s="4" t="str">
+        <x:v>需求</x:v>
+      </x:c>
+      <x:c r="I41" s="4" t="str">
+        <x:v>TEST-TM001-GOVERNANCE</x:v>
+      </x:c>
+      <x:c r="J41" s="4" t="str">
+        <x:v>historical_group_not_minimal_task</x:v>
+      </x:c>
+      <x:c r="K41" s="4" t="str">
+        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="42" customHeight="1">
+      <x:c r="A42" s="9" t="str">
+        <x:v>TASK-TM001-SERVER</x:v>
+      </x:c>
+      <x:c r="B42" s="9" t="str">
+        <x:v>历史分组</x:v>
+      </x:c>
+      <x:c r="C42" s="9" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="D42" s="9" t="str">
+        <x:v>REQ-TM001</x:v>
+      </x:c>
+      <x:c r="E42" s="9" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="F42" s="9" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="G42" s="9" t="str">
+        <x:v>FastAPI/SQLAlchemy/Alembic 工程、真实认证/权限/审计 API；随机可撤销 token 固定30天到期、不滑动，改密/重置/停用撤销旧会话</x:v>
+      </x:c>
+      <x:c r="H42" s="9" t="str">
+        <x:v>计划、数据/测试</x:v>
+      </x:c>
+      <x:c r="I42" s="9" t="str">
+        <x:v>E2E-TM001-001、E2E-TM001-002、E2E-TM001-003</x:v>
+      </x:c>
+      <x:c r="J42" s="9" t="str">
+        <x:v>historical_group_not_minimal_task</x:v>
+      </x:c>
+      <x:c r="K42" s="9" t="str">
+        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="42" customHeight="1">
+      <x:c r="A43" s="4" t="str">
+        <x:v>TASK-TM001-DATA</x:v>
+      </x:c>
+      <x:c r="B43" s="4" t="str">
+        <x:v>历史分组</x:v>
+      </x:c>
+      <x:c r="C43" s="4" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="D43" s="4" t="str">
+        <x:v>REQ-TM001</x:v>
+      </x:c>
+      <x:c r="E43" s="4" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="F43" s="4" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="G43" s="4" t="str">
+        <x:v>独立测试/生产 SQLite 文件、可执行造数 SQL、生产首建管理员、回归账号/独立预期及安全重置；已有生产密码不可被重建覆盖</x:v>
+      </x:c>
+      <x:c r="H43" s="4" t="str">
+        <x:v>计划、工程骨架</x:v>
+      </x:c>
+      <x:c r="I43" s="4" t="str">
+        <x:v>TEST-TM001-SERVER、E2E-TM001-001、E2E-TM001-005</x:v>
+      </x:c>
+      <x:c r="J43" s="4" t="str">
+        <x:v>historical_group_not_minimal_task</x:v>
+      </x:c>
+      <x:c r="K43" s="4" t="str">
+        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="72" customHeight="1">
+      <x:c r="A44" s="9" t="str">
         <x:v>TASK-TM001-MAC</x:v>
       </x:c>
-      <x:c r="B36" s="9" t="str">
+      <x:c r="B44" s="9" t="str">
         <x:v>历史分组</x:v>
       </x:c>
-      <x:c r="C36" s="9" t="str">
+      <x:c r="C44" s="9" t="str">
         <x:v>不适用</x:v>
       </x:c>
-      <x:c r="D36" s="9" t="str">
+      <x:c r="D44" s="9" t="str">
         <x:v>REQ-TM001</x:v>
       </x:c>
-      <x:c r="E36" s="9" t="str">
+      <x:c r="E44" s="9" t="str">
         <x:v>不适用</x:v>
       </x:c>
-      <x:c r="F36" s="9" t="str">
+      <x:c r="F44" s="9" t="str">
         <x:v>不适用</x:v>
       </x:c>
-      <x:c r="G36" s="9" t="str">
+      <x:c r="G44" s="9" t="str">
         <x:v>Electron React/TypeScript 登录/改密/主页/管理、默认本机 API/更新源地址与配置管理页的用户覆盖持久化；默认开启可关闭的设备自动登录、按规范化 origin 隔离的受保护凭据文件与内存会话、稳定 UI 标识、Playwright Electron工程</x:v>
       </x:c>
-      <x:c r="H36" s="9" t="str">
+      <x:c r="H44" s="9" t="str">
         <x:v>API 合同、工程骨架</x:v>
       </x:c>
-      <x:c r="I36" s="9" t="str">
+      <x:c r="I44" s="9" t="str">
         <x:v>E2E-TM001-001、E2E-TM001-002、E2E-TM001-003、E2E-TM001-004、E2E-TM001-005、E2E-TM001-006</x:v>
       </x:c>
-      <x:c r="J36" s="9" t="str">
+      <x:c r="J44" s="9" t="str">
         <x:v>historical_group_not_minimal_task</x:v>
       </x:c>
-      <x:c r="K36" s="9" t="str">
+      <x:c r="K44" s="9" t="str">
         <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:12</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="57" customHeight="1">
-      <x:c r="A37" s="4" t="str">
+    <x:row r="45" ht="57" customHeight="1">
+      <x:c r="A45" s="4" t="str">
         <x:v>TASK-TM001-UPDATE</x:v>
       </x:c>
-      <x:c r="B37" s="4" t="str">
+      <x:c r="B45" s="4" t="str">
         <x:v>历史分组</x:v>
       </x:c>
-      <x:c r="C37" s="4" t="str">
+      <x:c r="C45" s="4" t="str">
         <x:v>不适用</x:v>
       </x:c>
-      <x:c r="D37" s="4" t="str">
+      <x:c r="D45" s="4" t="str">
         <x:v>REQ-TM001</x:v>
       </x:c>
-      <x:c r="E37" s="4" t="str">
+      <x:c r="E45" s="4" t="str">
         <x:v>不适用</x:v>
       </x:c>
-      <x:c r="F37" s="4" t="str">
+      <x:c r="F45" s="4" t="str">
         <x:v>不适用</x:v>
       </x:c>
-      <x:c r="G37" s="4" t="str">
+      <x:c r="G45" s="4" t="str">
         <x:v>固定 Ed25519 公钥、同机回环更新源/签名测试包/失败包及真实更新用例；默认49177配置、URL安全校验与升级时锁定更新设置；两构建沿用经校验的同一隔离profile，升级后服务验证自动登录</x:v>
       </x:c>
-      <x:c r="H37" s="4" t="str">
+      <x:c r="H45" s="4" t="str">
         <x:v>Mac 工程</x:v>
       </x:c>
-      <x:c r="I37" s="4" t="str">
+      <x:c r="I45" s="4" t="str">
         <x:v>E2E-TM001-004</x:v>
       </x:c>
-      <x:c r="J37" s="4" t="str">
+      <x:c r="J45" s="4" t="str">
         <x:v>historical_group_not_minimal_task</x:v>
       </x:c>
-      <x:c r="K37" s="4" t="str">
+      <x:c r="K45" s="4" t="str">
         <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:13</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="57" customHeight="1">
-      <x:c r="A38" s="9" t="str">
+    <x:row r="46" ht="57" customHeight="1">
+      <x:c r="A46" s="9" t="str">
         <x:v>TASK-TM001-RUNNER</x:v>
       </x:c>
-      <x:c r="B38" s="9" t="str">
+      <x:c r="B46" s="9" t="str">
         <x:v>历史分组</x:v>
       </x:c>
-      <x:c r="C38" s="9" t="str">
+      <x:c r="C46" s="9" t="str">
         <x:v>不适用</x:v>
       </x:c>
-      <x:c r="D38" s="9" t="str">
+      <x:c r="D46" s="9" t="str">
         <x:v>REQ-TM001</x:v>
       </x:c>
-      <x:c r="E38" s="9" t="str">
+      <x:c r="E46" s="9" t="str">
         <x:v>不适用</x:v>
       </x:c>
-      <x:c r="F38" s="9" t="str">
+      <x:c r="F46" s="9" t="str">
         <x:v>不适用</x:v>
       </x:c>
-      <x:c r="G38" s="9" t="str">
+      <x:c r="G46" s="9" t="str">
         <x:v>本机Playwright从最终DMG安装App执行全部六例，原始JSON/trace/fixtureSQL/包摘要、父门禁复核；默认值与动态独占端口隔离测试；真实Squirrel自重启及profile、身份恢复</x:v>
       </x:c>
-      <x:c r="H38" s="9" t="str">
+      <x:c r="H46" s="9" t="str">
         <x:v>数据/桌面工程</x:v>
       </x:c>
-      <x:c r="I38" s="9" t="str">
+      <x:c r="I46" s="9" t="str">
         <x:v>E2E-TM001-001、E2E-TM001-002、E2E-TM001-003、E2E-TM001-004、E2E-TM001-005、E2E-TM001-006</x:v>
       </x:c>
-      <x:c r="J38" s="9" t="str">
+      <x:c r="J46" s="9" t="str">
         <x:v>historical_group_not_minimal_task</x:v>
       </x:c>
-      <x:c r="K38" s="9" t="str">
+      <x:c r="K46" s="9" t="str">
         <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:14</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="32" customHeight="1">
-      <x:c r="A39" s="4" t="str">
+    <x:row r="47" ht="32" customHeight="1">
+      <x:c r="A47" s="4" t="str">
         <x:v>TASK-TM001-REVIEW</x:v>
       </x:c>
-      <x:c r="B39" s="4" t="str">
+      <x:c r="B47" s="4" t="str">
         <x:v>历史分组</x:v>
       </x:c>
-      <x:c r="C39" s="4" t="str">
+      <x:c r="C47" s="4" t="str">
         <x:v>不适用</x:v>
       </x:c>
-      <x:c r="D39" s="4" t="str">
+      <x:c r="D47" s="4" t="str">
         <x:v>REQ-TM001</x:v>
       </x:c>
-      <x:c r="E39" s="4" t="str">
+      <x:c r="E47" s="4" t="str">
         <x:v>不适用</x:v>
       </x:c>
-      <x:c r="F39" s="4" t="str">
+      <x:c r="F47" s="4" t="str">
         <x:v>不适用</x:v>
       </x:c>
-      <x:c r="G39" s="4" t="str">
+      <x:c r="G47" s="4" t="str">
         <x:v>完整回归、流程复盘、PR 与合并判定、发布阻塞记录</x:v>
       </x:c>
-      <x:c r="H39" s="4" t="str">
+      <x:c r="H47" s="4" t="str">
         <x:v>全部实现任务</x:v>
       </x:c>
-      <x:c r="I39" s="4" t="str">
+      <x:c r="I47" s="4" t="str">
         <x:v>TEST-TM001-GOVERNANCE</x:v>
       </x:c>
-      <x:c r="J39" s="4" t="str">
+      <x:c r="J47" s="4" t="str">
         <x:v>historical_group_not_minimal_task</x:v>
       </x:c>
-      <x:c r="K39" s="4" t="str">
+      <x:c r="K47" s="4" t="str">
         <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:15</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="J5:J39">
+  <x:conditionalFormatting sqref="J5:J47">
     <x:cfRule type="containsText" dxfId="9" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="10" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="11" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37a03de48b1548e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re12022c604784224"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9451,517 +9755,550 @@
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
-    <x:row r="93" ht="57" customHeight="1">
+    <x:row r="93" ht="72" customHeight="1">
       <x:c r="A93" s="4" t="str">
-        <x:v>TM-005</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B93" s="4" t="str">
-        <x:v>E2E-TM005-001</x:v>
+        <x:v>TC-TM004-SOURCE-01</x:v>
       </x:c>
       <x:c r="C93" s="4" t="str">
-        <x:v>日期筛选、趋势和明细</x:v>
+        <x:v>授权根限定（TASK-TM004-SOURCE，AC-001，E2E-001）</x:v>
       </x:c>
       <x:c r="D93" s="4" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-SOURCE</x:v>
       </x:c>
       <x:c r="E93" s="4" t="str">
         <x:v>产品E2E</x:v>
       </x:c>
       <x:c r="F93" s="4" t="str">
-        <x:v>数据集 date_ranges；date_ranges 已由 scripts/test_data.py 提供标准化语义样例，固定2026-09-29T04:00:00Z、Asia/Shanghai、seed42；13行含1重复、12唯一。需另有已验证raw输入映射和真实App导入流程，当前未实现。</x:v>
+        <x:v>用户经 TM-002 UI 只选择隔离项目A目录；目录内有 M=100/10 完整原始行，旁边未授权目录有 X=999/99。</x:v>
       </x:c>
       <x:c r="G93" s="4" t="str">
-        <x:v>独立expected中的total依次16500、110、17380、27830、31130；custom=2200。today共5条、input15000、output1500、cache1700、reasoning170，cache/reasoning不再相加；custom-start包含、custom-end排除。趋势点及明细按expected事件时间逐条核对。</x:v>
+        <x:v>UI 显示待确认，事件表无新增
+UI 显示1次 M、total110，SQLite只读见唯一M
+调用数仍1、total110
+无X读取请求且事件表无X</x:v>
       </x:c>
       <x:c r="H93" s="4" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：只读按来源/项目统计 M 行数与 token，总数1/110；检查 X 键不存在；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I93" s="4" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J93" s="4" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K93" s="4" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L93" s="4" t="str">
-        <x:v>docs/testing/cases/05-TM-005-usage-statistics.md:15</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:87</x:v>
       </x:c>
       <x:c r="M93" s="4" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
-    <x:row r="94" ht="57" customHeight="1">
+    <x:row r="94" ht="72" customHeight="1">
       <x:c r="A94" s="9" t="str">
-        <x:v>TM-005</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B94" s="9" t="str">
-        <x:v>E2E-TM005-002</x:v>
+        <x:v>TC-TM004-SOURCE-02</x:v>
       </x:c>
       <x:c r="C94" s="9" t="str">
-        <x:v>时区、月边界与缺失值</x:v>
+        <x:v>撤权和重新授权（TASK-TM004-SOURCE，AC-004，E2E-004）</x:v>
       </x:c>
       <x:c r="D94" s="9" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-SOURCE</x:v>
       </x:c>
       <x:c r="E94" s="9" t="str">
         <x:v>产品E2E</x:v>
       </x:c>
       <x:c r="F94" s="9" t="str">
-        <x:v>数据集 date_ranges；复用date_ranges中的2026-09-28T15:59:59Z与16:00:00Z、2026-08-30T15:59:59Z与16:00:00Z边界。另需补充覆盖缺口、已覆盖零调用日、unknown字段三类状态；当前生成器未覆盖后面三类。</x:v>
+        <x:v>已扫描 M=100/10、S=200/20；撤权期间子代理新增 N=50/5。</x:v>
       </x:c>
       <x:c r="G94" s="9" t="str">
-        <x:v>Shanghai下15:59:59Z仍属前日、16:00:00Z属次日；UTC下二者同属UTC日期。无覆盖显示缺失，真实零可显示0，unknown字段显示未知；不得互相代替。各范围expected须独立按当地日期边界列出，不调用产品查询生成。</x:v>
+        <x:v>状态显示不可读且保留total330
+仍330且诊断为读取受阻
+唯一 M/S/N、total385
+M/S/N仍为三次且total385</x:v>
       </x:c>
       <x:c r="H94" s="9" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：只读唯一键数3与 token总385，撤权阶段无N。重置同共用配方；TM-002失权模拟与子目录绑定待补；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I94" s="9" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J94" s="9" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K94" s="9" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L94" s="9" t="str">
-        <x:v>docs/testing/cases/05-TM-005-usage-statistics.md:32</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:91</x:v>
       </x:c>
       <x:c r="M94" s="9" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
-    <x:row r="95" ht="57" customHeight="1">
+    <x:row r="95" ht="72" customHeight="1">
       <x:c r="A95" s="4" t="str">
-        <x:v>TM-006</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B95" s="4" t="str">
-        <x:v>E2E-TM006-001</x:v>
+        <x:v>TC-TM004-PARSER-01</x:v>
       </x:c>
       <x:c r="C95" s="4" t="str">
-        <x:v>Token子项与基础费用</x:v>
+        <x:v>主/子实际调用（TASK-TM004-PARSER，AC-001，E2E-001）</x:v>
       </x:c>
       <x:c r="D95" s="4" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-PARSER</x:v>
       </x:c>
       <x:c r="E95" s="4" t="str">
         <x:v>产品E2E</x:v>
       </x:c>
       <x:c r="F95" s="4" t="str">
-        <x:v>数据集 pricing；pricing由scripts/test_data.py生成合成非计费价格。gpt-5每百万input/cache/output为USD2/0.2/8；today-gpt input1000含cache200、output100含reasoning20。价格不是厂商现价。</x:v>
+        <x:v>同一项目原始主M100/10与子S200/20，模型各自保留，父关系有原始证据。</x:v>
       </x:c>
       <x:c r="G95" s="4" t="str">
-        <x:v>单调用total=1100；费用=(800×2+200×0.2+100×8)/1000000=USD0.002440，reasoning20不另加价。today已知费用USD0.015190且有1条无价格，alice今日USD0.010090。使用Decimal/十进制独立oracle，不以界面舍入反推底层精度。</x:v>
+        <x:v>可信total110
+可信input300/output30/total330
+仍2次调用/330</x:v>
       </x:c>
       <x:c r="H95" s="4" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：只读两条唯一事件和模型/父项目归属；不读取正文。版本化raw和模型字段待补；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I95" s="4" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J95" s="4" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K95" s="4" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L95" s="4" t="str">
-        <x:v>docs/testing/cases/06-TM-006-cost-estimates.md:15</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:95</x:v>
       </x:c>
       <x:c r="M95" s="4" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
-    <x:row r="96" ht="57" customHeight="1">
+    <x:row r="96" ht="102" customHeight="1">
       <x:c r="A96" s="9" t="str">
-        <x:v>TM-006</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B96" s="9" t="str">
-        <x:v>E2E-TM006-002</x:v>
+        <x:v>TC-TM004-PARSER-02</x:v>
       </x:c>
       <x:c r="C96" s="9" t="str">
-        <x:v>历史价格、多币种和未知费用</x:v>
+        <x:v>未知结构/缺字段（TASK-TM004-PARSER，AC-003，E2E-003）</x:v>
       </x:c>
       <x:c r="D96" s="9" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-PARSER</x:v>
       </x:c>
       <x:c r="E96" s="9" t="str">
         <x:v>产品E2E</x:v>
       </x:c>
       <x:c r="F96" s="9" t="str">
-        <x:v>数据集 pricing_extended；pricing_extended planned：同模型在生效时点T前后各一调用，两个独立价格版本；另有USD/CNY各一模型、无价模型和订阅估算模型。必须提供价格/订阅分摊规则及手算expected后才能实现。</x:v>
+        <x:v>已支持版本完整 M100/10、未知结构 U、JSONL 原始行真正缺 usage 的 Q。</x:v>
       </x:c>
       <x:c r="G96" s="9" t="str">
-        <x:v>T前后依各自生效版本计算，历史结果不会悄悄换价；USD与CNY分组，未约定汇率不得相加；无价格显示未知而非0；订阅必须明确估算口径。具体金额oracle依待定义订阅/价格合同生成，当前不得手填PASS。</x:v>
+        <x:v>可信total110
+可信仍110且出现未知结构诊断
+可信仍110、缺usage诊断新增
+诊断可见且不显示 U/Q 为零调用</x:v>
       </x:c>
       <x:c r="H96" s="9" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：只读可信事件1条/110，诊断各1条；具体版本标识、缺字段schema和SQL待补。隔离负测中 API SSE 省略 usage 后 CLI 仍在原生 JSONL 写0/0，**不是** Q 的原生缺字段样本；Q 需另证来源或标明故障注入，不得把0/0回填解释成已知零；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I96" s="9" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J96" s="9" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K96" s="9" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L96" s="9" t="str">
-        <x:v>docs/testing/cases/06-TM-006-cost-estimates.md:32</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:99</x:v>
       </x:c>
       <x:c r="M96" s="9" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
-    <x:row r="97" ht="57" customHeight="1">
+    <x:row r="97" ht="72" customHeight="1">
       <x:c r="A97" s="4" t="str">
-        <x:v>TM-007</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B97" s="4" t="str">
-        <x:v>E2E-TM007-001</x:v>
+        <x:v>TC-TM004-LINEAGE-01</x:v>
       </x:c>
       <x:c r="C97" s="4" t="str">
-        <x:v>离线、重启和补传幂等</x:v>
+        <x:v>子代理父项目（TASK-TM004-LINEAGE，AC-001，E2E-001）</x:v>
       </x:c>
       <x:c r="D97" s="4" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-LINEAGE</x:v>
       </x:c>
       <x:c r="E97" s="4" t="str">
         <x:v>产品E2E</x:v>
       </x:c>
       <x:c r="F97" s="4" t="str">
-        <x:v>数据集 sync_faults；sync_faults planned；alice两个隔离设备A/B，设备A调用100/10、B调用200/20；真实FastAPI/SQLite服务，可由外部fixture断网/恢复。账号继续用隔离测试fixture。</x:v>
+        <x:v>项目A主M100/10、子S200/20，另有项目B同名会话标识但无父关系。</x:v>
       </x:c>
       <x:c r="G97" s="4" t="str">
-        <x:v>离线重启不丢队列；恢复后2唯一调用、input300/output30/total330；重复批次不再加量。客户端只在真实确认后标已同步，个人合计与对应团队子集一致。</x:v>
+        <x:v>A=110
+A=330、B=0
+A仍330
+S标为子代理且使用原模型</x:v>
       </x:c>
       <x:c r="H97" s="4" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：只读S的父项目键为A、事件数2；原始父链线索缺失时不得假称通过；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I97" s="4" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J97" s="4" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K97" s="4" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L97" s="4" t="str">
-        <x:v>docs/testing/cases/07-TM-007-team-sync.md:11</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:103</x:v>
       </x:c>
       <x:c r="M97" s="4" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
-    <x:row r="98" ht="57" customHeight="1">
+    <x:row r="98" ht="72" customHeight="1">
       <x:c r="A98" s="9" t="str">
-        <x:v>TM-007</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B98" s="9" t="str">
-        <x:v>E2E-TM007-002</x:v>
+        <x:v>TC-TM004-LINEAGE-02</x:v>
       </x:c>
       <x:c r="C98" s="9" t="str">
-        <x:v>部分确认、中断和账号切换</x:v>
+        <x:v>fork继承和ID改写（TASK-TM004-LINEAGE，AC-002，E2E-002）</x:v>
       </x:c>
       <x:c r="D98" s="9" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-LINEAGE</x:v>
       </x:c>
       <x:c r="E98" s="9" t="str">
         <x:v>产品E2E</x:v>
       </x:c>
       <x:c r="F98" s="9" t="str">
-        <x:v>数据集 sync_faults；准备alice的三条唯一事件A/B/C，总量各110/220/330；控制服务仅确认A后断开，B可能已提交但响应丢失，C未提交。另有bob账号。故障注入必须在真实服务外部或明确测试环境中完成，不能绕过认证。</x:v>
+        <x:v>原M100/10、fork复制或引用M但消息ID改写、fork新N50/5。</x:v>
       </x:c>
       <x:c r="G98" s="9" t="str">
-        <x:v>最终alice的A/B/C各一次、total660；响应丢失不造成B重复；bob不能承接或篡改alice既有事件归属。切换时旧队列按已批准归属策略隔离，不能默认为新登录账号。</x:v>
+        <x:v>M仅入账一次且total110
+仍110
+total165且调用数2
+仍165</x:v>
       </x:c>
       <x:c r="H98" s="9" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：只读可信唯一调用2/165及继承诊断/关系；待schema确定；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I98" s="9" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J98" s="9" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K98" s="9" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L98" s="9" t="str">
-        <x:v>docs/testing/cases/07-TM-007-team-sync.md:28</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:107</x:v>
       </x:c>
       <x:c r="M98" s="9" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
-    <x:row r="99" ht="57" customHeight="1">
+    <x:row r="99" ht="72" customHeight="1">
       <x:c r="A99" s="4" t="str">
-        <x:v>TM-007</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B99" s="4" t="str">
-        <x:v>E2E-TM007-003</x:v>
+        <x:v>TC-TM004-INCREMENTAL-01</x:v>
       </x:c>
       <x:c r="C99" s="4" t="str">
-        <x:v>上传白名单与项目映射</x:v>
+        <x:v>半行完成（TASK-TM004-INCREMENTAL，AC-002，E2E-002）</x:v>
       </x:c>
       <x:c r="D99" s="4" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-INCREMENTAL</x:v>
       </x:c>
       <x:c r="E99" s="4" t="str">
         <x:v>产品E2E</x:v>
       </x:c>
       <x:c r="F99" s="4" t="str">
-        <x:v>数据集 sync_faults；合成日志包含唯一正文/代码/API-key/完整路径哨兵，以及合法用量/必要去重元数据；只用假值。准备已归属项目A和未归属事件B，待sync_faults生成。</x:v>
+        <x:v>已计M+N total165，P=20/2 原始JSONL行分成两次写入。</x:v>
       </x:c>
       <x:c r="G99" s="4" t="str">
-        <x:v>网络载荷/持久服务数据均不得含正文、代码、key或完整本机路径；只有批准用量/去重字段。B可明确分配，分配不增加事件量、也不跨团队归属。</x:v>
+        <x:v>扫描后仍165、读取游标未越过半行
+扫描后total187、调用数3
+P仅入账一次且total187</x:v>
       </x:c>
       <x:c r="H99" s="4" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：只读P只一条，可信事件3/187，游标处于完整行末；具体游标schema待补；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I99" s="4" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J99" s="4" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K99" s="4" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L99" s="4" t="str">
-        <x:v>docs/testing/cases/07-TM-007-team-sync.md:45</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:111</x:v>
       </x:c>
       <x:c r="M99" s="4" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
-    <x:row r="100" ht="57" customHeight="1">
+    <x:row r="100" ht="72" customHeight="1">
       <x:c r="A100" s="9" t="str">
-        <x:v>TM-007</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B100" s="9" t="str">
-        <x:v>E2E-TM007-004</x:v>
+        <x:v>TC-TM004-INCREMENTAL-02</x:v>
       </x:c>
       <x:c r="C100" s="9" t="str">
-        <x:v>统计越权与停用后上传</x:v>
+        <x:v>重复与事务恢复（TASK-TM004-INCREMENTAL，AC-002/004，E2E-002/004）</x:v>
       </x:c>
       <x:c r="D100" s="9" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-INCREMENTAL</x:v>
       </x:c>
       <x:c r="E100" s="9" t="str">
         <x:v>产品E2E</x:v>
       </x:c>
       <x:c r="F100" s="9" t="str">
-        <x:v>数据集 sync_faults；alice项目A调用100/10，bob项目B调用200/20；成员alice与管理员独立会话；alice另有一条未确认调用C=50/5。sync_faults与可重建统计SQL尚未实现。</x:v>
+        <x:v>完整M100/10、重复相同片段及移动/复制文件；在扫描提交边界中断App。</x:v>
       </x:c>
       <x:c r="G100" s="9" t="str">
-        <x:v>成员无权请求被服务端拒绝，UI不显示bob的220；停用后旧会话及上传拒绝，C不能标为已确认；合法历史不能被失败上传删除。此处补足TM-001仅身份/管理接口权限的范围。</x:v>
+        <x:v>M仅入账一次且total110
+仍110
+仍唯一M/110
+total165</x:v>
       </x:c>
       <x:c r="H100" s="9" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：只读唯一键数2/165且游标一致；故障注入不得绕过产品事务。TM-003事务接口待补；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I100" s="9" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J100" s="9" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K100" s="9" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L100" s="9" t="str">
-        <x:v>docs/testing/cases/07-TM-007-team-sync.md:62</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:115</x:v>
       </x:c>
       <x:c r="M100" s="9" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
-    <x:row r="101" ht="57" customHeight="1">
+    <x:row r="101" ht="87" customHeight="1">
       <x:c r="A101" s="4" t="str">
-        <x:v>TM-008</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B101" s="4" t="str">
-        <x:v>E2E-TM008-001</x:v>
+        <x:v>TC-TM004-DIAG-01</x:v>
       </x:c>
       <x:c r="C101" s="4" t="str">
-        <x:v>筛选一致的CSV导出</x:v>
+        <x:v>未知值不是零（TASK-TM004-DIAGNOSTIC，AC-003，E2E-003）</x:v>
       </x:c>
       <x:c r="D101" s="4" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-DIAGNOSTIC</x:v>
       </x:c>
       <x:c r="E101" s="4" t="str">
         <x:v>产品E2E</x:v>
       </x:c>
       <x:c r="F101" s="4" t="str">
-        <x:v>数据集 export_rows；export_rows planned；两成员、两个模型、时间范围内外各有事件，独立清单明确每条ID/字段/权限。先具备TM-005/007统计和授权。</x:v>
+        <x:v>可信M100/10、U未知格式、Q的JSONL原始行缺usage，以及另有独立来源证明的有效零usage记录Z。</x:v>
       </x:c>
       <x:c r="G101" s="4" t="str">
-        <x:v>每次CSV仅包含当次筛选且授权可见记录，行数/ID/汇总等于独立清单与界面；不混入旧筛选、其他成员或范围外记录。已知/未知费用语义一致。</x:v>
+        <x:v>显示110
+显示可信110和两个不同未覆盖提示
+零值记录可见但总量仍110
+三种状态不混淆</x:v>
       </x:c>
       <x:c r="H101" s="4" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：只读可信M和已证实的Z，U/Q仅诊断，不以0写入；Z的原始有效性仍 baseline_pending。2.1.126 遇到畸形合成 API 缺usage会自己写0/0，不能拿该行充当Z；未经额外证据不能由0/0 raw推断上游已知零；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I101" s="4" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J101" s="4" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K101" s="4" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L101" s="4" t="str">
-        <x:v>docs/testing/cases/08-TM-008-csv-export.md:11</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:119</x:v>
       </x:c>
       <x:c r="M101" s="4" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
-    <x:row r="102" ht="57" customHeight="1">
+    <x:row r="102" ht="72" customHeight="1">
       <x:c r="A102" s="9" t="str">
-        <x:v>TM-008</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B102" s="9" t="str">
-        <x:v>E2E-TM008-002</x:v>
+        <x:v>TC-TM004-DIAG-02</x:v>
       </x:c>
       <x:c r="C102" s="9" t="str">
-        <x:v>CSV转义、未知值及权限</x:v>
+        <x:v>失权提示及隐私（TASK-TM004-DIAGNOSTIC，AC-004，E2E-004）</x:v>
       </x:c>
       <x:c r="D102" s="9" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-DIAGNOSTIC</x:v>
       </x:c>
       <x:c r="E102" s="9" t="str">
         <x:v>产品E2E</x:v>
       </x:c>
       <x:c r="F102" s="9" t="str">
-        <x:v>数据集 export_rows；export_rows需含字段 a,b、say "hi"、带实际换行的项目名、未知费用与非ASCII模型名；两成员各有可区分哨兵事件。只在隔离数据中使用。</x:v>
+        <x:v>M已入账，撤权目录含合成 prompt、代码和密钥哨兵字符串。</x:v>
       </x:c>
       <x:c r="G102" s="9" t="str">
-        <x:v>逗号、双引号、嵌入换行均round-trip一致，Unicode不损坏；未知值不写成0；他人哨兵不出现在文件。若导出失败，不能留下看似完整的半文件。</x:v>
+        <x:v>UI显示读取受阻而非零用量，保留110
+无哨兵文本及完整源路径
+受阻提示消除且M不重计</x:v>
       </x:c>
       <x:c r="H102" s="9" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：只读事件1/110、诊断状态与仅白名单字段；隐私哨兵由固定生成器构造，不使用真实秘密；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I102" s="9" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J102" s="9" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K102" s="9" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L102" s="9" t="str">
-        <x:v>docs/testing/cases/08-TM-008-csv-export.md:28</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:123</x:v>
       </x:c>
       <x:c r="M102" s="9" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
-    <x:row r="103" ht="57" customHeight="1">
+    <x:row r="103" ht="72" customHeight="1">
       <x:c r="A103" s="4" t="str">
-        <x:v>TM-009</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B103" s="4" t="str">
-        <x:v>E2E-TM009-001</x:v>
+        <x:v>TC-TM004-DATA-01</x:v>
       </x:c>
       <x:c r="C103" s="4" t="str">
-        <x:v>80%/100%提醒幂等</x:v>
+        <x:v>原始fixture和独立oracle（TASK-TM004-DATA，AC-001–004，E2E-003）</x:v>
       </x:c>
       <x:c r="D103" s="4" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-DATA</x:v>
       </x:c>
       <x:c r="E103" s="4" t="str">
-        <x:v>产品E2E</x:v>
+        <x:v>data_fixture</x:v>
       </x:c>
       <x:c r="F103" s="4" t="str">
-        <x:v>数据集 budget_periods；budget_periods planned；独立个人、项目和团队预算分别100个合成USD单位，同周期使用量依次79→80→99→100；原始调用与价格要能精确形成这些费用。</x:v>
+        <x:v>固定版本 CLI/公开来源、隔离 CLAUDE_CONFIG_DIR、固定合成任务；禁止访问真实 ~/.claude。</x:v>
       </x:c>
       <x:c r="G103" s="4" t="str">
-        <x:v>每预算每周期80与100各最多一次，未达到不发；重扫/重启/重复上传不重发；预算仅提醒，不拦截模型调用。三层预算分别按其授权范围计算。</x:v>
+        <x:v>版本、来源、原始SHA及父子/fork证据有原件
+M/S/N/P的330、165、187、385在运行前记录
+SHA一致且SQL初态只有合成账号与零事件
+仅删除本次拥有目录且保留原始报告</x:v>
       </x:c>
       <x:c r="H103" s="4" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：本例不直接写入产品用量表；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I103" s="4" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J103" s="4" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K103" s="4" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L103" s="4" t="str">
-        <x:v>docs/testing/cases/09-TM-009-budget-alerts.md:11</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:127</x:v>
       </x:c>
       <x:c r="M103" s="4" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
-    <x:row r="104" ht="57" customHeight="1">
+    <x:row r="104" ht="72" customHeight="1">
       <x:c r="A104" s="9" t="str">
-        <x:v>TM-009</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B104" s="9" t="str">
-        <x:v>E2E-TM009-002</x:v>
+        <x:v>TC-TM004-E2E-01</x:v>
       </x:c>
       <x:c r="C104" s="9" t="str">
-        <x:v>新周期、币种与通知恢复</x:v>
+        <x:v>安装包真实链路（TASK-TM004-E2E，AC-001–004，E2E-001/004）</x:v>
       </x:c>
       <x:c r="D104" s="9" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-E2E</x:v>
       </x:c>
       <x:c r="E104" s="9" t="str">
         <x:v>产品E2E</x:v>
       </x:c>
       <x:c r="F104" s="9" t="str">
-        <x:v>数据集 budget_periods；两个币种独立预算；旧周期已发80/100阈值，参考时钟可由产品支持的测试配置推进；测试通知权限可以拒绝及恢复，不能修改用户其他App授权。</x:v>
+        <x:v>本版固定候选SHA、原DMG、TM-001–004完整必测TC清单。</x:v>
       </x:c>
       <x:c r="G104" s="9" t="str">
-        <x:v>系统拒绝不丢失应用内状态、不造成重试通知风暴；新周期独立重置，允许新一轮各阈值一次；币种分开计算。通知补发策略需在对应需求明确，不能由测试临时猜测。</x:v>
+        <x:v>仅连接本次独占服务和隔离授权根
+逐步断言UI、IPC后果和只读SQLite
+目标及历史已交付TC全部执行且无跳过/重试/失败
+结果与候选包一致且本次资源清理完成</x:v>
       </x:c>
       <x:c r="H104" s="9" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：本例不直接写入产品用量表；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I104" s="9" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J104" s="9" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K104" s="9" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L104" s="9" t="str">
-        <x:v>docs/testing/cases/09-TM-009-budget-alerts.md:28</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:131</x:v>
       </x:c>
       <x:c r="M104" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -9969,343 +10306,366 @@
     </x:row>
     <x:row r="105" ht="72" customHeight="1">
       <x:c r="A105" s="4" t="str">
-        <x:v>TM-010</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B105" s="4" t="str">
-        <x:v>E2E-TM010-001</x:v>
+        <x:v>TC-TM004-RELEASE-01</x:v>
       </x:c>
       <x:c r="C105" s="4" t="str">
-        <x:v>稳定版发现更新与数据保留</x:v>
+        <x:v>候选与证据一致（TASK-TM004-RELEASE，AC-001–004，E2E-004）</x:v>
       </x:c>
       <x:c r="D105" s="4" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-RELEASE</x:v>
       </x:c>
       <x:c r="E105" s="4" t="str">
-        <x:v>产品E2E</x:v>
+        <x:v>release_gate</x:v>
       </x:c>
       <x:c r="F105" s="4" t="str">
-        <x:v>数据集 update_packages；依赖TM-001/007；update_packages planned。需真实已分发稳定版、候选最终包及相同分发profile的签名/清单；旧版有账号设置、手动地址、统计/队列独立快照。首版无历史稳定版时使用SOP017规定的候选→受控高版，不伪称稳定升级。</x:v>
+        <x:v>同一已提交SHA/tree、DMG摘要、完整TM-001–004结果。</x:v>
       </x:c>
       <x:c r="G105" s="4" t="str">
-        <x:v>更新频率和说明可用；只有声明候选被安装，Sparkle自主重启；更新前后账号/设置/统计与快照一致，队列不丢失不重复。完整更新体验仍为未来功能，TM-001-004通过只证明最小更新路径。</x:v>
+        <x:v>SHA/tree和DMG摘要一致
+完整集合逐例PASS且清理完成，否则阻断
+Excel行和源摘要一致
+SOP-018真实PASS才进入SOP-019</x:v>
       </x:c>
       <x:c r="H105" s="4" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：本例不直接写入产品用量表；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I105" s="4" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J105" s="4" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K105" s="4" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L105" s="4" t="str">
-        <x:v>docs/testing/cases/10-TM-010-software-updates.md:11</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:135</x:v>
       </x:c>
       <x:c r="M105" s="4" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
-    <x:row r="106" ht="57" customHeight="1">
+    <x:row r="106" ht="72" customHeight="1">
       <x:c r="A106" s="9" t="str">
-        <x:v>TM-010</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B106" s="9" t="str">
-        <x:v>E2E-TM010-002</x:v>
+        <x:v>TC-TM004-SOURCE-03</x:v>
       </x:c>
       <x:c r="C106" s="9" t="str">
-        <x:v>签名、网络、空间和迁移失败恢复</x:v>
+        <x:v>嵌套子代理目录（TASK-TM004-SOURCE，AC-001，E2E-001）</x:v>
       </x:c>
       <x:c r="D106" s="9" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-SOURCE</x:v>
       </x:c>
       <x:c r="E106" s="9" t="str">
         <x:v>产品E2E</x:v>
       </x:c>
       <x:c r="F106" s="9" t="str">
-        <x:v>数据集 update_packages；对同一干净旧版分别建立四个隔离子场景：坏签名包、下载中断、受限测试卷空间不足、受控迁移失败；每个保存旧版包/DB/配置摘要。故障不能作用用户系统盘/生产库。</x:v>
+        <x:v>2.1.126 已安装二进制显示子代理路径可在 subagents/ 下继续嵌套；确切层级与父链由待取得的原始样本决定。固定数据应含项目A主M100/10、一级子S200/20、嵌套子T=50/5，以及授权根外同名文件X=999/99。</x:v>
       </x:c>
       <x:c r="G106" s="9" t="str">
-        <x:v>每个失败均不能形成半更新；原账号/统计和包的可用状态可验证。网络恢复后的成功需要完整包校验；迁移失败恢复来源与摘要明确。四个子场景全部为本case必需，不能挑一项通过。</x:v>
+        <x:v>项目A可信total385/3次调用
+不读取X
+总量和归属不变
+不猜A</x:v>
       </x:c>
       <x:c r="H106" s="9" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：只读事件唯一键、父项目与总量3/385；缺链变体的T不得纳入A可信聚合；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I106" s="9" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J106" s="9" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K106" s="9" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L106" s="9" t="str">
-        <x:v>docs/testing/cases/10-TM-010-software-updates.md:28</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:139</x:v>
       </x:c>
       <x:c r="M106" s="9" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
-    <x:row r="107" ht="57" customHeight="1">
+    <x:row r="107" ht="72" customHeight="1">
       <x:c r="A107" s="4" t="str">
-        <x:v>TM-010</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B107" s="4" t="str">
-        <x:v>E2E-TM010-003</x:v>
+        <x:v>TC-TM004-PARSER-03</x:v>
       </x:c>
       <x:c r="C107" s="4" t="str">
-        <x:v>升级默认地址和手动覆盖</x:v>
+        <x:v>同一消息多内容块和 Agent 摘要（TASK-TM004-PARSER，AC-001，E2E-001）</x:v>
       </x:c>
       <x:c r="D107" s="4" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-PARSER</x:v>
       </x:c>
       <x:c r="E107" s="4" t="str">
         <x:v>产品E2E</x:v>
       </x:c>
       <x:c r="F107" s="4" t="str">
-        <x:v>数据集 server_default_migration；server_default_migration planned；两套旧安装A从未设置地址、B已手动设置；候选内置一个届时确定且测试可访问的生产HTTPS默认地址。两源有独立账号/数据/会话，公钥不可随URL编辑。</x:v>
+        <x:v>同一次主调用M100/10拆为至少两个带相同 message.id 与 usage 的 assistant 内容块，另有 Agent 工具结果的 totalTokens/usage 摘要与子S200/20原始调用；本机独立结构探针已实际生成31/9双块，CLI 写两行相同 ID 和完整 usage，子代理19/6的父工具结果出现 total_tokens: 25。</x:v>
       </x:c>
       <x:c r="G107" s="4" t="str">
-        <x:v>只有无手动覆盖安装跟随新版默认；显式覆盖即使恰好等于旧默认也应按已经确定的配置来源规则处理。改变origin需重新服务认证，旧token不能跨源复用。</x:v>
+        <x:v>UI/SQLite为1次调用、total110
+可信为M+S两次、total330
+仍330</x:v>
       </x:c>
       <x:c r="H107" s="4" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：只读源消息调用键2个/330，父Agent汇总不能额外成为第三次调用；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I107" s="4" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J107" s="4" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K107" s="4" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L107" s="4" t="str">
-        <x:v>docs/testing/cases/10-TM-010-software-updates.md:45</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:143</x:v>
       </x:c>
       <x:c r="M107" s="4" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
-    <x:row r="108" ht="57" customHeight="1">
+    <x:row r="108" ht="72" customHeight="1">
       <x:c r="A108" s="9" t="str">
-        <x:v>TM-011</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B108" s="9" t="str">
-        <x:v>E2E-TM011-001</x:v>
+        <x:v>TC-TM004-LINEAGE-03</x:v>
       </x:c>
       <x:c r="C108" s="9" t="str">
-        <x:v>SQLite迁移与中断恢复</x:v>
+        <x:v>forkedFrom 复制与改写 UUID（TASK-TM004-LINEAGE，AC-002，E2E-002）</x:v>
       </x:c>
       <x:c r="D108" s="9" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-LINEAGE</x:v>
       </x:c>
       <x:c r="E108" s="9" t="str">
         <x:v>产品E2E</x:v>
       </x:c>
       <x:c r="F108" s="9" t="str">
-        <x:v>数据集 migration_snapshots；migration_snapshots planned；旧schema副本含固定账号/事件/队列、预计算记录数/Token/金额；候选迁移版本和明确故障点。全部作用私有临时库。</x:v>
+        <x:v>已计M100/10；分别用2.1.126真实生成的 fork 复制记录（保留 UUID）和改写 UUID 记录，依据实际 raw 的跨文件调用身份/父链判定，不能假定两者都含 forkedFrom；再追加真正新N50/5。</x:v>
       </x:c>
       <x:c r="G108" s="9" t="str">
-        <x:v>成功迁移只改变设计允许的schema/数据；账号、记录数、Token、费用/队列归属不丢。失败恢复到可启动一致状态，重复启动不重复迁移数据。不能以文件存在作为恢复成功。</x:v>
+        <x:v>M仅计一次且total110
+均仍110并在诊断/关系中可追溯原M
+total165/2次
+仍两次可信调用且total165</x:v>
       </x:c>
       <x:c r="H108" s="9" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：只读可信调用键2个、继承引用指向M；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I108" s="9" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J108" s="9" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K108" s="9" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L108" s="9" t="str">
-        <x:v>docs/testing/cases/11-TM-011-data-migration.md:11</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:147</x:v>
       </x:c>
       <x:c r="M108" s="9" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
-    <x:row r="109" ht="57" customHeight="1">
+    <x:row r="109" ht="72" customHeight="1">
       <x:c r="A109" s="4" t="str">
-        <x:v>TM-011</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B109" s="4" t="str">
-        <x:v>E2E-TM011-002</x:v>
+        <x:v>TC-TM004-LINEAGE-04</x:v>
       </x:c>
       <x:c r="C109" s="4" t="str">
-        <x:v>未来SQLite到MySQL迁移</x:v>
+        <x:v>fork-context-ref 父链（TASK-TM004-LINEAGE，AC-002，E2E-002）</x:v>
       </x:c>
       <x:c r="D109" s="4" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-LINEAGE</x:v>
       </x:c>
       <x:c r="E109" s="4" t="str">
         <x:v>产品E2E</x:v>
       </x:c>
       <x:c r="F109" s="4" t="str">
-        <x:v>数据集 migration_snapshots；仅后续独立版本适用；用户已确定v0.1.0继续SQLite。需要隔离源SQLite、目标MySQL、固定多成员/多项目用量快照、字符/时间/Decimal边界和独立expected。</x:v>
+        <x:v>2.1.126真实子代理 fork 记录中带 agentId,parentSessionId,parentLastUuid,contextLength；父会话存在M100/10，子代理仅新增S200/20。</x:v>
       </x:c>
       <x:c r="G109" s="4" t="str">
-        <x:v>源/目标记录数、Token、Decimal金额及权限结果一致，ID和幂等语义保持；不重复历史且旧源未被破坏。MySQL版本、字符集和迁移范围须在对应版本指定。</x:v>
+        <x:v>可信110
+可信330/2次而非440
+可信M/S两次且total330
+引用解析到M的既有调用键</x:v>
       </x:c>
       <x:c r="H109" s="4" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：只读M/S各一条及引用，total330；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I109" s="4" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J109" s="4" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K109" s="4" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L109" s="4" t="str">
-        <x:v>docs/testing/cases/11-TM-011-data-migration.md:28</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:151</x:v>
       </x:c>
       <x:c r="M109" s="4" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
-    <x:row r="110" ht="57" customHeight="1">
+    <x:row r="110" ht="72" customHeight="1">
       <x:c r="A110" s="9" t="str">
-        <x:v>TM-011</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B110" s="9" t="str">
-        <x:v>E2E-TM011-003</x:v>
+        <x:v>TC-TM004-LINEAGE-05</x:v>
       </x:c>
       <x:c r="C110" s="9" t="str">
-        <x:v>备份恢复与旧客户端补传</x:v>
+        <x:v>缺失或矛盾父链（TASK-TM004-LINEAGE，AC-002/003，E2E-002/003）</x:v>
       </x:c>
       <x:c r="D110" s="9" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-LINEAGE</x:v>
       </x:c>
       <x:c r="E110" s="9" t="str">
         <x:v>产品E2E</x:v>
       </x:c>
       <x:c r="F110" s="9" t="str">
-        <x:v>数据集 migration_snapshots；隔离服务已确认事件A/B与旧客户端未确认C；备份包含schema/数据/版本/摘要，另保存不在备份里的独立oracle。恢复目标必须为空且带测试标记。</x:v>
+        <x:v>在上一例的合成同构目录中分别移除引用父文件、指向不存在的 parentLastUuid、或提供无 forkedFrom 但UUID改写的复制历史；这些是测试故障注入，不能标为厂商实际输出。</x:v>
       </x:c>
       <x:c r="G110" s="9" t="str">
-        <x:v>备份能实际恢复而非只压缩成功；A/B不丢，重复补传不增加；C最终只出现一次，账号/权限符合恢复基线。队列与服务确认一致，旧客户端协议兼容。</x:v>
+        <x:v>M仅计一次且total110
+App显示未确定来源诊断，可信总量仍110、不能把不明副本计为新调用或有效零
+若真实新增S200/20可独立识别则总量330
+可信总量保持且诊断随恢复更新</x:v>
       </x:c>
       <x:c r="H110" s="9" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：只读未确定记录与可信M/S计数，不能借SQL灌成功；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I110" s="9" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J110" s="9" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K110" s="9" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L110" s="9" t="str">
-        <x:v>docs/testing/cases/11-TM-011-data-migration.md:45</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:155</x:v>
       </x:c>
       <x:c r="M110" s="9" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
-    <x:row r="111" ht="57" customHeight="1">
+    <x:row r="111" ht="102" customHeight="1">
       <x:c r="A111" s="4" t="str">
-        <x:v>TM-011</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B111" s="4" t="str">
-        <x:v>E2E-TM011-004</x:v>
+        <x:v>TC-TM004-SOURCE-04</x:v>
       </x:c>
       <x:c r="C111" s="4" t="str">
-        <x:v>保留时间边界与未同步保护</x:v>
+        <x:v>预览截断后的可续扫覆盖（TASK-TM004-SOURCE，AC-001/004，E2E-001/004）</x:v>
       </x:c>
       <x:c r="D111" s="4" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-SOURCE</x:v>
       </x:c>
       <x:c r="E111" s="4" t="str">
         <x:v>产品E2E</x:v>
       </x:c>
       <x:c r="F111" s="4" t="str">
-        <x:v>数据集 migration_snapshots；固定参考时间和Asia/Shanghai；本地90天/服务端365天。分别生成保留首日00:00、前一秒、前一天的已确认事件，以及同样超龄但未同步事件；具备可控时钟与独立边界oracle。</x:v>
+        <x:v>本例独占授权根，固定程序按 TM-002 已提交枚举顺序生成至少1025个普通 .jsonl 文件及足够目录项；前段有主M100/10，预览截断范围外且至少第五个256项采集页的深层 subagents/ 文件有子S50/5，其余文件没有可计量调用。另备可控制的页间撤权/恢复点。</x:v>
       </x:c>
       <x:c r="G111" s="4" t="str">
-        <x:v>保留首日00:00仍在，早一秒的已同步记录被清理；本地/服务按各自天数独立判定。未同步记录即使超龄仍保护，成功补传仅计一次；历史缺失不能显示真实0。</x:v>
+        <x:v>1000文件预览显示被截断，不声称全量
+UI 可显示已见M110，但 TM-003 coverage.scan_incomplete=1
+使用 openCandidateReadOnly(candidateToken) 读原始行；在另一次固定变体于页间撤权，下一页或打开须拒绝，cancelScan 后 scan_incomplete=1，重授后以新授权世代续扫
+可信 M+S 两调用、input150/output15/total165，scan_incomplete=0 才可显示本次覆盖完成；重启重扫总量不变</x:v>
       </x:c>
       <x:c r="H111" s="4" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：只读各来源事件键、聚合 (2,150,15)、游标及 coverage.scan_incomplete；中途必须为1；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I111" s="4" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J111" s="4" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K111" s="4" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L111" s="4" t="str">
-        <x:v>docs/testing/cases/11-TM-011-data-migration.md:62</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:159</x:v>
       </x:c>
       <x:c r="M111" s="4" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
-    <x:row r="112" ht="57" customHeight="1">
+    <x:row r="112" ht="102" customHeight="1">
       <x:c r="A112" s="9" t="str">
-        <x:v>TM-012</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B112" s="9" t="str">
-        <x:v>E2E-TM012-001</x:v>
+        <x:v>TC-TM004-INCREMENTAL-03</x:v>
       </x:c>
       <x:c r="C112" s="9" t="str">
-        <x:v>菜单栏摘要、暂停恢复与刷新</x:v>
+        <x:v>跨工具同 ID 与 Claude 复制历史（TASK-TM004-INCREMENTAL，AC-001/002，E2E-001/002）</x:v>
       </x:c>
       <x:c r="D112" s="9" t="str">
-        <x:v>待拆解</x:v>
+        <x:v>TASK-TM004-INCREMENTAL</x:v>
       </x:c>
       <x:c r="E112" s="9" t="str">
         <x:v>产品E2E</x:v>
       </x:c>
       <x:c r="F112" s="9" t="str">
-        <x:v>数据集 diagnostic_states；diagnostic_states planned；已采集A=100/10；暂停期间追加B=200/20并重放A。依赖实际采集、统计和同步功能，使用专用日志目录。</x:v>
+        <x:v>同一合成主体、各自经 UI 授权的 Codex 与 Claude 隔离根。固定本地响应使 Codex 原生 payload.response_id 与 Claude 主 assistant.message.id 字面均为 shared-call-01，分别有 C=11/1 与 M=100/10；Claude 原生 --fork-session 复制M，再有独立 Agent 子调用S=200/20（新 message.id、与父同 sessionId 但带 agentId）。另以明确标记的衍生故障数据令同一 Claude message.id 出现矛盾101/10，该行不冒称 CLI 原件。</x:v>
       </x:c>
       <x:c r="G112" s="9" t="str">
-        <x:v>初始total110、暂停期间仍110，恢复后唯一A/B、total330；手动刷新与重启不重复。菜单栏与主窗口同一筛选口径；暂停状态不伪装成没有日志。</x:v>
+        <x:v>可信1次/total12
+可信2次/input111/output11/total122，跨工具同字面 ID 不冲突
+可信3次/input311/output31/total342
+可信仍3次/342，出现 identity_conflict 与覆盖不完整</x:v>
       </x:c>
       <x:c r="H112" s="9" t="str">
-        <x:v>准备：待该功能的数据程序/SQL方案确定。
-变化：待具体任务及数据设计细化。
-核验：暂无可执行数据库核验绑定。</x:v>
+        <x:v>准备：按SOP-010新建隔离账号与SQLite；不得SQL直灌规范化成功事件
+变化：仅由真实App读取受控原始日志后按步骤产生事件或诊断；当前未执行
+核验：规划只读核对：只读同一 principal_key 下 source=codex 与 source=claude_code 各自事件数1/2、source_event_key 不同，Agent source_scope_key 与主来源可区分，复制M不多行，冲突不覆写原M；键与归属均不得存原生ID/完整路径；确切可执行SQL待TM-003稳定schema</x:v>
       </x:c>
       <x:c r="I112" s="9" t="str">
-        <x:v>未来规划</x:v>
+        <x:v>预期待明确</x:v>
       </x:c>
       <x:c r="J112" s="9" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K112" s="9" t="str">
-        <x:v>未来概要</x:v>
+        <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L112" s="9" t="str">
-        <x:v>docs/testing/cases/12-TM-012-menu-diagnostics.md:11</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:163</x:v>
       </x:c>
       <x:c r="M112" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -10313,13 +10673,13 @@
     </x:row>
     <x:row r="113" ht="57" customHeight="1">
       <x:c r="A113" s="4" t="str">
-        <x:v>TM-012</x:v>
+        <x:v>TM-005</x:v>
       </x:c>
       <x:c r="B113" s="4" t="str">
-        <x:v>E2E-TM012-002</x:v>
+        <x:v>E2E-TM005-001</x:v>
       </x:c>
       <x:c r="C113" s="4" t="str">
-        <x:v>诊断状态、恢复和登录启动</x:v>
+        <x:v>日期筛选、趋势和明细</x:v>
       </x:c>
       <x:c r="D113" s="4" t="str">
         <x:v>待拆解</x:v>
@@ -10328,10 +10688,10 @@
         <x:v>产品E2E</x:v>
       </x:c>
       <x:c r="F113" s="4" t="str">
-        <x:v>数据集 diagnostic_states；独立子场景：已授权目录失效、真实服务不可达/恢复、测试App登录启动开关。故障作用测试目录/进程；使用已登录桌面与可自动检查的系统设置。</x:v>
+        <x:v>数据集 date_ranges；date_ranges 已由 scripts/test_data.py 提供标准化语义样例，固定2026-09-29T04:00:00Z、Asia/Shanghai、seed42；13行含1重复、12唯一。需另有已验证raw输入映射和真实App导入流程，当前未实现。</x:v>
       </x:c>
       <x:c r="G113" s="4" t="str">
-        <x:v>错误与真实目录/网络故障一致，不能用旧缓存一直显示健康；恢复后状态及时更新，未同步数据不丢。启动设置与OS登记/实际启动行为一致，测试结束恢复本次测试前状态。</x:v>
+        <x:v>独立expected中的total依次16500、110、17380、27830、31130；custom=2200。today共5条、input15000、output1500、cache1700、reasoning170，cache/reasoning不再相加；custom-start包含、custom-end排除。趋势点及明细按expected事件时间逐条核对。</x:v>
       </x:c>
       <x:c r="H113" s="4" t="str">
         <x:v>准备：待该功能的数据程序/SQL方案确定。
@@ -10348,36 +10708,896 @@
         <x:v>未来概要</x:v>
       </x:c>
       <x:c r="L113" s="4" t="str">
-        <x:v>docs/testing/cases/12-TM-012-menu-diagnostics.md:28</x:v>
+        <x:v>docs/testing/cases/05-TM-005-usage-statistics.md:15</x:v>
       </x:c>
       <x:c r="M113" s="4" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
     </x:row>
+    <x:row r="114" ht="57" customHeight="1">
+      <x:c r="A114" s="9" t="str">
+        <x:v>TM-005</x:v>
+      </x:c>
+      <x:c r="B114" s="9" t="str">
+        <x:v>E2E-TM005-002</x:v>
+      </x:c>
+      <x:c r="C114" s="9" t="str">
+        <x:v>时区、月边界与缺失值</x:v>
+      </x:c>
+      <x:c r="D114" s="9" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E114" s="9" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F114" s="9" t="str">
+        <x:v>数据集 date_ranges；复用date_ranges中的2026-09-28T15:59:59Z与16:00:00Z、2026-08-30T15:59:59Z与16:00:00Z边界。另需补充覆盖缺口、已覆盖零调用日、unknown字段三类状态；当前生成器未覆盖后面三类。</x:v>
+      </x:c>
+      <x:c r="G114" s="9" t="str">
+        <x:v>Shanghai下15:59:59Z仍属前日、16:00:00Z属次日；UTC下二者同属UTC日期。无覆盖显示缺失，真实零可显示0，unknown字段显示未知；不得互相代替。各范围expected须独立按当地日期边界列出，不调用产品查询生成。</x:v>
+      </x:c>
+      <x:c r="H114" s="9" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I114" s="9" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J114" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K114" s="9" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L114" s="9" t="str">
+        <x:v>docs/testing/cases/05-TM-005-usage-statistics.md:32</x:v>
+      </x:c>
+      <x:c r="M114" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="57" customHeight="1">
+      <x:c r="A115" s="4" t="str">
+        <x:v>TM-006</x:v>
+      </x:c>
+      <x:c r="B115" s="4" t="str">
+        <x:v>E2E-TM006-001</x:v>
+      </x:c>
+      <x:c r="C115" s="4" t="str">
+        <x:v>Token子项与基础费用</x:v>
+      </x:c>
+      <x:c r="D115" s="4" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E115" s="4" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F115" s="4" t="str">
+        <x:v>数据集 pricing；pricing由scripts/test_data.py生成合成非计费价格。gpt-5每百万input/cache/output为USD2/0.2/8；today-gpt input1000含cache200、output100含reasoning20。价格不是厂商现价。</x:v>
+      </x:c>
+      <x:c r="G115" s="4" t="str">
+        <x:v>单调用total=1100；费用=(800×2+200×0.2+100×8)/1000000=USD0.002440，reasoning20不另加价。today已知费用USD0.015190且有1条无价格，alice今日USD0.010090。使用Decimal/十进制独立oracle，不以界面舍入反推底层精度。</x:v>
+      </x:c>
+      <x:c r="H115" s="4" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I115" s="4" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J115" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K115" s="4" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L115" s="4" t="str">
+        <x:v>docs/testing/cases/06-TM-006-cost-estimates.md:15</x:v>
+      </x:c>
+      <x:c r="M115" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="57" customHeight="1">
+      <x:c r="A116" s="9" t="str">
+        <x:v>TM-006</x:v>
+      </x:c>
+      <x:c r="B116" s="9" t="str">
+        <x:v>E2E-TM006-002</x:v>
+      </x:c>
+      <x:c r="C116" s="9" t="str">
+        <x:v>历史价格、多币种和未知费用</x:v>
+      </x:c>
+      <x:c r="D116" s="9" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E116" s="9" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F116" s="9" t="str">
+        <x:v>数据集 pricing_extended；pricing_extended planned：同模型在生效时点T前后各一调用，两个独立价格版本；另有USD/CNY各一模型、无价模型和订阅估算模型。必须提供价格/订阅分摊规则及手算expected后才能实现。</x:v>
+      </x:c>
+      <x:c r="G116" s="9" t="str">
+        <x:v>T前后依各自生效版本计算，历史结果不会悄悄换价；USD与CNY分组，未约定汇率不得相加；无价格显示未知而非0；订阅必须明确估算口径。具体金额oracle依待定义订阅/价格合同生成，当前不得手填PASS。</x:v>
+      </x:c>
+      <x:c r="H116" s="9" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I116" s="9" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J116" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K116" s="9" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L116" s="9" t="str">
+        <x:v>docs/testing/cases/06-TM-006-cost-estimates.md:32</x:v>
+      </x:c>
+      <x:c r="M116" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="57" customHeight="1">
+      <x:c r="A117" s="4" t="str">
+        <x:v>TM-007</x:v>
+      </x:c>
+      <x:c r="B117" s="4" t="str">
+        <x:v>E2E-TM007-001</x:v>
+      </x:c>
+      <x:c r="C117" s="4" t="str">
+        <x:v>离线、重启和补传幂等</x:v>
+      </x:c>
+      <x:c r="D117" s="4" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E117" s="4" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F117" s="4" t="str">
+        <x:v>数据集 sync_faults；sync_faults planned；alice两个隔离设备A/B，设备A调用100/10、B调用200/20；真实FastAPI/SQLite服务，可由外部fixture断网/恢复。账号继续用隔离测试fixture。</x:v>
+      </x:c>
+      <x:c r="G117" s="4" t="str">
+        <x:v>离线重启不丢队列；恢复后2唯一调用、input300/output30/total330；重复批次不再加量。客户端只在真实确认后标已同步，个人合计与对应团队子集一致。</x:v>
+      </x:c>
+      <x:c r="H117" s="4" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I117" s="4" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J117" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K117" s="4" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L117" s="4" t="str">
+        <x:v>docs/testing/cases/07-TM-007-team-sync.md:11</x:v>
+      </x:c>
+      <x:c r="M117" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="57" customHeight="1">
+      <x:c r="A118" s="9" t="str">
+        <x:v>TM-007</x:v>
+      </x:c>
+      <x:c r="B118" s="9" t="str">
+        <x:v>E2E-TM007-002</x:v>
+      </x:c>
+      <x:c r="C118" s="9" t="str">
+        <x:v>部分确认、中断和账号切换</x:v>
+      </x:c>
+      <x:c r="D118" s="9" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E118" s="9" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F118" s="9" t="str">
+        <x:v>数据集 sync_faults；准备alice的三条唯一事件A/B/C，总量各110/220/330；控制服务仅确认A后断开，B可能已提交但响应丢失，C未提交。另有bob账号。故障注入必须在真实服务外部或明确测试环境中完成，不能绕过认证。</x:v>
+      </x:c>
+      <x:c r="G118" s="9" t="str">
+        <x:v>最终alice的A/B/C各一次、total660；响应丢失不造成B重复；bob不能承接或篡改alice既有事件归属。切换时旧队列按已批准归属策略隔离，不能默认为新登录账号。</x:v>
+      </x:c>
+      <x:c r="H118" s="9" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I118" s="9" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J118" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K118" s="9" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L118" s="9" t="str">
+        <x:v>docs/testing/cases/07-TM-007-team-sync.md:28</x:v>
+      </x:c>
+      <x:c r="M118" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="57" customHeight="1">
+      <x:c r="A119" s="4" t="str">
+        <x:v>TM-007</x:v>
+      </x:c>
+      <x:c r="B119" s="4" t="str">
+        <x:v>E2E-TM007-003</x:v>
+      </x:c>
+      <x:c r="C119" s="4" t="str">
+        <x:v>上传白名单与项目映射</x:v>
+      </x:c>
+      <x:c r="D119" s="4" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E119" s="4" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F119" s="4" t="str">
+        <x:v>数据集 sync_faults；合成日志包含唯一正文/代码/API-key/完整路径哨兵，以及合法用量/必要去重元数据；只用假值。准备已归属项目A和未归属事件B，待sync_faults生成。</x:v>
+      </x:c>
+      <x:c r="G119" s="4" t="str">
+        <x:v>网络载荷/持久服务数据均不得含正文、代码、key或完整本机路径；只有批准用量/去重字段。B可明确分配，分配不增加事件量、也不跨团队归属。</x:v>
+      </x:c>
+      <x:c r="H119" s="4" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I119" s="4" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J119" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K119" s="4" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L119" s="4" t="str">
+        <x:v>docs/testing/cases/07-TM-007-team-sync.md:45</x:v>
+      </x:c>
+      <x:c r="M119" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="57" customHeight="1">
+      <x:c r="A120" s="9" t="str">
+        <x:v>TM-007</x:v>
+      </x:c>
+      <x:c r="B120" s="9" t="str">
+        <x:v>E2E-TM007-004</x:v>
+      </x:c>
+      <x:c r="C120" s="9" t="str">
+        <x:v>统计越权与停用后上传</x:v>
+      </x:c>
+      <x:c r="D120" s="9" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E120" s="9" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F120" s="9" t="str">
+        <x:v>数据集 sync_faults；alice项目A调用100/10，bob项目B调用200/20；成员alice与管理员独立会话；alice另有一条未确认调用C=50/5。sync_faults与可重建统计SQL尚未实现。</x:v>
+      </x:c>
+      <x:c r="G120" s="9" t="str">
+        <x:v>成员无权请求被服务端拒绝，UI不显示bob的220；停用后旧会话及上传拒绝，C不能标为已确认；合法历史不能被失败上传删除。此处补足TM-001仅身份/管理接口权限的范围。</x:v>
+      </x:c>
+      <x:c r="H120" s="9" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I120" s="9" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J120" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K120" s="9" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L120" s="9" t="str">
+        <x:v>docs/testing/cases/07-TM-007-team-sync.md:62</x:v>
+      </x:c>
+      <x:c r="M120" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="57" customHeight="1">
+      <x:c r="A121" s="4" t="str">
+        <x:v>TM-008</x:v>
+      </x:c>
+      <x:c r="B121" s="4" t="str">
+        <x:v>E2E-TM008-001</x:v>
+      </x:c>
+      <x:c r="C121" s="4" t="str">
+        <x:v>筛选一致的CSV导出</x:v>
+      </x:c>
+      <x:c r="D121" s="4" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E121" s="4" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F121" s="4" t="str">
+        <x:v>数据集 export_rows；export_rows planned；两成员、两个模型、时间范围内外各有事件，独立清单明确每条ID/字段/权限。先具备TM-005/007统计和授权。</x:v>
+      </x:c>
+      <x:c r="G121" s="4" t="str">
+        <x:v>每次CSV仅包含当次筛选且授权可见记录，行数/ID/汇总等于独立清单与界面；不混入旧筛选、其他成员或范围外记录。已知/未知费用语义一致。</x:v>
+      </x:c>
+      <x:c r="H121" s="4" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I121" s="4" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J121" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K121" s="4" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L121" s="4" t="str">
+        <x:v>docs/testing/cases/08-TM-008-csv-export.md:11</x:v>
+      </x:c>
+      <x:c r="M121" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="57" customHeight="1">
+      <x:c r="A122" s="9" t="str">
+        <x:v>TM-008</x:v>
+      </x:c>
+      <x:c r="B122" s="9" t="str">
+        <x:v>E2E-TM008-002</x:v>
+      </x:c>
+      <x:c r="C122" s="9" t="str">
+        <x:v>CSV转义、未知值及权限</x:v>
+      </x:c>
+      <x:c r="D122" s="9" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E122" s="9" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F122" s="9" t="str">
+        <x:v>数据集 export_rows；export_rows需含字段 a,b、say "hi"、带实际换行的项目名、未知费用与非ASCII模型名；两成员各有可区分哨兵事件。只在隔离数据中使用。</x:v>
+      </x:c>
+      <x:c r="G122" s="9" t="str">
+        <x:v>逗号、双引号、嵌入换行均round-trip一致，Unicode不损坏；未知值不写成0；他人哨兵不出现在文件。若导出失败，不能留下看似完整的半文件。</x:v>
+      </x:c>
+      <x:c r="H122" s="9" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I122" s="9" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J122" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K122" s="9" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L122" s="9" t="str">
+        <x:v>docs/testing/cases/08-TM-008-csv-export.md:28</x:v>
+      </x:c>
+      <x:c r="M122" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="57" customHeight="1">
+      <x:c r="A123" s="4" t="str">
+        <x:v>TM-009</x:v>
+      </x:c>
+      <x:c r="B123" s="4" t="str">
+        <x:v>E2E-TM009-001</x:v>
+      </x:c>
+      <x:c r="C123" s="4" t="str">
+        <x:v>80%/100%提醒幂等</x:v>
+      </x:c>
+      <x:c r="D123" s="4" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E123" s="4" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F123" s="4" t="str">
+        <x:v>数据集 budget_periods；budget_periods planned；独立个人、项目和团队预算分别100个合成USD单位，同周期使用量依次79→80→99→100；原始调用与价格要能精确形成这些费用。</x:v>
+      </x:c>
+      <x:c r="G123" s="4" t="str">
+        <x:v>每预算每周期80与100各最多一次，未达到不发；重扫/重启/重复上传不重发；预算仅提醒，不拦截模型调用。三层预算分别按其授权范围计算。</x:v>
+      </x:c>
+      <x:c r="H123" s="4" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I123" s="4" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J123" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K123" s="4" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L123" s="4" t="str">
+        <x:v>docs/testing/cases/09-TM-009-budget-alerts.md:11</x:v>
+      </x:c>
+      <x:c r="M123" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="57" customHeight="1">
+      <x:c r="A124" s="9" t="str">
+        <x:v>TM-009</x:v>
+      </x:c>
+      <x:c r="B124" s="9" t="str">
+        <x:v>E2E-TM009-002</x:v>
+      </x:c>
+      <x:c r="C124" s="9" t="str">
+        <x:v>新周期、币种与通知恢复</x:v>
+      </x:c>
+      <x:c r="D124" s="9" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E124" s="9" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F124" s="9" t="str">
+        <x:v>数据集 budget_periods；两个币种独立预算；旧周期已发80/100阈值，参考时钟可由产品支持的测试配置推进；测试通知权限可以拒绝及恢复，不能修改用户其他App授权。</x:v>
+      </x:c>
+      <x:c r="G124" s="9" t="str">
+        <x:v>系统拒绝不丢失应用内状态、不造成重试通知风暴；新周期独立重置，允许新一轮各阈值一次；币种分开计算。通知补发策略需在对应需求明确，不能由测试临时猜测。</x:v>
+      </x:c>
+      <x:c r="H124" s="9" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I124" s="9" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J124" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K124" s="9" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L124" s="9" t="str">
+        <x:v>docs/testing/cases/09-TM-009-budget-alerts.md:28</x:v>
+      </x:c>
+      <x:c r="M124" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="72" customHeight="1">
+      <x:c r="A125" s="4" t="str">
+        <x:v>TM-010</x:v>
+      </x:c>
+      <x:c r="B125" s="4" t="str">
+        <x:v>E2E-TM010-001</x:v>
+      </x:c>
+      <x:c r="C125" s="4" t="str">
+        <x:v>稳定版发现更新与数据保留</x:v>
+      </x:c>
+      <x:c r="D125" s="4" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E125" s="4" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F125" s="4" t="str">
+        <x:v>数据集 update_packages；依赖TM-001/007；update_packages planned。需真实已分发稳定版、候选最终包及相同分发profile的签名/清单；旧版有账号设置、手动地址、统计/队列独立快照。首版无历史稳定版时使用SOP017规定的候选→受控高版，不伪称稳定升级。</x:v>
+      </x:c>
+      <x:c r="G125" s="4" t="str">
+        <x:v>更新频率和说明可用；只有声明候选被安装，Sparkle自主重启；更新前后账号/设置/统计与快照一致，队列不丢失不重复。完整更新体验仍为未来功能，TM-001-004通过只证明最小更新路径。</x:v>
+      </x:c>
+      <x:c r="H125" s="4" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I125" s="4" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J125" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K125" s="4" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L125" s="4" t="str">
+        <x:v>docs/testing/cases/10-TM-010-software-updates.md:11</x:v>
+      </x:c>
+      <x:c r="M125" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="57" customHeight="1">
+      <x:c r="A126" s="9" t="str">
+        <x:v>TM-010</x:v>
+      </x:c>
+      <x:c r="B126" s="9" t="str">
+        <x:v>E2E-TM010-002</x:v>
+      </x:c>
+      <x:c r="C126" s="9" t="str">
+        <x:v>签名、网络、空间和迁移失败恢复</x:v>
+      </x:c>
+      <x:c r="D126" s="9" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E126" s="9" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F126" s="9" t="str">
+        <x:v>数据集 update_packages；对同一干净旧版分别建立四个隔离子场景：坏签名包、下载中断、受限测试卷空间不足、受控迁移失败；每个保存旧版包/DB/配置摘要。故障不能作用用户系统盘/生产库。</x:v>
+      </x:c>
+      <x:c r="G126" s="9" t="str">
+        <x:v>每个失败均不能形成半更新；原账号/统计和包的可用状态可验证。网络恢复后的成功需要完整包校验；迁移失败恢复来源与摘要明确。四个子场景全部为本case必需，不能挑一项通过。</x:v>
+      </x:c>
+      <x:c r="H126" s="9" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I126" s="9" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J126" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K126" s="9" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L126" s="9" t="str">
+        <x:v>docs/testing/cases/10-TM-010-software-updates.md:28</x:v>
+      </x:c>
+      <x:c r="M126" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="57" customHeight="1">
+      <x:c r="A127" s="4" t="str">
+        <x:v>TM-010</x:v>
+      </x:c>
+      <x:c r="B127" s="4" t="str">
+        <x:v>E2E-TM010-003</x:v>
+      </x:c>
+      <x:c r="C127" s="4" t="str">
+        <x:v>升级默认地址和手动覆盖</x:v>
+      </x:c>
+      <x:c r="D127" s="4" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E127" s="4" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F127" s="4" t="str">
+        <x:v>数据集 server_default_migration；server_default_migration planned；两套旧安装A从未设置地址、B已手动设置；候选内置一个届时确定且测试可访问的生产HTTPS默认地址。两源有独立账号/数据/会话，公钥不可随URL编辑。</x:v>
+      </x:c>
+      <x:c r="G127" s="4" t="str">
+        <x:v>只有无手动覆盖安装跟随新版默认；显式覆盖即使恰好等于旧默认也应按已经确定的配置来源规则处理。改变origin需重新服务认证，旧token不能跨源复用。</x:v>
+      </x:c>
+      <x:c r="H127" s="4" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I127" s="4" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J127" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K127" s="4" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L127" s="4" t="str">
+        <x:v>docs/testing/cases/10-TM-010-software-updates.md:45</x:v>
+      </x:c>
+      <x:c r="M127" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128" ht="57" customHeight="1">
+      <x:c r="A128" s="9" t="str">
+        <x:v>TM-011</x:v>
+      </x:c>
+      <x:c r="B128" s="9" t="str">
+        <x:v>E2E-TM011-001</x:v>
+      </x:c>
+      <x:c r="C128" s="9" t="str">
+        <x:v>SQLite迁移与中断恢复</x:v>
+      </x:c>
+      <x:c r="D128" s="9" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E128" s="9" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F128" s="9" t="str">
+        <x:v>数据集 migration_snapshots；migration_snapshots planned；旧schema副本含固定账号/事件/队列、预计算记录数/Token/金额；候选迁移版本和明确故障点。全部作用私有临时库。</x:v>
+      </x:c>
+      <x:c r="G128" s="9" t="str">
+        <x:v>成功迁移只改变设计允许的schema/数据；账号、记录数、Token、费用/队列归属不丢。失败恢复到可启动一致状态，重复启动不重复迁移数据。不能以文件存在作为恢复成功。</x:v>
+      </x:c>
+      <x:c r="H128" s="9" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I128" s="9" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J128" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K128" s="9" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L128" s="9" t="str">
+        <x:v>docs/testing/cases/11-TM-011-data-migration.md:11</x:v>
+      </x:c>
+      <x:c r="M128" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="57" customHeight="1">
+      <x:c r="A129" s="4" t="str">
+        <x:v>TM-011</x:v>
+      </x:c>
+      <x:c r="B129" s="4" t="str">
+        <x:v>E2E-TM011-002</x:v>
+      </x:c>
+      <x:c r="C129" s="4" t="str">
+        <x:v>未来SQLite到MySQL迁移</x:v>
+      </x:c>
+      <x:c r="D129" s="4" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E129" s="4" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F129" s="4" t="str">
+        <x:v>数据集 migration_snapshots；仅后续独立版本适用；用户已确定v0.1.0继续SQLite。需要隔离源SQLite、目标MySQL、固定多成员/多项目用量快照、字符/时间/Decimal边界和独立expected。</x:v>
+      </x:c>
+      <x:c r="G129" s="4" t="str">
+        <x:v>源/目标记录数、Token、Decimal金额及权限结果一致，ID和幂等语义保持；不重复历史且旧源未被破坏。MySQL版本、字符集和迁移范围须在对应版本指定。</x:v>
+      </x:c>
+      <x:c r="H129" s="4" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I129" s="4" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J129" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K129" s="4" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L129" s="4" t="str">
+        <x:v>docs/testing/cases/11-TM-011-data-migration.md:28</x:v>
+      </x:c>
+      <x:c r="M129" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130" ht="57" customHeight="1">
+      <x:c r="A130" s="9" t="str">
+        <x:v>TM-011</x:v>
+      </x:c>
+      <x:c r="B130" s="9" t="str">
+        <x:v>E2E-TM011-003</x:v>
+      </x:c>
+      <x:c r="C130" s="9" t="str">
+        <x:v>备份恢复与旧客户端补传</x:v>
+      </x:c>
+      <x:c r="D130" s="9" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E130" s="9" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F130" s="9" t="str">
+        <x:v>数据集 migration_snapshots；隔离服务已确认事件A/B与旧客户端未确认C；备份包含schema/数据/版本/摘要，另保存不在备份里的独立oracle。恢复目标必须为空且带测试标记。</x:v>
+      </x:c>
+      <x:c r="G130" s="9" t="str">
+        <x:v>备份能实际恢复而非只压缩成功；A/B不丢，重复补传不增加；C最终只出现一次，账号/权限符合恢复基线。队列与服务确认一致，旧客户端协议兼容。</x:v>
+      </x:c>
+      <x:c r="H130" s="9" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I130" s="9" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J130" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K130" s="9" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L130" s="9" t="str">
+        <x:v>docs/testing/cases/11-TM-011-data-migration.md:45</x:v>
+      </x:c>
+      <x:c r="M130" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="57" customHeight="1">
+      <x:c r="A131" s="4" t="str">
+        <x:v>TM-011</x:v>
+      </x:c>
+      <x:c r="B131" s="4" t="str">
+        <x:v>E2E-TM011-004</x:v>
+      </x:c>
+      <x:c r="C131" s="4" t="str">
+        <x:v>保留时间边界与未同步保护</x:v>
+      </x:c>
+      <x:c r="D131" s="4" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E131" s="4" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F131" s="4" t="str">
+        <x:v>数据集 migration_snapshots；固定参考时间和Asia/Shanghai；本地90天/服务端365天。分别生成保留首日00:00、前一秒、前一天的已确认事件，以及同样超龄但未同步事件；具备可控时钟与独立边界oracle。</x:v>
+      </x:c>
+      <x:c r="G131" s="4" t="str">
+        <x:v>保留首日00:00仍在，早一秒的已同步记录被清理；本地/服务按各自天数独立判定。未同步记录即使超龄仍保护，成功补传仅计一次；历史缺失不能显示真实0。</x:v>
+      </x:c>
+      <x:c r="H131" s="4" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I131" s="4" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J131" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K131" s="4" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L131" s="4" t="str">
+        <x:v>docs/testing/cases/11-TM-011-data-migration.md:62</x:v>
+      </x:c>
+      <x:c r="M131" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132" ht="57" customHeight="1">
+      <x:c r="A132" s="9" t="str">
+        <x:v>TM-012</x:v>
+      </x:c>
+      <x:c r="B132" s="9" t="str">
+        <x:v>E2E-TM012-001</x:v>
+      </x:c>
+      <x:c r="C132" s="9" t="str">
+        <x:v>菜单栏摘要、暂停恢复与刷新</x:v>
+      </x:c>
+      <x:c r="D132" s="9" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E132" s="9" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F132" s="9" t="str">
+        <x:v>数据集 diagnostic_states；diagnostic_states planned；已采集A=100/10；暂停期间追加B=200/20并重放A。依赖实际采集、统计和同步功能，使用专用日志目录。</x:v>
+      </x:c>
+      <x:c r="G132" s="9" t="str">
+        <x:v>初始total110、暂停期间仍110，恢复后唯一A/B、total330；手动刷新与重启不重复。菜单栏与主窗口同一筛选口径；暂停状态不伪装成没有日志。</x:v>
+      </x:c>
+      <x:c r="H132" s="9" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I132" s="9" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J132" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K132" s="9" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L132" s="9" t="str">
+        <x:v>docs/testing/cases/12-TM-012-menu-diagnostics.md:11</x:v>
+      </x:c>
+      <x:c r="M132" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133" ht="57" customHeight="1">
+      <x:c r="A133" s="4" t="str">
+        <x:v>TM-012</x:v>
+      </x:c>
+      <x:c r="B133" s="4" t="str">
+        <x:v>E2E-TM012-002</x:v>
+      </x:c>
+      <x:c r="C133" s="4" t="str">
+        <x:v>诊断状态、恢复和登录启动</x:v>
+      </x:c>
+      <x:c r="D133" s="4" t="str">
+        <x:v>待拆解</x:v>
+      </x:c>
+      <x:c r="E133" s="4" t="str">
+        <x:v>产品E2E</x:v>
+      </x:c>
+      <x:c r="F133" s="4" t="str">
+        <x:v>数据集 diagnostic_states；独立子场景：已授权目录失效、真实服务不可达/恢复、测试App登录启动开关。故障作用测试目录/进程；使用已登录桌面与可自动检查的系统设置。</x:v>
+      </x:c>
+      <x:c r="G133" s="4" t="str">
+        <x:v>错误与真实目录/网络故障一致，不能用旧缓存一直显示健康；恢复后状态及时更新，未同步数据不丢。启动设置与OS登记/实际启动行为一致，测试结束恢复本次测试前状态。</x:v>
+      </x:c>
+      <x:c r="H133" s="4" t="str">
+        <x:v>准备：待该功能的数据程序/SQL方案确定。
+变化：待具体任务及数据设计细化。
+核验：暂无可执行数据库核验绑定。</x:v>
+      </x:c>
+      <x:c r="I133" s="4" t="str">
+        <x:v>未来规划</x:v>
+      </x:c>
+      <x:c r="J133" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K133" s="4" t="str">
+        <x:v>未来概要</x:v>
+      </x:c>
+      <x:c r="L133" s="4" t="str">
+        <x:v>docs/testing/cases/12-TM-012-menu-diagnostics.md:28</x:v>
+      </x:c>
+      <x:c r="M133" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G5:G113">
+  <x:conditionalFormatting sqref="G5:G133">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="I5:I113">
+  <x:conditionalFormatting sqref="I5:I133">
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="16" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="17" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="J5:J113">
+  <x:conditionalFormatting sqref="J5:J133">
     <x:cfRule type="containsText" dxfId="18" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="19" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="20" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M113">
+  <x:conditionalFormatting sqref="M5:M133">
     <x:cfRule type="containsText" dxfId="21" priority="10" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="22" priority="11" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="23" priority="12" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46d0525f2c284244"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R981c725aa33a45e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10912,7 +12132,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R468164e844d040cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb916c68e4f6f40e5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11064,25 +12284,66 @@
         <x:v>releases/v0.1.0-20260929T074814Z/06-iteration-record.md</x:v>
       </x:c>
     </x:row>
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="4" t="str">
+        <x:v>v0.4.0-20261001T040433Z</x:v>
+      </x:c>
+      <x:c r="B7" s="4" t="str">
+        <x:v>0.4.0</x:v>
+      </x:c>
+      <x:c r="C7" s="16" t="n">
+        <x:v>46296.16982638889</x:v>
+      </x:c>
+      <x:c r="D7" s="4" t="str">
+        <x:v>产品功能</x:v>
+      </x:c>
+      <x:c r="E7" s="4" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="F7" s="4" t="str">
+        <x:v>未发布</x:v>
+      </x:c>
+      <x:c r="G7" s="4" t="str">
+        <x:v>internal</x:v>
+      </x:c>
+      <x:c r="H7" s="4" t="str">
+        <x:v>dmg/&lt;release_id&gt;/：仅门禁PASS后放正式DMG</x:v>
+      </x:c>
+      <x:c r="I7" s="15" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J7" s="4" t="str">
+        <x:v>设计草案：20条细TC已登记；程序、SQL、产品E2E与发布门禁尚未完成</x:v>
+      </x:c>
+      <x:c r="K7" s="4" t="str">
+        <x:v>Claude Code 2.1.126 隔离CLI原生投影与独立oracle；非产品通过证据</x:v>
+      </x:c>
+      <x:c r="L7" s="4" t="str">
+        <x:v>releases/v0.4.0-20261001T040433Z/00-manifest.json</x:v>
+      </x:c>
+      <x:c r="M7" s="4" t="str">
+        <x:v>releases/v0.4.0-20261001T040433Z/06-iteration-record.md</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="F5:F6">
+  <x:conditionalFormatting sqref="F5:F7">
     <x:cfRule type="containsText" dxfId="30" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="31" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="32" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="J5:J6">
+  <x:conditionalFormatting sqref="J5:J7">
     <x:cfRule type="containsText" dxfId="33" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="34" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="35" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M6">
+  <x:conditionalFormatting sqref="M5:M7">
     <x:cfRule type="containsText" dxfId="36" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="37" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="38" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R194caa4b70474ce0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd587e9eab8ff422e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11987,7 +13248,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93cbdb1e43044101"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ef76d0af5da48d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.1.0-20260929T074814Z][TM-000] docs: establish session ownership and update evidence index
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R273bfaa83b6049a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rbc6ef8bb2639460e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R040b0abcea5b431b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R6440d552f63d4ee6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Raf16677dbd7a4485"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rc1d784c2090d4389"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rf593c1d785cd445b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R6b7a1e7c3e3044e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R4341405b107e4236"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R1d84b9095f3648d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R2b6cc7a070834b86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R4cccc0ad4a264356"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R4797cc0c671342ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R7b218f9584464048"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R2d6080f09ca2464c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R17a6e08107a448e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R80d0806121a04480"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R1d83853b71cc4f58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Ra89beec5c33e407c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rc6b09aeb4829442b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Rbfee68823e604397"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Rfb7bba6be6364c78"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -816,8 +816,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="TMTable9" displayName="TMTable9" ref="A4:H36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:H36"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="TMTable9" displayName="TMTable9" ref="A4:H43" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:H43"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="复盘编号"/>
     <x:tableColumn id="2" name="名称"/>
@@ -1245,7 +1245,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f032e25c44a498a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R763d9cabeb79442f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1295,7 +1295,7 @@
         <x:v>依据</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="132" customHeight="1">
+    <x:row r="5" ht="162" customHeight="1">
       <x:c r="A5" s="4" t="str">
         <x:v>SOP-000</x:v>
       </x:c>
@@ -1306,16 +1306,16 @@
         <x:v>用户改变流程要求、现有 SOP 缺步骤/判据、规范冲突，或需要迁移 SOP 编号和位置。</x:v>
       </x:c>
       <x:c r="D5" s="4" t="str">
-        <x:v>读取当前[工作索引](README.md)、[文档规范](../docs/standards/documentation.md)及受影响流程；明确规则来源和当前 release_id。其他会话先向「SOP」管理会话（thread ID 01a0f5a5-63f7-76b0-aa53-ac6befec91ef）报告修订需求，由该会话执行本 SOP。迁移前按旧有效 SOP 执行，迁移后采用本目录。</x:v>
+        <x:v>读取当前[工作索引](README.md)、[文档规范](../docs/standards/documentation.md)及受影响流程；明确规则来源和当前 release_id。其他会话先向「SOP」管理会话（thread ID 01a0f5a5-63f7-76b0-aa53-ac6befec91ef）报告修订需求，由该会话执行本 SOP。非SOP文档的唯一编写者为「文档」会话（thread ID 01a0f14b-0888-7e93-bb85-a76b419f2ba7）；迁移前按旧有效 SOP 执行，迁移后采用本目录。</x:v>
       </x:c>
       <x:c r="E5" s="4" t="str">
-        <x:v>完整 SOP 索引、独立工作 SOP、同步的规范/模板/目录，以及变更与检查记录。</x:v>
+        <x:v>完整 SOP 索引、独立工作 SOP、向文档会话交接的非SOP变更清单及其提交/检查记录；整合后关联的规范、模板和目录。</x:v>
       </x:c>
       <x:c r="F5" s="4" t="str">
         <x:v>已基线</x:v>
       </x:c>
       <x:c r="G5" s="4" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H5" s="4" t="str">
         <x:v>sop/SOP-000-maintenance.md</x:v>
@@ -1471,7 +1471,7 @@
         <x:v>已基线</x:v>
       </x:c>
       <x:c r="G11" s="4" t="n">
-        <x:v>7</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H11" s="4" t="str">
         <x:v>sop/SOP-006-test-plan.md</x:v>
@@ -1601,7 +1601,7 @@
         <x:v>已基线</x:v>
       </x:c>
       <x:c r="G16" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H16" s="9" t="str">
         <x:v>sop/SOP-011-test-implementation.md</x:v>
@@ -1679,7 +1679,7 @@
         <x:v>已基线</x:v>
       </x:c>
       <x:c r="G19" s="4" t="n">
-        <x:v>23</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="H19" s="4" t="str">
         <x:v>sop/SOP-014-e2e.md</x:v>
@@ -1757,7 +1757,7 @@
         <x:v>已基线</x:v>
       </x:c>
       <x:c r="G22" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="H22" s="9" t="str">
         <x:v>sop/SOP-017-package-validation.md</x:v>
@@ -1783,7 +1783,7 @@
         <x:v>已基线</x:v>
       </x:c>
       <x:c r="G23" s="4" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H23" s="4" t="str">
         <x:v>sop/SOP-018-release-gate.md</x:v>
@@ -1919,7 +1919,7 @@
         <x:v>sop/SOP-023-iteration.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="57" customHeight="1">
+    <x:row r="29" ht="117" customHeight="1">
       <x:c r="A29" s="4" t="str">
         <x:v>SOP-024</x:v>
       </x:c>
@@ -1930,7 +1930,7 @@
         <x:v>新增文档、实现/接口/命令/测试变化、状态更新、链接迁移或记录关键决定。</x:v>
       </x:c>
       <x:c r="D29" s="4" t="str">
-        <x:v>先读 [文档规范](../docs/standards/documentation.md)、适用 SOP 和当前版本；变更规范/模板结构先经 SOP-000。</x:v>
+        <x:v>先读 [文档规范](../docs/standards/documentation.md)、适用 SOP 和当前版本；变更SOP定义先由SOP会话按SOP-000处理，非SOP规范/模板由文档会话编写。其他会话提供目标文件、具体内容/依据、版本、代码或原始证据及紧急依赖；已完成但未集成的旧非SOP改动须保留并交接，不丢弃。</x:v>
       </x:c>
       <x:c r="E29" s="4" t="str">
         <x:v>合规文档、目录/链接/追踪关系、准确状态与实际检查记录。</x:v>
@@ -1939,7 +1939,7 @@
         <x:v>已基线</x:v>
       </x:c>
       <x:c r="G29" s="4" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H29" s="4" t="str">
         <x:v>sop/SOP-024-document-change.md</x:v>
@@ -1953,7 +1953,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf83fc05e890d4999"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R661b6341359a462d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2102,7 +2102,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95753fc0b9574ea2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refacf0baad7d450b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2497,7 +2497,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc10d539c148d4de5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R163e906384534adc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3416,7 +3416,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6b51f9b912f4f1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R970291c4378548da"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4126,7 +4126,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R511cbb049ee44e39"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3660c153b5dd4a3d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5446,7 +5446,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37a03de48b1548e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb15f249c701f45ed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10377,7 +10377,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46d0525f2c284244"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf492ea58d26548f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10912,7 +10912,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R468164e844d040cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91e619ff28294f4c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11046,13 +11046,13 @@
         <x:v>internal</x:v>
       </x:c>
       <x:c r="H6" s="9" t="str">
-        <x:v>dmg/&lt;release_id&gt;/：当前仅开发包；正式DMG门禁PASS后保存</x:v>
+        <x:v>dmg/&lt;release_id&gt;/：当前有 d2db551 同摘要 CANDIDATE-NOT-RELEASED 便捷副本；正式原名 DMG 待最终整合门禁与归档</x:v>
       </x:c>
       <x:c r="I6" s="18" t="b">
         <x:v>0</x:v>
       </x:c>
       <x:c r="J6" s="9" t="str">
-        <x:v>Electron本机精细全量：78父用例62 PASS/9 FAIL/7 BLOCKED；38变体31 PASS/7 FAIL。开发候选未发布，未签发通行证；定向验证另存批次。</x:v>
+        <x:v>独立候选 d2db551 本机门禁 PASS，78父TC/38变体规范化全PASS，机器通行证已生成；最终 master 整合树尚未重验，未正式发布。旧3467dc1门禁FAIL原件保留。</x:v>
       </x:c>
       <x:c r="K6" s="9" t="str">
         <x:v>旧SwiftUI PR #2 已合并、历史双平台六例PASS；不继承给Electron</x:v>
@@ -11082,7 +11082,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R194caa4b70474ce0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5282f33019444cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11979,15 +11979,197 @@
         <x:v>docs/retrospectives/2026-09-29--2026-09-30-tokenmeter.md:478</x:v>
       </x:c>
     </x:row>
+    <x:row r="37" ht="117" customHeight="1">
+      <x:c r="A37" s="4" t="str">
+        <x:v>RET-032</x:v>
+      </x:c>
+      <x:c r="B37" s="4" t="str">
+        <x:v>本机测试决定与远端保护规则冲突</x:v>
+      </x:c>
+      <x:c r="C37" s="4" t="str">
+        <x:v>用户确认完整产品测试在本机执行，Git 只管理源码；远端 master 仍要求三项旧 Actions 检查且强制 PR。手动工作流不能稳定提供同一 PR head 的所需检查，已通过的本机门禁也不能冒充远端状态。</x:v>
+      </x:c>
+      <x:c r="D37" s="4" t="str">
+        <x:v>开发总控与 SOP 会话读取保护 API、工作流触发和旧检查的 App 来源，区分本机候选验收与远端合并条件。用户再次确认只在明确多环境要求时启动 Actions 完整测试。</x:v>
+      </x:c>
+      <x:c r="E37" s="4" t="str">
+        <x:v>由 SOP 会话修订 SOP-019，并保存保护规则迁移前后快照；移除旧三项 required checks，保留 PR、管理员执行、对话解决及禁强推/删除。每次整合仍需复读当前保护和远端树，最终本地 master 候选重新运行完整适用门禁。</x:v>
+      </x:c>
+      <x:c r="F37" s="4" t="str">
+        <x:v>规范分支 PR #4/#5 已先行进入远端 master 的历史见[TM-001 版本 06](../../releases/v0.1.0-20260929T074814Z/06-iteration-record.md)；当前最终产品整合和远端发布未据此自动完成。原始快照在本机 .local/git-sync/20261001T055756Z-local-only-protection/。</x:v>
+      </x:c>
+      <x:c r="G37" s="4" t="str">
+        <x:v>验收结果、远端分支保护和分发资格各需独立证明。更换执行地点时，同时核对保护规则与工作流触发，不能只改 SOP 文字。</x:v>
+      </x:c>
+      <x:c r="H37" s="4" t="str">
+        <x:v>docs/retrospectives/2026-10-01-development-and-governance.md:5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="102" customHeight="1">
+      <x:c r="A38" s="9" t="str">
+        <x:v>RET-033</x:v>
+      </x:c>
+      <x:c r="B38" s="9" t="str">
+        <x:v>主精细报告的辅助占位与最终结果口径不同</x:v>
+      </x:c>
+      <x:c r="C38" s="9" t="str">
+        <x:v>TM-001 主精细 run 的 116 行中，11 条辅助项只是待独立程序执行的占位，原始状态 BLOCKED。把后续辅助 PASS 回写到主报告，或只看主报告判最终失败，都会丢失真实来源。</x:v>
+      </x:c>
+      <x:c r="D38" s="9" t="str">
+        <x:v>核对精细、辅助、独立审计和六组补充 E2E 的原始报告及逐例 Excel，确定每份报告的候选、包、运行顺序和覆盖范围；旧主报告不改写。</x:v>
+      </x:c>
+      <x:c r="E38" s="9" t="str">
+        <x:v>固定门禁从各来源原件独立复算最终 78 父 TC、38 变体结果，保留主 run 的 11 条原始 BLOCKED，并在 final-product-result.json 写来源与规范化状态；缺原件、错候选或错摘要均阻断。</x:v>
+      </x:c>
+      <x:c r="F38" s="9" t="str">
+        <x:v>开发包联合复核曾得到逐项 PASS，但其主 run 仍为 BLOCKED 且包未发布；独立候选 d2db551 的新门禁原件最终为 PASS，见 .local/gates/tm001-final-gate-d2db551-20261001T0904Z/。最终总控整合仍待重验。</x:v>
+      </x:c>
+      <x:c r="G38" s="9" t="str">
+        <x:v>聚合结论要保留每个来源的原始状态和身份，不能把汇总表、截图或手工标记当作源测试结果。</x:v>
+      </x:c>
+      <x:c r="H38" s="9" t="str">
+        <x:v>docs/retrospectives/2026-10-01-development-and-governance.md:17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="117" customHeight="1">
+      <x:c r="A39" s="4" t="str">
+        <x:v>RET-034</x:v>
+      </x:c>
+      <x:c r="B39" s="4" t="str">
+        <x:v>首次干净候选缺管理员本人身份旁证</x:v>
+      </x:c>
+      <x:c r="C39" s="4" t="str">
+        <x:v>候选 3467dc1 的 95 个真实精细 Playwright 入口、辅助 11/11、审计 12/12、补充六组 6/6 分项通过，但最终门禁 FAIL。补充管理员场景只有被撤销成员 /v1/me 的预期 401，没有管理员本人有效 200 的原始旁证。</x:v>
+      </x:c>
+      <x:c r="D39" s="4" t="str">
+        <x:v>保留 .local/gates/tm001-final-gate-3467dc1-20261001T0730Z/gate.json 的 FAIL，按 SOP-015 对照既定身份验收与 service audit；判断为固定测试证据缺口，未把分项 PASS 推定为产品认证完成。</x:v>
+      </x:c>
+      <x:c r="E39" s="4" t="str">
+        <x:v>在固定 E2E-003 增加真实 App 重启后的管理员会话恢复、有效 /v1/me 200 及账号/角色断言，并给缺失 200 的门禁路径加负测；冻结新候选后完整重跑。</x:v>
+      </x:c>
+      <x:c r="F39" s="4" t="str">
+        <x:v>d2db551 的 E2E-003 原始 service audit 已出现有效 200，独立本机门禁 PASS；旧 FAIL 原件未覆盖。依据[本版结果](../../releases/v0.1.0-20260929T074814Z/07-test-results.md)及新旧 .local/gates/ 原件。正式整合发布仍待总控处理。</x:v>
+      </x:c>
+      <x:c r="G39" s="4" t="str">
+        <x:v>用例通过和门禁要求的证据链是两层检查。对关键身份行为，固定程序须采到正向与撤销后的反向原件。</x:v>
+      </x:c>
+      <x:c r="H39" s="4" t="str">
+        <x:v>docs/retrospectives/2026-10-01-development-and-governance.md:29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="72" customHeight="1">
+      <x:c r="A40" s="9" t="str">
+        <x:v>RET-035</x:v>
+      </x:c>
+      <x:c r="B40" s="9" t="str">
+        <x:v>系统打开文件列表含空名称项</x:v>
+      </x:c>
+      <x:c r="C40" s="9" t="str">
+        <x:v>lsof -Fn 可能产生无名称行。升级场景的采集器把它当成空路径，后续审计会报打开文件列表不完整；若简单丢弃整个列表，又会隐藏具名文件证据。</x:v>
+      </x:c>
+      <x:c r="D40" s="9" t="str">
+        <x:v>在首次门禁 FAIL 后只读核对 E2E-004 原始列表，确认有一条空名称；对照归档校验要求，区分命令输出占位与实际具名文件路径。</x:v>
+      </x:c>
+      <x:c r="E40" s="9" t="str">
+        <x:v>固定解析器只忽略无名称条目、保留全部具名路径；003 与精细更新采集器共用规则，并增加解析单元测试。</x:v>
+      </x:c>
+      <x:c r="F40" s="9" t="str">
+        <x:v>新候选 d2db551 的 E2E-004 原件记录 125 个具名路径、零空项，完整门禁 PASS；旧候选原件仍可复查。见版本 06 和两次门禁目录。</x:v>
+      </x:c>
+      <x:c r="G40" s="9" t="str">
+        <x:v>OS 工具的文本输出需按真实语法建模。修采集器时保留可审计的有效项，并用固定反例验证。</x:v>
+      </x:c>
+      <x:c r="H40" s="9" t="str">
+        <x:v>docs/retrospectives/2026-10-01-development-and-governance.md:41</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="87" customHeight="1">
+      <x:c r="A41" s="4" t="str">
+        <x:v>RET-036</x:v>
+      </x:c>
+      <x:c r="B41" s="4" t="str">
+        <x:v>后续版本不能沿用 TM-001 固定门禁总数</x:v>
+      </x:c>
+      <x:c r="C41" s="4" t="str">
+        <x:v>SOP-011/014/018 曾把 TM-001 的 116 主行、78 父 TC、38 变体、11 辅助、12 审计和六组场景写成通用候选数量。TM-002/003 新增用例后，该固定数会遗漏新需求，或让门禁错误地以旧集合判通过。</x:v>
+      </x:c>
+      <x:c r="D41" s="4" t="str">
+        <x:v>TM-002/003 报告各自草稿集合和门禁派生 TC 的自依赖；SOP 会话逐项核对来源 release、固定候选清单和既有 TM-001 历史原件，避免改写旧报告。</x:v>
+      </x:c>
+      <x:c r="E41" s="4" t="str">
+        <x:v>SOP 独立提交 3303c0b 定义目标版本加此前已交付功能的机器清单并集，逐来源核对父/变体/辅助/场景/审计；最终 gate 自身派生 TC 在其他原件及真实升级验真后计算。本会话接管其发布和用例规范等非 SOP 附件。</x:v>
+      </x:c>
+      <x:c r="F41" s="4" t="str">
+        <x:v>规范分支结构、基线、质量与治理 198/198 检查通过；产品跨版本执行器尚未在最终整合树实测，TM-002/003 产品验收仍 BLOCKED。原始规范检查在 .local/git-sync/20261001-cross-release-sop/。</x:v>
+      </x:c>
+      <x:c r="G41" s="4" t="str">
+        <x:v>历史版本的精确数量只约束其来源原件；后续发行范围必须从已确认版本的机器清单生成，并保存来源摘要。</x:v>
+      </x:c>
+      <x:c r="H41" s="4" t="str">
+        <x:v>docs/retrospectives/2026-10-01-development-and-governance.md:53</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="72" customHeight="1">
+      <x:c r="A42" s="9" t="str">
+        <x:v>RET-037</x:v>
+      </x:c>
+      <x:c r="B42" s="9" t="str">
+        <x:v>隔离 profile 不能证明 Keychain 凭据隔离</x:v>
+      </x:c>
+      <x:c r="C42" s="9" t="str">
+        <x:v>TM-002 的 safeStorage 在 macOS 涉及 Keychain。只使用独立 --user-data-dir 不能证明系统 item 与正式 App 分离，测试若误读、覆盖或清理已有凭据会污染用户环境。</x:v>
+      </x:c>
+      <x:c r="D42" s="9" t="str">
+        <x:v>总控和 SOP 会话区分浏览器 profile 与系统凭据命名空间，核对 Electron 源码仅能提供设计线索，不能替代最终 DMG 原生 item 身份证明。</x:v>
+      </x:c>
+      <x:c r="E42" s="9" t="str">
+        <x:v>在首次相关调用前，用同一最终 DMG 于隔离 macOS 测试账号或经证明独立的命名空间探查精确 service/account；要求预先不存在，记录 owner 与创建元数据，仅清理本次创建的精确 item。来源身份/密钥不可用时停读。相关规范和设计作为 TM-002/003/004 前置。</x:v>
+      </x:c>
+      <x:c r="F42" s="9" t="str">
+        <x:v>SOP 与非 SOP 设计约束已在分支形成；TM-002/003/004 尚无最终包原生探针和对应产品 E2E 原件，保持 BLOCKED。依据版本 06 及隔离规范交接。</x:v>
+      </x:c>
+      <x:c r="G42" s="9" t="str">
+        <x:v>测试隔离需覆盖操作系统共享资源，不只覆盖进程目录和 SQLite；不能从源码命名推断运行时凭据身份。</x:v>
+      </x:c>
+      <x:c r="H42" s="9" t="str">
+        <x:v>docs/retrospectives/2026-10-01-development-and-governance.md:65</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="72" customHeight="1">
+      <x:c r="A43" s="4" t="str">
+        <x:v>RET-038</x:v>
+      </x:c>
+      <x:c r="B43" s="4" t="str">
+        <x:v>并发开发造成文档草稿与候选状态交叉</x:v>
+      </x:c>
+      <x:c r="C43" s="4" t="str">
+        <x:v>TM-002 至 TM-005 并行形成需求、用例、机器目录和总表草稿；个别分支含已提交或未提交文档。不同分支中的用例数量、状态和来源行号在持续变化，直接合并可能覆盖 TM-001 原始批次，或把 baseline_pending 当作产品 PASS。</x:v>
+      </x:c>
+      <x:c r="D43" s="4" t="str">
+        <x:v>用户先指定“SOP”会话统一维护 SOP，随后指定“文档”会话统一编写其余文档与 Excel。文档会话核对可见会话、分支和交接输入，保留已形成的 diff 与原始检查，按来源需求逐项审阅。</x:v>
+      </x:c>
+      <x:c r="E43" s="4" t="str">
+        <x:v>建立[会话体系](../project-sessions.md)和单一文档入口；需求会话继续代码/固定测试并交付候选、TC、原件和阻断，文档会话在独立分支维护非 SOP 文档、目录和 Excel，总控整合后重验。未核实的分支不写成已创建会话。</x:v>
+      </x:c>
+      <x:c r="F43" s="4" t="str">
+        <x:v>归口规则已通知现有核心会话，交接队列已登记；TM-002 至 TM-005 的草稿仍在核对中，严格基线或产品门禁未通过的部分不升格。此次文档提交与检查结果见版本 06。</x:v>
+      </x:c>
+      <x:c r="G43" s="4" t="str">
+        <x:v>角色归口减少并发覆盖，但每条事实仍需要候选身份、原始证据和阶段状态。Excel 更新也须遵守候选输入先提交、批次在归档后索引的时序。</x:v>
+      </x:c>
+      <x:c r="H43" s="4" t="str">
+        <x:v>docs/retrospectives/2026-10-01-development-and-governance.md:77</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="F5:F36">
+  <x:conditionalFormatting sqref="F5:F43">
     <x:cfRule type="containsText" dxfId="39" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="40" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="41" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93cbdb1e43044101"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc07fa5317a0347a6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.1.0-20260929T074814Z][TM-000] docs: bind milestone archive and future upgrade contracts
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R5bcf6af7c2824aeb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R416d93558caa47ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R3eed2723341c4efe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R11eacf0c8a6847ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rd6c7c534ab26465b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R3c8710592e9c49c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R1b270a2dee4346ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R0a4b3a5aa47546dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rf888855f751947d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R32cead9b86ec4dda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R35c4bd608c694a0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Rb4069f2fb21043b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rf2621ab51edf4918"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rd0eded506b6f4e16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R5cc396c4723c4ea4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Ra228ac68a0294779"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R63749ec98d05495f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R5dee996be0e14721"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Rb6b6c6cf83be4879"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Ref2df82fe2b34886"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R8cd258111ab14bc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R8f05ebc6ecf14392"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1251,7 +1251,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c8e4c6871c9448d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb073f7078ced4335"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1959,7 +1959,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02f8fd2b66bf4042"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc22714fd11ab424f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2108,7 +2108,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85c0fee1613347c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1928780e08ea4590"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2543,7 +2543,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f0aa82aa5844cbf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbce28c71569f41b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3590,7 +3590,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5407363040844d1a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ebaf172ae7842c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4367,7 +4367,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R490ea09385ac40b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb908851cdca0420f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6150,7 +6150,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R857f4be4041d474b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5b7618679c74cdf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12970,7 +12970,7 @@
         <x:v>v0.2.0-20261001T034118Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="147" ht="132" customHeight="1">
+    <x:row r="147" ht="177" customHeight="1">
       <x:c r="A147" s="4" t="str">
         <x:v>TM-002</x:v>
       </x:c>
@@ -12987,17 +12987,17 @@
         <x:v>交付门禁</x:v>
       </x:c>
       <x:c r="F147" s="4" t="str">
-        <x:v>已锁定候选 SHA/tree、0.2.0 最终 DMG 原件/清单、上一0.1本机正式稳定DMG及其SOP-018通行证、SOP-020归档收据、来源里程碑SHA/tree、签名和原包摘要、同机隔离签名更新源与每例隔离服务；若没有这些前置或真实升级入口，本例为 BLOCKED，不能用开发/候选包、受控101或同源码测试高版冒充。远端源码登记与Tag可待最终统一办理。TM-001 全部已交付 TC 和 除本例外 TM-002 其余 27 条父 TC 与 35 个稳定变体的固定清单在运行前确定。</x:v>
+        <x:v>已锁定候选 SHA/tree、0.2.0 最终 DMG 原件/清单、上一0.1本机正式稳定DMG及其SOP-018通行证、SOP-020 schema 2 release-index.json（milestone_sha/tree、master_tip_sha、remote_source_state=PENDING、原DMG/manifest/passport摘要）、签名、同机隔离签名更新源与每例隔离服务；若没有这些前置或真实升级入口，本例为 BLOCKED，不能用开发/候选包、受控101或同源码测试高版冒充。远端源码登记与Tag可待最终统一办理。TM-001 全部已交付 TC 和 除本例外 TM-002 其余 27 条父 TC 与 35 个稳定变体的固定清单在运行前确定。</x:v>
       </x:c>
       <x:c r="G147" s="4" t="str">
         <x:v>TM-001 全部已交付 TC、其他 27 条 TM-002 父 TC/35 变体的真实 UI、原生面板、服务与隔离 DB 由各自固定程序执行；原始记录各有唯一尝试和清理；本例结果此时仍为 BLOCKED。
-上一0.1本机稳定原包来源与通行证一致，App 自主升级；0.2显示新版本、保留TM-001合成账号/配置且 /v1/me 复核身份；来源初态 none，真实面板确认A后重启恢复本版密文来源；两端包签名、摘要和进程版本吻合。
+上一0.1本机稳定原包schema 2归档、里程碑来源、通行证与实际摘要一致，负测按既定拒绝，App 自主升级；0.2显示新版本、保留TM-001合成账号/配置且 /v1/me 复核身份；来源初态 none，真实面板确认A后重启恢复本版密文来源；两端包签名、摘要和进程版本吻合。
 本例不自我依赖：只有 TM-001 全部、其他 27 条 TM-002 父 TC/35 变体及升级真实结果均 PASS，且本例自身包/升级/证据核验 PASS，才记本例 PASS 并由最终 gate 签发通行证；计算前为 BLOCKED；本步骤无业务 DB 写入。</x:v>
       </x:c>
       <x:c r="H147" s="4" t="str">
-        <x:v>准备：每个产品 TC 由共同 R 独立准备合成账号、隔离 SQLite 与来源；本门禁只读这些运行的原始摘要及 SQL/数据证据引用，并核对最终 DMG、升级源和候选 SHA/tree。 上一稳定0.1包须有SOP-018/020原件及来源里程碑身份，远端登记可待办。
+        <x:v>准备：每个产品 TC 由共同 R 独立准备合成账号、隔离 SQLite 与来源；本门禁只读这些运行的原始摘要及 SQL/数据证据引用，并核对最终 DMG、升级源和候选 SHA/tree。 上一稳定0.1包须有SOP-018/020原件及来源里程碑身份，远端登记可待办。 稳定升级源消费者还须有旧schema/候选包/错误里程碑和摘要的固定拒绝负测。
 变化：本门禁自身无服务业务 SQL 写入；逐个产品 TC 的认证 sessions/audit 变化只按各自 NDA 与只读证据解释。
-核验：只读复核 TM-001 全部已交付 TC、其他 27 条 TM-002 父 TC/35 变体的隔离 DB/SQL 引用与原始逐步结果，并核对最终包、升级、清理和候选一致性；本例结果由这些原件派生，不连接生产库。 核对上一0.1稳定原包的通行证、归档、来源SHA/tree及真实升级链。</x:v>
+核验：只读复核 TM-001 全部已交付 TC、其他 27 条 TM-002 父 TC/35 变体的隔离 DB/SQL 引用与原始逐步结果，并核对最终包、升级、清理和候选一致性；本例结果由这些原件派生，不连接生产库。 核对上一0.1稳定原包的通行证、归档、来源SHA/tree及真实升级链。 只读核对schema 2 release-index.json的milestone_sha/tree、master_tip_sha、remote_source_state及原件摘要。</x:v>
       </x:c>
       <x:c r="I147" s="4" t="str">
         <x:v>预期待明确</x:v>
@@ -14375,7 +14375,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a349a07c4ad4ae4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec35cff4aad5459b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14910,7 +14910,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf2738bc8d4d43e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc77e3f313c004fe0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15072,7 +15072,7 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="72" customHeight="1">
+    <x:row r="7" ht="117" customHeight="1">
       <x:c r="A7" s="4" t="str">
         <x:v>v0.2.0-20261001T034118Z</x:v>
       </x:c>
@@ -15101,7 +15101,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J7" s="4" t="str">
-        <x:v>0.2设计草稿：3功能点/9 TASK、28父TC/35变体已编制，SOP-008基线与固定程序未完成；需上一实际本机稳定0.1原包。产品E2E NOT_RUN、未发布。</x:v>
+        <x:v>0.2设计草稿：3功能点/9 TASK、28父TC/35变体已编制，SOP-008基线与固定程序未完成；需上一实际本机稳定0.1原包和schema 2归档消费者。最终包Keychain身份探针缺隔离测试账号或已实测独立命名空间，相关E2E BLOCKED；产品E2E NOT_RUN、未发布。</x:v>
       </x:c>
       <x:c r="K7" s="4" t="str">
         <x:v>TM001独立候选d2门禁PASS；本地master整合树尚未完成同树门禁或SOP-020稳定归档，不能继承为0.2升级源；本版无实际产品运行。</x:v>
@@ -15134,7 +15134,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R330cfc4c7212448f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34c190857069430d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16221,7 +16221,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52eacc33365f495f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94073158d3cc4eaf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.3.0-20261001T034652Z][TM-003] Record CORE development slice readiness
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Ra702d9032419454f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R3ccf785cff824031"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rc0e266b44e8e4387"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R2fe9df2ed8484af4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Ra1d3832d77d44954"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R6b490de23f5b4254"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R73a9f7a1a4ff407e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R61d060e006c441d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R91607a3954054080"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R18ffc2a61fbe4df2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Ra9834d7a84304806"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R04a09d8054e24439"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Ra8b6d438e10e4cc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R6744e6d3400e4dbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R2ba2051075b449cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rde15358f574c431e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R828cd351cd3f4a6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R9c2d956194f14733"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R1b84a2ea719747e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Ra3337ccae59b4978"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R8b1eb842c9be4df6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R9db3c10219b94070"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1255,7 +1255,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c3c3941a6734fa6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad2356804e564194"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1963,7 +1963,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R966c6dcd4d42499a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c6ce5ad2d3f4c4e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2112,7 +2112,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97878ac8d0cc498c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbabee8887f5246c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2547,7 +2547,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b83207a825a41b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb60bcb58940a449d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3594,7 +3594,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd029f162ac214e85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd30be25a417f4e6e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4701,7 +4701,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39a6e7bac47e4ea0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9ab17abf0d0427a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7486,7 +7486,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec70bb3810934e65"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf769948b070a4b80"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19938,7 +19938,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f9309e62ac44ebc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R912ecfc95f1a4378"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20511,7 +20511,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0297172083574cbe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d8dfb9ad96d493c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20769,7 +20769,7 @@
         <x:v>releases/v0.2.0-20261001T034118Z/01-requirements.md:32</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="117" customHeight="1">
+    <x:row r="8" ht="132" customHeight="1">
       <x:c r="A8" s="9" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
       </x:c>
@@ -20798,7 +20798,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J8" s="9" t="str">
-        <x:v>整版draft、未发布。原27条目标TC与3条无授权CORE辅助TC设计固定但程序绑定和运行未完成；CORE切片文档检查PASS，Git提交SHA因主对象库不可见而缺，development_slice_ready仍BLOCKED。TM002授权与产品Keychain依赖未齐，产品E2E未执行；正式发行完整门禁NOT_RUN。</x:v>
+        <x:v>整版draft、未发布。原27条目标TC保留，新增3条无授权CORE辅助TC在恢复新仓库候选7d77d63按SOP-008独立切片判为development_slice_ready；固定程序绑定与实际运行仍缺，30条TM003目标/辅助TC均未获得产品PASS。授权/真实App/服务/Keychain及产品E2E仍BLOCKED，0.3整版baseline和正式发行完整门禁NOT_RUN。</x:v>
       </x:c>
       <x:c r="K8" s="9" t="str">
         <x:v>TM-001 干净源码候选为技术基底；其产品门禁不继承给TM-003</x:v>
@@ -20955,7 +20955,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d04cecde8da4866"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc08e1a26493946c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22120,7 +22120,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ff906f63aba4039"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra38b2a0da86e45e9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.5.0-20261001T034729Z][TM-005] Freeze pure statistics CORE slice and sync project workbook
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R04a09d8054e24439"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Ra8b6d438e10e4cc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R6744e6d3400e4dbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R2ba2051075b449cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rde15358f574c431e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R828cd351cd3f4a6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R9c2d956194f14733"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R1b84a2ea719747e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Ra3337ccae59b4978"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R8b1eb842c9be4df6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R9db3c10219b94070"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R49697d2c441d464b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R5d12880f2ce24702"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R60e45e41e1234871"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rf8797fb3cdf7496a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R82b1eb0351634d5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R95cfb4f1d6ac42bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rabfd9323da1c4b9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R1d58ab70850b4c19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rdd0b166202e346e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Rd589207889cc4343"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Rd07e33eea4e84bed"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -755,8 +755,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N264" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N264"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N267" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N267"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="功能编号"/>
     <x:tableColumn id="2" name="用例编号"/>
@@ -1101,8 +1101,8 @@
         <x:v>已登记用例</x:v>
       </x:c>
       <x:c r="B8" s="11" t="n">
-        <x:f>COUNTA('05测试用例'!B5:B264)</x:f>
-        <x:v>260</x:v>
+        <x:f>COUNTA('05测试用例'!B5:B267)</x:f>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>父用例与具有稳定 ID 的变体各占一行；含未来概要场景</x:v>
@@ -1125,7 +1125,7 @@
         <x:v>细化产品用例</x:v>
       </x:c>
       <x:c r="B10" s="11" t="n">
-        <x:v>190</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
         <x:v>逐条结果按运行批次记录；稳定变体独立列出</x:v>
@@ -1255,7 +1255,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad2356804e564194"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa21f6bd2e694056"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1963,7 +1963,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c6ce5ad2d3f4c4e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc2f0e39e73241d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2112,7 +2112,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbabee8887f5246c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17a35b4f5f0d417e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2547,7 +2547,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb60bcb58940a449d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R961caa3c423e4d07"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3594,7 +3594,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd30be25a417f4e6e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93b416a951454bb2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4701,7 +4701,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9ab17abf0d0427a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1338d444aef4cb7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7486,7 +7486,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf769948b070a4b80"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R961f62463f854144"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19915,30 +19915,176 @@
         <x:v>v0.3.0-20261001T034652Z</x:v>
       </x:c>
     </x:row>
+    <x:row r="265" ht="72" customHeight="1">
+      <x:c r="A265" s="4" t="str">
+        <x:v>TM-005</x:v>
+      </x:c>
+      <x:c r="B265" s="4" t="str">
+        <x:v>TC-TM005-CORE-01</x:v>
+      </x:c>
+      <x:c r="C265" s="4" t="str">
+        <x:v>双来源可信事件与半开日汇总</x:v>
+      </x:c>
+      <x:c r="D265" s="4" t="str">
+        <x:v>TASK-TM005-EVENT-CONTRACT
+TASK-TM005-RANGE-QUERY</x:v>
+      </x:c>
+      <x:c r="E265" s="4" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="F265" s="4" t="str">
+        <x:v>fixture的A/B、跨主体C、界外D/E；synthetic-p1、Asia/Shanghai当地日2026-09-29</x:v>
+      </x:c>
+      <x:c r="G265" s="4" t="str">
+        <x:v>1. 按固定主体/当地日查询纯统计函数；仅A/B被选、C/D/E排除；输入数组和键不变
+2. 核对来源、模型、Token和三个子项；input300/output30/total330；Codex110/Claude220；未知模型110/sonnet-test220；缓存读20但部分未知、缓存写未知、推理2但部分未知，子项不加总
+3. 逐个输入非法来源、负数、超范围缓存和坏UTC；各自被拒绝，无完整零或有效汇总输出；原fixture不变</x:v>
+      </x:c>
+      <x:c r="H265" s="4" t="str">
+        <x:v>准备：无产品DB写入；每例从新内存输入开始
+变化：不适用；纯统计返回值与输入未变
+核验：固定fixture摘要、事件筛选、各字段与状态逐步核对；无SQL</x:v>
+      </x:c>
+      <x:c r="I265" s="4" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J265" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K265" s="4" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L265" s="4" t="str">
+        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:326</x:v>
+      </x:c>
+      <x:c r="M265" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N265" s="4" t="str">
+        <x:v>v0.5.0-20261001T034729Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="266" ht="57" customHeight="1">
+      <x:c r="A266" s="9" t="str">
+        <x:v>TM-005</x:v>
+      </x:c>
+      <x:c r="B266" s="9" t="str">
+        <x:v>TC-TM005-CORE-02</x:v>
+      </x:c>
+      <x:c r="C266" s="9" t="str">
+        <x:v>未知用量诊断不补零</x:v>
+      </x:c>
+      <x:c r="D266" s="9" t="str">
+        <x:v>TASK-TM005-EVENT-CONTRACT
+TASK-TM005-COVERAGE</x:v>
+      </x:c>
+      <x:c r="E266" s="9" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="F266" s="9" t="str">
+        <x:v>fixture A/B及同范围Claude missing_usage诊断；双来源complete仅为模块合成覆盖假设</x:v>
+      </x:c>
+      <x:c r="G266" s="9" t="str">
+        <x:v>1. 先仅统计A/B；已知330，未知模型110保留，来源Codex110/Claude220
+2. 加入诊断重新统计；partial、known_tokens330、total_tokens=null；诊断不增调用或零Token
+3. 移除A/B仅保留诊断；unknown、known_tokens0、total_tokens=null，不能写已确认零</x:v>
+      </x:c>
+      <x:c r="H266" s="9" t="str">
+        <x:v>准备：无产品DB写入；每例从新内存输入开始
+变化：不适用；纯统计返回值与输入未变
+核验：固定fixture摘要、事件筛选、各字段与状态逐步核对；无SQL</x:v>
+      </x:c>
+      <x:c r="I266" s="9" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J266" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K266" s="9" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L266" s="9" t="str">
+        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:334</x:v>
+      </x:c>
+      <x:c r="M266" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N266" s="9" t="str">
+        <x:v>v0.5.0-20261001T034729Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="267" ht="87" customHeight="1">
+      <x:c r="A267" s="4" t="str">
+        <x:v>TM-005</x:v>
+      </x:c>
+      <x:c r="B267" s="4" t="str">
+        <x:v>TC-TM005-CORE-03</x:v>
+      </x:c>
+      <x:c r="C267" s="4" t="str">
+        <x:v>声明式覆盖状态代数</x:v>
+      </x:c>
+      <x:c r="D267" s="4" t="str">
+        <x:v>TASK-TM005-COVERAGE</x:v>
+      </x:c>
+      <x:c r="E267" s="4" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="F267" s="4" t="str">
+        <x:v>fixture五行coverage_algebra；complete仅为模块合成输入，product_coverage_proven=false</x:v>
+      </x:c>
+      <x:c r="G267" s="4" t="str">
+        <x:v>1. 两来源complete且无事件、随后移除覆盖事实；前者complete/known0/total0；后者不得自行推断complete
+2. 一来源missing，分别给空事件与可信110；空事件missing/known0/total null；可信110为partial/known110/total null
+3. 两来源complete，分别给可信110+未知诊断、仅未知诊断；前者partial/known110/total null；后者unknown/known0/total null</x:v>
+      </x:c>
+      <x:c r="H267" s="4" t="str">
+        <x:v>准备：无产品DB写入；每例从新内存输入开始
+变化：不适用；纯统计返回值与输入未变
+核验：固定fixture摘要、事件筛选、各字段与状态逐步核对；无SQL</x:v>
+      </x:c>
+      <x:c r="I267" s="4" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J267" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K267" s="4" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L267" s="4" t="str">
+        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:342</x:v>
+      </x:c>
+      <x:c r="M267" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N267" s="4" t="str">
+        <x:v>v0.5.0-20261001T034729Z</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G5:G264">
+  <x:conditionalFormatting sqref="G5:G267">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="I5:I264">
+  <x:conditionalFormatting sqref="I5:I267">
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="16" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="17" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="J5:J264">
+  <x:conditionalFormatting sqref="J5:J267">
     <x:cfRule type="containsText" dxfId="18" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="19" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="20" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M264">
+  <x:conditionalFormatting sqref="M5:M267">
     <x:cfRule type="containsText" dxfId="21" priority="10" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="22" priority="11" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="23" priority="12" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R912ecfc95f1a4378"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73e815c9d86a4064"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20511,7 +20657,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d8dfb9ad96d493c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d75d2e9f55f4cfc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20798,7 +20944,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J8" s="9" t="str">
-        <x:v>整版draft、未发布。原27条目标TC保留，新增3条无授权CORE辅助TC在恢复新仓库候选7d77d63按SOP-008独立切片判为development_slice_ready；固定程序绑定与实际运行仍缺，30条TM003目标/辅助TC均未获得产品PASS。授权/真实App/服务/Keychain及产品E2E仍BLOCKED，0.3整版baseline和正式发行完整门禁NOT_RUN。</x:v>
+        <x:v>整版draft、未发布。27条产品TC未执行；3条CORE辅助TC已在文档提交48ca089独立切片就绪，在开发分支311deedf运行模块3/3 PASS，原始receipt在该分支.local/ci/tm003-core-20261001/。代码尚未合入本文档树，机器绑定保持空；模块报告不能作为产品E2E或发行门禁，结果Excel规范待SOP修订。</x:v>
       </x:c>
       <x:c r="K8" s="9" t="str">
         <x:v>TM-001 干净源码候选为技术基底；其产品门禁不继承给TM-003</x:v>
@@ -20813,7 +20959,7 @@
         <x:v>未核实同名功能分支SHA/tree读回</x:v>
       </x:c>
       <x:c r="O8" s="9" t="str">
-        <x:v>产品E2E未执行；本机稳定包未归档</x:v>
+        <x:v>CORE模块3/3只在独立开发分支PASS；真实安装App产品E2E未运行；本机稳定包未归档</x:v>
       </x:c>
       <x:c r="P8" s="9" t="str">
         <x:v>本轮五版稳定后一次受保护PR；待办</x:v>
@@ -20881,7 +21027,7 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="102" customHeight="1">
+    <x:row r="10" ht="117" customHeight="1">
       <x:c r="A10" s="9" t="str">
         <x:v>v0.5.0-20261001T034729Z</x:v>
       </x:c>
@@ -20910,7 +21056,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J10" s="9" t="str">
-        <x:v>整版draft、未发布。6 TASK、32父TC、6稳定变体及两组摘要已登记；纯统计语义oracle仅可验证算术/覆盖合同，不证明双来源真实采集。固定产品数据、SQLite/IPC、安装App逐TC绑定未完成；正式发行完整门禁NOT_RUN。</x:v>
+        <x:v>整版draft、未发布。原32条产品父TC、6稳定变体和两组摘要保留；新增3条纯统计CORE辅助TC，合成fixture与逐步预期已冻结，切片核对尚在进行。静态oracle不证明真实双来源采集或产品E2E；固定产品数据、SQLite/IPC、安装App逐TC绑定未完成，正式发行完整门禁NOT_RUN。</x:v>
       </x:c>
       <x:c r="K10" s="9" t="str">
         <x:v>TM005语义oracle只验证规范化样例；0.4及此前稳定原包尚未形成，真实升级BLOCKED。</x:v>
@@ -20955,7 +21101,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc08e1a26493946c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7977dad8fd6645e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22120,7 +22266,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra38b2a0da86e45e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf611e281df2443f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.5.0-20261001T034729Z][TM-005] Record pure statistics development slice readiness
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R49697d2c441d464b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R5d12880f2ce24702"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R60e45e41e1234871"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rf8797fb3cdf7496a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R82b1eb0351634d5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R95cfb4f1d6ac42bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rabfd9323da1c4b9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R1d58ab70850b4c19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rdd0b166202e346e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Rd589207889cc4343"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Rd07e33eea4e84bed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Ra34cb97649fe4064"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Ra70c794b2e164466"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rfb3048600da248a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R7e5a4ada29ae4937"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Re2b75bfe9fed4bc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rb81226098b1e4536"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Re24460cc44ea476b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R18122656c3bd40c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R93ce1a3f21084943"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Rbacb2c3887dc4b14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R363d3736582d4f08"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1255,7 +1255,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa21f6bd2e694056"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e400cb931d046ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1963,7 +1963,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc2f0e39e73241d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re66a8b0da047414e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2112,7 +2112,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17a35b4f5f0d417e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref49158206c0495c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2547,7 +2547,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R961caa3c423e4d07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b318a29ab9c4d3d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3594,7 +3594,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93b416a951454bb2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37d2691052f64f9a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4701,7 +4701,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1338d444aef4cb7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ff245d7da434fbd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7486,7 +7486,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R961f62463f854144"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd75cc4e2fd4745e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20084,7 +20084,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73e815c9d86a4064"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8f0538f57bf4f6c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20657,7 +20657,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d75d2e9f55f4cfc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55c211e1a3b04821"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21027,7 +21027,7 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="117" customHeight="1">
+    <x:row r="10" ht="162" customHeight="1">
       <x:c r="A10" s="9" t="str">
         <x:v>v0.5.0-20261001T034729Z</x:v>
       </x:c>
@@ -21056,7 +21056,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J10" s="9" t="str">
-        <x:v>整版draft、未发布。原32条产品父TC、6稳定变体和两组摘要保留；新增3条纯统计CORE辅助TC，合成fixture与逐步预期已冻结，切片核对尚在进行。静态oracle不证明真实双来源采集或产品E2E；固定产品数据、SQLite/IPC、安装App逐TC绑定未完成，正式发行完整门禁NOT_RUN。</x:v>
+        <x:v>整版draft、未发布。原32条产品父TC、6稳定变体和两组摘要保留；纯统计CORE-01/02/03辅助TC在输入提交061c759后，经SOP-008内容核对及结构/治理457项PASS，独立切片development_slice_ready，程序绑定仍为空、模块实际运行unexecuted。静态oracle与切片就绪不证明真实双来源采集或产品E2E；固定产品数据、SQLite/IPC、安装App逐TC绑定未完成，正式发行完整门禁NOT_RUN。</x:v>
       </x:c>
       <x:c r="K10" s="9" t="str">
         <x:v>TM005语义oracle只验证规范化样例；0.4及此前稳定原包尚未形成，真实升级BLOCKED。</x:v>
@@ -21101,7 +21101,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7977dad8fd6645e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra17d60bf792243b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22266,7 +22266,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf611e281df2443f1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R110a0b1237ef4333"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.4.0-20261001T040433Z][TM-004] Freeze reader CORE cases and sync workbook
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Ra34cb97649fe4064"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Ra70c794b2e164466"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rfb3048600da248a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R7e5a4ada29ae4937"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Re2b75bfe9fed4bc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rb81226098b1e4536"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Re24460cc44ea476b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R18122656c3bd40c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R93ce1a3f21084943"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Rbacb2c3887dc4b14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R363d3736582d4f08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R37ace6a3945f47b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rceed6940fe764674"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R84b4961f62504997"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R6a82d18c33fc49e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R7bc52af645e44234"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R6c9210257dd648a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R9f2c216a24f34eba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Rd412b793cfec432a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R5eba53e2586c47e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R539ced6782444afc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Rc0c3595293ea42bc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -755,8 +755,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N267" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N267"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N270" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N270"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="功能编号"/>
     <x:tableColumn id="2" name="用例编号"/>
@@ -1101,8 +1101,8 @@
         <x:v>已登记用例</x:v>
       </x:c>
       <x:c r="B8" s="11" t="n">
-        <x:f>COUNTA('05测试用例'!B5:B267)</x:f>
-        <x:v>263</x:v>
+        <x:f>COUNTA('05测试用例'!B5:B270)</x:f>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>父用例与具有稳定 ID 的变体各占一行；含未来概要场景</x:v>
@@ -1125,7 +1125,7 @@
         <x:v>细化产品用例</x:v>
       </x:c>
       <x:c r="B10" s="11" t="n">
-        <x:v>193</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
         <x:v>逐条结果按运行批次记录；稳定变体独立列出</x:v>
@@ -1255,7 +1255,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e400cb931d046ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc08057c18b414774"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1963,7 +1963,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re66a8b0da047414e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7630e691777f4a17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2112,7 +2112,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref49158206c0495c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R595d16cdd3e04f9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2547,7 +2547,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b318a29ab9c4d3d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9b039b9e42a452e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3594,7 +3594,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37d2691052f64f9a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc7e50be55244892"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4701,7 +4701,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ff245d7da434fbd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9144ed7a373426b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7486,7 +7486,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd75cc4e2fd4745e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76db2900f6da4213"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15735,7 +15735,7 @@
         <x:v>未来概要</x:v>
       </x:c>
       <x:c r="L176" s="9" t="str">
-        <x:v>docs/testing/cases/05-TM-005-usage-statistics.md:19</x:v>
+        <x:v>docs/testing/cases/05-TM-005-usage-statistics.md:21</x:v>
       </x:c>
       <x:c r="M176" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -15781,7 +15781,7 @@
         <x:v>未来概要</x:v>
       </x:c>
       <x:c r="L177" s="4" t="str">
-        <x:v>docs/testing/cases/05-TM-005-usage-statistics.md:36</x:v>
+        <x:v>docs/testing/cases/05-TM-005-usage-statistics.md:38</x:v>
       </x:c>
       <x:c r="M177" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -20061,30 +20061,175 @@
         <x:v>v0.5.0-20261001T034729Z</x:v>
       </x:c>
     </x:row>
+    <x:row r="268" ht="72" customHeight="1">
+      <x:c r="A268" s="9" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="B268" s="9" t="str">
+        <x:v>TC-TM004-CORE-01</x:v>
+      </x:c>
+      <x:c r="C268" s="9" t="str">
+        <x:v>完整LF、半行与限额续读</x:v>
+      </x:c>
+      <x:c r="D268" s="9" t="str">
+        <x:v>TASK-TM004-INCREMENTAL</x:v>
+      </x:c>
+      <x:c r="E268" s="9" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="F268" s="9" t="str">
+        <x:v>固定746字节13/7 assistant行、前半字节、两条不同ID完整行、首读上限754字节</x:v>
+      </x:c>
+      <x:c r="G268" s="9" t="str">
+        <x:v>1. 读未写完的前半行；调用0、偏移0、scanIncomplete=true，不作可信零结论
+2. 补齐LF、重复读取；补齐后一次13/7=20、偏移746、前缀MAC匹配；重复读取0调用且游标不变
+3. 两完整行首读754字节后续读；首读只第一条、偏移746、read_limit且未完成；续读只第二条、偏移为总字节长、完成</x:v>
+      </x:c>
+      <x:c r="H268" s="9" t="str">
+        <x:v>准备：无产品DB；每例新建自有临时文件
+变化：不适用；只返回模块调用、诊断与游标
+核验：固定fixture/行摘要和逐步返回值、前缀MAC及失败时无新游标；无SQL</x:v>
+      </x:c>
+      <x:c r="I268" s="9" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J268" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K268" s="9" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L268" s="9" t="str">
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:170</x:v>
+      </x:c>
+      <x:c r="M268" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N268" s="9" t="str">
+        <x:v>v0.4.0-20261001T040433Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="269" ht="72" customHeight="1">
+      <x:c r="A269" s="4" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="B269" s="4" t="str">
+        <x:v>TC-TM004-CORE-02</x:v>
+      </x:c>
+      <x:c r="C269" s="4" t="str">
+        <x:v>前缀MAC、变更和密钥失败</x:v>
+      </x:c>
+      <x:c r="D269" s="4" t="str">
+        <x:v>TASK-TM004-INCREMENTAL</x:v>
+      </x:c>
+      <x:c r="E269" s="4" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="F269" s="4" t="str">
+        <x:v>已提交首行，追加不同ID第二行、同长度ID改写并复原mtime、截短、身份改变、秘密缺失或错误</x:v>
+      </x:c>
+      <x:c r="G269" s="4" t="str">
+        <x:v>1. 首行后追加第二完整行；快照digest变化但稳定身份/前缀MAC相同，续读只第二调用，无cursor_reset
+2. 同长度前缀改写、截短及稳定身份变更；分别报cursor_reset并从0重扫；同inode/size/mtime也不能忽略MAC不符
+3. 秘密无效或读中源变化；拒绝且没有可提交新游标/可信调用/成功零；输出不含路径正文秘密</x:v>
+      </x:c>
+      <x:c r="H269" s="4" t="str">
+        <x:v>准备：无产品DB；每例新建自有临时文件
+变化：不适用；只返回模块调用、诊断与游标
+核验：固定fixture/行摘要和逐步返回值、前缀MAC及失败时无新游标；无SQL</x:v>
+      </x:c>
+      <x:c r="I269" s="4" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J269" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K269" s="4" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L269" s="4" t="str">
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:178</x:v>
+      </x:c>
+      <x:c r="M269" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N269" s="4" t="str">
+        <x:v>v0.4.0-20261001T040433Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="270" ht="57" customHeight="1">
+      <x:c r="A270" s="9" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="B270" s="9" t="str">
+        <x:v>TC-TM004-CORE-03</x:v>
+      </x:c>
+      <x:c r="C270" s="9" t="str">
+        <x:v>损坏完整行与未知结构</x:v>
+      </x:c>
+      <x:c r="D270" s="9" t="str">
+        <x:v>TASK-TM004-PARSER
+TASK-TM004-INCREMENTAL</x:v>
+      </x:c>
+      <x:c r="E270" s="9" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="F270" s="9" t="str">
+        <x:v>固定13/7行前置非法UTF8完整行和版本2.1.127完整行，尾部再追加无LF坏字节</x:v>
+      </x:c>
+      <x:c r="G270" s="9" t="str">
+        <x:v>1. 读三条完整LF行；仅合法2.1.126一条调用13/7=20；invalid_utf8及unsupported_version各一次
+2. 核对游标、重复读取及隐私；游标到三行LF末，MAC匹配且完成；重复读取0；输出无路径、正文、秘密
+3. 追加无LF坏字节再补LF；未补LF前偏移不动且未完成；补LF后仅诊断推进，无伪调用</x:v>
+      </x:c>
+      <x:c r="H270" s="9" t="str">
+        <x:v>准备：无产品DB；每例新建自有临时文件
+变化：不适用；只返回模块调用、诊断与游标
+核验：固定fixture/行摘要和逐步返回值、前缀MAC及失败时无新游标；无SQL</x:v>
+      </x:c>
+      <x:c r="I270" s="9" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J270" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K270" s="9" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L270" s="9" t="str">
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:186</x:v>
+      </x:c>
+      <x:c r="M270" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N270" s="9" t="str">
+        <x:v>v0.4.0-20261001T040433Z</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G5:G267">
+  <x:conditionalFormatting sqref="G5:G270">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="I5:I267">
+  <x:conditionalFormatting sqref="I5:I270">
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="16" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="17" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="J5:J267">
+  <x:conditionalFormatting sqref="J5:J270">
     <x:cfRule type="containsText" dxfId="18" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="19" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="20" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M267">
+  <x:conditionalFormatting sqref="M5:M270">
     <x:cfRule type="containsText" dxfId="21" priority="10" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="22" priority="11" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="23" priority="12" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8f0538f57bf4f6c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf20fbd45b564c07"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20657,7 +20802,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55c211e1a3b04821"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad61b66a93d64781"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21000,7 +21145,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J9" s="4" t="str">
-        <x:v>整版draft、未发布。8 TASK、20细TC及四组摘要已登记；纯内存Claude 2.1.126解析器f2c3972覆盖已验证主会话、复制fork、同ID双块及可核实单层Agent，单元36/36、治理452/452PASS。改写UUID、fork-context-ref、嵌套Agent、有效零及授权/身份/SQLite仍缺证据或集成；20条产品TC未执行，正式发行完整门禁NOT_RUN。</x:v>
+        <x:v>整版draft、未发布。原20产品细TC及四组摘要保留，新增3条已打开只读句柄的reader CORE辅助TC，固定LF、前缀MAC/重扫和损坏行输入，切片检查未完成。开发树模块红0/3与绿3/3仅是交接证据，且代码未形成干净提交；产品授权、稳定文件身份、SQLite原子事务、IPC/App E2E未验证，正式发行门禁NOT_RUN。</x:v>
       </x:c>
       <x:c r="K9" s="4" t="str">
         <x:v>TM004源分支原生零/缺失与nested Agent定向探针仅为研究证据；0.3及此前稳定原包尚未形成，真实升级BLOCKED。</x:v>
@@ -21101,7 +21246,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra17d60bf792243b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c2f4c5085bc46f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22266,7 +22411,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R110a0b1237ef4333"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73a7e994b1c249cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.3.0-20261001T034652Z][TM-000] Sync module result SOP with documentation and workbook
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R37ace6a3945f47b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rceed6940fe764674"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R84b4961f62504997"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R6a82d18c33fc49e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R7bc52af645e44234"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R6c9210257dd648a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R9f2c216a24f34eba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Rd412b793cfec432a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R5eba53e2586c47e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R539ced6782444afc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Rc0c3595293ea42bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Ra6f210bcb0454295"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R79f1b1bb8c7d4c88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R169ebc8165914139"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rcdd98965e7164734"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R670eb371060f4511"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R216314e6083e425e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R50b9ebef16624a75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R8ac6150839b04d13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rbb98a582fe514638"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R50d19ea48f5644bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R64aaf28c83be4b22"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1255,7 +1255,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc08057c18b414774"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re175f6a10d684b84"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1611,7 +1611,7 @@
         <x:v>已基线</x:v>
       </x:c>
       <x:c r="G16" s="9" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="H16" s="9" t="str">
         <x:v>sop/SOP-011-test-implementation.md</x:v>
@@ -1657,13 +1657,13 @@
         <x:v>012实现、009本机运行时和锁文件就绪。</x:v>
       </x:c>
       <x:c r="E18" s="9" t="str">
-        <x:v>构建物和基础原始结果或精确缺项。</x:v>
+        <x:v>构建物、基础及固定模块TC原始结果、独立批次Excel和导出收据，或精确缺项。</x:v>
       </x:c>
       <x:c r="F18" s="9" t="str">
         <x:v>已基线</x:v>
       </x:c>
       <x:c r="G18" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H18" s="9" t="str">
         <x:v>sop/SOP-013-build-and-check.md</x:v>
@@ -1689,7 +1689,7 @@
         <x:v>已基线</x:v>
       </x:c>
       <x:c r="G19" s="4" t="n">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="H19" s="4" t="str">
         <x:v>sop/SOP-014-e2e.md</x:v>
@@ -1949,7 +1949,7 @@
         <x:v>已基线</x:v>
       </x:c>
       <x:c r="G29" s="4" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H29" s="4" t="str">
         <x:v>sop/SOP-024-document-change.md</x:v>
@@ -1963,7 +1963,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7630e691777f4a17"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01d20f25691a4d3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2112,7 +2112,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R595d16cdd3e04f9f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d4100c370ca43ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2547,7 +2547,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9b039b9e42a452e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58ce105b0ad34683"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3594,7 +3594,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc7e50be55244892"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcea4c46319904a25"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4701,7 +4701,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9144ed7a373426b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57f6c1e9dfc540fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7486,7 +7486,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76db2900f6da4213"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R865e9e7bfd724203"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20229,7 +20229,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf20fbd45b564c07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafe0914c2e5f4e3d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20802,7 +20802,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad61b66a93d64781"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a1d865dd2024f4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21060,7 +21060,7 @@
         <x:v>releases/v0.2.0-20261001T034118Z/01-requirements.md:32</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="132" customHeight="1">
+    <x:row r="8" ht="192" customHeight="1">
       <x:c r="A8" s="9" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
       </x:c>
@@ -21089,7 +21089,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J8" s="9" t="str">
-        <x:v>整版draft、未发布。27条产品TC未执行；3条CORE辅助TC已在文档提交48ca089独立切片就绪，在开发分支311deedf运行模块3/3 PASS，原始receipt在该分支.local/ci/tm003-core-20261001/。代码尚未合入本文档树，机器绑定保持空；模块报告不能作为产品E2E或发行门禁，结果Excel规范待SOP修订。</x:v>
+        <x:v>整版draft、未发布。27条产品TC未执行；3条CORE辅助TC已在文档提交48ca089独立切片就绪，在开发分支311deedf运行模块3/3 PASS，原始receipt在该分支.local/ci/tm003-core-20261001/。代码尚未合入本文档树，机器绑定保持空；模块报告不能作为产品E2E或发行门禁，结果Excel规范待SOP修订。 2026-10-02新代码候选44379e6已有逐步模块3/3与桌面29/29/typecheck/build原件；source_check独立Excel导出程序仍缺，批次登记BLOCKED，产品E2E仍NOT_RUN。</x:v>
       </x:c>
       <x:c r="K8" s="9" t="str">
         <x:v>TM-001 干净源码候选为技术基底；其产品门禁不继承给TM-003</x:v>
@@ -21172,7 +21172,7 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="162" customHeight="1">
+    <x:row r="10" ht="237" customHeight="1">
       <x:c r="A10" s="9" t="str">
         <x:v>v0.5.0-20261001T034729Z</x:v>
       </x:c>
@@ -21201,7 +21201,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J10" s="9" t="str">
-        <x:v>整版draft、未发布。原32条产品父TC、6稳定变体和两组摘要保留；纯统计CORE-01/02/03辅助TC在输入提交061c759后，经SOP-008内容核对及结构/治理457项PASS，独立切片development_slice_ready，程序绑定仍为空、模块实际运行unexecuted。静态oracle与切片就绪不证明真实双来源采集或产品E2E；固定产品数据、SQLite/IPC、安装App逐TC绑定未完成，正式发行完整门禁NOT_RUN。</x:v>
+        <x:v>整版draft、未发布。原32条产品父TC、6稳定变体和两组摘要保留；纯统计CORE-01/02/03辅助TC在输入提交061c759后，经SOP-008内容核对及结构/治理457项PASS，独立切片development_slice_ready，程序绑定仍为空、模块实际运行unexecuted。静态oracle与切片就绪不证明真实双来源采集或产品E2E；固定产品数据、SQLite/IPC、安装App逐TC绑定未完成，正式发行完整门禁NOT_RUN。 独立代码提交6a0f6f的source_check CORE3/3、桌面29/29、build PASS，原件在TM005工作树.local/tm005-core-postcommit-20261001T162401Z；程序尚未进入本文档树、模块Excel导出/批次登记BLOCKED，产品E2E仍NOT_RUN。</x:v>
       </x:c>
       <x:c r="K10" s="9" t="str">
         <x:v>TM005语义oracle只验证规范化样例；0.4及此前稳定原包尚未形成，真实升级BLOCKED。</x:v>
@@ -21246,7 +21246,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c2f4c5085bc46f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raad3cfddeeb34401"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22411,7 +22411,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73a7e994b1c249cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31d38ae98c06435d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.3.0-20261001T034652Z][TM-000] Index verified module runs and sync live documentation
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Ra6f210bcb0454295"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R79f1b1bb8c7d4c88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R169ebc8165914139"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rcdd98965e7164734"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R670eb371060f4511"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R216314e6083e425e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R50b9ebef16624a75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R8ac6150839b04d13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rbb98a582fe514638"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R50d19ea48f5644bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R64aaf28c83be4b22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Rbf12aa18b3554001"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R0df86ad125c847cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rb1d655ac537243bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R02ea4983c9c44775"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rcf6a862be63b4235"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R2503d345bbf645c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rb9fac209113c41ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R929989622c2e47b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rabd4aa5c6f0f4350"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R63d60e02ad764d31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R79b31b47b30a4cc3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -152,7 +152,38 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="45">
+  <x:dxfs count="48">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9A201B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFDE8E7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF754E00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CD"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF754E00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF6DF"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
@@ -778,21 +809,23 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:L17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:L17"/>
-  <x:tableColumns count="12">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N19"/>
+  <x:tableColumns count="14">
     <x:tableColumn id="1" name="运行批次"/>
     <x:tableColumn id="2" name="版本"/>
-    <x:tableColumn id="3" name="范围"/>
-    <x:tableColumn id="4" name="结果"/>
-    <x:tableColumn id="5" name="父用例/场景数"/>
-    <x:tableColumn id="6" name="通过数"/>
-    <x:tableColumn id="7" name="失败数"/>
-    <x:tableColumn id="8" name="阻塞数"/>
-    <x:tableColumn id="9" name="候选提交"/>
-    <x:tableColumn id="10" name="发布资格"/>
-    <x:tableColumn id="11" name="批次摘要"/>
-    <x:tableColumn id="12" name="独立结果Excel（本机）"/>
+    <x:tableColumn id="3" name="执行类型"/>
+    <x:tableColumn id="4" name="范围"/>
+    <x:tableColumn id="5" name="结果"/>
+    <x:tableColumn id="6" name="父用例/场景数"/>
+    <x:tableColumn id="7" name="通过数"/>
+    <x:tableColumn id="8" name="失败数"/>
+    <x:tableColumn id="9" name="阻塞数"/>
+    <x:tableColumn id="10" name="候选提交"/>
+    <x:tableColumn id="11" name="发布资格"/>
+    <x:tableColumn id="12" name="批次摘要"/>
+    <x:tableColumn id="13" name="独立结果Excel（本机）"/>
+    <x:tableColumn id="14" name="产品E2E状态"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1113,8 +1146,8 @@
         <x:v>测试批次</x:v>
       </x:c>
       <x:c r="B9" s="10" t="n">
-        <x:f>COUNTA('06测试批次'!A5:A17)</x:f>
-        <x:v>13</x:v>
+        <x:f>COUNTA('06测试批次'!A5:A19)</x:f>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>06测试批次，每次运行一行，记录独立结果Excel位置</x:v>
@@ -1125,7 +1158,7 @@
         <x:v>细化产品用例</x:v>
       </x:c>
       <x:c r="B10" s="11" t="n">
-        <x:v>196</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
         <x:v>逐条结果按运行批次记录；稳定变体独立列出</x:v>
@@ -1136,7 +1169,7 @@
         <x:v>界面与治理检查</x:v>
       </x:c>
       <x:c r="B11" s="10" t="n">
-        <x:v>41</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C11" s="4" t="str">
         <x:v>辅助检查不能替代产品E2E；稳定变体独立列出</x:v>
@@ -1235,10 +1268,10 @@
         <x:v>最近登记批次</x:v>
       </x:c>
       <x:c r="B20" s="9" t="str">
-        <x:v>FAIL</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>本地master固定候选最终包首次精细门禁：固定本地master候选门禁FAIL；原始116项91 PASS/14 FAIL/11 BLOCKED，UPDATE-05父项与13变体缺签名输入。逐例模型78父TC 66 PASS/1 FAIL/11 BLOCKED，38变体25 PASS/13 FAIL；无正式稳定包。；是否覆盖完整回归以批次范围和原始证据为准。</x:v>
+        <x:v>source_check · TM-003 CORE-01/02/03 固定模块验证；非产品E2E：共享source_check清理合同扩展后的新候选：CORE固定3/3、九步PASS，owned_root清理逐例PASS；独立Excel/verification回读PASS。旧ea6b187批次保留；原27条产品TC与正式发行仍NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
@@ -1255,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re175f6a10d684b84"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25d759ba0397462f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1957,13 +1990,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F5:F29">
-    <x:cfRule type="containsText" dxfId="42" priority="1" operator="containsText" text="FAIL"/>
-    <x:cfRule type="containsText" dxfId="43" priority="2" operator="containsText" text="预期待明确"/>
-    <x:cfRule type="containsText" dxfId="44" priority="3" operator="containsText" text="未执行"/>
+    <x:cfRule type="containsText" dxfId="45" priority="1" operator="containsText" text="FAIL"/>
+    <x:cfRule type="containsText" dxfId="46" priority="2" operator="containsText" text="预期待明确"/>
+    <x:cfRule type="containsText" dxfId="47" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01d20f25691a4d3c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R569059b8ca0b4736"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2112,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d4100c370ca43ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6025bfdd02894eb7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2547,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58ce105b0ad34683"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf28121b6afbb43f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3594,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcea4c46319904a25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9e3695a17444599"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4701,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57f6c1e9dfc540fa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89bf59096c52401f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7486,7 +7519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R865e9e7bfd724203"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf24b92a7a9c4ba9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13395,15 +13428,13 @@
         <x:v>安全单元</x:v>
       </x:c>
       <x:c r="F127" s="4" t="str">
-        <x:v>七个独立变体：四个恶意 IPC 参数分别为 B 绝对路径、B 的 file:// URL、../B/sessions/2026/10/01/b-01.jsonl、伪造 selectionId 00000000-0000-4000-8000-000000000099；三个受控竞态为过期选择、撤销期间刷新、切换账号期间刷新。全部只用自有 A/B 与同一主进程业务代码。</x:v>
+        <x:v>七个独立变体：B路径攻击使用独占短根R=/tmp/t2-&lt;8位十六进制&gt;、R/A/a.jsonl与R/B/b.jsonl；ABSOLUTE/FILE_URL/DOTDOT分别调用tokenmeter:invoke(previewSource,{selectionId:B绝对路径/file URL/../B/b.jsonl})，TOKEN调用同method并传未签发UUID；三竞态保持原输入。路径字串事前断言≤64，仅本例拥有A/B。</x:v>
       </x:c>
       <x:c r="G127" s="4" t="str">
-        <x:v>测试 UI 不适用，原因是本例为主进程参数安全层；A/B 文件未被读取，无网络/DB 操作。
-主进程返回安全错误码，不返回内容、绝对路径或 locator；不存在 renderer 任意文件读取 API，A/B open/read=0、B 元数据访问=0；无网络/DB 操作。
-四个恶意参数变体均未确认来源、未修改 A/B 字节；分别保存脱敏错误码和文件审计，不记录路径或 token；无网络/DB 操作。</x:v>
+        <x:v>ABSOLUTE/FILE_URL/DOTDOT/TOKEN均调用previewSource.selectionId，返回snapshot.error=invalid_selection且不打开A/B、无来源状态变化；竞态变体沿既定屏障判据。</x:v>
       </x:c>
       <x:c r="H127" s="4" t="str">
-        <x:v>准备：七变体各自 R 与独立 A/B/profile；仅内存主进程 handler、受控异步屏障和隔离文件；无服务/DB，SQL 不适用。四恶意参数安全拒绝，三竞态过期结果不提交。
+        <x:v>准备：七变体各自短根R=/tmp/t2-&lt;8位十六进制&gt;、A/B/profile及owner marker；恶意字串≤64，实际业务previewSource IPC、受控异步屏障和隔离文件；无服务/DB，SQL不适用。
 变化：不适用：辅助检查不写服务业务库。
 核验：不适用：本例按内存输入、自有副本或原始结果核验，没有 DB 连接或 SQL。</x:v>
       </x:c>
@@ -13443,13 +13474,13 @@
         <x:v>安全单元</x:v>
       </x:c>
       <x:c r="F128" s="9" t="str">
-        <x:v>renderer传B绝对路径</x:v>
+        <x:v>tokenmeter:invoke('previewSource',{selectionId:R+'/B/b.jsonl'})；R=/tmp/t2-&lt;8位十六进制&gt;独占短根，输入≤64字符</x:v>
       </x:c>
       <x:c r="G128" s="9" t="str">
-        <x:v>主进程安全拒绝，不返回内容、绝对路径或 locator；B 元数据/open/read=0，sources 无确认记录。</x:v>
+        <x:v>snapshot.error=invalid_selection；无pending/confirmed变化，不返回路径/locator/正文；A/B open/read=0、B metadata=0</x:v>
       </x:c>
       <x:c r="H128" s="9" t="str">
-        <x:v>准备：七变体各自 R 与独立 A/B/profile；仅内存主进程 handler、受控异步屏障和隔离文件；无服务/DB，SQL 不适用。四恶意参数安全拒绝，三竞态过期结果不提交。
+        <x:v>准备：七变体各自短根R=/tmp/t2-&lt;8位十六进制&gt;、A/B/profile及owner marker；恶意字串≤64，实际业务previewSource IPC、受控异步屏障和隔离文件；无服务/DB，SQL不适用。
 变化：不适用：辅助检查不写服务业务库。
 核验：不适用：本例按内存输入、自有副本或原始结果核验，没有 DB 连接或 SQL。</x:v>
       </x:c>
@@ -13489,13 +13520,13 @@
         <x:v>安全单元</x:v>
       </x:c>
       <x:c r="F129" s="4" t="str">
-        <x:v>renderer传指向B的file:// URL</x:v>
+        <x:v>tokenmeter:invoke('previewSource',{selectionId:pathToFileURL(R+'/B/b.jsonl').href})；R=/tmp/t2-&lt;8位十六进制&gt;独占短根，输入≤64字符</x:v>
       </x:c>
       <x:c r="G129" s="4" t="str">
-        <x:v>主进程安全拒绝，不返回内容、绝对路径或 locator；B 元数据/open/read=0，sources 无确认记录。</x:v>
+        <x:v>snapshot.error=invalid_selection；无pending/confirmed变化，不返回路径/locator/正文；A/B open/read=0、B metadata=0</x:v>
       </x:c>
       <x:c r="H129" s="4" t="str">
-        <x:v>准备：七变体各自 R 与独立 A/B/profile；仅内存主进程 handler、受控异步屏障和隔离文件；无服务/DB，SQL 不适用。四恶意参数安全拒绝，三竞态过期结果不提交。
+        <x:v>准备：七变体各自短根R=/tmp/t2-&lt;8位十六进制&gt;、A/B/profile及owner marker；恶意字串≤64，实际业务previewSource IPC、受控异步屏障和隔离文件；无服务/DB，SQL不适用。
 变化：不适用：辅助检查不写服务业务库。
 核验：不适用：本例按内存输入、自有副本或原始结果核验，没有 DB 连接或 SQL。</x:v>
       </x:c>
@@ -13535,13 +13566,13 @@
         <x:v>安全单元</x:v>
       </x:c>
       <x:c r="F130" s="9" t="str">
-        <x:v>renderer传../B/sessions/2026/10/01/b-01.jsonl</x:v>
+        <x:v>tokenmeter:invoke('previewSource',{selectionId:'../B/b.jsonl'})；R=/tmp/t2-&lt;8位十六进制&gt;独占短根，输入≤64字符</x:v>
       </x:c>
       <x:c r="G130" s="9" t="str">
-        <x:v>主进程安全拒绝，不返回内容、绝对路径或 locator；B 元数据/open/read=0，sources 无确认记录。</x:v>
+        <x:v>snapshot.error=invalid_selection；无pending/confirmed变化，不返回路径/locator/正文；A/B open/read=0、B metadata=0</x:v>
       </x:c>
       <x:c r="H130" s="9" t="str">
-        <x:v>准备：七变体各自 R 与独立 A/B/profile；仅内存主进程 handler、受控异步屏障和隔离文件；无服务/DB，SQL 不适用。四恶意参数安全拒绝，三竞态过期结果不提交。
+        <x:v>准备：七变体各自短根R=/tmp/t2-&lt;8位十六进制&gt;、A/B/profile及owner marker；恶意字串≤64，实际业务previewSource IPC、受控异步屏障和隔离文件；无服务/DB，SQL不适用。
 变化：不适用：辅助检查不写服务业务库。
 核验：不适用：本例按内存输入、自有副本或原始结果核验，没有 DB 连接或 SQL。</x:v>
       </x:c>
@@ -13587,7 +13618,7 @@
         <x:v>主进程安全拒绝，不返回内容、绝对路径或 locator；B 元数据/open/read=0，sources 无确认记录。</x:v>
       </x:c>
       <x:c r="H131" s="4" t="str">
-        <x:v>准备：七变体各自 R 与独立 A/B/profile；仅内存主进程 handler、受控异步屏障和隔离文件；无服务/DB，SQL 不适用。四恶意参数安全拒绝，三竞态过期结果不提交。
+        <x:v>准备：七变体各自短根R=/tmp/t2-&lt;8位十六进制&gt;、A/B/profile及owner marker；恶意字串≤64，实际业务previewSource IPC、受控异步屏障和隔离文件；无服务/DB，SQL不适用。
 变化：不适用：辅助检查不写服务业务库。
 核验：不适用：本例按内存输入、自有副本或原始结果核验，没有 DB 连接或 SQL。</x:v>
       </x:c>
@@ -13633,7 +13664,7 @@
         <x:v>旧 Alice 结果拒绝，Bob 不得建暂选/确认 A；Alice/Bob 无新增来源，A/B 零读取。</x:v>
       </x:c>
       <x:c r="H132" s="9" t="str">
-        <x:v>准备：七变体各自 R 与独立 A/B/profile；仅内存主进程 handler、受控异步屏障和隔离文件；无服务/DB，SQL 不适用。四恶意参数安全拒绝，三竞态过期结果不提交。
+        <x:v>准备：七变体各自短根R=/tmp/t2-&lt;8位十六进制&gt;、A/B/profile及owner marker；恶意字串≤64，实际业务previewSource IPC、受控异步屏障和隔离文件；无服务/DB，SQL不适用。
 变化：不适用：辅助检查不写服务业务库。
 核验：不适用：本例按内存输入、自有副本或原始结果核验，没有 DB 连接或 SQL。</x:v>
       </x:c>
@@ -13679,7 +13710,7 @@
         <x:v>撤销删密文和读取能力，旧 Promise 不提交候选或 complete=true；撤销后 A/B 后续操作为零。</x:v>
       </x:c>
       <x:c r="H133" s="4" t="str">
-        <x:v>准备：七变体各自 R 与独立 A/B/profile；仅内存主进程 handler、受控异步屏障和隔离文件；无服务/DB，SQL 不适用。四恶意参数安全拒绝，三竞态过期结果不提交。
+        <x:v>准备：七变体各自短根R=/tmp/t2-&lt;8位十六进制&gt;、A/B/profile及owner marker；恶意字串≤64，实际业务previewSource IPC、受控异步屏障和隔离文件；无服务/DB，SQL不适用。
 变化：不适用：辅助检查不写服务业务库。
 核验：不适用：本例按内存输入、自有副本或原始结果核验，没有 DB 连接或 SQL。</x:v>
       </x:c>
@@ -13725,7 +13756,7 @@
         <x:v>Bob 不得见旧 Alice 候选或得到来源；切换后 A/B 后续零访问；Bob 请求 Alice 来源 ID 被拒绝。</x:v>
       </x:c>
       <x:c r="H134" s="9" t="str">
-        <x:v>准备：七变体各自 R 与独立 A/B/profile；仅内存主进程 handler、受控异步屏障和隔离文件；无服务/DB，SQL 不适用。四恶意参数安全拒绝，三竞态过期结果不提交。
+        <x:v>准备：七变体各自短根R=/tmp/t2-&lt;8位十六进制&gt;、A/B/profile及owner marker；恶意字串≤64，实际业务previewSource IPC、受控异步屏障和隔离文件；无服务/DB，SQL不适用。
 变化：不适用：辅助检查不写服务业务库。
 核验：不适用：本例按内存输入、自有副本或原始结果核验，没有 DB 连接或 SQL。</x:v>
       </x:c>
@@ -18485,7 +18516,7 @@
         <x:v>TASK-TM003-SOURCE</x:v>
       </x:c>
       <x:c r="E235" s="4" t="str">
-        <x:v>source_check</x:v>
+        <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F235" s="4" t="str">
         <x:v>1. 对照本版声明的 CLI build、官方结构与 sessions/YYYY/MM/DD/*.jsonl 受控原生样例→样例有 session_meta.id、token_usage_record.payload.response_id/usage，版本和 SHA 有记录。2. 换一个未声明 build→该 build 不列为已支持，显示 unsupported_source_version。</x:v>
@@ -18772,7 +18803,7 @@
         <x:v>TASK-TM003-SOURCE</x:v>
       </x:c>
       <x:c r="E241" s="4" t="str">
-        <x:v>source_check</x:v>
+        <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F241" s="4" t="str">
         <x:v>1. 输入只有 event_msg.token_count.info.total_token_usage=100/10 且无 response_id→诊断 unverified_cumulative、可信事件0。2. 加 rate-limit-only 的 info=null→诊断 missing_usage，不生成0值用量事件。</x:v>
@@ -19012,7 +19043,7 @@
         <x:v>TASK-TM003-IDENTITY</x:v>
       </x:c>
       <x:c r="E246" s="9" t="str">
-        <x:v>source_check</x:v>
+        <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F246" s="9" t="str">
         <x:v>本例私有 schema 与tests/fixtures/tm004/identity-v1-vectors.json 中的公开测试 HMAC key（仅固定向量，绝不进入产品 profile）；标准事件 Codex provider-response/shared-call-01=100/10/cached20，Claude provider-message/shared-call-01=30/3/cached0；随后同 Codex 事件重放、另一 Agent 无复制链同 Claude ID 重用、同 Codex ID 但用量或模型冲突。</x:v>
@@ -19784,7 +19815,7 @@
         <x:v>TASK-TM003-PARSE</x:v>
       </x:c>
       <x:c r="E262" s="9" t="str">
-        <x:v>source_check</x:v>
+        <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F262" s="9" t="str">
         <x:v>原生形状完整A=100/10/cached20；B=200/20/cached40半行后补LF；C=300/30/cached60完整行及累计快照；固定种子和T0。</x:v>
@@ -19803,7 +19834,7 @@
         <x:v>draft</x:v>
       </x:c>
       <x:c r="J262" s="9" t="str">
-        <x:v>未执行</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="K262" s="9" t="str">
         <x:v>细化用例</x:v>
@@ -19812,7 +19843,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:315</x:v>
       </x:c>
       <x:c r="M262" s="9" t="str">
-        <x:v>尚未执行</x:v>
+        <x:v>tm003-core-20261001T165439Z (source_check；产品E2E未运行)</x:v>
       </x:c>
       <x:c r="N262" s="9" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -19833,7 +19864,7 @@
 TASK-TM003-PARSE</x:v>
       </x:c>
       <x:c r="E263" s="4" t="str">
-        <x:v>source_check</x:v>
+        <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F263" s="4" t="str">
         <x:v>无ID累计100/10和rate-limit info=null；合法A；缺usage、负input、cached111&gt;input100、total111四条不同ID完整LF行；未知build。</x:v>
@@ -19852,7 +19883,7 @@
         <x:v>draft</x:v>
       </x:c>
       <x:c r="J263" s="4" t="str">
-        <x:v>未执行</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="K263" s="4" t="str">
         <x:v>细化用例</x:v>
@@ -19861,7 +19892,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:319</x:v>
       </x:c>
       <x:c r="M263" s="4" t="str">
-        <x:v>尚未执行</x:v>
+        <x:v>tm003-core-20261001T165439Z (source_check；产品E2E未运行)</x:v>
       </x:c>
       <x:c r="N263" s="4" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -19881,7 +19912,7 @@
         <x:v>TASK-TM003-IDENTITY</x:v>
       </x:c>
       <x:c r="E264" s="9" t="str">
-        <x:v>source_check</x:v>
+        <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F264" s="9" t="str">
         <x:v>公开identity-v1测试key；codex/provider-response/shared-call-01的A=100/10/cached20；同ID重放；shared-call-02同usage；shared-call-01冲突999/99；claude_code/provider-message/shared-call-01仅求键。</x:v>
@@ -19900,7 +19931,7 @@
         <x:v>draft</x:v>
       </x:c>
       <x:c r="J264" s="9" t="str">
-        <x:v>未执行</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="K264" s="9" t="str">
         <x:v>细化用例</x:v>
@@ -19909,13 +19940,13 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:323</x:v>
       </x:c>
       <x:c r="M264" s="9" t="str">
-        <x:v>尚未执行</x:v>
+        <x:v>tm003-core-20261001T165439Z (source_check；产品E2E未运行)</x:v>
       </x:c>
       <x:c r="N264" s="9" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="265" ht="72" customHeight="1">
+    <x:row r="265" ht="87" customHeight="1">
       <x:c r="A265" s="4" t="str">
         <x:v>TM-005</x:v>
       </x:c>
@@ -19930,13 +19961,13 @@
 TASK-TM005-RANGE-QUERY</x:v>
       </x:c>
       <x:c r="E265" s="4" t="str">
-        <x:v>source_check</x:v>
+        <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F265" s="4" t="str">
         <x:v>fixture的A/B、跨主体C、界外D/E；synthetic-p1、Asia/Shanghai当地日2026-09-29</x:v>
       </x:c>
       <x:c r="G265" s="4" t="str">
-        <x:v>1. 按固定主体/当地日查询纯统计函数；仅A/B被选、C/D/E排除；输入数组和键不变
+        <x:v>1. 按固定主体和fixture固定UTC半开界查询纯统计函数，不做IANA日期换算；仅A/B被选、C/D/E排除；输入数组和键不变
 2. 核对来源、模型、Token和三个子项；input300/output30/total330；Codex110/Claude220；未知模型110/sonnet-test220；缓存读20但部分未知、缓存写未知、推理2但部分未知，子项不加总
 3. 逐个输入非法来源、负数、超范围缓存和坏UTC；各自被拒绝，无完整零或有效汇总输出；原fixture不变</x:v>
       </x:c>
@@ -19979,7 +20010,7 @@
 TASK-TM005-COVERAGE</x:v>
       </x:c>
       <x:c r="E266" s="9" t="str">
-        <x:v>source_check</x:v>
+        <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F266" s="9" t="str">
         <x:v>fixture A/B及同范围Claude missing_usage诊断；双来源complete仅为模块合成覆盖假设</x:v>
@@ -20027,7 +20058,7 @@
         <x:v>TASK-TM005-COVERAGE</x:v>
       </x:c>
       <x:c r="E267" s="4" t="str">
-        <x:v>source_check</x:v>
+        <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F267" s="4" t="str">
         <x:v>fixture五行coverage_algebra；complete仅为模块合成输入，product_coverage_proven=false</x:v>
@@ -20075,7 +20106,7 @@
         <x:v>TASK-TM004-INCREMENTAL</x:v>
       </x:c>
       <x:c r="E268" s="9" t="str">
-        <x:v>source_check</x:v>
+        <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F268" s="9" t="str">
         <x:v>固定746字节13/7 assistant行、前半字节、两条不同ID完整行、首读上限754字节</x:v>
@@ -20123,7 +20154,7 @@
         <x:v>TASK-TM004-INCREMENTAL</x:v>
       </x:c>
       <x:c r="E269" s="4" t="str">
-        <x:v>source_check</x:v>
+        <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F269" s="4" t="str">
         <x:v>已提交首行，追加不同ID第二行、同长度ID改写并复原mtime、截短、身份改变、秘密缺失或错误</x:v>
@@ -20172,7 +20203,7 @@
 TASK-TM004-INCREMENTAL</x:v>
       </x:c>
       <x:c r="E270" s="9" t="str">
-        <x:v>source_check</x:v>
+        <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F270" s="9" t="str">
         <x:v>固定13/7行前置非法UTF8完整行和版本2.1.127完整行，尾部再追加无LF坏字节</x:v>
@@ -20229,7 +20260,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafe0914c2e5f4e3d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53d132cdb12b4b3f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20240,21 +20271,23 @@
   <x:cols>
     <x:col min="1" max="1" width="55" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="52" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="43" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="55" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="95" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="55" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="95" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="95" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="2">
       <x:c r="A2" s="1" t="str">
-        <x:v>测试批次索引 · 详细结果单独保存</x:v>
+        <x:v>测试批次索引 · 模块与产品结果分别计数</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
@@ -20265,34 +20298,40 @@
         <x:v>版本</x:v>
       </x:c>
       <x:c r="C4" s="8" t="str">
+        <x:v>执行类型</x:v>
+      </x:c>
+      <x:c r="D4" s="8" t="str">
         <x:v>范围</x:v>
       </x:c>
-      <x:c r="D4" s="8" t="str">
+      <x:c r="E4" s="8" t="str">
         <x:v>结果</x:v>
       </x:c>
-      <x:c r="E4" s="8" t="str">
+      <x:c r="F4" s="8" t="str">
         <x:v>父用例/场景数</x:v>
       </x:c>
-      <x:c r="F4" s="8" t="str">
+      <x:c r="G4" s="8" t="str">
         <x:v>通过数</x:v>
       </x:c>
-      <x:c r="G4" s="8" t="str">
+      <x:c r="H4" s="8" t="str">
         <x:v>失败数</x:v>
       </x:c>
-      <x:c r="H4" s="8" t="str">
+      <x:c r="I4" s="8" t="str">
         <x:v>阻塞数</x:v>
       </x:c>
-      <x:c r="I4" s="8" t="str">
+      <x:c r="J4" s="8" t="str">
         <x:v>候选提交</x:v>
       </x:c>
-      <x:c r="J4" s="8" t="str">
+      <x:c r="K4" s="8" t="str">
         <x:v>发布资格</x:v>
       </x:c>
-      <x:c r="K4" s="8" t="str">
+      <x:c r="L4" s="8" t="str">
         <x:v>批次摘要</x:v>
       </x:c>
-      <x:c r="L4" s="8" t="str">
+      <x:c r="M4" s="8" t="str">
         <x:v>独立结果Excel（本机）</x:v>
+      </x:c>
+      <x:c r="N4" s="8" t="str">
+        <x:v>产品E2E状态</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
@@ -20303,34 +20342,40 @@
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
       <x:c r="C5" s="4" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="str">
         <x:v>开发包诊断 / dirty</x:v>
       </x:c>
-      <x:c r="D5" s="4" t="str">
+      <x:c r="E5" s="4" t="str">
         <x:v>FAIL</x:v>
       </x:c>
-      <x:c r="E5" s="4" t="n">
+      <x:c r="F5" s="4" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="F5" s="4" t="n">
+      <x:c r="G5" s="4" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G5" s="4" t="n">
+      <x:c r="H5" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H5" s="4" t="n">
+      <x:c r="I5" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I5" s="4" t="str">
+      <x:c r="J5" s="4" t="str">
         <x:v>6e80dd12d60ee5dad641bca030445a2153a269c9</x:v>
       </x:c>
-      <x:c r="J5" s="4" t="str">
+      <x:c r="K5" s="4" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="K5" s="4" t="str">
+      <x:c r="L5" s="4" t="str">
         <x:v>六个历史聚合场景，升级004失败；不回填新增TC。结果表修订02修正时间显示，原表和测试证据保留；未新增测试运行。</x:v>
       </x:c>
-      <x:c r="L5" s="4" t="str">
+      <x:c r="M5" s="4" t="str">
         <x:v>.local/test-results/local-a1b2c3d4e5f60718293a4b5c6d7e8f94/revisions/02/TokenMeter测试结果-local-a1b2c3d4e5f60718293a4b5c6d7e8f94.xlsx</x:v>
+      </x:c>
+      <x:c r="N5" s="4" t="str">
+        <x:v>FAIL</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
@@ -20341,34 +20386,40 @@
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D6" s="9" t="str">
         <x:v>精细开发包回归（测试造数中断）</x:v>
       </x:c>
-      <x:c r="D6" s="9" t="str">
+      <x:c r="E6" s="9" t="str">
         <x:v>BLOCKED</x:v>
       </x:c>
-      <x:c r="E6" s="9" t="n">
+      <x:c r="F6" s="9" t="n">
         <x:v>78</x:v>
       </x:c>
-      <x:c r="F6" s="9" t="n">
+      <x:c r="G6" s="9" t="n">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="G6" s="9" t="n">
+      <x:c r="H6" s="9" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H6" s="9" t="n">
+      <x:c r="I6" s="9" t="n">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="I6" s="9" t="str">
+      <x:c r="J6" s="9" t="str">
         <x:v>6e80dd12d60ee5dad641bca030445a2153a269c9</x:v>
       </x:c>
-      <x:c r="J6" s="9" t="str">
+      <x:c r="K6" s="9" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="K6" s="9" t="str">
+      <x:c r="L6" s="9" t="str">
         <x:v>前16条登录实际PASS；第17条参数路径中的#被SQLite URI截断，准备阶段中断。78父TC为16 PASS/62 BLOCKED；31变体未完成。清理全真，缺项未以旧场景通过代替。</x:v>
       </x:c>
-      <x:c r="L6" s="9" t="str">
+      <x:c r="M6" s="9" t="str">
         <x:v>.local/test-results/local-7feea03dd72e4eddba0651cede8fd23d-frozen/TokenMeter测试结果-local-7feea03dd72e4eddba0651cede8fd23d.xlsx</x:v>
+      </x:c>
+      <x:c r="N6" s="9" t="str">
+        <x:v>BLOCKED</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="57" customHeight="1">
@@ -20379,34 +20430,40 @@
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
       <x:c r="C7" s="4" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D7" s="4" t="str">
         <x:v>完整精细回归及同候选辅助检查</x:v>
       </x:c>
-      <x:c r="D7" s="4" t="str">
+      <x:c r="E7" s="4" t="str">
         <x:v>FAIL</x:v>
       </x:c>
-      <x:c r="E7" s="4" t="n">
+      <x:c r="F7" s="4" t="n">
         <x:v>78</x:v>
       </x:c>
-      <x:c r="F7" s="4" t="n">
+      <x:c r="G7" s="4" t="n">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="G7" s="4" t="n">
+      <x:c r="H7" s="4" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="H7" s="4" t="n">
+      <x:c r="I7" s="4" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="I7" s="4" t="str">
+      <x:c r="J7" s="4" t="str">
         <x:v>6e80dd12d60ee5dad641bca030445a2153a269c9</x:v>
       </x:c>
-      <x:c r="J7" s="4" t="str">
+      <x:c r="K7" s="4" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="K7" s="4" t="str">
+      <x:c r="L7" s="4" t="str">
         <x:v>78父用例：62 PASS、9 FAIL、7 BLOCKED；38参数变体：31 PASS、7 FAIL（不与父用例相加）。真实产品95个执行入口，另11条辅助检查。独立代码复核保留原始失败，证据不足降BLOCKED。含3,397条证据链接和12张截图。</x:v>
       </x:c>
-      <x:c r="L7" s="4" t="str">
+      <x:c r="M7" s="4" t="str">
         <x:v>.local/test-results/local-343e54113b0b442383e80f137013014b-reviewed/TokenMeter测试结果-local-343e54113b0b442383e80f137013014b.xlsx</x:v>
+      </x:c>
+      <x:c r="N7" s="4" t="str">
+        <x:v>FAIL</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="57" customHeight="1">
@@ -20417,34 +20474,40 @@
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D8" s="9" t="str">
         <x:v>PASSWORD05/ADMIN03/UPDATE05脚本修复后定向验证</x:v>
       </x:c>
-      <x:c r="D8" s="9" t="str">
+      <x:c r="E8" s="9" t="str">
         <x:v>FAIL</x:v>
       </x:c>
-      <x:c r="E8" s="9" t="n">
+      <x:c r="F8" s="9" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="F8" s="9" t="n">
+      <x:c r="G8" s="9" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="G8" s="9" t="n">
+      <x:c r="H8" s="9" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H8" s="9" t="n">
+      <x:c r="I8" s="9" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I8" s="9" t="str">
+      <x:c r="J8" s="9" t="str">
         <x:v>6e80dd12d60ee5dad641bca030445a2153a269c9</x:v>
       </x:c>
-      <x:c r="J8" s="9" t="str">
+      <x:c r="K8" s="9" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="K8" s="9" t="str">
+      <x:c r="L8" s="9" t="str">
         <x:v>15个实际Playwright入口；3父用例2 PASS/1 FAIL，13变体8 PASS/5 FAIL。PASSWORD05独立peer与ADMIN03收尾脚本修复验证通过；UPDATE05五个解压身份场景20秒后仍有临时目录残留。其余75父用例范围外。原全量失败保留，本次不构成全量发布回归。</x:v>
       </x:c>
-      <x:c r="L8" s="9" t="str">
+      <x:c r="M8" s="9" t="str">
         <x:v>.local/test-results/local-877830fb340a4d12b4e29cf76fa422ed-reviewed/TokenMeter测试结果-local-877830fb340a4d12b4e29cf76fa422ed.xlsx</x:v>
+      </x:c>
+      <x:c r="N8" s="9" t="str">
+        <x:v>FAIL</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="57" customHeight="1">
@@ -20455,34 +20518,40 @@
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="str">
         <x:v>UI01颜色检查脚本修复后单例验证</x:v>
       </x:c>
-      <x:c r="D9" s="4" t="str">
+      <x:c r="E9" s="4" t="str">
         <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="E9" s="4" t="n">
-        <x:v>1</x:v>
       </x:c>
       <x:c r="F9" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G9" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H9" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I9" s="4" t="str">
+      <x:c r="I9" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J9" s="4" t="str">
         <x:v>6e80dd12d60ee5dad641bca030445a2153a269c9</x:v>
       </x:c>
-      <x:c r="J9" s="4" t="str">
+      <x:c r="K9" s="4" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="K9" s="4" t="str">
+      <x:c r="L9" s="4" t="str">
         <x:v>仅UI01一条PASS，77条TM001不在本次范围。修复#fff缩写颜色解析后，程序测得浅色对比度16.235、深色12.513，6页无溢出。7张截图、53条证据链接；不覆盖首次FAIL，不代表完整产品回归通过。</x:v>
       </x:c>
-      <x:c r="L9" s="4" t="str">
+      <x:c r="M9" s="4" t="str">
         <x:v>.local/test-results/aux-ui01-local-343e54113b0b442383e80f137013014b-02-reviewed/TokenMeter测试结果-aux-ui01-local-343e54113b0b442383e80f137013014b-02.xlsx</x:v>
+      </x:c>
+      <x:c r="N9" s="4" t="str">
+        <x:v>PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="57" customHeight="1">
@@ -20493,34 +20562,40 @@
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D10" s="9" t="str">
         <x:v>完整精细主回归（辅助11项未绑定）</x:v>
       </x:c>
-      <x:c r="D10" s="9" t="str">
+      <x:c r="E10" s="9" t="str">
         <x:v>FAIL</x:v>
       </x:c>
-      <x:c r="E10" s="9" t="n">
+      <x:c r="F10" s="9" t="n">
         <x:v>78</x:v>
       </x:c>
-      <x:c r="F10" s="9" t="n">
+      <x:c r="G10" s="9" t="n">
         <x:v>66</x:v>
       </x:c>
-      <x:c r="G10" s="9" t="n">
+      <x:c r="H10" s="9" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H10" s="9" t="n">
+      <x:c r="I10" s="9" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="I10" s="9" t="str">
+      <x:c r="J10" s="9" t="str">
         <x:v>6e80dd12d60ee5dad641bca030445a2153a269c9</x:v>
       </x:c>
-      <x:c r="J10" s="9" t="str">
+      <x:c r="K10" s="9" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="K10" s="9" t="str">
+      <x:c r="L10" s="9" t="str">
         <x:v>78父TC：66 PASS、1 FAIL（SESSION-09）、11辅助占位BLOCKED；38参数变体全部PASS。原始运行FAIL，清理完成；独立审计PASS只证明被审计旁证，不改变产品结论。 参数变体另计：38 PASS、0 FAIL、0 BLOCKED。</x:v>
       </x:c>
-      <x:c r="L10" s="9" t="str">
+      <x:c r="M10" s="9" t="str">
         <x:v>.local/test-results/local-571dd63bfe5b4d90a95ed9c70d80de07-reviewed/TokenMeter测试结果-local-571dd63bfe5b4d90a95ed9c70d80de07.xlsx</x:v>
+      </x:c>
+      <x:c r="N10" s="9" t="str">
+        <x:v>FAIL</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
@@ -20531,34 +20606,40 @@
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
       <x:c r="C11" s="4" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="str">
         <x:v>SESSION-09脚本修正后单例定向验证</x:v>
       </x:c>
-      <x:c r="D11" s="4" t="str">
+      <x:c r="E11" s="4" t="str">
         <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="E11" s="4" t="n">
-        <x:v>1</x:v>
       </x:c>
       <x:c r="F11" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G11" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H11" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I11" s="4" t="str">
+      <x:c r="I11" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J11" s="4" t="str">
         <x:v>6e80dd12d60ee5dad641bca030445a2153a269c9</x:v>
       </x:c>
-      <x:c r="J11" s="4" t="str">
+      <x:c r="K11" s="4" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="K11" s="4" t="str">
+      <x:c r="L11" s="4" t="str">
         <x:v>SESSION-09一例PASS、清理完成；其余77父TC范围外。仅定位前次禁用按钮点击失败，不覆盖完整回归FAIL。</x:v>
       </x:c>
-      <x:c r="L11" s="4" t="str">
+      <x:c r="M11" s="4" t="str">
         <x:v>.local/test-results/local-4a8815e9d61e4b4bbdd41f7a2f897c52-reviewed/TokenMeter测试结果-local-4a8815e9d61e4b4bbdd41f7a2f897c52.xlsx</x:v>
+      </x:c>
+      <x:c r="N11" s="4" t="str">
+        <x:v>PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="57" customHeight="1">
@@ -20569,34 +20650,40 @@
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
       <x:c r="C12" s="9" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D12" s="9" t="str">
         <x:v>完整精细主回归（升级清理失败）</x:v>
       </x:c>
-      <x:c r="D12" s="9" t="str">
+      <x:c r="E12" s="9" t="str">
         <x:v>FAIL</x:v>
       </x:c>
-      <x:c r="E12" s="9" t="n">
+      <x:c r="F12" s="9" t="n">
         <x:v>78</x:v>
       </x:c>
-      <x:c r="F12" s="9" t="n">
+      <x:c r="G12" s="9" t="n">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="G12" s="9" t="n">
+      <x:c r="H12" s="9" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H12" s="9" t="n">
+      <x:c r="I12" s="9" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="I12" s="9" t="str">
+      <x:c r="J12" s="9" t="str">
         <x:v>6e80dd12d60ee5dad641bca030445a2153a269c9</x:v>
       </x:c>
-      <x:c r="J12" s="9" t="str">
+      <x:c r="K12" s="9" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="K12" s="9" t="str">
+      <x:c r="L12" s="9" t="str">
         <x:v>78父TC：65 PASS、1 FAIL（UPDATE-07清理不完整）、12 BLOCKED（UPDATE-08及11辅助占位）；38参数变体全部PASS。原始运行FAIL、cleanup_completed=false；不能放行。 参数变体另计：38 PASS、0 FAIL、0 BLOCKED。</x:v>
       </x:c>
-      <x:c r="L12" s="9" t="str">
+      <x:c r="M12" s="9" t="str">
         <x:v>.local/test-results/local-f47f8257607c48458cc52b886d281d70-reviewed/TokenMeter测试结果-local-f47f8257607c48458cc52b886d281d70.xlsx</x:v>
+      </x:c>
+      <x:c r="N12" s="9" t="str">
+        <x:v>FAIL</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
@@ -20607,34 +20694,40 @@
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
       <x:c r="C13" s="4" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="str">
         <x:v>UPDATE-07/08清理问题定向复现</x:v>
       </x:c>
-      <x:c r="D13" s="4" t="str">
+      <x:c r="E13" s="4" t="str">
         <x:v>FAIL</x:v>
       </x:c>
-      <x:c r="E13" s="4" t="n">
+      <x:c r="F13" s="4" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="F13" s="4" t="n">
+      <x:c r="G13" s="4" t="n">
         <x:v>0</x:v>
-      </x:c>
-      <x:c r="G13" s="4" t="n">
-        <x:v>1</x:v>
       </x:c>
       <x:c r="H13" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I13" s="4" t="str">
+      <x:c r="I13" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J13" s="4" t="str">
         <x:v>6e80dd12d60ee5dad641bca030445a2153a269c9</x:v>
       </x:c>
-      <x:c r="J13" s="4" t="str">
+      <x:c r="K13" s="4" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="K13" s="4" t="str">
+      <x:c r="L13" s="4" t="str">
         <x:v>UPDATE-07因本轮拥有资源未完全清理而FAIL，UPDATE-08为避免接管残留而BLOCKED；cleanup_completed=false。其余76父TC范围外，原始失败保留。</x:v>
       </x:c>
-      <x:c r="L13" s="4" t="str">
+      <x:c r="M13" s="4" t="str">
         <x:v>.local/test-results/local-c8e31657d5e4428584a6f316936113e1-reviewed/TokenMeter测试结果-local-c8e31657d5e4428584a6f316936113e1.xlsx</x:v>
+      </x:c>
+      <x:c r="N13" s="4" t="str">
+        <x:v>FAIL</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
@@ -20645,34 +20738,40 @@
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
       <x:c r="C14" s="9" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D14" s="9" t="str">
         <x:v>UPDATE-07/08测试环境阻断定向批次</x:v>
       </x:c>
-      <x:c r="D14" s="9" t="str">
+      <x:c r="E14" s="9" t="str">
         <x:v>BLOCKED</x:v>
       </x:c>
-      <x:c r="E14" s="9" t="n">
+      <x:c r="F14" s="9" t="n">
         <x:v>2</x:v>
-      </x:c>
-      <x:c r="F14" s="9" t="n">
-        <x:v>0</x:v>
       </x:c>
       <x:c r="G14" s="9" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H14" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I14" s="9" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="I14" s="9" t="str">
+      <x:c r="J14" s="9" t="str">
         <x:v>6e80dd12d60ee5dad641bca030445a2153a269c9</x:v>
       </x:c>
-      <x:c r="J14" s="9" t="str">
+      <x:c r="K14" s="9" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="K14" s="9" t="str">
+      <x:c r="L14" s="9" t="str">
         <x:v>启动时使用系统Python，缺少alembic；UPDATE-07/08均在准备阶段BLOCKED，实际执行0例。原始BLOCKED及环境原因保留，清理完成。</x:v>
       </x:c>
-      <x:c r="L14" s="9" t="str">
+      <x:c r="M14" s="9" t="str">
         <x:v>.local/test-results/local-70e531d3092c4cbea30160117c379287-reviewed/TokenMeter测试结果-local-70e531d3092c4cbea30160117c379287.xlsx</x:v>
+      </x:c>
+      <x:c r="N14" s="9" t="str">
+        <x:v>BLOCKED</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
@@ -20683,34 +20782,40 @@
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
       <x:c r="C15" s="4" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D15" s="4" t="str">
         <x:v>UPDATE-07/08隔离环境定向验证</x:v>
       </x:c>
-      <x:c r="D15" s="4" t="str">
+      <x:c r="E15" s="4" t="str">
         <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="E15" s="4" t="n">
-        <x:v>2</x:v>
       </x:c>
       <x:c r="F15" s="4" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G15" s="4" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H15" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I15" s="4" t="str">
+      <x:c r="I15" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J15" s="4" t="str">
         <x:v>6e80dd12d60ee5dad641bca030445a2153a269c9</x:v>
       </x:c>
-      <x:c r="J15" s="4" t="str">
+      <x:c r="K15" s="4" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="K15" s="4" t="str">
+      <x:c r="L15" s="4" t="str">
         <x:v>使用项目venv执行UPDATE-07/08，2例PASS、清理完成；UPDATE-07独立旁证审计PASS。其余76父TC范围外，不覆盖此前完整回归FAIL。</x:v>
       </x:c>
-      <x:c r="L15" s="4" t="str">
+      <x:c r="M15" s="4" t="str">
         <x:v>.local/test-results/local-b6627e4379c64386bfc1a535fb432c16-reviewed/TokenMeter测试结果-local-b6627e4379c64386bfc1a535fb432c16.xlsx</x:v>
+      </x:c>
+      <x:c r="N15" s="4" t="str">
+        <x:v>PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="57" customHeight="1">
@@ -20721,34 +20826,40 @@
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
       <x:c r="C16" s="9" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D16" s="9" t="str">
         <x:v>同候选完整联合复核（本机开发包）</x:v>
       </x:c>
-      <x:c r="D16" s="9" t="str">
+      <x:c r="E16" s="9" t="str">
         <x:v>PASS</x:v>
-      </x:c>
-      <x:c r="E16" s="9" t="n">
-        <x:v>78</x:v>
       </x:c>
       <x:c r="F16" s="9" t="n">
         <x:v>78</x:v>
       </x:c>
       <x:c r="G16" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="H16" s="9" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I16" s="9" t="str">
+      <x:c r="I16" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J16" s="9" t="str">
         <x:v>6e80dd12d60ee5dad641bca030445a2153a269c9</x:v>
       </x:c>
-      <x:c r="J16" s="9" t="str">
+      <x:c r="K16" s="9" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="K16" s="9" t="str">
+      <x:c r="L16" s="9" t="str">
         <x:v>主原始BLOCKED：67产品父TC与38参数变体PASS，11辅助仅占位BLOCKED。独立辅助11/11 PASS并绑定同候选，六组6/6 PASS，审计v2 12/12 PASS；联合审核后78父TC和38变体全PASS。原件未改，开发包与dirty源码不具发布资格。</x:v>
       </x:c>
-      <x:c r="L16" s="9" t="str">
+      <x:c r="M16" s="9" t="str">
         <x:v>.local/test-results/local-534748ff47cb44229183a6bd878c1674-reviewed/TokenMeter测试结果-local-534748ff47cb44229183a6bd878c1674.xlsx</x:v>
+      </x:c>
+      <x:c r="N16" s="9" t="str">
+        <x:v>PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="57" customHeight="1">
@@ -20759,50 +20870,149 @@
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
       <x:c r="C17" s="4" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D17" s="4" t="str">
         <x:v>本地master固定候选最终包首次精细门禁</x:v>
       </x:c>
-      <x:c r="D17" s="4" t="str">
+      <x:c r="E17" s="4" t="str">
         <x:v>FAIL</x:v>
       </x:c>
-      <x:c r="E17" s="4" t="n">
+      <x:c r="F17" s="4" t="n">
         <x:v>78</x:v>
       </x:c>
-      <x:c r="F17" s="4" t="n">
+      <x:c r="G17" s="4" t="n">
         <x:v>66</x:v>
       </x:c>
-      <x:c r="G17" s="4" t="n">
+      <x:c r="H17" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H17" s="4" t="n">
+      <x:c r="I17" s="4" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="I17" s="4" t="str">
+      <x:c r="J17" s="4" t="str">
         <x:v>c2911bc65d55579fcf71e5ba11db87357a01a5e4</x:v>
       </x:c>
-      <x:c r="J17" s="4" t="str">
+      <x:c r="K17" s="4" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="K17" s="4" t="str">
+      <x:c r="L17" s="4" t="str">
         <x:v>固定本地master候选门禁FAIL；原始116项91 PASS/14 FAIL/11 BLOCKED，UPDATE-05父项与13变体缺签名输入。逐例模型78父TC 66 PASS/1 FAIL/11 BLOCKED，38变体25 PASS/13 FAIL；无正式稳定包。</x:v>
       </x:c>
-      <x:c r="L17" s="4" t="str">
+      <x:c r="M17" s="4" t="str">
         <x:v>.local/test-results/local-0512d4fc44544eba97f9d1ae79cbfc37-reviewed/TokenMeter测试结果-local-0512d4fc44544eba97f9d1ae79cbfc37.xlsx</x:v>
       </x:c>
+      <x:c r="N17" s="4" t="str">
+        <x:v>FAIL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="42" customHeight="1">
+      <x:c r="A18" s="9" t="str">
+        <x:v>tm003-core-20261001T163807Z</x:v>
+      </x:c>
+      <x:c r="B18" s="9" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="C18" s="9" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D18" s="9" t="str">
+        <x:v>TM-003 CORE-01/02/03 固定模块验证；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E18" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F18" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G18" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H18" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I18" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J18" s="9" t="str">
+        <x:v>ea6b18765ce63a5b32b7de0488de5d2a4647de94</x:v>
+      </x:c>
+      <x:c r="K18" s="9" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L18" s="9" t="str">
+        <x:v>source_check固定3条/9步骤PASS，逐例清理PASS；独立结果Excel/verification回读PASS。仅模块，不覆盖TM003原27条产品TC；产品E2E和发行门禁NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M18" s="9" t="str">
+        <x:v>.local/test-results/tm003-core-20261001T163807Z/TokenMeter测试结果-tm003-core-20261001T163807Z.xlsx</x:v>
+      </x:c>
+      <x:c r="N18" s="9" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="57" customHeight="1">
+      <x:c r="A19" s="4" t="str">
+        <x:v>tm003-core-20261001T165439Z</x:v>
+      </x:c>
+      <x:c r="B19" s="4" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="C19" s="4" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D19" s="4" t="str">
+        <x:v>TM-003 CORE-01/02/03 固定模块验证；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E19" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F19" s="4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G19" s="4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H19" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I19" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J19" s="4" t="str">
+        <x:v>d7c3d39ac0a007f0e16f55bbb3cfc9b15fd9fe34</x:v>
+      </x:c>
+      <x:c r="K19" s="4" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L19" s="4" t="str">
+        <x:v>共享source_check清理合同扩展后的新候选：CORE固定3/3、九步PASS，owned_root清理逐例PASS；独立Excel/verification回读PASS。旧ea6b187批次保留；原27条产品TC与正式发行仍NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M19" s="4" t="str">
+        <x:v>.local/test-results/tm003-core-20261001T165439Z/TokenMeter测试结果-tm003-core-20261001T165439Z.xlsx</x:v>
+      </x:c>
+      <x:c r="N19" s="4" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D5:D17">
+  <x:conditionalFormatting sqref="E5:E19">
     <x:cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="26" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="L5:L17">
+  <x:conditionalFormatting sqref="M5:M19">
     <x:cfRule type="containsText" dxfId="27" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="29" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="N5:N19">
+    <x:cfRule type="containsText" dxfId="30" priority="7" operator="containsText" text="FAIL"/>
+    <x:cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="预期待明确"/>
+    <x:cfRule type="containsText" dxfId="32" priority="9" operator="containsText" text="未执行"/>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a1d865dd2024f4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5d2095136964585"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21004,7 +21214,7 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="192" customHeight="1">
+    <x:row r="7" ht="237" customHeight="1">
       <x:c r="A7" s="4" t="str">
         <x:v>v0.2.0-20261001T034118Z</x:v>
       </x:c>
@@ -21033,7 +21243,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J7" s="4" t="str">
-        <x:v>设计基线已完成：3功能点、9 TASK、28父TC、35变体。开发工作树已有原生目录面板、加密locator、根FD受限读取、React授权UI及33个固定E2E叶入口（28可执行、5场景摘要）；报告单元59/59、治理473/473、构建PASS。产品E2E因AX trusted=false及隔离标准测试账号不可用BLOCKED，Keychain最终包隔离未证实。本独立文档树未合该代码，机器绑定仍planned；正式发行完整门禁NOT_RUN、未发布。0.2公开配置为version0.2.0/build200及测试高版0.2.1/build201，实际0.2包尚未证明。</x:v>
+        <x:v>设计基线已完成：3功能点、9 TASK、28父TC、35变体。开发工作树已有原生目录面板、加密locator、根FD受限读取、React授权UI及33个固定E2E叶入口（28可执行、5场景摘要）；报告单元59/59、治理473/473、构建PASS。产品E2E因AX trusted=false及隔离标准测试账号不可用BLOCKED，Keychain最终包隔离未证实。本独立文档树未合该代码，机器绑定仍planned；正式发行完整门禁NOT_RUN、未发布。0.2公开配置为version0.2.0/build200及测试高版0.2.1/build201，实际0.2包尚未证明。 2026-10-02修订SECURITY-01三个恶意字串变体的固定IPC method/字段/错误码，产品状态不变；需在整合候选重核基线及固定程序。</x:v>
       </x:c>
       <x:c r="K7" s="4" t="str">
         <x:v>TM001独立候选d2门禁PASS只属历史；本地master c2911bc首次最终包门禁FAIL、无SOP-020稳定原包，不能作为0.2升级源；本版无实际产品运行。</x:v>
@@ -21060,7 +21270,7 @@
         <x:v>releases/v0.2.0-20261001T034118Z/01-requirements.md:32</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="192" customHeight="1">
+    <x:row r="8" ht="297" customHeight="1">
       <x:c r="A8" s="9" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
       </x:c>
@@ -21089,7 +21299,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J8" s="9" t="str">
-        <x:v>整版draft、未发布。27条产品TC未执行；3条CORE辅助TC已在文档提交48ca089独立切片就绪，在开发分支311deedf运行模块3/3 PASS，原始receipt在该分支.local/ci/tm003-core-20261001/。代码尚未合入本文档树，机器绑定保持空；模块报告不能作为产品E2E或发行门禁，结果Excel规范待SOP修订。 2026-10-02新代码候选44379e6已有逐步模块3/3与桌面29/29/typecheck/build原件；source_check独立Excel导出程序仍缺，批次登记BLOCKED，产品E2E仍NOT_RUN。</x:v>
+        <x:v>整版draft、未发布。27条产品TC未执行；3条CORE辅助TC已在文档提交48ca089独立切片就绪，在开发分支311deedf运行模块3/3 PASS，原始receipt在该分支.local/ci/tm003-core-20261001/。代码尚未合入本文档树，机器绑定保持空；模块报告不能作为产品E2E或发行门禁，结果Excel规范待SOP修订。 2026-10-02新代码候选44379e6已有逐步模块3/3与桌面29/29/typecheck/build原件；source_check独立Excel导出程序仍缺，批次登记BLOCKED，产品E2E仍NOT_RUN。 固定导出器新run tm003-core-20261001T163807Z在ea6b187候选生成3/3/9步source_check独立Excel并回读PASS，现已按被测SHA登记模块批次；原27条产品TC与发行仍NOT_RUN。 新清理合同候选d7c3d39的独立run tm003-core-20261001T165439Z亦3/3/9步及Excel回读PASS，作为最新模块批次；旧ea6批次保留。</x:v>
       </x:c>
       <x:c r="K8" s="9" t="str">
         <x:v>TM-001 干净源码候选为技术基底；其产品门禁不继承给TM-003</x:v>
@@ -21116,7 +21326,7 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="132" customHeight="1">
+    <x:row r="9" ht="162" customHeight="1">
       <x:c r="A9" s="4" t="str">
         <x:v>v0.4.0-20261001T040433Z</x:v>
       </x:c>
@@ -21145,7 +21355,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J9" s="4" t="str">
-        <x:v>整版draft、未发布。原20产品细TC及四组摘要保留，新增3条已打开只读句柄的reader CORE辅助TC，固定LF、前缀MAC/重扫和损坏行输入，切片检查未完成。开发树模块红0/3与绿3/3仅是交接证据，且代码未形成干净提交；产品授权、稳定文件身份、SQLite原子事务、IPC/App E2E未验证，正式发行门禁NOT_RUN。</x:v>
+        <x:v>整版draft、未发布。原20产品细TC及四组摘要保留，3条reader CORE辅助TC在输入提交fea41fe/同步SOP后的干净候选ebbcfd0上按SOP-008独立判为development_slice_ready；程序绑定仍空。本版代码分支e52b62e报告reader目标9/9、桌面49/49和build PASS，仅为模块原件，Excel/总表批次尚无固定导出器。产品授权、稳定文件身份最终接口、SQLite原子事务、IPC/App E2E未验证，正式发行门禁NOT_RUN。</x:v>
       </x:c>
       <x:c r="K9" s="4" t="str">
         <x:v>TM004源分支原生零/缺失与nested Agent定向探针仅为研究证据；0.3及此前稳定原包尚未形成，真实升级BLOCKED。</x:v>
@@ -21172,7 +21382,7 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="237" customHeight="1">
+    <x:row r="10" ht="267" customHeight="1">
       <x:c r="A10" s="9" t="str">
         <x:v>v0.5.0-20261001T034729Z</x:v>
       </x:c>
@@ -21201,7 +21411,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J10" s="9" t="str">
-        <x:v>整版draft、未发布。原32条产品父TC、6稳定变体和两组摘要保留；纯统计CORE-01/02/03辅助TC在输入提交061c759后，经SOP-008内容核对及结构/治理457项PASS，独立切片development_slice_ready，程序绑定仍为空、模块实际运行unexecuted。静态oracle与切片就绪不证明真实双来源采集或产品E2E；固定产品数据、SQLite/IPC、安装App逐TC绑定未完成，正式发行完整门禁NOT_RUN。 独立代码提交6a0f6f的source_check CORE3/3、桌面29/29、build PASS，原件在TM005工作树.local/tm005-core-postcommit-20261001T162401Z；程序尚未进入本文档树、模块Excel导出/批次登记BLOCKED，产品E2E仍NOT_RUN。</x:v>
+        <x:v>整版draft、未发布。原32条产品父TC、6稳定变体和两组摘要保留；纯统计CORE-01/02/03辅助TC在输入提交061c759后，经SOP-008内容核对及结构/治理457项PASS，独立切片development_slice_ready，程序绑定仍为空、模块实际运行unexecuted。静态oracle与切片就绪不证明真实双来源采集或产品E2E；固定产品数据、SQLite/IPC、安装App逐TC绑定未完成，正式发行完整门禁NOT_RUN。 独立代码提交6a0f6f的source_check CORE3/3、桌面29/29、build PASS，原件在TM005工作树.local/tm005-core-postcommit-20261001T162401Z；程序尚未进入本文档树、模块Excel导出/批次登记BLOCKED，产品E2E仍NOT_RUN。 CORE-01仅验证已给UTC半开界聚合，不验证IANA日期换算；该单独辅助TC待固定。</x:v>
       </x:c>
       <x:c r="K10" s="9" t="str">
         <x:v>TM005语义oracle只验证规范化样例；0.4及此前稳定原包尚未形成，真实升级BLOCKED。</x:v>
@@ -21230,23 +21440,23 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F5:F10">
-    <x:cfRule type="containsText" dxfId="30" priority="1" operator="containsText" text="FAIL"/>
-    <x:cfRule type="containsText" dxfId="31" priority="2" operator="containsText" text="预期待明确"/>
-    <x:cfRule type="containsText" dxfId="32" priority="3" operator="containsText" text="未执行"/>
+    <x:cfRule type="containsText" dxfId="33" priority="1" operator="containsText" text="FAIL"/>
+    <x:cfRule type="containsText" dxfId="34" priority="2" operator="containsText" text="预期待明确"/>
+    <x:cfRule type="containsText" dxfId="35" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="J5:J10">
-    <x:cfRule type="containsText" dxfId="33" priority="4" operator="containsText" text="FAIL"/>
-    <x:cfRule type="containsText" dxfId="34" priority="5" operator="containsText" text="预期待明确"/>
-    <x:cfRule type="containsText" dxfId="35" priority="6" operator="containsText" text="未执行"/>
+    <x:cfRule type="containsText" dxfId="36" priority="4" operator="containsText" text="FAIL"/>
+    <x:cfRule type="containsText" dxfId="37" priority="5" operator="containsText" text="预期待明确"/>
+    <x:cfRule type="containsText" dxfId="38" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="M5:M10">
-    <x:cfRule type="containsText" dxfId="36" priority="7" operator="containsText" text="FAIL"/>
-    <x:cfRule type="containsText" dxfId="37" priority="8" operator="containsText" text="预期待明确"/>
-    <x:cfRule type="containsText" dxfId="38" priority="9" operator="containsText" text="未执行"/>
+    <x:cfRule type="containsText" dxfId="39" priority="7" operator="containsText" text="FAIL"/>
+    <x:cfRule type="containsText" dxfId="40" priority="8" operator="containsText" text="预期待明确"/>
+    <x:cfRule type="containsText" dxfId="41" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raad3cfddeeb34401"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22babf438e234005"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22405,13 +22615,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F5:F46">
-    <x:cfRule type="containsText" dxfId="39" priority="1" operator="containsText" text="FAIL"/>
-    <x:cfRule type="containsText" dxfId="40" priority="2" operator="containsText" text="预期待明确"/>
-    <x:cfRule type="containsText" dxfId="41" priority="3" operator="containsText" text="未执行"/>
+    <x:cfRule type="containsText" dxfId="42" priority="1" operator="containsText" text="FAIL"/>
+    <x:cfRule type="containsText" dxfId="43" priority="2" operator="containsText" text="预期待明确"/>
+    <x:cfRule type="containsText" dxfId="44" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31d38ae98c06435d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3f8606679304557"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.3.0-20261001T034652Z][TM-003] Freeze atomic store and cursor CORE test inputs
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Rbf12aa18b3554001"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R0df86ad125c847cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rb1d655ac537243bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R02ea4983c9c44775"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rcf6a862be63b4235"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R2503d345bbf645c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rb9fac209113c41ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R929989622c2e47b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rabd4aa5c6f0f4350"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R63d60e02ad764d31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R79b31b47b30a4cc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R7bcf00d865dd4eb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R156bab950efc4f5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rc9c5081c5e674fc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rf6b5cfbd3ec349c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R85fc27840feb49b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R4a1341aeefab4aac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rd777e0187db64e0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R4a3ebf10cd5f4340"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R7016dc8cac4844f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R999fe6c93ae14b6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Rdeebd0e96c5f4903"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -786,8 +786,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N270" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N270"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N272" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N272"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="功能编号"/>
     <x:tableColumn id="2" name="用例编号"/>
@@ -1134,8 +1134,8 @@
         <x:v>已登记用例</x:v>
       </x:c>
       <x:c r="B8" s="11" t="n">
-        <x:f>COUNTA('05测试用例'!B5:B270)</x:f>
-        <x:v>266</x:v>
+        <x:f>COUNTA('05测试用例'!B5:B272)</x:f>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>父用例与具有稳定 ID 的变体各占一行；含未来概要场景</x:v>
@@ -1169,7 +1169,7 @@
         <x:v>界面与治理检查</x:v>
       </x:c>
       <x:c r="B11" s="10" t="n">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C11" s="4" t="str">
         <x:v>辅助检查不能替代产品E2E；稳定变体独立列出</x:v>
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25d759ba0397462f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45392368bbda4a2d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R569059b8ca0b4736"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19b2f7e0dda74ebc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6025bfdd02894eb7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6300d3a562d543fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf28121b6afbb43f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8eb61670ecc40d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9e3695a17444599"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra55d6dc8b0a34b63"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89bf59096c52401f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5e4f1c98b7d43cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7519,7 +7519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf24b92a7a9c4ba9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R168a1387b8454b44"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18540,7 +18540,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L235" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:207</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:238</x:v>
       </x:c>
       <x:c r="M235" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18587,7 +18587,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L236" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:211</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:242</x:v>
       </x:c>
       <x:c r="M236" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18634,7 +18634,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L237" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:215</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:246</x:v>
       </x:c>
       <x:c r="M237" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18682,7 +18682,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L238" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:219</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:250</x:v>
       </x:c>
       <x:c r="M238" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18732,7 +18732,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L239" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:223</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:254</x:v>
       </x:c>
       <x:c r="M239" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18780,7 +18780,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L240" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:227</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:258</x:v>
       </x:c>
       <x:c r="M240" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18827,7 +18827,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L241" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:231</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:262</x:v>
       </x:c>
       <x:c r="M241" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18874,7 +18874,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L242" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:235</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:266</x:v>
       </x:c>
       <x:c r="M242" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18922,7 +18922,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L243" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:239</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:270</x:v>
       </x:c>
       <x:c r="M243" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18971,7 +18971,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L244" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:243</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:274</x:v>
       </x:c>
       <x:c r="M244" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19020,7 +19020,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L245" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:247</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:278</x:v>
       </x:c>
       <x:c r="M245" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19069,7 +19069,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L246" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:251</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:282</x:v>
       </x:c>
       <x:c r="M246" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19116,7 +19116,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L247" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:255</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:286</x:v>
       </x:c>
       <x:c r="M247" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19164,7 +19164,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L248" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:259</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:290</x:v>
       </x:c>
       <x:c r="M248" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19212,7 +19212,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L249" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:263</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:294</x:v>
       </x:c>
       <x:c r="M249" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19260,7 +19260,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L250" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:267</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:298</x:v>
       </x:c>
       <x:c r="M250" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19308,7 +19308,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L251" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:271</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:302</x:v>
       </x:c>
       <x:c r="M251" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19358,7 +19358,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L252" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:275</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:306</x:v>
       </x:c>
       <x:c r="M252" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19405,7 +19405,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L253" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:279</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:310</x:v>
       </x:c>
       <x:c r="M253" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19452,7 +19452,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L254" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:283</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:314</x:v>
       </x:c>
       <x:c r="M254" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19500,7 +19500,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L255" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:287</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:318</x:v>
       </x:c>
       <x:c r="M255" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19549,7 +19549,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L256" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:291</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:322</x:v>
       </x:c>
       <x:c r="M256" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19599,7 +19599,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L257" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:295</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:326</x:v>
       </x:c>
       <x:c r="M257" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19647,7 +19647,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L258" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:299</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:330</x:v>
       </x:c>
       <x:c r="M258" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19696,7 +19696,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L259" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:303</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:334</x:v>
       </x:c>
       <x:c r="M259" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19744,7 +19744,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L260" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:307</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:338</x:v>
       </x:c>
       <x:c r="M260" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19792,7 +19792,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L261" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:311</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:342</x:v>
       </x:c>
       <x:c r="M261" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19840,7 +19840,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L262" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:315</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:346</x:v>
       </x:c>
       <x:c r="M262" s="9" t="str">
         <x:v>tm003-core-20261001T165439Z (source_check；产品E2E未运行)</x:v>
@@ -19889,7 +19889,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L263" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:319</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:350</x:v>
       </x:c>
       <x:c r="M263" s="4" t="str">
         <x:v>tm003-core-20261001T165439Z (source_check；产品E2E未运行)</x:v>
@@ -19937,7 +19937,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L264" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:323</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:354</x:v>
       </x:c>
       <x:c r="M264" s="9" t="str">
         <x:v>tm003-core-20261001T165439Z (source_check；产品E2E未运行)</x:v>
@@ -19946,127 +19946,130 @@
         <x:v>v0.3.0-20261001T034652Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="265" ht="87" customHeight="1">
+    <x:row r="265" ht="117" customHeight="1">
       <x:c r="A265" s="4" t="str">
+        <x:v>TM-003</x:v>
+      </x:c>
+      <x:c r="B265" s="4" t="str">
+        <x:v>TC-TM003-CORE-04</x:v>
+      </x:c>
+      <x:c r="C265" s="4" t="str">
+        <x:v>同步批次原子提交与密钥标记</x:v>
+      </x:c>
+      <x:c r="D265" s="4" t="str">
+        <x:v>TASK-TM003-STORE</x:v>
+      </x:c>
+      <x:c r="E265" s="4" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F265" s="4" t="str">
+        <x:v>header+A=410字节、补B=750字节；A100/10/cached20、B200/20/cached40；公开key1=00..1f及不同有效key2=20..3f；owner SQLite上的INSERT和UPDATE失败触发器</x:v>
+      </x:c>
+      <x:c r="G265" s="4" t="str">
+        <x:v>一行A，(count,input,output,cached)=(1,100,10,20)，total110，诊断0，cursor410，key1标记，scan_incomplete=1；重开不变
+批次失败且全回滚；仍仅A/total110/诊断0/cursor410/原MAC/key1标记/scan_incomplete=1；重开仍相同
+B仅新增一次；(2,300,30,60)、total330、invalid_record诊断1、cursor750及新MAC、scan_incomplete=0；重开不重计
+明确密钥标记不匹配并停采集；A/B两行/total330/诊断1/cursor750/覆盖/key1标记均不变，无key2重键或已知零</x:v>
+      </x:c>
+      <x:c r="H265" s="4" t="str">
+        <x:v>准备：新建本例owner SQLite；业务行只由模块API插入；步骤2在本例库创建两条失败触发器
+变化：步骤1 A+cursor/coverage/key标记原子提交；步骤2全回滚；步骤3 B+一诊断+cursor/coverage原子提交；步骤4不变
+核验：每步只读usage_event数量与SUM、collection_diagnostic代码数、source_cursor offset/prefix_mac、coverage.scan_incomplete、identity_key_state.key_marker；关闭重开复查；仅清理owner库</x:v>
+      </x:c>
+      <x:c r="I265" s="4" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J265" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K265" s="4" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L265" s="4" t="str">
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:203</x:v>
+      </x:c>
+      <x:c r="M265" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N265" s="4" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="266" ht="117" customHeight="1">
+      <x:c r="A266" s="9" t="str">
+        <x:v>TM-003</x:v>
+      </x:c>
+      <x:c r="B266" s="9" t="str">
+        <x:v>TC-TM003-CORE-05</x:v>
+      </x:c>
+      <x:c r="C266" s="9" t="str">
+        <x:v>追加、半行、前缀改写与截短游标</x:v>
+      </x:c>
+      <x:c r="D266" s="9" t="str">
+        <x:v>TASK-TM003-SCAN
+TASK-TM003-STORE</x:v>
+      </x:c>
+      <x:c r="E266" s="9" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F266" s="9" t="str">
+        <x:v>fixture header+A410、+B750、+C1090；B半行；A.padding 0→1同长度原地改写且mtime不变；合成稳定文件身份恒定，可变快照digest随修改；公开key1</x:v>
+      </x:c>
+      <x:c r="G266" s="9" t="str">
+        <x:v>A一行total110，cursor410，保存对410字节prefixMAC及稳定身份，输出不含路径/正文/密钥
+B不提交；A一行total110，cursor410，前缀MAC相同，无cursor_reset
+只消费B/C；(count,input,output,cached)=(3,600,60,120)，total660，cursor1090，A不重计，无cursor_reset
+fixture新旧SHA不同；prefixMAC不符，cursor_reset且从0重扫；A/B/C唯一三行、total660、旧行不删，coverage.missing_before=1
+长度小于游标而从0重扫；历史A/B/C三行与total660保留；cursor410，coverage缺口为真，B/C不填零不删除</x:v>
+      </x:c>
+      <x:c r="H266" s="9" t="str">
+        <x:v>准备：新建owner文件/空SQLite；模块读取固定原始行；不访问TM-002目录能力
+变化：A/B/C仅通过正式模块API入库；追加推进完整LF游标；改写/截短重扫仅改变游标和覆盖缺口、不删可信旧行
+核验：只读按(principal_key,source,source_event_key)核对唯一三行及SUM、source_cursor offset/prefix_mac、coverage.missing_before、cursor_reset诊断；比较fixture新旧SHA/长度/mtime；结束仅清理owner资源</x:v>
+      </x:c>
+      <x:c r="I266" s="9" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J266" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K266" s="9" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L266" s="9" t="str">
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:216</x:v>
+      </x:c>
+      <x:c r="M266" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N266" s="9" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="267" ht="87" customHeight="1">
+      <x:c r="A267" s="4" t="str">
         <x:v>TM-005</x:v>
       </x:c>
-      <x:c r="B265" s="4" t="str">
+      <x:c r="B267" s="4" t="str">
         <x:v>TC-TM005-CORE-01</x:v>
       </x:c>
-      <x:c r="C265" s="4" t="str">
+      <x:c r="C267" s="4" t="str">
         <x:v>双来源可信事件与半开日汇总</x:v>
       </x:c>
-      <x:c r="D265" s="4" t="str">
+      <x:c r="D267" s="4" t="str">
         <x:v>TASK-TM005-EVENT-CONTRACT
 TASK-TM005-RANGE-QUERY</x:v>
       </x:c>
-      <x:c r="E265" s="4" t="str">
+      <x:c r="E267" s="4" t="str">
         <x:v>模块检查</x:v>
       </x:c>
-      <x:c r="F265" s="4" t="str">
+      <x:c r="F267" s="4" t="str">
         <x:v>fixture的A/B、跨主体C、界外D/E；synthetic-p1、Asia/Shanghai当地日2026-09-29</x:v>
       </x:c>
-      <x:c r="G265" s="4" t="str">
+      <x:c r="G267" s="4" t="str">
         <x:v>1. 按固定主体和fixture固定UTC半开界查询纯统计函数，不做IANA日期换算；仅A/B被选、C/D/E排除；输入数组和键不变
 2. 核对来源、模型、Token和三个子项；input300/output30/total330；Codex110/Claude220；未知模型110/sonnet-test220；缓存读20但部分未知、缓存写未知、推理2但部分未知，子项不加总
 3. 逐个输入非法来源、负数、超范围缓存和坏UTC；各自被拒绝，无完整零或有效汇总输出；原fixture不变</x:v>
-      </x:c>
-      <x:c r="H265" s="4" t="str">
-        <x:v>准备：无产品DB写入；每例从新内存输入开始
-变化：不适用；纯统计返回值与输入未变
-核验：固定fixture摘要、事件筛选、各字段与状态逐步核对；无SQL</x:v>
-      </x:c>
-      <x:c r="I265" s="4" t="str">
-        <x:v>draft</x:v>
-      </x:c>
-      <x:c r="J265" s="4" t="str">
-        <x:v>未执行</x:v>
-      </x:c>
-      <x:c r="K265" s="4" t="str">
-        <x:v>细化用例</x:v>
-      </x:c>
-      <x:c r="L265" s="4" t="str">
-        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:326</x:v>
-      </x:c>
-      <x:c r="M265" s="4" t="str">
-        <x:v>尚未执行</x:v>
-      </x:c>
-      <x:c r="N265" s="4" t="str">
-        <x:v>v0.5.0-20261001T034729Z</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="266" ht="57" customHeight="1">
-      <x:c r="A266" s="9" t="str">
-        <x:v>TM-005</x:v>
-      </x:c>
-      <x:c r="B266" s="9" t="str">
-        <x:v>TC-TM005-CORE-02</x:v>
-      </x:c>
-      <x:c r="C266" s="9" t="str">
-        <x:v>未知用量诊断不补零</x:v>
-      </x:c>
-      <x:c r="D266" s="9" t="str">
-        <x:v>TASK-TM005-EVENT-CONTRACT
-TASK-TM005-COVERAGE</x:v>
-      </x:c>
-      <x:c r="E266" s="9" t="str">
-        <x:v>模块检查</x:v>
-      </x:c>
-      <x:c r="F266" s="9" t="str">
-        <x:v>fixture A/B及同范围Claude missing_usage诊断；双来源complete仅为模块合成覆盖假设</x:v>
-      </x:c>
-      <x:c r="G266" s="9" t="str">
-        <x:v>1. 先仅统计A/B；已知330，未知模型110保留，来源Codex110/Claude220
-2. 加入诊断重新统计；partial、known_tokens330、total_tokens=null；诊断不增调用或零Token
-3. 移除A/B仅保留诊断；unknown、known_tokens0、total_tokens=null，不能写已确认零</x:v>
-      </x:c>
-      <x:c r="H266" s="9" t="str">
-        <x:v>准备：无产品DB写入；每例从新内存输入开始
-变化：不适用；纯统计返回值与输入未变
-核验：固定fixture摘要、事件筛选、各字段与状态逐步核对；无SQL</x:v>
-      </x:c>
-      <x:c r="I266" s="9" t="str">
-        <x:v>draft</x:v>
-      </x:c>
-      <x:c r="J266" s="9" t="str">
-        <x:v>未执行</x:v>
-      </x:c>
-      <x:c r="K266" s="9" t="str">
-        <x:v>细化用例</x:v>
-      </x:c>
-      <x:c r="L266" s="9" t="str">
-        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:334</x:v>
-      </x:c>
-      <x:c r="M266" s="9" t="str">
-        <x:v>尚未执行</x:v>
-      </x:c>
-      <x:c r="N266" s="9" t="str">
-        <x:v>v0.5.0-20261001T034729Z</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="267" ht="87" customHeight="1">
-      <x:c r="A267" s="4" t="str">
-        <x:v>TM-005</x:v>
-      </x:c>
-      <x:c r="B267" s="4" t="str">
-        <x:v>TC-TM005-CORE-03</x:v>
-      </x:c>
-      <x:c r="C267" s="4" t="str">
-        <x:v>声明式覆盖状态代数</x:v>
-      </x:c>
-      <x:c r="D267" s="4" t="str">
-        <x:v>TASK-TM005-COVERAGE</x:v>
-      </x:c>
-      <x:c r="E267" s="4" t="str">
-        <x:v>模块检查</x:v>
-      </x:c>
-      <x:c r="F267" s="4" t="str">
-        <x:v>fixture五行coverage_algebra；complete仅为模块合成输入，product_coverage_proven=false</x:v>
-      </x:c>
-      <x:c r="G267" s="4" t="str">
-        <x:v>1. 两来源complete且无事件、随后移除覆盖事实；前者complete/known0/total0；后者不得自行推断complete
-2. 一来源missing，分别给空事件与可信110；空事件missing/known0/total null；可信110为partial/known110/total null
-3. 两来源complete，分别给可信110+未知诊断、仅未知诊断；前者partial/known110/total null；后者unknown/known0/total null</x:v>
       </x:c>
       <x:c r="H267" s="4" t="str">
         <x:v>准备：无产品DB写入；每例从新内存输入开始
@@ -20083,7 +20086,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L267" s="4" t="str">
-        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:342</x:v>
+        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:326</x:v>
       </x:c>
       <x:c r="M267" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -20092,126 +20095,126 @@
         <x:v>v0.5.0-20261001T034729Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="268" ht="72" customHeight="1">
+    <x:row r="268" ht="57" customHeight="1">
       <x:c r="A268" s="9" t="str">
-        <x:v>TM-004</x:v>
+        <x:v>TM-005</x:v>
       </x:c>
       <x:c r="B268" s="9" t="str">
-        <x:v>TC-TM004-CORE-01</x:v>
+        <x:v>TC-TM005-CORE-02</x:v>
       </x:c>
       <x:c r="C268" s="9" t="str">
-        <x:v>完整LF、半行与限额续读</x:v>
+        <x:v>未知用量诊断不补零</x:v>
       </x:c>
       <x:c r="D268" s="9" t="str">
-        <x:v>TASK-TM004-INCREMENTAL</x:v>
+        <x:v>TASK-TM005-EVENT-CONTRACT
+TASK-TM005-COVERAGE</x:v>
       </x:c>
       <x:c r="E268" s="9" t="str">
         <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F268" s="9" t="str">
+        <x:v>fixture A/B及同范围Claude missing_usage诊断；双来源complete仅为模块合成覆盖假设</x:v>
+      </x:c>
+      <x:c r="G268" s="9" t="str">
+        <x:v>1. 先仅统计A/B；已知330，未知模型110保留，来源Codex110/Claude220
+2. 加入诊断重新统计；partial、known_tokens330、total_tokens=null；诊断不增调用或零Token
+3. 移除A/B仅保留诊断；unknown、known_tokens0、total_tokens=null，不能写已确认零</x:v>
+      </x:c>
+      <x:c r="H268" s="9" t="str">
+        <x:v>准备：无产品DB写入；每例从新内存输入开始
+变化：不适用；纯统计返回值与输入未变
+核验：固定fixture摘要、事件筛选、各字段与状态逐步核对；无SQL</x:v>
+      </x:c>
+      <x:c r="I268" s="9" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J268" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K268" s="9" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L268" s="9" t="str">
+        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:334</x:v>
+      </x:c>
+      <x:c r="M268" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N268" s="9" t="str">
+        <x:v>v0.5.0-20261001T034729Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="269" ht="87" customHeight="1">
+      <x:c r="A269" s="4" t="str">
+        <x:v>TM-005</x:v>
+      </x:c>
+      <x:c r="B269" s="4" t="str">
+        <x:v>TC-TM005-CORE-03</x:v>
+      </x:c>
+      <x:c r="C269" s="4" t="str">
+        <x:v>声明式覆盖状态代数</x:v>
+      </x:c>
+      <x:c r="D269" s="4" t="str">
+        <x:v>TASK-TM005-COVERAGE</x:v>
+      </x:c>
+      <x:c r="E269" s="4" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F269" s="4" t="str">
+        <x:v>fixture五行coverage_algebra；complete仅为模块合成输入，product_coverage_proven=false</x:v>
+      </x:c>
+      <x:c r="G269" s="4" t="str">
+        <x:v>1. 两来源complete且无事件、随后移除覆盖事实；前者complete/known0/total0；后者不得自行推断complete
+2. 一来源missing，分别给空事件与可信110；空事件missing/known0/total null；可信110为partial/known110/total null
+3. 两来源complete，分别给可信110+未知诊断、仅未知诊断；前者partial/known110/total null；后者unknown/known0/total null</x:v>
+      </x:c>
+      <x:c r="H269" s="4" t="str">
+        <x:v>准备：无产品DB写入；每例从新内存输入开始
+变化：不适用；纯统计返回值与输入未变
+核验：固定fixture摘要、事件筛选、各字段与状态逐步核对；无SQL</x:v>
+      </x:c>
+      <x:c r="I269" s="4" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J269" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K269" s="4" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L269" s="4" t="str">
+        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:342</x:v>
+      </x:c>
+      <x:c r="M269" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N269" s="4" t="str">
+        <x:v>v0.5.0-20261001T034729Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="270" ht="72" customHeight="1">
+      <x:c r="A270" s="9" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="B270" s="9" t="str">
+        <x:v>TC-TM004-CORE-01</x:v>
+      </x:c>
+      <x:c r="C270" s="9" t="str">
+        <x:v>完整LF、半行与限额续读</x:v>
+      </x:c>
+      <x:c r="D270" s="9" t="str">
+        <x:v>TASK-TM004-INCREMENTAL</x:v>
+      </x:c>
+      <x:c r="E270" s="9" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F270" s="9" t="str">
         <x:v>固定746字节13/7 assistant行、前半字节、两条不同ID完整行、首读上限754字节</x:v>
       </x:c>
-      <x:c r="G268" s="9" t="str">
+      <x:c r="G270" s="9" t="str">
         <x:v>1. 读未写完的前半行；调用0、偏移0、scanIncomplete=true，不作可信零结论
 2. 补齐LF、重复读取；补齐后一次13/7=20、偏移746、前缀MAC匹配；重复读取0调用且游标不变
 3. 两完整行首读754字节后续读；首读只第一条、偏移746、read_limit且未完成；续读只第二条、偏移为总字节长、完成</x:v>
-      </x:c>
-      <x:c r="H268" s="9" t="str">
-        <x:v>准备：无产品DB；每例新建自有临时文件
-变化：不适用；只返回模块调用、诊断与游标
-核验：固定fixture/行摘要和逐步返回值、前缀MAC及失败时无新游标；无SQL</x:v>
-      </x:c>
-      <x:c r="I268" s="9" t="str">
-        <x:v>draft</x:v>
-      </x:c>
-      <x:c r="J268" s="9" t="str">
-        <x:v>未执行</x:v>
-      </x:c>
-      <x:c r="K268" s="9" t="str">
-        <x:v>细化用例</x:v>
-      </x:c>
-      <x:c r="L268" s="9" t="str">
-        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:170</x:v>
-      </x:c>
-      <x:c r="M268" s="9" t="str">
-        <x:v>尚未执行</x:v>
-      </x:c>
-      <x:c r="N268" s="9" t="str">
-        <x:v>v0.4.0-20261001T040433Z</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="269" ht="72" customHeight="1">
-      <x:c r="A269" s="4" t="str">
-        <x:v>TM-004</x:v>
-      </x:c>
-      <x:c r="B269" s="4" t="str">
-        <x:v>TC-TM004-CORE-02</x:v>
-      </x:c>
-      <x:c r="C269" s="4" t="str">
-        <x:v>前缀MAC、变更和密钥失败</x:v>
-      </x:c>
-      <x:c r="D269" s="4" t="str">
-        <x:v>TASK-TM004-INCREMENTAL</x:v>
-      </x:c>
-      <x:c r="E269" s="4" t="str">
-        <x:v>模块检查</x:v>
-      </x:c>
-      <x:c r="F269" s="4" t="str">
-        <x:v>已提交首行，追加不同ID第二行、同长度ID改写并复原mtime、截短、身份改变、秘密缺失或错误</x:v>
-      </x:c>
-      <x:c r="G269" s="4" t="str">
-        <x:v>1. 首行后追加第二完整行；快照digest变化但稳定身份/前缀MAC相同，续读只第二调用，无cursor_reset
-2. 同长度前缀改写、截短及稳定身份变更；分别报cursor_reset并从0重扫；同inode/size/mtime也不能忽略MAC不符
-3. 秘密无效或读中源变化；拒绝且没有可提交新游标/可信调用/成功零；输出不含路径正文秘密</x:v>
-      </x:c>
-      <x:c r="H269" s="4" t="str">
-        <x:v>准备：无产品DB；每例新建自有临时文件
-变化：不适用；只返回模块调用、诊断与游标
-核验：固定fixture/行摘要和逐步返回值、前缀MAC及失败时无新游标；无SQL</x:v>
-      </x:c>
-      <x:c r="I269" s="4" t="str">
-        <x:v>draft</x:v>
-      </x:c>
-      <x:c r="J269" s="4" t="str">
-        <x:v>未执行</x:v>
-      </x:c>
-      <x:c r="K269" s="4" t="str">
-        <x:v>细化用例</x:v>
-      </x:c>
-      <x:c r="L269" s="4" t="str">
-        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:178</x:v>
-      </x:c>
-      <x:c r="M269" s="4" t="str">
-        <x:v>尚未执行</x:v>
-      </x:c>
-      <x:c r="N269" s="4" t="str">
-        <x:v>v0.4.0-20261001T040433Z</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="270" ht="57" customHeight="1">
-      <x:c r="A270" s="9" t="str">
-        <x:v>TM-004</x:v>
-      </x:c>
-      <x:c r="B270" s="9" t="str">
-        <x:v>TC-TM004-CORE-03</x:v>
-      </x:c>
-      <x:c r="C270" s="9" t="str">
-        <x:v>损坏完整行与未知结构</x:v>
-      </x:c>
-      <x:c r="D270" s="9" t="str">
-        <x:v>TASK-TM004-PARSER
-TASK-TM004-INCREMENTAL</x:v>
-      </x:c>
-      <x:c r="E270" s="9" t="str">
-        <x:v>模块检查</x:v>
-      </x:c>
-      <x:c r="F270" s="9" t="str">
-        <x:v>固定13/7行前置非法UTF8完整行和版本2.1.127完整行，尾部再追加无LF坏字节</x:v>
-      </x:c>
-      <x:c r="G270" s="9" t="str">
-        <x:v>1. 读三条完整LF行；仅合法2.1.126一条调用13/7=20；invalid_utf8及unsupported_version各一次
-2. 核对游标、重复读取及隐私；游标到三行LF末，MAC匹配且完成；重复读取0；输出无路径、正文、秘密
-3. 追加无LF坏字节再补LF；未补LF前偏移不动且未完成；补LF后仅诊断推进，无伪调用</x:v>
       </x:c>
       <x:c r="H270" s="9" t="str">
         <x:v>准备：无产品DB；每例新建自有临时文件
@@ -20228,7 +20231,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L270" s="9" t="str">
-        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:186</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:170</x:v>
       </x:c>
       <x:c r="M270" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -20237,30 +20240,127 @@
         <x:v>v0.4.0-20261001T040433Z</x:v>
       </x:c>
     </x:row>
+    <x:row r="271" ht="72" customHeight="1">
+      <x:c r="A271" s="4" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="B271" s="4" t="str">
+        <x:v>TC-TM004-CORE-02</x:v>
+      </x:c>
+      <x:c r="C271" s="4" t="str">
+        <x:v>前缀MAC、变更和密钥失败</x:v>
+      </x:c>
+      <x:c r="D271" s="4" t="str">
+        <x:v>TASK-TM004-INCREMENTAL</x:v>
+      </x:c>
+      <x:c r="E271" s="4" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F271" s="4" t="str">
+        <x:v>已提交首行，追加不同ID第二行、同长度ID改写并复原mtime、截短、身份改变、秘密缺失或错误</x:v>
+      </x:c>
+      <x:c r="G271" s="4" t="str">
+        <x:v>1. 首行后追加第二完整行；快照digest变化但稳定身份/前缀MAC相同，续读只第二调用，无cursor_reset
+2. 同长度前缀改写、截短及稳定身份变更；分别报cursor_reset并从0重扫；同inode/size/mtime也不能忽略MAC不符
+3. 秘密无效或读中源变化；拒绝且没有可提交新游标/可信调用/成功零；输出不含路径正文秘密</x:v>
+      </x:c>
+      <x:c r="H271" s="4" t="str">
+        <x:v>准备：无产品DB；每例新建自有临时文件
+变化：不适用；只返回模块调用、诊断与游标
+核验：固定fixture/行摘要和逐步返回值、前缀MAC及失败时无新游标；无SQL</x:v>
+      </x:c>
+      <x:c r="I271" s="4" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J271" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K271" s="4" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L271" s="4" t="str">
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:178</x:v>
+      </x:c>
+      <x:c r="M271" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N271" s="4" t="str">
+        <x:v>v0.4.0-20261001T040433Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="272" ht="57" customHeight="1">
+      <x:c r="A272" s="9" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="B272" s="9" t="str">
+        <x:v>TC-TM004-CORE-03</x:v>
+      </x:c>
+      <x:c r="C272" s="9" t="str">
+        <x:v>损坏完整行与未知结构</x:v>
+      </x:c>
+      <x:c r="D272" s="9" t="str">
+        <x:v>TASK-TM004-PARSER
+TASK-TM004-INCREMENTAL</x:v>
+      </x:c>
+      <x:c r="E272" s="9" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F272" s="9" t="str">
+        <x:v>固定13/7行前置非法UTF8完整行和版本2.1.127完整行，尾部再追加无LF坏字节</x:v>
+      </x:c>
+      <x:c r="G272" s="9" t="str">
+        <x:v>1. 读三条完整LF行；仅合法2.1.126一条调用13/7=20；invalid_utf8及unsupported_version各一次
+2. 核对游标、重复读取及隐私；游标到三行LF末，MAC匹配且完成；重复读取0；输出无路径、正文、秘密
+3. 追加无LF坏字节再补LF；未补LF前偏移不动且未完成；补LF后仅诊断推进，无伪调用</x:v>
+      </x:c>
+      <x:c r="H272" s="9" t="str">
+        <x:v>准备：无产品DB；每例新建自有临时文件
+变化：不适用；只返回模块调用、诊断与游标
+核验：固定fixture/行摘要和逐步返回值、前缀MAC及失败时无新游标；无SQL</x:v>
+      </x:c>
+      <x:c r="I272" s="9" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J272" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K272" s="9" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L272" s="9" t="str">
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:186</x:v>
+      </x:c>
+      <x:c r="M272" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N272" s="9" t="str">
+        <x:v>v0.4.0-20261001T040433Z</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G5:G270">
+  <x:conditionalFormatting sqref="G5:G272">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="I5:I270">
+  <x:conditionalFormatting sqref="I5:I272">
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="16" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="17" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="J5:J270">
+  <x:conditionalFormatting sqref="J5:J272">
     <x:cfRule type="containsText" dxfId="18" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="19" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="20" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M270">
+  <x:conditionalFormatting sqref="M5:M272">
     <x:cfRule type="containsText" dxfId="21" priority="10" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="22" priority="11" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="23" priority="12" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53d132cdb12b4b3f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b5bad41f7cb43fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21012,7 +21112,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5d2095136964585"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1c226c53dd74dcc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21270,7 +21370,7 @@
         <x:v>releases/v0.2.0-20261001T034118Z/01-requirements.md:32</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="297" customHeight="1">
+    <x:row r="8" ht="342" customHeight="1">
       <x:c r="A8" s="9" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
       </x:c>
@@ -21299,7 +21399,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J8" s="9" t="str">
-        <x:v>整版draft、未发布。27条产品TC未执行；3条CORE辅助TC已在文档提交48ca089独立切片就绪，在开发分支311deedf运行模块3/3 PASS，原始receipt在该分支.local/ci/tm003-core-20261001/。代码尚未合入本文档树，机器绑定保持空；模块报告不能作为产品E2E或发行门禁，结果Excel规范待SOP修订。 2026-10-02新代码候选44379e6已有逐步模块3/3与桌面29/29/typecheck/build原件；source_check独立Excel导出程序仍缺，批次登记BLOCKED，产品E2E仍NOT_RUN。 固定导出器新run tm003-core-20261001T163807Z在ea6b187候选生成3/3/9步source_check独立Excel并回读PASS，现已按被测SHA登记模块批次；原27条产品TC与发行仍NOT_RUN。 新清理合同候选d7c3d39的独立run tm003-core-20261001T165439Z亦3/3/9步及Excel回读PASS，作为最新模块批次；旧ea6批次保留。</x:v>
+        <x:v>整版draft、未发布。27条产品TC未执行；3条CORE辅助TC已在文档提交48ca089独立切片就绪，在开发分支311deedf运行模块3/3 PASS，原始receipt在该分支.local/ci/tm003-core-20261001/。代码尚未合入本文档树，机器绑定保持空；模块报告不能作为产品E2E或发行门禁，结果Excel规范待SOP修订。 2026-10-02新代码候选44379e6已有逐步模块3/3与桌面29/29/typecheck/build原件；source_check独立Excel导出程序仍缺，批次登记BLOCKED，产品E2E仍NOT_RUN。 固定导出器新run tm003-core-20261001T163807Z在ea6b187候选生成3/3/9步source_check独立Excel并回读PASS，现已按被测SHA登记模块批次；原27条产品TC与发行仍NOT_RUN。 新清理合同候选d7c3d39的独立run tm003-core-20261001T165439Z亦3/3/9步及Excel回读PASS，作为最新模块批次；旧ea6批次保留。 后续CORE-04/05的测试输入已编制，程序未绑定、未执行；独立SOP-008切片复核待文档干净提交。</x:v>
       </x:c>
       <x:c r="K8" s="9" t="str">
         <x:v>TM-001 干净源码候选为技术基底；其产品门禁不继承给TM-003</x:v>
@@ -21456,7 +21556,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22babf438e234005"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4158954b7951482d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22621,7 +22721,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3f8606679304557"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf359d27351742cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.1.0-20260929T074814Z][TM-001] Index verified UPDATE-05 targeted result workbook
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R7bcf00d865dd4eb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R156bab950efc4f5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rc9c5081c5e674fc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rf6b5cfbd3ec349c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R85fc27840feb49b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R4a1341aeefab4aac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rd777e0187db64e0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R4a3ebf10cd5f4340"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R7016dc8cac4844f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R999fe6c93ae14b6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Rdeebd0e96c5f4903"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R0af57b27871f4093"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rc785ec2bd08349ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R9da2d755809c4ca2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rf609cc11a3c14d1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R6bf838a9f9584f80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R379f8348e51344d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R3518c44d508c4867"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R29618a27bc994739"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rff51e22708124cb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Rd9e1c0f3ca2f432e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R36c8450f06cd4cc9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -809,8 +809,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N19"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N20"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="运行批次"/>
     <x:tableColumn id="2" name="版本"/>
@@ -1146,8 +1146,8 @@
         <x:v>测试批次</x:v>
       </x:c>
       <x:c r="B9" s="10" t="n">
-        <x:f>COUNTA('06测试批次'!A5:A19)</x:f>
-        <x:v>15</x:v>
+        <x:f>COUNTA('06测试批次'!A5:A20)</x:f>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>06测试批次，每次运行一行，记录独立结果Excel位置</x:v>
@@ -1271,7 +1271,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>source_check · TM-003 CORE-01/02/03 固定模块验证；非产品E2E：共享source_check清理合同扩展后的新候选：CORE固定3/3、九步PASS，owned_root清理逐例PASS；独立Excel/verification回读PASS。旧ea6b187批次保留；原27条产品TC与正式发行仍NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
+        <x:v>product_e2e · granular_targeted_probe；仅TC-TM001-UPDATE-05父例及13固定变体：UPDATE-05父例1 PASS、13固定变体13 PASS、26逐步记录，77条TM001父例范围外；清理完成。仅709d候选定向探针，不覆盖旧c291完整门禁FAIL或授予发行资格；Excel为后置de081a6导出修复从原报告生成，非重跑App。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45392368bbda4a2d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb45b5bde48c74523"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19b2f7e0dda74ebc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06bc7c770cc6441a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6300d3a562d543fa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R897949901cd54d89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8eb61670ecc40d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra14f9d99992246ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra55d6dc8b0a34b63"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2770688113524adb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5e4f1c98b7d43cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d1f5a873b2c4094"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7519,7 +7519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R168a1387b8454b44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57f30b7f7d394d9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10661,7 +10661,7 @@
         <x:v>已设计</x:v>
       </x:c>
       <x:c r="J68" s="9" t="str">
-        <x:v>FAIL</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="K68" s="9" t="str">
         <x:v>细化用例</x:v>
@@ -10670,7 +10670,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:609</x:v>
       </x:c>
       <x:c r="M68" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-65796d0033704e3988cd7174dec93c81 (仅定向探针；完整门禁仍FAIL)</x:v>
       </x:c>
       <x:c r="N68" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -20360,7 +20360,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b5bad41f7cb43fa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15026631cc374e50"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21094,25 +21094,69 @@
         <x:v>NOT_RUN</x:v>
       </x:c>
     </x:row>
+    <x:row r="20" ht="57" customHeight="1">
+      <x:c r="A20" s="9" t="str">
+        <x:v>local-65796d0033704e3988cd7174dec93c81</x:v>
+      </x:c>
+      <x:c r="B20" s="9" t="str">
+        <x:v>v0.1.0-20260929T074814Z</x:v>
+      </x:c>
+      <x:c r="C20" s="9" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D20" s="9" t="str">
+        <x:v>granular_targeted_probe；仅TC-TM001-UPDATE-05父例及13固定变体</x:v>
+      </x:c>
+      <x:c r="E20" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F20" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G20" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H20" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I20" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J20" s="9" t="str">
+        <x:v>709d21253a0f88bc703a431cbf3adba3df17e508</x:v>
+      </x:c>
+      <x:c r="K20" s="9" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L20" s="9" t="str">
+        <x:v>UPDATE-05父例1 PASS、13固定变体13 PASS、26逐步记录，77条TM001父例范围外；清理完成。仅709d候选定向探针，不覆盖旧c291完整门禁FAIL或授予发行资格；Excel为后置de081a6导出修复从原报告生成，非重跑App。</x:v>
+      </x:c>
+      <x:c r="M20" s="9" t="str">
+        <x:v>.local/test-results/local-65796d0033704e3988cd7174dec93c81/TokenMeter测试结果-local-65796d0033704e3988cd7174dec93c81.xlsx</x:v>
+      </x:c>
+      <x:c r="N20" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E5:E19">
+  <x:conditionalFormatting sqref="E5:E20">
     <x:cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="26" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M19">
+  <x:conditionalFormatting sqref="M5:M20">
     <x:cfRule type="containsText" dxfId="27" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="29" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="N5:N19">
+  <x:conditionalFormatting sqref="N5:N20">
     <x:cfRule type="containsText" dxfId="30" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="32" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1c226c53dd74dcc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46c847e7fec346f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21258,7 +21302,7 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="117" customHeight="1">
+    <x:row r="6" ht="177" customHeight="1">
       <x:c r="A6" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
@@ -21287,7 +21331,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J6" s="9" t="str">
-        <x:v>开发中，未发布。c291本地master最终包门禁FAIL：116项91 PASS/14 FAIL/11 BLOCKED；9f06cb1修复私有签名输入后开发检查PASS，但新定向App仍FAIL/BLOCKED并有ENOSPC，功能回归未完成。旧d2db551独立候选PASS不转用于新候选。正式发行完整门禁NOT_RUN，无稳定0.1原包。</x:v>
+        <x:v>开发中，未发布。c291本地master最终包门禁FAIL：116项91 PASS/14 FAIL/11 BLOCKED；9f06cb1修复私有签名输入后开发检查PASS，但新定向App仍FAIL/BLOCKED并有ENOSPC，功能回归未完成。旧d2db551独立候选PASS不转用于新候选。正式发行完整门禁NOT_RUN，无稳定0.1原包。 709d UPDATE-05定向父1+变体13 PASS，后置de081a6导出Excel回读PASS；仅定向，77父TC范围外，旧c291完整门禁FAIL及未发行不变。</x:v>
       </x:c>
       <x:c r="K6" s="9" t="str">
         <x:v>旧SwiftUI PR #2 已合并、历史双平台六例PASS；不继承给Electron</x:v>
@@ -21556,7 +21600,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4158954b7951482d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6453414550ec48c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22721,7 +22765,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf359d27351742cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra37c7c299a6c4c35"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.3.0-20261001T034652Z][TM-003] Freeze multi-file generation atomicity case
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Rbde94a1a5ca34e1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R284aa9f88a2e4034"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rc25a6238ae194d71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rcc997e240d914aa6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R08667b0399ca47da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R48cbdec366684311"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rf5c7c974eace4aa0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Rf8cb85b19dcf4653"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R50a4e122758c41f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R57a9fa2ad59a4f1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R0b814b45870a4298"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R7215fc6f93a443cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R742d88c8de894ce7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R12c572f106d8457a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R1044b23d2bc74f6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R323f0c37591644ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R9de02a0f67a4441b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R900b662389ba48b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Ra5304fed28d54022"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rda36ae4456dd4866"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R1c8d52062e24401f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Rbae19fa2c4fb4f57"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -786,8 +786,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N273" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N273"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N274" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N274"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="功能编号"/>
     <x:tableColumn id="2" name="用例编号"/>
@@ -809,8 +809,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N20"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N21"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="运行批次"/>
     <x:tableColumn id="2" name="版本"/>
@@ -1134,8 +1134,8 @@
         <x:v>已登记用例</x:v>
       </x:c>
       <x:c r="B8" s="11" t="n">
-        <x:f>COUNTA('05测试用例'!B5:B273)</x:f>
-        <x:v>269</x:v>
+        <x:f>COUNTA('05测试用例'!B5:B274)</x:f>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>父用例与具有稳定 ID 的变体各占一行；含未来概要场景</x:v>
@@ -1146,8 +1146,8 @@
         <x:v>测试批次</x:v>
       </x:c>
       <x:c r="B9" s="10" t="n">
-        <x:f>COUNTA('06测试批次'!A5:A20)</x:f>
-        <x:v>16</x:v>
+        <x:f>COUNTA('06测试批次'!A5:A21)</x:f>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>06测试批次，每次运行一行，记录独立结果Excel位置</x:v>
@@ -1169,7 +1169,7 @@
         <x:v>界面与治理检查</x:v>
       </x:c>
       <x:c r="B11" s="10" t="n">
-        <x:v>56</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="C11" s="4" t="str">
         <x:v>辅助检查不能替代产品E2E；稳定变体独立列出</x:v>
@@ -1271,7 +1271,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>product_e2e · granular_targeted_probe；仅TC-TM001-UPDATE-05父例及13固定变体：UPDATE-05父例1 PASS、13固定变体13 PASS、26逐步记录，77条TM001父例范围外；清理完成。仅709d候选定向探针，不覆盖旧c291完整门禁FAIL或授予发行资格；Excel为后置de081a6导出修复从原报告生成，非重跑App。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
+        <x:v>source_check · TM-003 CORE-04/05 固定模块事务与游标验证；非产品E2E：source_check固定CORE04/05 2/2、9步、各例owner清理PASS；独立Excel/verification回读PASS。仅模块，原27条产品TC未执行，正式发行NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6034ed23f6dd49f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9093cd2d7ca74824"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8da03928fcd14244"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R968100f766774b29"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9c873e73bb3444f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2973a4fdff544a29"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76cc21639a444669"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b8deead0e034697"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc99b01a21c74a59"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra90d29cb501c470c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48b80fb90b69440a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3377c092b5cb4c90"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7519,7 +7519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3fc4ce55b6b4ada"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe889e98a7904ae5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18586,7 +18586,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L236" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:238</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:251</x:v>
       </x:c>
       <x:c r="M236" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18633,7 +18633,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L237" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:242</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:255</x:v>
       </x:c>
       <x:c r="M237" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18680,7 +18680,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L238" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:246</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:259</x:v>
       </x:c>
       <x:c r="M238" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18728,7 +18728,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L239" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:250</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:263</x:v>
       </x:c>
       <x:c r="M239" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18778,7 +18778,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L240" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:254</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:267</x:v>
       </x:c>
       <x:c r="M240" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18826,7 +18826,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L241" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:258</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:271</x:v>
       </x:c>
       <x:c r="M241" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18873,7 +18873,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L242" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:262</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:275</x:v>
       </x:c>
       <x:c r="M242" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18920,7 +18920,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L243" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:266</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:279</x:v>
       </x:c>
       <x:c r="M243" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18968,7 +18968,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L244" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:270</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:283</x:v>
       </x:c>
       <x:c r="M244" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19017,7 +19017,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L245" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:274</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:287</x:v>
       </x:c>
       <x:c r="M245" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19066,7 +19066,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L246" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:278</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:291</x:v>
       </x:c>
       <x:c r="M246" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19115,7 +19115,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L247" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:282</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:295</x:v>
       </x:c>
       <x:c r="M247" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19162,7 +19162,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L248" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:286</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:299</x:v>
       </x:c>
       <x:c r="M248" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19210,7 +19210,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L249" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:290</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:303</x:v>
       </x:c>
       <x:c r="M249" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19258,7 +19258,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L250" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:294</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:307</x:v>
       </x:c>
       <x:c r="M250" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19306,7 +19306,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L251" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:298</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:311</x:v>
       </x:c>
       <x:c r="M251" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19354,7 +19354,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L252" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:302</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:315</x:v>
       </x:c>
       <x:c r="M252" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19404,7 +19404,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L253" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:306</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:319</x:v>
       </x:c>
       <x:c r="M253" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19451,7 +19451,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L254" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:310</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:323</x:v>
       </x:c>
       <x:c r="M254" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19498,7 +19498,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L255" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:314</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:327</x:v>
       </x:c>
       <x:c r="M255" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19546,7 +19546,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L256" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:318</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:331</x:v>
       </x:c>
       <x:c r="M256" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19595,7 +19595,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L257" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:322</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:335</x:v>
       </x:c>
       <x:c r="M257" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19645,7 +19645,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L258" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:326</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:339</x:v>
       </x:c>
       <x:c r="M258" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19693,7 +19693,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L259" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:330</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:343</x:v>
       </x:c>
       <x:c r="M259" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19742,7 +19742,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L260" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:334</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:347</x:v>
       </x:c>
       <x:c r="M260" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19790,7 +19790,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L261" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:338</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:351</x:v>
       </x:c>
       <x:c r="M261" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19838,7 +19838,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L262" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:342</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:355</x:v>
       </x:c>
       <x:c r="M262" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19886,7 +19886,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L263" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:346</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:359</x:v>
       </x:c>
       <x:c r="M263" s="4" t="str">
         <x:v>tm003-core-20261001T165439Z (source_check；产品E2E未运行)</x:v>
@@ -19935,7 +19935,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L264" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:350</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:363</x:v>
       </x:c>
       <x:c r="M264" s="9" t="str">
         <x:v>tm003-core-20261001T165439Z (source_check；产品E2E未运行)</x:v>
@@ -19983,7 +19983,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L265" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:354</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:367</x:v>
       </x:c>
       <x:c r="M265" s="4" t="str">
         <x:v>tm003-core-20261001T165439Z (source_check；产品E2E未运行)</x:v>
@@ -20026,7 +20026,7 @@
         <x:v>draft</x:v>
       </x:c>
       <x:c r="J266" s="9" t="str">
-        <x:v>未执行</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="K266" s="9" t="str">
         <x:v>细化用例</x:v>
@@ -20035,7 +20035,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:203</x:v>
       </x:c>
       <x:c r="M266" s="9" t="str">
-        <x:v>尚未执行</x:v>
+        <x:v>tm003-core45-20261001T175000Z (source_check；产品E2E未运行)</x:v>
       </x:c>
       <x:c r="N266" s="9" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -20077,7 +20077,7 @@
         <x:v>draft</x:v>
       </x:c>
       <x:c r="J267" s="4" t="str">
-        <x:v>未执行</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="K267" s="4" t="str">
         <x:v>细化用例</x:v>
@@ -20086,85 +20086,86 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:216</x:v>
       </x:c>
       <x:c r="M267" s="4" t="str">
-        <x:v>尚未执行</x:v>
+        <x:v>tm003-core45-20261001T175000Z (source_check；产品E2E未运行)</x:v>
       </x:c>
       <x:c r="N267" s="4" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="268" ht="87" customHeight="1">
+    <x:row r="268" ht="117" customHeight="1">
       <x:c r="A268" s="9" t="str">
+        <x:v>TM-003</x:v>
+      </x:c>
+      <x:c r="B268" s="9" t="str">
+        <x:v>TC-TM003-CORE-06</x:v>
+      </x:c>
+      <x:c r="C268" s="9" t="str">
+        <x:v>多文件代际一次提交与全回滚</x:v>
+      </x:c>
+      <x:c r="D268" s="9" t="str">
+        <x:v>TASK-TM003-SCAN
+TASK-TM003-STORE</x:v>
+      </x:c>
+      <x:c r="E268" s="9" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F268" s="9" t="str">
+        <x:v>固定tm003-core-generation.json：同一generation两页file-a/file-b，各header+完整LF调用、各410字节；第1页complete=false，末页complete=true；owner空SQLite、公开key1、假scan capability/guard；四步各新空库。</x:v>
+      </x:c>
+      <x:c r="G268" s="9" t="str">
+        <x:v>A仅内存暂存；commitScanBatch调用0次，事件/游标/诊断/覆盖无本代际行，complete=false不称完整
+批次失败并全回滚：A/B事件、两个游标、诊断、覆盖、首次key标记均0或不存在；重开库仍空
+guard拒绝或取消，cancelScan调用1次，commitScanBatch调用0次；暂存清空，事件/两个游标/诊断/覆盖/密钥标记均未提交
+A/B唯一两行，(count,input,output,cached,total)=(2,300,30,60,330)；两游标各410及prefixMAC、coverage.scan_incomplete=0；重启不重复，不输出路径/正文/密钥</x:v>
+      </x:c>
+      <x:c r="H268" s="9" t="str">
+        <x:v>准备：每路径独立owner 0700根/0600空SQLite；事件只由正式模块API提交；步骤2仅创建本例游标失败触发器
+变化：未完成无提交；第二游标失败或guard撤权全代际回滚；完整稳定代际原子提交A/B两个事件、两个游标和覆盖
+核验：逐步只读usage_event唯一键/聚合、source_cursor数量及偏移/prefixMAC、collection_diagnostic、coverage和identity_key_state；重开验证失败仍空、成功不重计；owner清理</x:v>
+      </x:c>
+      <x:c r="I268" s="9" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J268" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K268" s="9" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L268" s="9" t="str">
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:230</x:v>
+      </x:c>
+      <x:c r="M268" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N268" s="9" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="269" ht="87" customHeight="1">
+      <x:c r="A269" s="4" t="str">
         <x:v>TM-005</x:v>
       </x:c>
-      <x:c r="B268" s="9" t="str">
+      <x:c r="B269" s="4" t="str">
         <x:v>TC-TM005-CORE-01</x:v>
       </x:c>
-      <x:c r="C268" s="9" t="str">
+      <x:c r="C269" s="4" t="str">
         <x:v>双来源可信事件与半开日汇总</x:v>
       </x:c>
-      <x:c r="D268" s="9" t="str">
+      <x:c r="D269" s="4" t="str">
         <x:v>TASK-TM005-EVENT-CONTRACT
 TASK-TM005-RANGE-QUERY</x:v>
       </x:c>
-      <x:c r="E268" s="9" t="str">
+      <x:c r="E269" s="4" t="str">
         <x:v>模块检查</x:v>
       </x:c>
-      <x:c r="F268" s="9" t="str">
+      <x:c r="F269" s="4" t="str">
         <x:v>fixture的A/B、跨主体C、界外D/E；synthetic-p1、Asia/Shanghai当地日2026-09-29</x:v>
       </x:c>
-      <x:c r="G268" s="9" t="str">
+      <x:c r="G269" s="4" t="str">
         <x:v>1. 按固定主体和fixture固定UTC半开界查询纯统计函数，不做IANA日期换算；仅A/B被选、C/D/E排除；输入数组和键不变
 2. 核对来源、模型、Token和三个子项；input300/output30/total330；Codex110/Claude220；未知模型110/sonnet-test220；缓存读20但部分未知、缓存写未知、推理2但部分未知，子项不加总
 3. 逐个输入非法来源、负数、超范围缓存和坏UTC；各自被拒绝，无完整零或有效汇总输出；原fixture不变</x:v>
-      </x:c>
-      <x:c r="H268" s="9" t="str">
-        <x:v>准备：无产品DB写入；每例从新内存输入开始
-变化：不适用；纯统计返回值与输入未变
-核验：固定fixture摘要、事件筛选、各字段与状态逐步核对；无SQL</x:v>
-      </x:c>
-      <x:c r="I268" s="9" t="str">
-        <x:v>draft</x:v>
-      </x:c>
-      <x:c r="J268" s="9" t="str">
-        <x:v>未执行</x:v>
-      </x:c>
-      <x:c r="K268" s="9" t="str">
-        <x:v>细化用例</x:v>
-      </x:c>
-      <x:c r="L268" s="9" t="str">
-        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:326</x:v>
-      </x:c>
-      <x:c r="M268" s="9" t="str">
-        <x:v>尚未执行</x:v>
-      </x:c>
-      <x:c r="N268" s="9" t="str">
-        <x:v>v0.5.0-20261001T034729Z</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="269" ht="57" customHeight="1">
-      <x:c r="A269" s="4" t="str">
-        <x:v>TM-005</x:v>
-      </x:c>
-      <x:c r="B269" s="4" t="str">
-        <x:v>TC-TM005-CORE-02</x:v>
-      </x:c>
-      <x:c r="C269" s="4" t="str">
-        <x:v>未知用量诊断不补零</x:v>
-      </x:c>
-      <x:c r="D269" s="4" t="str">
-        <x:v>TASK-TM005-EVENT-CONTRACT
-TASK-TM005-COVERAGE</x:v>
-      </x:c>
-      <x:c r="E269" s="4" t="str">
-        <x:v>模块检查</x:v>
-      </x:c>
-      <x:c r="F269" s="4" t="str">
-        <x:v>fixture A/B及同范围Claude missing_usage诊断；双来源complete仅为模块合成覆盖假设</x:v>
-      </x:c>
-      <x:c r="G269" s="4" t="str">
-        <x:v>1. 先仅统计A/B；已知330，未知模型110保留，来源Codex110/Claude220
-2. 加入诊断重新统计；partial、known_tokens330、total_tokens=null；诊断不增调用或零Token
-3. 移除A/B仅保留诊断；unknown、known_tokens0、total_tokens=null，不能写已确认零</x:v>
       </x:c>
       <x:c r="H269" s="4" t="str">
         <x:v>准备：无产品DB写入；每例从新内存输入开始
@@ -20181,7 +20182,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L269" s="4" t="str">
-        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:334</x:v>
+        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:326</x:v>
       </x:c>
       <x:c r="M269" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -20190,29 +20191,30 @@
         <x:v>v0.5.0-20261001T034729Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="270" ht="87" customHeight="1">
+    <x:row r="270" ht="57" customHeight="1">
       <x:c r="A270" s="9" t="str">
         <x:v>TM-005</x:v>
       </x:c>
       <x:c r="B270" s="9" t="str">
-        <x:v>TC-TM005-CORE-03</x:v>
+        <x:v>TC-TM005-CORE-02</x:v>
       </x:c>
       <x:c r="C270" s="9" t="str">
-        <x:v>声明式覆盖状态代数</x:v>
+        <x:v>未知用量诊断不补零</x:v>
       </x:c>
       <x:c r="D270" s="9" t="str">
-        <x:v>TASK-TM005-COVERAGE</x:v>
+        <x:v>TASK-TM005-EVENT-CONTRACT
+TASK-TM005-COVERAGE</x:v>
       </x:c>
       <x:c r="E270" s="9" t="str">
         <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F270" s="9" t="str">
-        <x:v>fixture五行coverage_algebra；complete仅为模块合成输入，product_coverage_proven=false</x:v>
+        <x:v>fixture A/B及同范围Claude missing_usage诊断；双来源complete仅为模块合成覆盖假设</x:v>
       </x:c>
       <x:c r="G270" s="9" t="str">
-        <x:v>1. 两来源complete且无事件、随后移除覆盖事实；前者complete/known0/total0；后者不得自行推断complete
-2. 一来源missing，分别给空事件与可信110；空事件missing/known0/total null；可信110为partial/known110/total null
-3. 两来源complete，分别给可信110+未知诊断、仅未知诊断；前者partial/known110/total null；后者unknown/known0/total null</x:v>
+        <x:v>1. 先仅统计A/B；已知330，未知模型110保留，来源Codex110/Claude220
+2. 加入诊断重新统计；partial、known_tokens330、total_tokens=null；诊断不增调用或零Token
+3. 移除A/B仅保留诊断；unknown、known_tokens0、total_tokens=null，不能写已确认零</x:v>
       </x:c>
       <x:c r="H270" s="9" t="str">
         <x:v>准备：无产品DB写入；每例从新内存输入开始
@@ -20229,7 +20231,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L270" s="9" t="str">
-        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:342</x:v>
+        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:334</x:v>
       </x:c>
       <x:c r="M270" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -20238,77 +20240,77 @@
         <x:v>v0.5.0-20261001T034729Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="271" ht="72" customHeight="1">
+    <x:row r="271" ht="87" customHeight="1">
       <x:c r="A271" s="4" t="str">
-        <x:v>TM-004</x:v>
+        <x:v>TM-005</x:v>
       </x:c>
       <x:c r="B271" s="4" t="str">
-        <x:v>TC-TM004-CORE-01</x:v>
+        <x:v>TC-TM005-CORE-03</x:v>
       </x:c>
       <x:c r="C271" s="4" t="str">
-        <x:v>完整LF、半行与限额续读</x:v>
+        <x:v>声明式覆盖状态代数</x:v>
       </x:c>
       <x:c r="D271" s="4" t="str">
-        <x:v>TASK-TM004-INCREMENTAL</x:v>
+        <x:v>TASK-TM005-COVERAGE</x:v>
       </x:c>
       <x:c r="E271" s="4" t="str">
         <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F271" s="4" t="str">
+        <x:v>fixture五行coverage_algebra；complete仅为模块合成输入，product_coverage_proven=false</x:v>
+      </x:c>
+      <x:c r="G271" s="4" t="str">
+        <x:v>1. 两来源complete且无事件、随后移除覆盖事实；前者complete/known0/total0；后者不得自行推断complete
+2. 一来源missing，分别给空事件与可信110；空事件missing/known0/total null；可信110为partial/known110/total null
+3. 两来源complete，分别给可信110+未知诊断、仅未知诊断；前者partial/known110/total null；后者unknown/known0/total null</x:v>
+      </x:c>
+      <x:c r="H271" s="4" t="str">
+        <x:v>准备：无产品DB写入；每例从新内存输入开始
+变化：不适用；纯统计返回值与输入未变
+核验：固定fixture摘要、事件筛选、各字段与状态逐步核对；无SQL</x:v>
+      </x:c>
+      <x:c r="I271" s="4" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J271" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K271" s="4" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L271" s="4" t="str">
+        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:342</x:v>
+      </x:c>
+      <x:c r="M271" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N271" s="4" t="str">
+        <x:v>v0.5.0-20261001T034729Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="272" ht="72" customHeight="1">
+      <x:c r="A272" s="9" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="B272" s="9" t="str">
+        <x:v>TC-TM004-CORE-01</x:v>
+      </x:c>
+      <x:c r="C272" s="9" t="str">
+        <x:v>完整LF、半行与限额续读</x:v>
+      </x:c>
+      <x:c r="D272" s="9" t="str">
+        <x:v>TASK-TM004-INCREMENTAL</x:v>
+      </x:c>
+      <x:c r="E272" s="9" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F272" s="9" t="str">
         <x:v>固定746字节13/7 assistant行、前半字节、两条不同ID完整行、首读上限754字节</x:v>
       </x:c>
-      <x:c r="G271" s="4" t="str">
+      <x:c r="G272" s="9" t="str">
         <x:v>1. 读未写完的前半行；调用0、偏移0、scanIncomplete=true，不作可信零结论
 2. 补齐LF、重复读取；补齐后一次13/7=20、偏移746、前缀MAC匹配；重复读取0调用且游标不变
 3. 两完整行首读754字节后续读；首读只第一条、偏移746、read_limit且未完成；续读只第二条、偏移为总字节长、完成</x:v>
-      </x:c>
-      <x:c r="H271" s="4" t="str">
-        <x:v>准备：无产品DB；每例新建自有临时文件
-变化：不适用；只返回模块调用、诊断与游标
-核验：固定fixture/行摘要和逐步返回值、前缀MAC及失败时无新游标；无SQL</x:v>
-      </x:c>
-      <x:c r="I271" s="4" t="str">
-        <x:v>draft</x:v>
-      </x:c>
-      <x:c r="J271" s="4" t="str">
-        <x:v>未执行</x:v>
-      </x:c>
-      <x:c r="K271" s="4" t="str">
-        <x:v>细化用例</x:v>
-      </x:c>
-      <x:c r="L271" s="4" t="str">
-        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:170</x:v>
-      </x:c>
-      <x:c r="M271" s="4" t="str">
-        <x:v>尚未执行</x:v>
-      </x:c>
-      <x:c r="N271" s="4" t="str">
-        <x:v>v0.4.0-20261001T040433Z</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="272" ht="72" customHeight="1">
-      <x:c r="A272" s="9" t="str">
-        <x:v>TM-004</x:v>
-      </x:c>
-      <x:c r="B272" s="9" t="str">
-        <x:v>TC-TM004-CORE-02</x:v>
-      </x:c>
-      <x:c r="C272" s="9" t="str">
-        <x:v>前缀MAC、变更和密钥失败</x:v>
-      </x:c>
-      <x:c r="D272" s="9" t="str">
-        <x:v>TASK-TM004-INCREMENTAL</x:v>
-      </x:c>
-      <x:c r="E272" s="9" t="str">
-        <x:v>模块检查</x:v>
-      </x:c>
-      <x:c r="F272" s="9" t="str">
-        <x:v>已提交首行，追加不同ID第二行、同长度ID改写并复原mtime、截短、身份改变、秘密缺失或错误</x:v>
-      </x:c>
-      <x:c r="G272" s="9" t="str">
-        <x:v>1. 首行后追加第二完整行；快照digest变化但稳定身份/前缀MAC相同，续读只第二调用，无cursor_reset
-2. 同长度前缀改写、截短及稳定身份变更；分别报cursor_reset并从0重扫；同inode/size/mtime也不能忽略MAC不符
-3. 秘密无效或读中源变化；拒绝且没有可提交新游标/可信调用/成功零；输出不含路径正文秘密</x:v>
       </x:c>
       <x:c r="H272" s="9" t="str">
         <x:v>准备：无产品DB；每例新建自有临时文件
@@ -20325,7 +20327,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L272" s="9" t="str">
-        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:178</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:170</x:v>
       </x:c>
       <x:c r="M272" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -20334,30 +20336,29 @@
         <x:v>v0.4.0-20261001T040433Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="273" ht="57" customHeight="1">
+    <x:row r="273" ht="72" customHeight="1">
       <x:c r="A273" s="4" t="str">
         <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B273" s="4" t="str">
-        <x:v>TC-TM004-CORE-03</x:v>
+        <x:v>TC-TM004-CORE-02</x:v>
       </x:c>
       <x:c r="C273" s="4" t="str">
-        <x:v>损坏完整行与未知结构</x:v>
+        <x:v>前缀MAC、变更和密钥失败</x:v>
       </x:c>
       <x:c r="D273" s="4" t="str">
-        <x:v>TASK-TM004-PARSER
-TASK-TM004-INCREMENTAL</x:v>
+        <x:v>TASK-TM004-INCREMENTAL</x:v>
       </x:c>
       <x:c r="E273" s="4" t="str">
         <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F273" s="4" t="str">
-        <x:v>固定13/7行前置非法UTF8完整行和版本2.1.127完整行，尾部再追加无LF坏字节</x:v>
+        <x:v>已提交首行，追加不同ID第二行、同长度ID改写并复原mtime、截短、身份改变、秘密缺失或错误</x:v>
       </x:c>
       <x:c r="G273" s="4" t="str">
-        <x:v>1. 读三条完整LF行；仅合法2.1.126一条调用13/7=20；invalid_utf8及unsupported_version各一次
-2. 核对游标、重复读取及隐私；游标到三行LF末，MAC匹配且完成；重复读取0；输出无路径、正文、秘密
-3. 追加无LF坏字节再补LF；未补LF前偏移不动且未完成；补LF后仅诊断推进，无伪调用</x:v>
+        <x:v>1. 首行后追加第二完整行；快照digest变化但稳定身份/前缀MAC相同，续读只第二调用，无cursor_reset
+2. 同长度前缀改写、截短及稳定身份变更；分别报cursor_reset并从0重扫；同inode/size/mtime也不能忽略MAC不符
+3. 秘密无效或读中源变化；拒绝且没有可提交新游标/可信调用/成功零；输出不含路径正文秘密</x:v>
       </x:c>
       <x:c r="H273" s="4" t="str">
         <x:v>准备：无产品DB；每例新建自有临时文件
@@ -20374,7 +20375,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L273" s="4" t="str">
-        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:186</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:178</x:v>
       </x:c>
       <x:c r="M273" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -20383,30 +20384,79 @@
         <x:v>v0.4.0-20261001T040433Z</x:v>
       </x:c>
     </x:row>
+    <x:row r="274" ht="57" customHeight="1">
+      <x:c r="A274" s="9" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="B274" s="9" t="str">
+        <x:v>TC-TM004-CORE-03</x:v>
+      </x:c>
+      <x:c r="C274" s="9" t="str">
+        <x:v>损坏完整行与未知结构</x:v>
+      </x:c>
+      <x:c r="D274" s="9" t="str">
+        <x:v>TASK-TM004-PARSER
+TASK-TM004-INCREMENTAL</x:v>
+      </x:c>
+      <x:c r="E274" s="9" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F274" s="9" t="str">
+        <x:v>固定13/7行前置非法UTF8完整行和版本2.1.127完整行，尾部再追加无LF坏字节</x:v>
+      </x:c>
+      <x:c r="G274" s="9" t="str">
+        <x:v>1. 读三条完整LF行；仅合法2.1.126一条调用13/7=20；invalid_utf8及unsupported_version各一次
+2. 核对游标、重复读取及隐私；游标到三行LF末，MAC匹配且完成；重复读取0；输出无路径、正文、秘密
+3. 追加无LF坏字节再补LF；未补LF前偏移不动且未完成；补LF后仅诊断推进，无伪调用</x:v>
+      </x:c>
+      <x:c r="H274" s="9" t="str">
+        <x:v>准备：无产品DB；每例新建自有临时文件
+变化：不适用；只返回模块调用、诊断与游标
+核验：固定fixture/行摘要和逐步返回值、前缀MAC及失败时无新游标；无SQL</x:v>
+      </x:c>
+      <x:c r="I274" s="9" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J274" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K274" s="9" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L274" s="9" t="str">
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:186</x:v>
+      </x:c>
+      <x:c r="M274" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N274" s="9" t="str">
+        <x:v>v0.4.0-20261001T040433Z</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G5:G273">
+  <x:conditionalFormatting sqref="G5:G274">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="I5:I273">
+  <x:conditionalFormatting sqref="I5:I274">
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="16" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="17" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="J5:J273">
+  <x:conditionalFormatting sqref="J5:J274">
     <x:cfRule type="containsText" dxfId="18" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="19" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="20" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M273">
+  <x:conditionalFormatting sqref="M5:M274">
     <x:cfRule type="containsText" dxfId="21" priority="10" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="22" priority="11" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="23" priority="12" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad33f5b1dcfb4e67"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfaad12eebafd4f06"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21184,25 +21234,69 @@
         <x:v>PASS</x:v>
       </x:c>
     </x:row>
+    <x:row r="21" ht="42" customHeight="1">
+      <x:c r="A21" s="4" t="str">
+        <x:v>tm003-core45-20261001T175000Z</x:v>
+      </x:c>
+      <x:c r="B21" s="4" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="C21" s="4" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D21" s="4" t="str">
+        <x:v>TM-003 CORE-04/05 固定模块事务与游标验证；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E21" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F21" s="4" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G21" s="4" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H21" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I21" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J21" s="4" t="str">
+        <x:v>9efc6fa9d8523f30dfc20f4cfb8282cc54f18dd0</x:v>
+      </x:c>
+      <x:c r="K21" s="4" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L21" s="4" t="str">
+        <x:v>source_check固定CORE04/05 2/2、9步、各例owner清理PASS；独立Excel/verification回读PASS。仅模块，原27条产品TC未执行，正式发行NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M21" s="4" t="str">
+        <x:v>.local/test-results/tm003-core45-20261001T175000Z/TokenMeter测试结果-tm003-core45-20261001T175000Z.xlsx</x:v>
+      </x:c>
+      <x:c r="N21" s="4" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E5:E20">
+  <x:conditionalFormatting sqref="E5:E21">
     <x:cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="26" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M20">
+  <x:conditionalFormatting sqref="M5:M21">
     <x:cfRule type="containsText" dxfId="27" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="29" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="N5:N20">
+  <x:conditionalFormatting sqref="N5:N21">
     <x:cfRule type="containsText" dxfId="30" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="32" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e7a2a8d48c543ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f0916034fad42d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21460,7 +21554,7 @@
         <x:v>releases/v0.2.0-20261001T034118Z/01-requirements.md:32</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="342" customHeight="1">
+    <x:row r="8" ht="387" customHeight="1">
       <x:c r="A8" s="9" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
       </x:c>
@@ -21489,7 +21583,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J8" s="9" t="str">
-        <x:v>整版draft、未发布。27条产品TC未执行；3条CORE辅助TC已在文档提交48ca089独立切片就绪，在开发分支311deedf运行模块3/3 PASS，原始receipt在该分支.local/ci/tm003-core-20261001/。代码尚未合入本文档树，机器绑定保持空；模块报告不能作为产品E2E或发行门禁，结果Excel规范待SOP修订。 2026-10-02新代码候选44379e6已有逐步模块3/3与桌面29/29/typecheck/build原件；source_check独立Excel导出程序仍缺，批次登记BLOCKED，产品E2E仍NOT_RUN。 固定导出器新run tm003-core-20261001T163807Z在ea6b187候选生成3/3/9步source_check独立Excel并回读PASS，现已按被测SHA登记模块批次；原27条产品TC与发行仍NOT_RUN。 新清理合同候选d7c3d39的独立run tm003-core-20261001T165439Z亦3/3/9步及Excel回读PASS，作为最新模块批次；旧ea6批次保留。 后续CORE-04/05的测试输入已编制，程序未绑定、未执行；独立SOP-008切片复核待文档干净提交。</x:v>
+        <x:v>整版draft、未发布。27条产品TC未执行；3条CORE辅助TC已在文档提交48ca089独立切片就绪，在开发分支311deedf运行模块3/3 PASS，原始receipt在该分支.local/ci/tm003-core-20261001/。代码尚未合入本文档树，机器绑定保持空；模块报告不能作为产品E2E或发行门禁，结果Excel规范待SOP修订。 2026-10-02新代码候选44379e6已有逐步模块3/3与桌面29/29/typecheck/build原件；source_check独立Excel导出程序仍缺，批次登记BLOCKED，产品E2E仍NOT_RUN。 固定导出器新run tm003-core-20261001T163807Z在ea6b187候选生成3/3/9步source_check独立Excel并回读PASS，现已按被测SHA登记模块批次；原27条产品TC与发行仍NOT_RUN。 新清理合同候选d7c3d39的独立run tm003-core-20261001T165439Z亦3/3/9步及Excel回读PASS，作为最新模块批次；旧ea6批次保留。 后续CORE-04/05的测试输入已编制，程序未绑定、未执行；独立SOP-008切片复核待文档干净提交。 CORE04/05基于9efc6fa独立source_check 2/2、9步和Excel回读PASS，第17批次；CORE06新输入未执行，产品E2E NOT_RUN。</x:v>
       </x:c>
       <x:c r="K8" s="9" t="str">
         <x:v>TM-001 干净源码候选为技术基底；其产品门禁不继承给TM-003</x:v>
@@ -21646,7 +21740,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc5d10965c904b6d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4791341f513d4308"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22811,7 +22905,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e806a9fd13a4224"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52c4b647f49e45f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.4.0-20261001T040433Z][TM-004] Freeze trigger port auxiliary test
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R7215fc6f93a443cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R742d88c8de894ce7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R12c572f106d8457a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R1044b23d2bc74f6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R323f0c37591644ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R9de02a0f67a4441b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R900b662389ba48b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Ra5304fed28d54022"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rda36ae4456dd4866"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R1c8d52062e24401f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Rbae19fa2c4fb4f57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Rcb2e6197ef514bde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R3d396230446642d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R0b857d5ae06a45ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R586e9306229e404c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rf581f41391f54e9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rdfefec032dd34f3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rac338ac978374a73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Rfea48e2e580f413c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Ra6d9dd69c3c940c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R032275ad43524de5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R6d66857b2eac4403"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -786,8 +786,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N274" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N274"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N275" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N275"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="功能编号"/>
     <x:tableColumn id="2" name="用例编号"/>
@@ -1134,8 +1134,8 @@
         <x:v>已登记用例</x:v>
       </x:c>
       <x:c r="B8" s="11" t="n">
-        <x:f>COUNTA('05测试用例'!B5:B274)</x:f>
-        <x:v>270</x:v>
+        <x:f>COUNTA('05测试用例'!B5:B275)</x:f>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>父用例与具有稳定 ID 的变体各占一行；含未来概要场景</x:v>
@@ -1169,7 +1169,7 @@
         <x:v>界面与治理检查</x:v>
       </x:c>
       <x:c r="B11" s="10" t="n">
-        <x:v>57</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C11" s="4" t="str">
         <x:v>辅助检查不能替代产品E2E；稳定变体独立列出</x:v>
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9093cd2d7ca74824"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf232f8d41fe34f5e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R968100f766774b29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra712f0d0e8f24eb3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2973a4fdff544a29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7511311acf0f4c69"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b8deead0e034697"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5b3683e4c874f2c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra90d29cb501c470c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55ac6f0a777c4164"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3377c092b5cb4c90"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b0b80079f74487c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7519,7 +7519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe889e98a7904ae5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R526d9b71940b4a85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20433,30 +20433,79 @@
         <x:v>v0.4.0-20261001T040433Z</x:v>
       </x:c>
     </x:row>
+    <x:row r="275" ht="87" customHeight="1">
+      <x:c r="A275" s="4" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="B275" s="4" t="str">
+        <x:v>TC-TM004-CORE-04</x:v>
+      </x:c>
+      <x:c r="C275" s="4" t="str">
+        <x:v>授权主体与扫描事务触发</x:v>
+      </x:c>
+      <x:c r="D275" s="4" t="str">
+        <x:v>TASK-TM004-SOURCE
+TASK-TM004-INCREMENTAL</x:v>
+      </x:c>
+      <x:c r="E275" s="4" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F275" s="4" t="str">
+        <x:v>tests/fixtures/tm004-trigger-core-slice.json；固定UUID、M=100/10、无效路径/主体/来源、三种屏障事件</x:v>
+      </x:c>
+      <x:c r="G275" s="4" t="str">
+        <x:v>1. 拒绝路径字段、无效主体/来源和预先取消的请求；明确拒绝；beginCandidateScan=0，commitSync=0，无成功零值
+2. 扫描开始后在固定屏障分别换账号、撤权和取消；每次cancelScan被调用；commitSync=0；缓冲数据不外露
+3. 健康主体和授权世代扫描完整M并通过提交守卫；commitSync恰一次；返回1次调用、100/10/110、覆盖完整；无私密哨兵/原生标识</x:v>
+      </x:c>
+      <x:c r="H275" s="4" t="str">
+        <x:v>准备：无产品DB；每子变体新建假端口与计数器
+变化：无SQLite；只观察假同步提交次数及数值
+核验：逐步断言扫描、取消、守卫、提交次数与返回白名单；无SQL</x:v>
+      </x:c>
+      <x:c r="I275" s="4" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J275" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K275" s="4" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L275" s="4" t="str">
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:198</x:v>
+      </x:c>
+      <x:c r="M275" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N275" s="4" t="str">
+        <x:v>v0.4.0-20261001T040433Z</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G5:G274">
+  <x:conditionalFormatting sqref="G5:G275">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="I5:I274">
+  <x:conditionalFormatting sqref="I5:I275">
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="16" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="17" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="J5:J274">
+  <x:conditionalFormatting sqref="J5:J275">
     <x:cfRule type="containsText" dxfId="18" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="19" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="20" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M274">
+  <x:conditionalFormatting sqref="M5:M275">
     <x:cfRule type="containsText" dxfId="21" priority="10" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="22" priority="11" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="23" priority="12" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfaad12eebafd4f06"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62b3220ccbf44a10"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21296,7 +21345,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f0916034fad42d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0455fdbf79064229"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21740,7 +21789,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4791341f513d4308"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6603ff5ad4b1416a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22905,7 +22954,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52c4b647f49e45f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7dfc65debf24da0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.4.0-20261001T040433Z][TM-004] Freeze source and storage port slices
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Rcb2e6197ef514bde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R3d396230446642d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R0b857d5ae06a45ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R586e9306229e404c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rf581f41391f54e9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rdfefec032dd34f3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rac338ac978374a73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Rfea48e2e580f413c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Ra6d9dd69c3c940c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R032275ad43524de5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R6d66857b2eac4403"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Rd2a6d09f77894779"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rf4e156a1925645dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Red0433e6efb741c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R86b940aabb4d473e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R9846e0924699427f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R87d79ff2e74b42de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rf30adb9bddbd4df5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R33be556776a34e79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R1fac0a087b6e4e85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R7291e1ae66594553"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Re295b36e23cc4b12"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -786,8 +786,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N275" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N275"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N276" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N276"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="功能编号"/>
     <x:tableColumn id="2" name="用例编号"/>
@@ -809,8 +809,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N21"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N22"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="运行批次"/>
     <x:tableColumn id="2" name="版本"/>
@@ -832,8 +832,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="TMTable8" displayName="TMTable8" ref="A4:R10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:R10"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="TMTable8" displayName="TMTable8" ref="A4:R11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:R11"/>
   <x:tableColumns count="18">
     <x:tableColumn id="1" name="发布编号"/>
     <x:tableColumn id="2" name="版本"/>
@@ -1134,8 +1134,8 @@
         <x:v>已登记用例</x:v>
       </x:c>
       <x:c r="B8" s="11" t="n">
-        <x:f>COUNTA('05测试用例'!B5:B275)</x:f>
-        <x:v>271</x:v>
+        <x:f>COUNTA('05测试用例'!B5:B276)</x:f>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>父用例与具有稳定 ID 的变体各占一行；含未来概要场景</x:v>
@@ -1146,8 +1146,8 @@
         <x:v>测试批次</x:v>
       </x:c>
       <x:c r="B9" s="10" t="n">
-        <x:f>COUNTA('06测试批次'!A5:A21)</x:f>
-        <x:v>17</x:v>
+        <x:f>COUNTA('06测试批次'!A5:A22)</x:f>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>06测试批次，每次运行一行，记录独立结果Excel位置</x:v>
@@ -1169,7 +1169,7 @@
         <x:v>界面与治理检查</x:v>
       </x:c>
       <x:c r="B11" s="10" t="n">
-        <x:v>58</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C11" s="4" t="str">
         <x:v>辅助检查不能替代产品E2E；稳定变体独立列出</x:v>
@@ -1271,7 +1271,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>source_check · TM-003 CORE-04/05 固定模块事务与游标验证；非产品E2E：source_check固定CORE04/05 2/2、9步、各例owner清理PASS；独立Excel/verification回读PASS。仅模块，原27条产品TC未执行，正式发行NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
+        <x:v>source_check · TM-003 CORE-06 固定多文件代际提交与全回滚；非产品E2E：source_check固定CORE06 1/1、四步及owner清理PASS；此前408ebf8红测步骤2 FAIL保留。独立Excel/verification回读PASS。原27条产品TC、App E2E与发行均NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf232f8d41fe34f5e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R112308681a85490a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra712f0d0e8f24eb3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b0d3089fa0541b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7511311acf0f4c69"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6b07d381f0c44e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5b3683e4c874f2c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf01dd68b6584e30"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55ac6f0a777c4164"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc237592fa63497d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b0b80079f74487c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8580111f2c5649f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7519,7 +7519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R526d9b71940b4a85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3aa2b3bcebe74fdd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20127,7 +20127,7 @@
         <x:v>draft</x:v>
       </x:c>
       <x:c r="J268" s="9" t="str">
-        <x:v>未执行</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="K268" s="9" t="str">
         <x:v>细化用例</x:v>
@@ -20136,7 +20136,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:230</x:v>
       </x:c>
       <x:c r="M268" s="9" t="str">
-        <x:v>尚未执行</x:v>
+        <x:v>tm003-core06-20261001T182500Z (source_check；产品E2E未运行)</x:v>
       </x:c>
       <x:c r="N268" s="9" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -20336,7 +20336,7 @@
         <x:v>v0.4.0-20261001T040433Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="273" ht="72" customHeight="1">
+    <x:row r="273" ht="87" customHeight="1">
       <x:c r="A273" s="4" t="str">
         <x:v>TM-004</x:v>
       </x:c>
@@ -20356,7 +20356,7 @@
         <x:v>已提交首行，追加不同ID第二行、同长度ID改写并复原mtime、截短、身份改变、秘密缺失或错误</x:v>
       </x:c>
       <x:c r="G273" s="4" t="str">
-        <x:v>1. 首行后追加第二完整行；快照digest变化但稳定身份/前缀MAC相同，续读只第二调用，无cursor_reset
+        <x:v>1. 首行后追加第二完整行；size/mtime变化但TM-002 dev/ino摘要和前缀MAC相同，续读只第二调用，无cursor_reset
 2. 同长度前缀改写、截短及稳定身份变更；分别报cursor_reset并从0重扫；同inode/size/mtime也不能忽略MAC不符
 3. 秘密无效或读中源变化；拒绝且没有可提交新游标/可信调用/成功零；输出不含路径正文秘密</x:v>
       </x:c>
@@ -20433,7 +20433,7 @@
         <x:v>v0.4.0-20261001T040433Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="275" ht="87" customHeight="1">
+    <x:row r="275" ht="132" customHeight="1">
       <x:c r="A275" s="4" t="str">
         <x:v>TM-004</x:v>
       </x:c>
@@ -20451,12 +20451,12 @@
         <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F275" s="4" t="str">
-        <x:v>tests/fixtures/tm004-trigger-core-slice.json；固定UUID、M=100/10、无效路径/主体/来源、三种屏障事件</x:v>
+        <x:v>tests/fixtures/tm004-trigger-core-slice.json；固定UUID、M=100/10、各错误码、三种屏障事件及成功返回形状</x:v>
       </x:c>
       <x:c r="G275" s="4" t="str">
-        <x:v>1. 拒绝路径字段、无效主体/来源和预先取消的请求；明确拒绝；beginCandidateScan=0，commitSync=0，无成功零值
-2. 扫描开始后在固定屏障分别换账号、撤权和取消；每次cancelScan被调用；commitSync=0；缓冲数据不外露
-3. 健康主体和授权世代扫描完整M并通过提交守卫；commitSync恰一次；返回1次调用、100/10/110、覆盖完整；无私密哨兵/原生标识</x:v>
+        <x:v>1. 拒绝路径字段、无效主体/来源和预先取消的请求；路径字段/坏UUID为invalid_collection_request；账号不可用为collection_unavailable；异主体来源为source_not_authorized；预先取消为collection_cancelled；均扫描0、提交0
+2. 扫描开始后在固定屏障分别换账号、撤权和取消；换账号/撤权为collection_stale，取消为collection_cancelled；每次cancelScan、commitSync=0、缓冲不外露
+3. 健康主体和授权世代扫描完整M并通过提交守卫；commitSync恰一次；返回summary{callCount:1,inputTokens:100,outputTokens:10,totalTokens:110,scanIncomplete:false},diagnostics:[]，无私密哨兵/原生标识</x:v>
       </x:c>
       <x:c r="H275" s="4" t="str">
         <x:v>准备：无产品DB；每子变体新建假端口与计数器
@@ -20482,30 +20482,80 @@
         <x:v>v0.4.0-20261001T040433Z</x:v>
       </x:c>
     </x:row>
+    <x:row r="276" ht="147" customHeight="1">
+      <x:c r="A276" s="9" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="B276" s="9" t="str">
+        <x:v>TC-TM004-CORE-05</x:v>
+      </x:c>
+      <x:c r="C276" s="9" t="str">
+        <x:v>多文件来源键与整代持久映射</x:v>
+      </x:c>
+      <x:c r="D276" s="9" t="str">
+        <x:v>TASK-TM004-INCREMENTAL
+TASK-TM004-LINEAGE</x:v>
+      </x:c>
+      <x:c r="E276" s="9" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F276" s="9" t="str">
+        <x:v>tests/fixtures/tm004-storage-port-slice.json；合成M100/10、S200/20、Q50/5，三文件HMAC/游标/诊断与隔离SQLite；异常model_id哨兵与invalid_model_id诊断</x:v>
+      </x:c>
+      <x:c r="G276" s="9" t="str">
+        <x:v>1. 计算三个文件来源键、根键及换源/追加/替换向量；64hex键逐一等于fixture；普通追加键不变，换sourceId/文件摘要改变；数据库不收原摘要/相对名
+2. 构造完整三文件generation并核对文件归属与turnId代号；a/b/c各有自己的M/S/Q、游标和诊断；c异常model_id置null并增加invalid_model_id，SQLite/WAL无哨兵；turn代号仅进scope HMAC；未到末页/正文不稳零提交
+3. 分别在新库注入第二游标写失败与guard撤权；每次整代回滚或零开始，事件/游标/诊断/覆盖/密钥标记全空；取消并清缓冲
+4. 稳定末页通过guard后一次同步commitScanBatch并重扫；唯一3调用、input350/output35/total385、3游标/4诊断按文件归属、scan_incomplete=1；scope键匹配向量，重扫不增；SQLite/WAL无模型哨兵/原生标识</x:v>
+      </x:c>
+      <x:c r="H276" s="9" t="str">
+        <x:v>准备：每故障子场景新建本例空SQLite；故障注入只在本例库设置第二游标写入RAISE(ABORT)
+变化：成功一次事务新增三事件、三个游标、三诊断与根覆盖；失败和撤权零提交
+核验：只读查询usage_event、source_cursor、collection_diagnostic、coverage的数量/键/数值；核对源键和scope HMAC向量及无原生标识；关闭并核对SQLite/WAL无合成prompt/路径哨兵</x:v>
+      </x:c>
+      <x:c r="I276" s="9" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J276" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K276" s="9" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L276" s="9" t="str">
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:206</x:v>
+      </x:c>
+      <x:c r="M276" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N276" s="9" t="str">
+        <x:v>v0.4.0-20261001T040433Z</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G5:G275">
+  <x:conditionalFormatting sqref="G5:G276">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="I5:I275">
+  <x:conditionalFormatting sqref="I5:I276">
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="16" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="17" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="J5:J275">
+  <x:conditionalFormatting sqref="J5:J276">
     <x:cfRule type="containsText" dxfId="18" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="19" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="20" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M275">
+  <x:conditionalFormatting sqref="M5:M276">
     <x:cfRule type="containsText" dxfId="21" priority="10" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="22" priority="11" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="23" priority="12" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62b3220ccbf44a10"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07055277d0114c75"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21327,25 +21377,69 @@
         <x:v>NOT_RUN</x:v>
       </x:c>
     </x:row>
+    <x:row r="22" ht="42" customHeight="1">
+      <x:c r="A22" s="9" t="str">
+        <x:v>tm003-core06-20261001T182500Z</x:v>
+      </x:c>
+      <x:c r="B22" s="9" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="C22" s="9" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D22" s="9" t="str">
+        <x:v>TM-003 CORE-06 固定多文件代际提交与全回滚；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E22" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F22" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G22" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H22" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I22" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J22" s="9" t="str">
+        <x:v>eef956b877ebe60f53e605db861f738533837f8b</x:v>
+      </x:c>
+      <x:c r="K22" s="9" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L22" s="9" t="str">
+        <x:v>source_check固定CORE06 1/1、四步及owner清理PASS；此前408ebf8红测步骤2 FAIL保留。独立Excel/verification回读PASS。原27条产品TC、App E2E与发行均NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M22" s="9" t="str">
+        <x:v>.local/test-results/tm003-core06-20261001T182500Z/TokenMeter测试结果-tm003-core06-20261001T182500Z.xlsx</x:v>
+      </x:c>
+      <x:c r="N22" s="9" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E5:E21">
+  <x:conditionalFormatting sqref="E5:E22">
     <x:cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="26" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M21">
+  <x:conditionalFormatting sqref="M5:M22">
     <x:cfRule type="containsText" dxfId="27" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="29" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="N5:N21">
+  <x:conditionalFormatting sqref="N5:N22">
     <x:cfRule type="containsText" dxfId="30" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="32" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0455fdbf79064229"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfef00fe67eeb4ddb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21632,7 +21726,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J8" s="9" t="str">
-        <x:v>整版draft、未发布。27条产品TC未执行；3条CORE辅助TC已在文档提交48ca089独立切片就绪，在开发分支311deedf运行模块3/3 PASS，原始receipt在该分支.local/ci/tm003-core-20261001/。代码尚未合入本文档树，机器绑定保持空；模块报告不能作为产品E2E或发行门禁，结果Excel规范待SOP修订。 2026-10-02新代码候选44379e6已有逐步模块3/3与桌面29/29/typecheck/build原件；source_check独立Excel导出程序仍缺，批次登记BLOCKED，产品E2E仍NOT_RUN。 固定导出器新run tm003-core-20261001T163807Z在ea6b187候选生成3/3/9步source_check独立Excel并回读PASS，现已按被测SHA登记模块批次；原27条产品TC与发行仍NOT_RUN。 新清理合同候选d7c3d39的独立run tm003-core-20261001T165439Z亦3/3/9步及Excel回读PASS，作为最新模块批次；旧ea6批次保留。 后续CORE-04/05的测试输入已编制，程序未绑定、未执行；独立SOP-008切片复核待文档干净提交。 CORE04/05基于9efc6fa独立source_check 2/2、9步和Excel回读PASS，第17批次；CORE06新输入未执行，产品E2E NOT_RUN。</x:v>
+        <x:v>整版draft、未发布。27条产品TC未执行；3条CORE辅助TC已在文档提交48ca089独立切片就绪，在开发分支311deedf运行模块3/3 PASS，原始receipt在该分支.local/ci/tm003-core-20261001/。代码尚未合入本文档树，机器绑定保持空；模块报告不能作为产品E2E或发行门禁，结果Excel规范待SOP修订。 2026-10-02新代码候选44379e6已有逐步模块3/3与桌面29/29/typecheck/build原件；source_check独立Excel导出程序仍缺，批次登记BLOCKED，产品E2E仍NOT_RUN。 固定导出器新run tm003-core-20261001T163807Z在ea6b187候选生成3/3/9步source_check独立Excel并回读PASS，现已按被测SHA登记模块批次；原27条产品TC与发行仍NOT_RUN。 新清理合同候选d7c3d39的独立run tm003-core-20261001T165439Z亦3/3/9步及Excel回读PASS，作为最新模块批次；旧ea6批次保留。 后续CORE-04/05的测试输入已编制，程序未绑定、未执行；独立SOP-008切片复核待文档干净提交。 CORE04/05基于9efc6fa独立source_check 2/2、9步和Excel回读PASS，第17批次；CORE06新输入未执行，产品E2E NOT_RUN。 CORE06在eef956b的固定</x:v>
       </x:c>
       <x:c r="K8" s="9" t="str">
         <x:v>TM-001 干净源码候选为技术基底；其产品门禁不继承给TM-003</x:v>
@@ -21659,101 +21753,69 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="162" customHeight="1">
+    <x:row r="9" ht="72" customHeight="1">
       <x:c r="A9" s="4" t="str">
+        <x:v>v0.3.0-20261001T034652Z（续1）</x:v>
+      </x:c>
+      <x:c r="B9" s="4" t="str"/>
+      <x:c r="C9" s="16" t="str"/>
+      <x:c r="D9" s="4" t="str"/>
+      <x:c r="E9" s="4" t="str"/>
+      <x:c r="F9" s="4" t="str"/>
+      <x:c r="G9" s="4" t="str"/>
+      <x:c r="H9" s="4" t="str"/>
+      <x:c r="I9" s="4" t="str"/>
+      <x:c r="J9" s="4" t="str">
+        <x:v>source_check 1/1、四步与清理PASS，独立Excel回读PASS，第18批次；此前408ebf8红测失败保留。仅多文件模块，原27条产品TC与正式发行NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="K9" s="4" t="str"/>
+      <x:c r="L9" s="4" t="str"/>
+      <x:c r="M9" s="4" t="str"/>
+      <x:c r="N9" s="4" t="str"/>
+      <x:c r="O9" s="4" t="str"/>
+      <x:c r="P9" s="4" t="str"/>
+      <x:c r="Q9" s="4" t="str"/>
+      <x:c r="R9" s="4" t="str"/>
+    </x:row>
+    <x:row r="10" ht="237" customHeight="1">
+      <x:c r="A10" s="9" t="str">
         <x:v>v0.4.0-20261001T040433Z</x:v>
       </x:c>
-      <x:c r="B9" s="4" t="str">
+      <x:c r="B10" s="9" t="str">
         <x:v>0.4.0</x:v>
       </x:c>
-      <x:c r="C9" s="16" t="n">
+      <x:c r="C10" s="17" t="n">
         <x:v>46296.16982638889</x:v>
-      </x:c>
-      <x:c r="D9" s="4" t="str">
-        <x:v>产品功能</x:v>
-      </x:c>
-      <x:c r="E9" s="4" t="str">
-        <x:v>TM-004</x:v>
-      </x:c>
-      <x:c r="F9" s="4" t="str">
-        <x:v>未发布</x:v>
-      </x:c>
-      <x:c r="G9" s="4" t="str">
-        <x:v>internal</x:v>
-      </x:c>
-      <x:c r="H9" s="4" t="str">
-        <x:v>dmg/&lt;release_id&gt;/：仅门禁PASS后放正式DMG</x:v>
-      </x:c>
-      <x:c r="I9" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J9" s="4" t="str">
-        <x:v>整版draft、未发布。原20产品细TC及四组摘要保留，3条reader CORE辅助TC在输入提交fea41fe/同步SOP后的干净候选ebbcfd0上按SOP-008独立判为development_slice_ready；程序绑定仍空。本版代码分支e52b62e报告reader目标9/9、桌面49/49和build PASS，仅为模块原件，Excel/总表批次尚无固定导出器。产品授权、稳定文件身份最终接口、SQLite原子事务、IPC/App E2E未验证，正式发行门禁NOT_RUN。</x:v>
-      </x:c>
-      <x:c r="K9" s="4" t="str">
-        <x:v>TM004源分支原生零/缺失与nested Agent定向探针仅为研究证据；0.3及此前稳定原包尚未形成，真实升级BLOCKED。</x:v>
-      </x:c>
-      <x:c r="L9" s="4" t="str">
-        <x:v>releases/v0.4.0-20261001T040433Z/00-manifest.json</x:v>
-      </x:c>
-      <x:c r="M9" s="4" t="str">
-        <x:v>releases/v0.4.0-20261001T040433Z/06-iteration-record.md</x:v>
-      </x:c>
-      <x:c r="N9" s="4" t="str">
-        <x:v>未核实同名远端功能分支SHA/tree</x:v>
-      </x:c>
-      <x:c r="O9" s="4" t="str">
-        <x:v>最终包产品E2E未执行；本机稳定包未归档</x:v>
-      </x:c>
-      <x:c r="P9" s="4" t="str">
-        <x:v>全部目标版本稳定后待办</x:v>
-      </x:c>
-      <x:c r="Q9" s="4" t="str">
-        <x:v>远端master读回后逐版待办</x:v>
-      </x:c>
-      <x:c r="R9" s="4" t="str">
-        <x:v>未提供</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="267" customHeight="1">
-      <x:c r="A10" s="9" t="str">
-        <x:v>v0.5.0-20261001T034729Z</x:v>
-      </x:c>
-      <x:c r="B10" s="9" t="str">
-        <x:v>0.5.0</x:v>
-      </x:c>
-      <x:c r="C10" s="17" t="n">
-        <x:v>46296.15797453704</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
         <x:v>产品功能</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
-        <x:v>TM-005</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="F10" s="9" t="str">
-        <x:v>draft</x:v>
+        <x:v>未发布</x:v>
       </x:c>
       <x:c r="G10" s="9" t="str">
         <x:v>internal</x:v>
       </x:c>
       <x:c r="H10" s="9" t="str">
-        <x:v>dmg/&lt;release_id&gt;/：仅门禁PASS后放正式原名包</x:v>
+        <x:v>dmg/&lt;release_id&gt;/：仅门禁PASS后放正式DMG</x:v>
       </x:c>
       <x:c r="I10" s="18" t="b">
         <x:v>0</x:v>
       </x:c>
       <x:c r="J10" s="9" t="str">
-        <x:v>整版draft、未发布。原32条产品父TC、6稳定变体和两组摘要保留；纯统计CORE-01/02/03辅助TC在输入提交061c759后，经SOP-008内容核对及结构/治理457项PASS，独立切片development_slice_ready，程序绑定仍为空、模块实际运行unexecuted。静态oracle与切片就绪不证明真实双来源采集或产品E2E；固定产品数据、SQLite/IPC、安装App逐TC绑定未完成，正式发行完整门禁NOT_RUN。 独立代码提交6a0f6f的source_check CORE3/3、桌面29/29、build PASS，原件在TM005工作树.local/tm005-core-postcommit-20261001T162401Z；程序尚未进入本文档树、模块Excel导出/批次登记BLOCKED，产品E2E仍NOT_RUN。 CORE-01仅验证已给UTC半开界聚合，不验证IANA日期换算；该单独辅助TC待固定。</x:v>
+        <x:v>整版draft、未发布。原20产品细TC及四组摘要保留，3条reader CORE辅助TC在输入提交fea41fe/同步SOP后的干净候选ebbcfd0上按SOP-008独立判为development_slice_ready；程序绑定仍空。本版代码分支e52b62e报告reader目标9/9、桌面49/49和build PASS，仅为模块原件，Excel/总表批次尚无固定导出器。产品授权、稳定文件身份最终接口、SQLite原子事务、IPC/App E2E未验证，正式发行门禁NOT_RUN。 新增CORE04/05合成主进程触发及三文件存储辅助输入：拒绝码、提交守卫、来源/根分域HMAC、scope代号、modelId哨兵与整代事务；两例程序未绑定/未运行，原20条产品TC与正式发行NOT_RUN。</x:v>
       </x:c>
       <x:c r="K10" s="9" t="str">
-        <x:v>TM005语义oracle只验证规范化样例；0.4及此前稳定原包尚未形成，真实升级BLOCKED。</x:v>
+        <x:v>TM004源分支原生零/缺失与nested Agent定向探针仅为研究证据；0.3及此前稳定原包尚未形成，真实升级BLOCKED。</x:v>
       </x:c>
       <x:c r="L10" s="9" t="str">
-        <x:v>releases/v0.5.0-20261001T034729Z/00-manifest.json</x:v>
+        <x:v>releases/v0.4.0-20261001T040433Z/00-manifest.json</x:v>
       </x:c>
       <x:c r="M10" s="9" t="str">
-        <x:v>releases/v0.5.0-20261001T034729Z/06-iteration-record.md</x:v>
+        <x:v>releases/v0.4.0-20261001T040433Z/06-iteration-record.md</x:v>
       </x:c>
       <x:c r="N10" s="9" t="str">
         <x:v>未核实同名远端功能分支SHA/tree</x:v>
@@ -21771,25 +21833,81 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
+    <x:row r="11" ht="267" customHeight="1">
+      <x:c r="A11" s="4" t="str">
+        <x:v>v0.5.0-20261001T034729Z</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="str">
+        <x:v>0.5.0</x:v>
+      </x:c>
+      <x:c r="C11" s="16" t="n">
+        <x:v>46296.15797453704</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="str">
+        <x:v>产品功能</x:v>
+      </x:c>
+      <x:c r="E11" s="4" t="str">
+        <x:v>TM-005</x:v>
+      </x:c>
+      <x:c r="F11" s="4" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="G11" s="4" t="str">
+        <x:v>internal</x:v>
+      </x:c>
+      <x:c r="H11" s="4" t="str">
+        <x:v>dmg/&lt;release_id&gt;/：仅门禁PASS后放正式原名包</x:v>
+      </x:c>
+      <x:c r="I11" s="15" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J11" s="4" t="str">
+        <x:v>整版draft、未发布。原32条产品父TC、6稳定变体和两组摘要保留；纯统计CORE-01/02/03辅助TC在输入提交061c759后，经SOP-008内容核对及结构/治理457项PASS，独立切片development_slice_ready，程序绑定仍为空、模块实际运行unexecuted。静态oracle与切片就绪不证明真实双来源采集或产品E2E；固定产品数据、SQLite/IPC、安装App逐TC绑定未完成，正式发行完整门禁NOT_RUN。 独立代码提交6a0f6f的source_check CORE3/3、桌面29/29、build PASS，原件在TM005工作树.local/tm005-core-postcommit-20261001T162401Z；程序尚未进入本文档树、模块Excel导出/批次登记BLOCKED，产品E2E仍NOT_RUN。 CORE-01仅验证已给UTC半开界聚合，不验证IANA日期换算；该单独辅助TC待固定。</x:v>
+      </x:c>
+      <x:c r="K11" s="4" t="str">
+        <x:v>TM005语义oracle只验证规范化样例；0.4及此前稳定原包尚未形成，真实升级BLOCKED。</x:v>
+      </x:c>
+      <x:c r="L11" s="4" t="str">
+        <x:v>releases/v0.5.0-20261001T034729Z/00-manifest.json</x:v>
+      </x:c>
+      <x:c r="M11" s="4" t="str">
+        <x:v>releases/v0.5.0-20261001T034729Z/06-iteration-record.md</x:v>
+      </x:c>
+      <x:c r="N11" s="4" t="str">
+        <x:v>未核实同名远端功能分支SHA/tree</x:v>
+      </x:c>
+      <x:c r="O11" s="4" t="str">
+        <x:v>最终包产品E2E未执行；本机稳定包未归档</x:v>
+      </x:c>
+      <x:c r="P11" s="4" t="str">
+        <x:v>全部目标版本稳定后待办</x:v>
+      </x:c>
+      <x:c r="Q11" s="4" t="str">
+        <x:v>远端master读回后逐版待办</x:v>
+      </x:c>
+      <x:c r="R11" s="4" t="str">
+        <x:v>未提供</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="F5:F10">
+  <x:conditionalFormatting sqref="F5:F11">
     <x:cfRule type="containsText" dxfId="33" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="34" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="35" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="J5:J10">
+  <x:conditionalFormatting sqref="J5:J11">
     <x:cfRule type="containsText" dxfId="36" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="37" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="38" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M10">
+  <x:conditionalFormatting sqref="M5:M11">
     <x:cfRule type="containsText" dxfId="39" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="40" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="41" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6603ff5ad4b1416a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05ae6df2a6ec496f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22954,7 +23072,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7dfc65debf24da0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fd0a65e9add4415"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.5.0-20261001T034729Z][TM-005] Freeze IANA and SQLite snapshot slices
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Rd2a6d09f77894779"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rf4e156a1925645dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Red0433e6efb741c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R86b940aabb4d473e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R9846e0924699427f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R87d79ff2e74b42de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rf30adb9bddbd4df5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R33be556776a34e79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R1fac0a087b6e4e85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R7291e1ae66594553"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Re295b36e23cc4b12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R03da98a060ab4d87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rc913b7e1ddc34fd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R5be28f3e8f744c1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R5fb38f2805654721"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R59404c9513e44933"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rb1e39f2374b54239"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rb5d78ab00f3c4599"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Rb1c69ee60a984249"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R171637a30f9a4bbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R57f8bb6c4f834705"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R4d4ccaff825d4813"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -786,8 +786,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N276" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N276"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N278" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N278"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="功能编号"/>
     <x:tableColumn id="2" name="用例编号"/>
@@ -1134,8 +1134,8 @@
         <x:v>已登记用例</x:v>
       </x:c>
       <x:c r="B8" s="11" t="n">
-        <x:f>COUNTA('05测试用例'!B5:B276)</x:f>
-        <x:v>272</x:v>
+        <x:f>COUNTA('05测试用例'!B5:B278)</x:f>
+        <x:v>274</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>父用例与具有稳定 ID 的变体各占一行；含未来概要场景</x:v>
@@ -1169,7 +1169,7 @@
         <x:v>界面与治理检查</x:v>
       </x:c>
       <x:c r="B11" s="10" t="n">
-        <x:v>59</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C11" s="4" t="str">
         <x:v>辅助检查不能替代产品E2E；稳定变体独立列出</x:v>
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R112308681a85490a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f67fcf0e7364c95"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b0d3089fa0541b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95f5f982d560437b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6b07d381f0c44e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R165491c43adf4f37"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf01dd68b6584e30"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R665d6ed9fa6a4dfe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc237592fa63497d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68ffe26ec25d4c6d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8580111f2c5649f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdaf1cb19a5694eb9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7519,7 +7519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3aa2b3bcebe74fdd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf26d95603cd64ac9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15812,7 +15812,7 @@
         <x:v>未来概要</x:v>
       </x:c>
       <x:c r="L177" s="4" t="str">
-        <x:v>docs/testing/cases/05-TM-005-usage-statistics.md:21</x:v>
+        <x:v>docs/testing/cases/05-TM-005-usage-statistics.md:23</x:v>
       </x:c>
       <x:c r="M177" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -15858,7 +15858,7 @@
         <x:v>未来概要</x:v>
       </x:c>
       <x:c r="L178" s="9" t="str">
-        <x:v>docs/testing/cases/05-TM-005-usage-statistics.md:38</x:v>
+        <x:v>docs/testing/cases/05-TM-005-usage-statistics.md:40</x:v>
       </x:c>
       <x:c r="M178" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -20532,30 +20532,128 @@
         <x:v>v0.4.0-20261001T040433Z</x:v>
       </x:c>
     </x:row>
+    <x:row r="277" ht="87" customHeight="1">
+      <x:c r="A277" s="4" t="str">
+        <x:v>TM-005</x:v>
+      </x:c>
+      <x:c r="B277" s="4" t="str">
+        <x:v>TC-TM005-CORE-04</x:v>
+      </x:c>
+      <x:c r="C277" s="4" t="str">
+        <x:v>IANA当地日半开UTC界</x:v>
+      </x:c>
+      <x:c r="D277" s="4" t="str">
+        <x:v>TASK-TM005-RANGE-QUERY</x:v>
+      </x:c>
+      <x:c r="E277" s="4" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F277" s="4" t="str">
+        <x:v>tests/fixtures/tm005-iana-core-slice.json；上海/UTC与纽约春秋四日、三种无效输入</x:v>
+      </x:c>
+      <x:c r="G277" s="4" t="str">
+        <x:v>1. 转换上海与UTC固定当地日；分别得到fixture固定24小时UTC半开界，传入事件UTC时刻不变
+2. 转换纽约春秋DST当地日及四类边界时刻；春23小时/秋25小时；before/at_end排除，at_start/before_end纳入
+3. 分别提交无效时区、无效日和非规范日期；invalid_timezone或invalid_local_day；无默认UTC范围/成功零</x:v>
+      </x:c>
+      <x:c r="H277" s="4" t="str">
+        <x:v>准备：无DB
+变化：无DB或系统时间变化
+核验：固定IANA各日UTC半开界、23/25小时、边界包含关系及错误码；无SQL</x:v>
+      </x:c>
+      <x:c r="I277" s="4" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J277" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K277" s="4" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L277" s="4" t="str">
+        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:354</x:v>
+      </x:c>
+      <x:c r="M277" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N277" s="4" t="str">
+        <x:v>v0.5.0-20261001T034729Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="278" ht="132" customHeight="1">
+      <x:c r="A278" s="9" t="str">
+        <x:v>TM-005</x:v>
+      </x:c>
+      <x:c r="B278" s="9" t="str">
+        <x:v>TC-TM005-CORE-05</x:v>
+      </x:c>
+      <x:c r="C278" s="9" t="str">
+        <x:v>双来源隔离SQLite同窗只读快照</x:v>
+      </x:c>
+      <x:c r="D278" s="9" t="str">
+        <x:v>TASK-TM005-EVENT-CONTRACT
+TASK-TM005-RANGE-QUERY</x:v>
+      </x:c>
+      <x:c r="E278" s="9" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F278" s="9" t="str">
+        <x:v>tests/fixtures/tm005-sqlite-snapshot-slice.json；A/B双来源330、C异主体、D/E界外、F并发后新快照+55</x:v>
+      </x:c>
+      <x:c r="G278" s="9" t="str">
+        <x:v>1. 固定插入A–E并开启同一读事务；选A/B两调用，input300/output30/total330；C/D/E分别被主体或半开界排除，查询零写
+2. 在同一读事务取来源、模型、明细与逐日点；Codex110/Claude220；未知模型110/sonnet-test220；明细A/B和日点330；缓存读known20+unknown1，子项不加总
+3. 另一连接提交F后复查旧快照，再开新快照；旧事务各视图仍A/B和330；新事务A/B/F三调用、input350/output35/total385、Codex165/Claude220
+4. 查询空日及隐私边界；现有coverage不证明当地空日完整，不能报产品零；库/WAL/输出无原生ID、路径、正文或秘密</x:v>
+      </x:c>
+      <x:c r="H278" s="9" t="str">
+        <x:v>准备：固定准备程序仅在本例owner SQLite经UsageStore.commitBatch提交A–E；启用WAL并记录前态
+变化：查询零写入；另一连接固定提交F后旧读事务仍330，新读事务385
+核验：只读usage_event按主体/source/UTC半开界核对事件、来源/模型/明细/日点与子项未知数；coverage不能证明完整空日</x:v>
+      </x:c>
+      <x:c r="I278" s="9" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J278" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K278" s="9" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L278" s="9" t="str">
+        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:362</x:v>
+      </x:c>
+      <x:c r="M278" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N278" s="9" t="str">
+        <x:v>v0.5.0-20261001T034729Z</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G5:G276">
+  <x:conditionalFormatting sqref="G5:G278">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="I5:I276">
+  <x:conditionalFormatting sqref="I5:I278">
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="16" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="17" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="J5:J276">
+  <x:conditionalFormatting sqref="J5:J278">
     <x:cfRule type="containsText" dxfId="18" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="19" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="20" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M276">
+  <x:conditionalFormatting sqref="M5:M278">
     <x:cfRule type="containsText" dxfId="21" priority="10" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="22" priority="11" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="23" priority="12" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07055277d0114c75"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50ad1a979e9f49c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21439,7 +21537,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfef00fe67eeb4ddb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2673db9b28934247"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21833,7 +21931,7 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="267" customHeight="1">
+    <x:row r="11" ht="327" customHeight="1">
       <x:c r="A11" s="4" t="str">
         <x:v>v0.5.0-20261001T034729Z</x:v>
       </x:c>
@@ -21862,7 +21960,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J11" s="4" t="str">
-        <x:v>整版draft、未发布。原32条产品父TC、6稳定变体和两组摘要保留；纯统计CORE-01/02/03辅助TC在输入提交061c759后，经SOP-008内容核对及结构/治理457项PASS，独立切片development_slice_ready，程序绑定仍为空、模块实际运行unexecuted。静态oracle与切片就绪不证明真实双来源采集或产品E2E；固定产品数据、SQLite/IPC、安装App逐TC绑定未完成，正式发行完整门禁NOT_RUN。 独立代码提交6a0f6f的source_check CORE3/3、桌面29/29、build PASS，原件在TM005工作树.local/tm005-core-postcommit-20261001T162401Z；程序尚未进入本文档树、模块Excel导出/批次登记BLOCKED，产品E2E仍NOT_RUN。 CORE-01仅验证已给UTC半开界聚合，不验证IANA日期换算；该单独辅助TC待固定。</x:v>
+        <x:v>整版draft、未发布。原32条产品父TC、6稳定变体和两组摘要保留；纯统计CORE-01/02/03辅助TC在输入提交061c759后，经SOP-008内容核对及结构/治理457项PASS，独立切片development_slice_ready，程序绑定仍为空、模块实际运行unexecuted。静态oracle与切片就绪不证明真实双来源采集或产品E2E；固定产品数据、SQLite/IPC、安装App逐TC绑定未完成，正式发行完整门禁NOT_RUN。 独立代码提交6a0f6f的source_check CORE3/3、桌面29/29、build PASS，原件在TM005工作树.local/tm005-core-postcommit-20261001T162401Z；程序尚未进入本文档树、模块Excel导出/批次登记BLOCKED，产品E2E仍NOT_RUN。 CORE-01仅验证已给UTC半开界聚合，不验证IANA日期换算；该单独辅助TC待固定。 新增CORE04/05固定IANA当地日与合成双来源SQLite只读快照辅助TC，程序null/unexecuted；coverage表无连续空日证明，原32产品TC/6变体与发行仍BLOCKED/NOT_RUN。</x:v>
       </x:c>
       <x:c r="K11" s="4" t="str">
         <x:v>TM005语义oracle只验证规范化样例；0.4及此前稳定原包尚未形成，真实升级BLOCKED。</x:v>
@@ -21907,7 +22005,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05ae6df2a6ec496f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40c2610ef7584128"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23072,7 +23170,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fd0a65e9add4415"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19dc7b9740c5447e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.1.0-20260929T074814Z][TM-001] Index login probe and correct bootstrap binding
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R03da98a060ab4d87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rc913b7e1ddc34fd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R5be28f3e8f744c1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R5fb38f2805654721"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R59404c9513e44933"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rb1e39f2374b54239"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rb5d78ab00f3c4599"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Rb1c69ee60a984249"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R171637a30f9a4bbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R57f8bb6c4f834705"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R4d4ccaff825d4813"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Rfe05154a975845bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Ra3b4b22b95ac43e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R7f533fc21dc34947"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rcbce82796618482d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R4acab15c44c645bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R439bef78c4784c60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rfb32810f08f8448a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R9d4b22d3f2c3492d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R5fb85447064a443b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Reecff22380fc45ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R18d2afb9c5d7434a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -809,8 +809,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N22"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N23"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="运行批次"/>
     <x:tableColumn id="2" name="版本"/>
@@ -1146,8 +1146,8 @@
         <x:v>测试批次</x:v>
       </x:c>
       <x:c r="B9" s="10" t="n">
-        <x:f>COUNTA('06测试批次'!A5:A22)</x:f>
-        <x:v>18</x:v>
+        <x:f>COUNTA('06测试批次'!A5:A23)</x:f>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>06测试批次，每次运行一行，记录独立结果Excel位置</x:v>
@@ -1263,7 +1263,7 @@
         <x:v>DMG及原始证据留本机；Git保存代码、文档和此工作簿</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="72" customHeight="1">
+    <x:row r="20" ht="87" customHeight="1">
       <x:c r="A20" s="9" t="str">
         <x:v>最近登记批次</x:v>
       </x:c>
@@ -1271,7 +1271,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>source_check · TM-003 CORE-06 固定多文件代际提交与全回滚；非产品E2E：source_check固定CORE06 1/1、四步及owner清理PASS；此前408ebf8红测步骤2 FAIL保留。独立Excel/verification回读PASS。原27条产品TC、App E2E与发行均NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
+        <x:v>product_e2e · TASK-TM001-LOGIN-AUTH；仅LOGIN-01/02/03/04/08五条固定父TC，安装原DMG的真实App定向回归：原始App定向run五条父TC、11步骤PASS，cleanup_completed=true；前置误加--development的独立run local-7ce07b71ca1240de93c16a437ab7e292在清单预检处5例BLOCKED且App未启动，保留原件不混入本批PASS。其余TM001父TC在709d未运行，旧c291完整门禁FAIL及正式发行NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f67fcf0e7364c95"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2a6a9990ee74b4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95f5f982d560437b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51fd4f6cad34451f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R165491c43adf4f37"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbfdd2f932b9450c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R665d6ed9fa6a4dfe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3156454378504541"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68ffe26ec25d4c6d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97ed798623cb46cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdaf1cb19a5694eb9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b9e21e2ae78491c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7519,7 +7519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf26d95603cd64ac9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59eb394ef4834d88"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7635,7 +7635,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:76</x:v>
       </x:c>
       <x:c r="M5" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-2aa05fb7b2754289a1d77b9ef89bd321</x:v>
       </x:c>
       <x:c r="N5" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -7682,7 +7682,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:92</x:v>
       </x:c>
       <x:c r="M6" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-2aa05fb7b2754289a1d77b9ef89bd321</x:v>
       </x:c>
       <x:c r="N6" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -7729,7 +7729,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:107</x:v>
       </x:c>
       <x:c r="M7" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-2aa05fb7b2754289a1d77b9ef89bd321</x:v>
       </x:c>
       <x:c r="N7" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -7776,7 +7776,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:122</x:v>
       </x:c>
       <x:c r="M8" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-2aa05fb7b2754289a1d77b9ef89bd321</x:v>
       </x:c>
       <x:c r="N8" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -7964,7 +7964,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:182</x:v>
       </x:c>
       <x:c r="M12" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-2aa05fb7b2754289a1d77b9ef89bd321</x:v>
       </x:c>
       <x:c r="N12" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -10061,7 +10061,7 @@
 新成员及admin改后状态完整保留，首建不是每次启动清库</x:v>
       </x:c>
       <x:c r="H56" s="9" t="str">
-        <x:v>准备：D-PROD先真实改密；额外成员用批准provision输入，数据绑定待补
+        <x:v>准备：D-PROD先在真实UI改密；固定Playwright程序以离线provision向本例拥有的库添加尾0007的test-extra成员，再读回与重启核对；不接触用户生产库。
 变化：重启不重置散列/账号；重复初始化/错误seed事务拒绝且原行保留；123456仍失效
 只读核验：Q-OWNER、Q-SCHEMA、Q-USERS、Q-AUDIT、Q-INTEGRITY</x:v>
       </x:c>
@@ -20653,7 +20653,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50ad1a979e9f49c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46bf37bcf6b24826"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21519,25 +21519,69 @@
         <x:v>NOT_RUN</x:v>
       </x:c>
     </x:row>
+    <x:row r="23" ht="72" customHeight="1">
+      <x:c r="A23" s="4" t="str">
+        <x:v>local-2aa05fb7b2754289a1d77b9ef89bd321</x:v>
+      </x:c>
+      <x:c r="B23" s="4" t="str">
+        <x:v>v0.1.0-20260929T074814Z</x:v>
+      </x:c>
+      <x:c r="C23" s="4" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D23" s="4" t="str">
+        <x:v>TASK-TM001-LOGIN-AUTH；仅LOGIN-01/02/03/04/08五条固定父TC，安装原DMG的真实App定向回归</x:v>
+      </x:c>
+      <x:c r="E23" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F23" s="4" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G23" s="4" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H23" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I23" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J23" s="4" t="str">
+        <x:v>709d21253a0f88bc703a431cbf3adba3df17e508</x:v>
+      </x:c>
+      <x:c r="K23" s="4" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L23" s="4" t="str">
+        <x:v>原始App定向run五条父TC、11步骤PASS，cleanup_completed=true；前置误加--development的独立run local-7ce07b71ca1240de93c16a437ab7e292在清单预检处5例BLOCKED且App未启动，保留原件不混入本批PASS。其余TM001父TC在709d未运行，旧c291完整门禁FAIL及正式发行NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M23" s="4" t="str">
+        <x:v>.local/test-results/local-2aa05fb7b2754289a1d77b9ef89bd321/TokenMeter测试结果-local-2aa05fb7b2754289a1d77b9ef89bd321.xlsx</x:v>
+      </x:c>
+      <x:c r="N23" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E5:E22">
+  <x:conditionalFormatting sqref="E5:E23">
     <x:cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="26" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M22">
+  <x:conditionalFormatting sqref="M5:M23">
     <x:cfRule type="containsText" dxfId="27" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="29" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="N5:N22">
+  <x:conditionalFormatting sqref="N5:N23">
     <x:cfRule type="containsText" dxfId="30" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="32" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2673db9b28934247"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b1053466448425a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21683,7 +21727,7 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="177" customHeight="1">
+    <x:row r="6" ht="207" customHeight="1">
       <x:c r="A6" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
@@ -21712,7 +21756,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J6" s="9" t="str">
-        <x:v>开发中，未发布。c291本地master最终包门禁FAIL：116项91 PASS/14 FAIL/11 BLOCKED；9f06cb1修复私有签名输入后开发检查PASS，但新定向App仍FAIL/BLOCKED并有ENOSPC，功能回归未完成。旧d2db551独立候选PASS不转用于新候选。正式发行完整门禁NOT_RUN，无稳定0.1原包。 709d UPDATE-05定向父1+变体13 PASS，后置de081a6导出Excel回读PASS；仅定向，77父TC范围外，旧c291完整门禁FAIL及未发行不变。</x:v>
+        <x:v>开发中，未发布。c291本地master最终包门禁FAIL：116项91 PASS/14 FAIL/11 BLOCKED；9f06cb1修复私有签名输入后开发检查PASS，但新定向App仍FAIL/BLOCKED并有ENOSPC，功能回归未完成。旧d2db551独立候选PASS不转用于新候选。正式发行完整门禁NOT_RUN，无稳定0.1原包。 709d UPDATE-05定向父1+变体13 PASS，后置de081a6导出Excel回读PASS；仅定向，77父TC范围外，旧c291完整门禁FAIL及未发行不变。 709d安装DMG的登录定向五父例/11步原始PASS，独立Excel回读PASS；仍非整版回归，旧c291完整门禁FAIL。</x:v>
       </x:c>
       <x:c r="K6" s="9" t="str">
         <x:v>旧SwiftUI PR #2 已合并、历史双平台六例PASS；不继承给Electron</x:v>
@@ -22005,7 +22049,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40c2610ef7584128"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde003fe1710f4bf0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23170,7 +23214,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19dc7b9740c5447e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8033685bd13348ed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.1.0-20260929T074814Z][TM-001] Index login session probe
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Rfe05154a975845bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Ra3b4b22b95ac43e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R7f533fc21dc34947"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rcbce82796618482d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R4acab15c44c645bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R439bef78c4784c60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rfb32810f08f8448a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R9d4b22d3f2c3492d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R5fb85447064a443b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Reecff22380fc45ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R18d2afb9c5d7434a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R40eec56730e94cb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R2d0243dab96f4272"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R4f7c2e65804d429e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R7432be5ea61948a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R62b52c4fd3d4449e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Ra062c60b9f1f4b1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R5304bf93fcdc463c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R88d16b11c9c24d8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R2033abd9b4934d9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Raa7b5685110e4847"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R8f4259f914264c18"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -809,8 +809,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N23"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N24"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="运行批次"/>
     <x:tableColumn id="2" name="版本"/>
@@ -1146,8 +1146,8 @@
         <x:v>测试批次</x:v>
       </x:c>
       <x:c r="B9" s="10" t="n">
-        <x:f>COUNTA('06测试批次'!A5:A23)</x:f>
-        <x:v>19</x:v>
+        <x:f>COUNTA('06测试批次'!A5:A24)</x:f>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>06测试批次，每次运行一行，记录独立结果Excel位置</x:v>
@@ -1263,7 +1263,7 @@
         <x:v>DMG及原始证据留本机；Git保存代码、文档和此工作簿</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="87" customHeight="1">
+    <x:row r="20" ht="72" customHeight="1">
       <x:c r="A20" s="9" t="str">
         <x:v>最近登记批次</x:v>
       </x:c>
@@ -1271,7 +1271,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>product_e2e · TASK-TM001-LOGIN-AUTH；仅LOGIN-01/02/03/04/08五条固定父TC，安装原DMG的真实App定向回归：原始App定向run五条父TC、11步骤PASS，cleanup_completed=true；前置误加--development的独立run local-7ce07b71ca1240de93c16a437ab7e292在清单预检处5例BLOCKED且App未启动，保留原件不混入本批PASS。其余TM001父TC在709d未运行，旧c291完整门禁FAIL及正式发行NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
+        <x:v>product_e2e · TASK-TM001-LOGIN-SESSION；仅LOGIN-10/11/12/13/14/15六条固定父TC，真实App定向回归：原始真实App定向run六条父TC、14步骤PASS，cleanup_completed=true；独立Excel/verification PASS。与LOGIN-AUTH为不同run，709d其余TM001父TC未运行；旧c291完整门禁FAIL及正式发行NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2a6a9990ee74b4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R723af0d63ca24a15"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51fd4f6cad34451f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R808cf99423ce413b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbfdd2f932b9450c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1136ecb951694a09"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3156454378504541"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f769844bef445eb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97ed798623cb46cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34b9211cc0704e14"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b9e21e2ae78491c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c3b6d4310d04cf4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7519,7 +7519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59eb394ef4834d88"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reefe618ae2574f9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8058,7 +8058,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:212</x:v>
       </x:c>
       <x:c r="M14" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-1d7d9238f9fd4d389e27cad990a6cb97</x:v>
       </x:c>
       <x:c r="N14" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -8106,7 +8106,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:227</x:v>
       </x:c>
       <x:c r="M15" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-1d7d9238f9fd4d389e27cad990a6cb97</x:v>
       </x:c>
       <x:c r="N15" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -8154,7 +8154,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:243</x:v>
       </x:c>
       <x:c r="M16" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-1d7d9238f9fd4d389e27cad990a6cb97</x:v>
       </x:c>
       <x:c r="N16" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -8201,7 +8201,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:259</x:v>
       </x:c>
       <x:c r="M17" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-1d7d9238f9fd4d389e27cad990a6cb97</x:v>
       </x:c>
       <x:c r="N17" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -8248,7 +8248,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:274</x:v>
       </x:c>
       <x:c r="M18" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-1d7d9238f9fd4d389e27cad990a6cb97</x:v>
       </x:c>
       <x:c r="N18" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -8295,7 +8295,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:289</x:v>
       </x:c>
       <x:c r="M19" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-1d7d9238f9fd4d389e27cad990a6cb97</x:v>
       </x:c>
       <x:c r="N19" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -20653,7 +20653,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46bf37bcf6b24826"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a6423fa3c604459"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21563,25 +21563,69 @@
         <x:v>PASS</x:v>
       </x:c>
     </x:row>
+    <x:row r="24" ht="57" customHeight="1">
+      <x:c r="A24" s="9" t="str">
+        <x:v>local-1d7d9238f9fd4d389e27cad990a6cb97</x:v>
+      </x:c>
+      <x:c r="B24" s="9" t="str">
+        <x:v>v0.1.0-20260929T074814Z</x:v>
+      </x:c>
+      <x:c r="C24" s="9" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D24" s="9" t="str">
+        <x:v>TASK-TM001-LOGIN-SESSION；仅LOGIN-10/11/12/13/14/15六条固定父TC，真实App定向回归</x:v>
+      </x:c>
+      <x:c r="E24" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F24" s="9" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G24" s="9" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H24" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I24" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J24" s="9" t="str">
+        <x:v>709d21253a0f88bc703a431cbf3adba3df17e508</x:v>
+      </x:c>
+      <x:c r="K24" s="9" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L24" s="9" t="str">
+        <x:v>原始真实App定向run六条父TC、14步骤PASS，cleanup_completed=true；独立Excel/verification PASS。与LOGIN-AUTH为不同run，709d其余TM001父TC未运行；旧c291完整门禁FAIL及正式发行NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M24" s="9" t="str">
+        <x:v>.local/test-results/local-1d7d9238f9fd4d389e27cad990a6cb97/TokenMeter测试结果-local-1d7d9238f9fd4d389e27cad990a6cb97.xlsx</x:v>
+      </x:c>
+      <x:c r="N24" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E5:E23">
+  <x:conditionalFormatting sqref="E5:E24">
     <x:cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="26" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M23">
+  <x:conditionalFormatting sqref="M5:M24">
     <x:cfRule type="containsText" dxfId="27" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="29" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="N5:N23">
+  <x:conditionalFormatting sqref="N5:N24">
     <x:cfRule type="containsText" dxfId="30" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="32" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b1053466448425a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06d2cb7561004b00"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21727,7 +21771,7 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="207" customHeight="1">
+    <x:row r="6" ht="237" customHeight="1">
       <x:c r="A6" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
@@ -21756,7 +21800,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J6" s="9" t="str">
-        <x:v>开发中，未发布。c291本地master最终包门禁FAIL：116项91 PASS/14 FAIL/11 BLOCKED；9f06cb1修复私有签名输入后开发检查PASS，但新定向App仍FAIL/BLOCKED并有ENOSPC，功能回归未完成。旧d2db551独立候选PASS不转用于新候选。正式发行完整门禁NOT_RUN，无稳定0.1原包。 709d UPDATE-05定向父1+变体13 PASS，后置de081a6导出Excel回读PASS；仅定向，77父TC范围外，旧c291完整门禁FAIL及未发行不变。 709d安装DMG的登录定向五父例/11步原始PASS，独立Excel回读PASS；仍非整版回归，旧c291完整门禁FAIL。</x:v>
+        <x:v>开发中，未发布。c291本地master最终包门禁FAIL：116项91 PASS/14 FAIL/11 BLOCKED；9f06cb1修复私有签名输入后开发检查PASS，但新定向App仍FAIL/BLOCKED并有ENOSPC，功能回归未完成。旧d2db551独立候选PASS不转用于新候选。正式发行完整门禁NOT_RUN，无稳定0.1原包。 709d UPDATE-05定向父1+变体13 PASS，后置de081a6导出Excel回读PASS；仅定向，77父TC范围外，旧c291完整门禁FAIL及未发行不变。 709d安装DMG的登录定向五父例/11步原始PASS，独立Excel回读PASS；仍非整版回归，旧c291完整门禁FAIL。 709d LOGIN-SESSION另六父例/14步原始PASS并单独导出Excel；未完成整版回归。</x:v>
       </x:c>
       <x:c r="K6" s="9" t="str">
         <x:v>旧SwiftUI PR #2 已合并、历史双平台六例PASS；不继承给Electron</x:v>
@@ -22049,7 +22093,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde003fe1710f4bf0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45b56c3c45a94b44"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23214,7 +23258,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8033685bd13348ed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fffb01a21df4546"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.2.0-20261001T034118Z][TM-002] Record blocked package preflight
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R40eec56730e94cb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R2d0243dab96f4272"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R4f7c2e65804d429e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R7432be5ea61948a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R62b52c4fd3d4449e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Ra062c60b9f1f4b1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R5304bf93fcdc463c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R88d16b11c9c24d8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R2033abd9b4934d9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Raa7b5685110e4847"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R8f4259f914264c18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R8cdafae5ccab484a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rcb8f66cdc3514d53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R28ce7a812c584bb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Ra0fe381165cd4a19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R4533929afd8f4c9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rf65a19c6ff634f23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R7f4d35d8ac554b24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R84e315dc370e4a55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R73cb57d499cc4b22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Re986d5fc29994387"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Re668346564824b45"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R723af0d63ca24a15"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a2e04e222b54c30"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R808cf99423ce413b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81c65f4b63f14b8f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1136ecb951694a09"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c51b6908a3a4dc2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f769844bef445eb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf58f71e53f784f76"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34b9211cc0704e14"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc659f5cd08f4353"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c3b6d4310d04cf4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc94bbc0bb40546f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7519,7 +7519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reefe618ae2574f9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R931bb2c1ca274f7b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20653,7 +20653,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a6423fa3c604459"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc90cfc758c1542e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21625,7 +21625,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06d2cb7561004b00"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c8c0c3c927249f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21827,7 +21827,7 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="282" customHeight="1">
+    <x:row r="7" ht="342" customHeight="1">
       <x:c r="A7" s="4" t="str">
         <x:v>v0.2.0-20261001T034118Z</x:v>
       </x:c>
@@ -21856,7 +21856,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J7" s="4" t="str">
-        <x:v>设计基线已完成：3功能点、9 TASK、28父TC、35变体。开发工作树已有原生目录面板、加密locator、根FD受限读取、React授权UI及33个固定E2E叶入口（28可执行、5场景摘要）；报告单元59/59、治理473/473、构建PASS。产品E2E因AX trusted=false及隔离标准测试账号不可用BLOCKED，Keychain最终包隔离未证实。本独立文档树未合该代码，机器绑定仍planned；正式发行完整门禁NOT_RUN、未发布。0.2公开配置为version0.2.0/build200及测试高版0.2.1/build201，实际0.2包尚未证明。 2026-10-02修订SECURITY-01三个恶意字串变体的固定IPC method/字段/错误码，产品状态不变；需在整合候选重核基线及固定程序。 EVIDENCE-01新增第七固定负例，本版36变体；SECURITY-01仅profile准备目录纠错。新输入未执行，产品E2E仍NOT_RUN。</x:v>
+        <x:v>设计基线已完成：3功能点、9 TASK、28父TC、35变体。开发工作树已有原生目录面板、加密locator、根FD受限读取、React授权UI及33个固定E2E叶入口（28可执行、5场景摘要）；报告单元59/59、治理473/473、构建PASS。产品E2E因AX trusted=false及隔离标准测试账号不可用BLOCKED，Keychain最终包隔离未证实。本独立文档树未合该代码，机器绑定仍planned；正式发行完整门禁NOT_RUN、未发布。0.2公开配置为version0.2.0/build200及测试高版0.2.1/build201，实际0.2包尚未证明。 2026-10-02修订SECURITY-01三个恶意字串变体的固定IPC method/字段/错误码，产品状态不变；需在整合候选重核基线及固定程序。 EVIDENCE-01新增第七固定负例，本版36变体；SECURITY-01仅profile准备目录纠错。新输入未执行，产品E2E仍NOT_RUN。 0cc4f3e候选包预检33条全BLOCKED、零产品步骤；缺显式独立test/excluded账号，App未启动；固定结果Excel缺失，根总表批次待登记。</x:v>
       </x:c>
       <x:c r="K7" s="4" t="str">
         <x:v>TM001独立候选d2门禁PASS只属历史；本地master c2911bc首次最终包门禁FAIL、无SOP-020稳定原包，不能作为0.2升级源；本版无实际产品运行。</x:v>
@@ -22093,7 +22093,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45b56c3c45a94b44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ef5d7f22e44442b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23258,7 +23258,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fffb01a21df4546"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8347536de86f4d49"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.3.0-20261001T034652Z][TM-003] Freeze main collector source check slice
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R8cdafae5ccab484a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rcb8f66cdc3514d53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R28ce7a812c584bb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Ra0fe381165cd4a19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R4533929afd8f4c9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rf65a19c6ff634f23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R7f4d35d8ac554b24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R84e315dc370e4a55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R73cb57d499cc4b22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Re986d5fc29994387"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Re668346564824b45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R6859e9789eaa4df4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R4640075aba8a46ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R60a530bf23a54544"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R2359c002b9c04b97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R576e404900d24273"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R4abac05370484d31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R404411f10c8b4644"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R42b671ea6dee41d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Red5216beacbc41fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R980a7298878d4026"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R55e5b945aebc4eb0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -786,8 +786,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N278" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N278"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N279" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N279"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="功能编号"/>
     <x:tableColumn id="2" name="用例编号"/>
@@ -1134,8 +1134,8 @@
         <x:v>已登记用例</x:v>
       </x:c>
       <x:c r="B8" s="11" t="n">
-        <x:f>COUNTA('05测试用例'!B5:B278)</x:f>
-        <x:v>274</x:v>
+        <x:f>COUNTA('05测试用例'!B5:B279)</x:f>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>父用例与具有稳定 ID 的变体各占一行；含未来概要场景</x:v>
@@ -1169,7 +1169,7 @@
         <x:v>界面与治理检查</x:v>
       </x:c>
       <x:c r="B11" s="10" t="n">
-        <x:v>61</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C11" s="4" t="str">
         <x:v>辅助检查不能替代产品E2E；稳定变体独立列出</x:v>
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a2e04e222b54c30"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86fe8959df4e4996"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81c65f4b63f14b8f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8261aaa075b24b03"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c51b6908a3a4dc2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6de93d56ad0c49f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf58f71e53f784f76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc67abf79e706473f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc659f5cd08f4353"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14b7815ba70e4401"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc94bbc0bb40546f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc59ced9c7c9e4ae9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7519,7 +7519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R931bb2c1ca274f7b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R417c62f167974b9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18586,7 +18586,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L236" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:251</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:265</x:v>
       </x:c>
       <x:c r="M236" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18633,7 +18633,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L237" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:255</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:269</x:v>
       </x:c>
       <x:c r="M237" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18680,7 +18680,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L238" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:259</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:273</x:v>
       </x:c>
       <x:c r="M238" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18728,7 +18728,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L239" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:263</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:277</x:v>
       </x:c>
       <x:c r="M239" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18778,7 +18778,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L240" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:267</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:281</x:v>
       </x:c>
       <x:c r="M240" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18826,7 +18826,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L241" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:271</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:285</x:v>
       </x:c>
       <x:c r="M241" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18873,7 +18873,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L242" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:275</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:289</x:v>
       </x:c>
       <x:c r="M242" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18920,7 +18920,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L243" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:279</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:293</x:v>
       </x:c>
       <x:c r="M243" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18968,7 +18968,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L244" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:283</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:297</x:v>
       </x:c>
       <x:c r="M244" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19017,7 +19017,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L245" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:287</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:301</x:v>
       </x:c>
       <x:c r="M245" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19066,7 +19066,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L246" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:291</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:305</x:v>
       </x:c>
       <x:c r="M246" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19115,7 +19115,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L247" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:295</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:309</x:v>
       </x:c>
       <x:c r="M247" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19162,7 +19162,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L248" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:299</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:313</x:v>
       </x:c>
       <x:c r="M248" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19210,7 +19210,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L249" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:303</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:317</x:v>
       </x:c>
       <x:c r="M249" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19258,7 +19258,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L250" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:307</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:321</x:v>
       </x:c>
       <x:c r="M250" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19306,7 +19306,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L251" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:311</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:325</x:v>
       </x:c>
       <x:c r="M251" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19354,7 +19354,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L252" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:315</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:329</x:v>
       </x:c>
       <x:c r="M252" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19404,7 +19404,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L253" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:319</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:333</x:v>
       </x:c>
       <x:c r="M253" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19451,7 +19451,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L254" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:323</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:337</x:v>
       </x:c>
       <x:c r="M254" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19498,7 +19498,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L255" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:327</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:341</x:v>
       </x:c>
       <x:c r="M255" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19546,7 +19546,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L256" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:331</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:345</x:v>
       </x:c>
       <x:c r="M256" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19595,7 +19595,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L257" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:335</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:349</x:v>
       </x:c>
       <x:c r="M257" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19645,7 +19645,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L258" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:339</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:353</x:v>
       </x:c>
       <x:c r="M258" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19693,7 +19693,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L259" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:343</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:357</x:v>
       </x:c>
       <x:c r="M259" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19742,7 +19742,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L260" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:347</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:361</x:v>
       </x:c>
       <x:c r="M260" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19790,7 +19790,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L261" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:351</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:365</x:v>
       </x:c>
       <x:c r="M261" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19838,7 +19838,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L262" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:355</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:369</x:v>
       </x:c>
       <x:c r="M262" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19886,7 +19886,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L263" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:359</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:373</x:v>
       </x:c>
       <x:c r="M263" s="4" t="str">
         <x:v>tm003-core-20261001T165439Z (source_check；产品E2E未运行)</x:v>
@@ -19935,7 +19935,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L264" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:363</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:377</x:v>
       </x:c>
       <x:c r="M264" s="9" t="str">
         <x:v>tm003-core-20261001T165439Z (source_check；产品E2E未运行)</x:v>
@@ -19983,7 +19983,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L265" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:367</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:381</x:v>
       </x:c>
       <x:c r="M265" s="4" t="str">
         <x:v>tm003-core-20261001T165439Z (source_check；产品E2E未运行)</x:v>
@@ -20142,79 +20142,81 @@
         <x:v>v0.3.0-20261001T034652Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="269" ht="87" customHeight="1">
+    <x:row r="269" ht="117" customHeight="1">
       <x:c r="A269" s="4" t="str">
+        <x:v>TM-003</x:v>
+      </x:c>
+      <x:c r="B269" s="4" t="str">
+        <x:v>TC-TM003-CORE-07</x:v>
+      </x:c>
+      <x:c r="C269" s="4" t="str">
+        <x:v>主进程采集编排与能力失效</x:v>
+      </x:c>
+      <x:c r="D269" s="4" t="str">
+        <x:v>TASK-TM003-SCAN
+TASK-TM003-STORE</x:v>
+      </x:c>
+      <x:c r="E269" s="4" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F269" s="4" t="str">
+        <x:v>固定同代际两页file-a/file-b各410字节、假readCandidateChunk每次最多返128字节、65536请求上限、公开HMAC root/file键向量；坏sourceId/主体/采集授权、提前EOF/读异常/1025字节元数据对1024注入暂存预算、撤权/切换主体；五步。</x:v>
+      </x:c>
+      <x:c r="G269" s="4" t="str">
+        <x:v>扫描前拒绝；beginCandidateScan与commitScanBatch调用0次，不写事件/游标/覆盖，不接受renderer路径/账号/密钥
+第一页无落库；末页完整稳定后A/B两事件、input300/output30/cached60/total330，两游标各410、coverage.scan_incomplete=0，commitScanBatch1次，cancelScan1次且无私密哨兵
+三路径均取消、提交0次、四表无行；请求≤65536，超预算在完整Buffer分配前失败，不截断正文后提交
+守卫拒绝、cancelScan各1次、同步提交0次，旧主体暂存不写新主体
+根/文件HMAC键及调用身份稳定，A/B仍各一、total330、游标各410，重扫仍经守卫和关闭，不输出私密哨兵</x:v>
+      </x:c>
+      <x:c r="H269" s="4" t="str">
+        <x:v>准备：每个故障变体本例owner0700根/0600新SQLite；事件只经正式解析/UsageStore；公开测试key不进入产品profile
+变化：仅完整稳定且guard通过的两页代际一次事务入A/B；所有预检、读取、容量和失权故障零提交；重扫去重
+核验：逐步只读usage_event数量/聚合/HMAC键、source_cursor两个偏移/prefixMAC、collection_diagnostic、coverage和库/WAL私密哨兵；核fake端口调用顺序/次数及owner清理</x:v>
+      </x:c>
+      <x:c r="I269" s="4" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J269" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K269" s="4" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L269" s="4" t="str">
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:243</x:v>
+      </x:c>
+      <x:c r="M269" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N269" s="4" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="270" ht="87" customHeight="1">
+      <x:c r="A270" s="9" t="str">
         <x:v>TM-005</x:v>
       </x:c>
-      <x:c r="B269" s="4" t="str">
+      <x:c r="B270" s="9" t="str">
         <x:v>TC-TM005-CORE-01</x:v>
       </x:c>
-      <x:c r="C269" s="4" t="str">
+      <x:c r="C270" s="9" t="str">
         <x:v>双来源可信事件与半开日汇总</x:v>
       </x:c>
-      <x:c r="D269" s="4" t="str">
+      <x:c r="D270" s="9" t="str">
         <x:v>TASK-TM005-EVENT-CONTRACT
 TASK-TM005-RANGE-QUERY</x:v>
       </x:c>
-      <x:c r="E269" s="4" t="str">
+      <x:c r="E270" s="9" t="str">
         <x:v>模块检查</x:v>
       </x:c>
-      <x:c r="F269" s="4" t="str">
+      <x:c r="F270" s="9" t="str">
         <x:v>fixture的A/B、跨主体C、界外D/E；synthetic-p1、Asia/Shanghai当地日2026-09-29</x:v>
       </x:c>
-      <x:c r="G269" s="4" t="str">
+      <x:c r="G270" s="9" t="str">
         <x:v>1. 按固定主体和fixture固定UTC半开界查询纯统计函数，不做IANA日期换算；仅A/B被选、C/D/E排除；输入数组和键不变
 2. 核对来源、模型、Token和三个子项；input300/output30/total330；Codex110/Claude220；未知模型110/sonnet-test220；缓存读20但部分未知、缓存写未知、推理2但部分未知，子项不加总
 3. 逐个输入非法来源、负数、超范围缓存和坏UTC；各自被拒绝，无完整零或有效汇总输出；原fixture不变</x:v>
-      </x:c>
-      <x:c r="H269" s="4" t="str">
-        <x:v>准备：无产品DB写入；每例从新内存输入开始
-变化：不适用；纯统计返回值与输入未变
-核验：固定fixture摘要、事件筛选、各字段与状态逐步核对；无SQL</x:v>
-      </x:c>
-      <x:c r="I269" s="4" t="str">
-        <x:v>draft</x:v>
-      </x:c>
-      <x:c r="J269" s="4" t="str">
-        <x:v>未执行</x:v>
-      </x:c>
-      <x:c r="K269" s="4" t="str">
-        <x:v>细化用例</x:v>
-      </x:c>
-      <x:c r="L269" s="4" t="str">
-        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:326</x:v>
-      </x:c>
-      <x:c r="M269" s="4" t="str">
-        <x:v>尚未执行</x:v>
-      </x:c>
-      <x:c r="N269" s="4" t="str">
-        <x:v>v0.5.0-20261001T034729Z</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="270" ht="57" customHeight="1">
-      <x:c r="A270" s="9" t="str">
-        <x:v>TM-005</x:v>
-      </x:c>
-      <x:c r="B270" s="9" t="str">
-        <x:v>TC-TM005-CORE-02</x:v>
-      </x:c>
-      <x:c r="C270" s="9" t="str">
-        <x:v>未知用量诊断不补零</x:v>
-      </x:c>
-      <x:c r="D270" s="9" t="str">
-        <x:v>TASK-TM005-EVENT-CONTRACT
-TASK-TM005-COVERAGE</x:v>
-      </x:c>
-      <x:c r="E270" s="9" t="str">
-        <x:v>模块检查</x:v>
-      </x:c>
-      <x:c r="F270" s="9" t="str">
-        <x:v>fixture A/B及同范围Claude missing_usage诊断；双来源complete仅为模块合成覆盖假设</x:v>
-      </x:c>
-      <x:c r="G270" s="9" t="str">
-        <x:v>1. 先仅统计A/B；已知330，未知模型110保留，来源Codex110/Claude220
-2. 加入诊断重新统计；partial、known_tokens330、total_tokens=null；诊断不增调用或零Token
-3. 移除A/B仅保留诊断；unknown、known_tokens0、total_tokens=null，不能写已确认零</x:v>
       </x:c>
       <x:c r="H270" s="9" t="str">
         <x:v>准备：无产品DB写入；每例从新内存输入开始
@@ -20231,7 +20233,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L270" s="9" t="str">
-        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:334</x:v>
+        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:326</x:v>
       </x:c>
       <x:c r="M270" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -20240,29 +20242,30 @@
         <x:v>v0.5.0-20261001T034729Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="271" ht="87" customHeight="1">
+    <x:row r="271" ht="57" customHeight="1">
       <x:c r="A271" s="4" t="str">
         <x:v>TM-005</x:v>
       </x:c>
       <x:c r="B271" s="4" t="str">
-        <x:v>TC-TM005-CORE-03</x:v>
+        <x:v>TC-TM005-CORE-02</x:v>
       </x:c>
       <x:c r="C271" s="4" t="str">
-        <x:v>声明式覆盖状态代数</x:v>
+        <x:v>未知用量诊断不补零</x:v>
       </x:c>
       <x:c r="D271" s="4" t="str">
-        <x:v>TASK-TM005-COVERAGE</x:v>
+        <x:v>TASK-TM005-EVENT-CONTRACT
+TASK-TM005-COVERAGE</x:v>
       </x:c>
       <x:c r="E271" s="4" t="str">
         <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F271" s="4" t="str">
-        <x:v>fixture五行coverage_algebra；complete仅为模块合成输入，product_coverage_proven=false</x:v>
+        <x:v>fixture A/B及同范围Claude missing_usage诊断；双来源complete仅为模块合成覆盖假设</x:v>
       </x:c>
       <x:c r="G271" s="4" t="str">
-        <x:v>1. 两来源complete且无事件、随后移除覆盖事实；前者complete/known0/total0；后者不得自行推断complete
-2. 一来源missing，分别给空事件与可信110；空事件missing/known0/total null；可信110为partial/known110/total null
-3. 两来源complete，分别给可信110+未知诊断、仅未知诊断；前者partial/known110/total null；后者unknown/known0/total null</x:v>
+        <x:v>1. 先仅统计A/B；已知330，未知模型110保留，来源Codex110/Claude220
+2. 加入诊断重新统计；partial、known_tokens330、total_tokens=null；诊断不增调用或零Token
+3. 移除A/B仅保留诊断；unknown、known_tokens0、total_tokens=null，不能写已确认零</x:v>
       </x:c>
       <x:c r="H271" s="4" t="str">
         <x:v>准备：无产品DB写入；每例从新内存输入开始
@@ -20279,7 +20282,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L271" s="4" t="str">
-        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:342</x:v>
+        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:334</x:v>
       </x:c>
       <x:c r="M271" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -20288,77 +20291,77 @@
         <x:v>v0.5.0-20261001T034729Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="272" ht="72" customHeight="1">
+    <x:row r="272" ht="87" customHeight="1">
       <x:c r="A272" s="9" t="str">
-        <x:v>TM-004</x:v>
+        <x:v>TM-005</x:v>
       </x:c>
       <x:c r="B272" s="9" t="str">
-        <x:v>TC-TM004-CORE-01</x:v>
+        <x:v>TC-TM005-CORE-03</x:v>
       </x:c>
       <x:c r="C272" s="9" t="str">
-        <x:v>完整LF、半行与限额续读</x:v>
+        <x:v>声明式覆盖状态代数</x:v>
       </x:c>
       <x:c r="D272" s="9" t="str">
-        <x:v>TASK-TM004-INCREMENTAL</x:v>
+        <x:v>TASK-TM005-COVERAGE</x:v>
       </x:c>
       <x:c r="E272" s="9" t="str">
         <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F272" s="9" t="str">
+        <x:v>fixture五行coverage_algebra；complete仅为模块合成输入，product_coverage_proven=false</x:v>
+      </x:c>
+      <x:c r="G272" s="9" t="str">
+        <x:v>1. 两来源complete且无事件、随后移除覆盖事实；前者complete/known0/total0；后者不得自行推断complete
+2. 一来源missing，分别给空事件与可信110；空事件missing/known0/total null；可信110为partial/known110/total null
+3. 两来源complete，分别给可信110+未知诊断、仅未知诊断；前者partial/known110/total null；后者unknown/known0/total null</x:v>
+      </x:c>
+      <x:c r="H272" s="9" t="str">
+        <x:v>准备：无产品DB写入；每例从新内存输入开始
+变化：不适用；纯统计返回值与输入未变
+核验：固定fixture摘要、事件筛选、各字段与状态逐步核对；无SQL</x:v>
+      </x:c>
+      <x:c r="I272" s="9" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J272" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K272" s="9" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L272" s="9" t="str">
+        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:342</x:v>
+      </x:c>
+      <x:c r="M272" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N272" s="9" t="str">
+        <x:v>v0.5.0-20261001T034729Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="273" ht="72" customHeight="1">
+      <x:c r="A273" s="4" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="B273" s="4" t="str">
+        <x:v>TC-TM004-CORE-01</x:v>
+      </x:c>
+      <x:c r="C273" s="4" t="str">
+        <x:v>完整LF、半行与限额续读</x:v>
+      </x:c>
+      <x:c r="D273" s="4" t="str">
+        <x:v>TASK-TM004-INCREMENTAL</x:v>
+      </x:c>
+      <x:c r="E273" s="4" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F273" s="4" t="str">
         <x:v>固定746字节13/7 assistant行、前半字节、两条不同ID完整行、首读上限754字节</x:v>
       </x:c>
-      <x:c r="G272" s="9" t="str">
+      <x:c r="G273" s="4" t="str">
         <x:v>1. 读未写完的前半行；调用0、偏移0、scanIncomplete=true，不作可信零结论
 2. 补齐LF、重复读取；补齐后一次13/7=20、偏移746、前缀MAC匹配；重复读取0调用且游标不变
 3. 两完整行首读754字节后续读；首读只第一条、偏移746、read_limit且未完成；续读只第二条、偏移为总字节长、完成</x:v>
-      </x:c>
-      <x:c r="H272" s="9" t="str">
-        <x:v>准备：无产品DB；每例新建自有临时文件
-变化：不适用；只返回模块调用、诊断与游标
-核验：固定fixture/行摘要和逐步返回值、前缀MAC及失败时无新游标；无SQL</x:v>
-      </x:c>
-      <x:c r="I272" s="9" t="str">
-        <x:v>draft</x:v>
-      </x:c>
-      <x:c r="J272" s="9" t="str">
-        <x:v>未执行</x:v>
-      </x:c>
-      <x:c r="K272" s="9" t="str">
-        <x:v>细化用例</x:v>
-      </x:c>
-      <x:c r="L272" s="9" t="str">
-        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:170</x:v>
-      </x:c>
-      <x:c r="M272" s="9" t="str">
-        <x:v>尚未执行</x:v>
-      </x:c>
-      <x:c r="N272" s="9" t="str">
-        <x:v>v0.4.0-20261001T040433Z</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="273" ht="87" customHeight="1">
-      <x:c r="A273" s="4" t="str">
-        <x:v>TM-004</x:v>
-      </x:c>
-      <x:c r="B273" s="4" t="str">
-        <x:v>TC-TM004-CORE-02</x:v>
-      </x:c>
-      <x:c r="C273" s="4" t="str">
-        <x:v>前缀MAC、变更和密钥失败</x:v>
-      </x:c>
-      <x:c r="D273" s="4" t="str">
-        <x:v>TASK-TM004-INCREMENTAL</x:v>
-      </x:c>
-      <x:c r="E273" s="4" t="str">
-        <x:v>模块检查</x:v>
-      </x:c>
-      <x:c r="F273" s="4" t="str">
-        <x:v>已提交首行，追加不同ID第二行、同长度ID改写并复原mtime、截短、身份改变、秘密缺失或错误</x:v>
-      </x:c>
-      <x:c r="G273" s="4" t="str">
-        <x:v>1. 首行后追加第二完整行；size/mtime变化但TM-002 dev/ino摘要和前缀MAC相同，续读只第二调用，无cursor_reset
-2. 同长度前缀改写、截短及稳定身份变更；分别报cursor_reset并从0重扫；同inode/size/mtime也不能忽略MAC不符
-3. 秘密无效或读中源变化；拒绝且没有可提交新游标/可信调用/成功零；输出不含路径正文秘密</x:v>
       </x:c>
       <x:c r="H273" s="4" t="str">
         <x:v>准备：无产品DB；每例新建自有临时文件
@@ -20375,7 +20378,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L273" s="4" t="str">
-        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:178</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:170</x:v>
       </x:c>
       <x:c r="M273" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -20384,30 +20387,29 @@
         <x:v>v0.4.0-20261001T040433Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="274" ht="57" customHeight="1">
+    <x:row r="274" ht="87" customHeight="1">
       <x:c r="A274" s="9" t="str">
         <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B274" s="9" t="str">
-        <x:v>TC-TM004-CORE-03</x:v>
+        <x:v>TC-TM004-CORE-02</x:v>
       </x:c>
       <x:c r="C274" s="9" t="str">
-        <x:v>损坏完整行与未知结构</x:v>
+        <x:v>前缀MAC、变更和密钥失败</x:v>
       </x:c>
       <x:c r="D274" s="9" t="str">
-        <x:v>TASK-TM004-PARSER
-TASK-TM004-INCREMENTAL</x:v>
+        <x:v>TASK-TM004-INCREMENTAL</x:v>
       </x:c>
       <x:c r="E274" s="9" t="str">
         <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F274" s="9" t="str">
-        <x:v>固定13/7行前置非法UTF8完整行和版本2.1.127完整行，尾部再追加无LF坏字节</x:v>
+        <x:v>已提交首行，追加不同ID第二行、同长度ID改写并复原mtime、截短、身份改变、秘密缺失或错误</x:v>
       </x:c>
       <x:c r="G274" s="9" t="str">
-        <x:v>1. 读三条完整LF行；仅合法2.1.126一条调用13/7=20；invalid_utf8及unsupported_version各一次
-2. 核对游标、重复读取及隐私；游标到三行LF末，MAC匹配且完成；重复读取0；输出无路径、正文、秘密
-3. 追加无LF坏字节再补LF；未补LF前偏移不动且未完成；补LF后仅诊断推进，无伪调用</x:v>
+        <x:v>1. 首行后追加第二完整行；size/mtime变化但TM-002 dev/ino摘要和前缀MAC相同，续读只第二调用，无cursor_reset
+2. 同长度前缀改写、截短及稳定身份变更；分别报cursor_reset并从0重扫；同inode/size/mtime也不能忽略MAC不符
+3. 秘密无效或读中源变化；拒绝且没有可提交新游标/可信调用/成功零；输出不含路径正文秘密</x:v>
       </x:c>
       <x:c r="H274" s="9" t="str">
         <x:v>准备：无产品DB；每例新建自有临时文件
@@ -20424,7 +20426,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L274" s="9" t="str">
-        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:186</x:v>
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:178</x:v>
       </x:c>
       <x:c r="M274" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -20433,227 +20435,276 @@
         <x:v>v0.4.0-20261001T040433Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="275" ht="132" customHeight="1">
+    <x:row r="275" ht="57" customHeight="1">
       <x:c r="A275" s="4" t="str">
         <x:v>TM-004</x:v>
       </x:c>
       <x:c r="B275" s="4" t="str">
+        <x:v>TC-TM004-CORE-03</x:v>
+      </x:c>
+      <x:c r="C275" s="4" t="str">
+        <x:v>损坏完整行与未知结构</x:v>
+      </x:c>
+      <x:c r="D275" s="4" t="str">
+        <x:v>TASK-TM004-PARSER
+TASK-TM004-INCREMENTAL</x:v>
+      </x:c>
+      <x:c r="E275" s="4" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F275" s="4" t="str">
+        <x:v>固定13/7行前置非法UTF8完整行和版本2.1.127完整行，尾部再追加无LF坏字节</x:v>
+      </x:c>
+      <x:c r="G275" s="4" t="str">
+        <x:v>1. 读三条完整LF行；仅合法2.1.126一条调用13/7=20；invalid_utf8及unsupported_version各一次
+2. 核对游标、重复读取及隐私；游标到三行LF末，MAC匹配且完成；重复读取0；输出无路径、正文、秘密
+3. 追加无LF坏字节再补LF；未补LF前偏移不动且未完成；补LF后仅诊断推进，无伪调用</x:v>
+      </x:c>
+      <x:c r="H275" s="4" t="str">
+        <x:v>准备：无产品DB；每例新建自有临时文件
+变化：不适用；只返回模块调用、诊断与游标
+核验：固定fixture/行摘要和逐步返回值、前缀MAC及失败时无新游标；无SQL</x:v>
+      </x:c>
+      <x:c r="I275" s="4" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J275" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K275" s="4" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L275" s="4" t="str">
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:186</x:v>
+      </x:c>
+      <x:c r="M275" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N275" s="4" t="str">
+        <x:v>v0.4.0-20261001T040433Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="276" ht="132" customHeight="1">
+      <x:c r="A276" s="9" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="B276" s="9" t="str">
         <x:v>TC-TM004-CORE-04</x:v>
       </x:c>
-      <x:c r="C275" s="4" t="str">
+      <x:c r="C276" s="9" t="str">
         <x:v>授权主体与扫描事务触发</x:v>
       </x:c>
-      <x:c r="D275" s="4" t="str">
+      <x:c r="D276" s="9" t="str">
         <x:v>TASK-TM004-SOURCE
 TASK-TM004-INCREMENTAL</x:v>
       </x:c>
-      <x:c r="E275" s="4" t="str">
+      <x:c r="E276" s="9" t="str">
         <x:v>模块检查</x:v>
       </x:c>
-      <x:c r="F275" s="4" t="str">
+      <x:c r="F276" s="9" t="str">
         <x:v>tests/fixtures/tm004-trigger-core-slice.json；固定UUID、M=100/10、各错误码、三种屏障事件及成功返回形状</x:v>
       </x:c>
-      <x:c r="G275" s="4" t="str">
+      <x:c r="G276" s="9" t="str">
         <x:v>1. 拒绝路径字段、无效主体/来源和预先取消的请求；路径字段/坏UUID为invalid_collection_request；账号不可用为collection_unavailable；异主体来源为source_not_authorized；预先取消为collection_cancelled；均扫描0、提交0
 2. 扫描开始后在固定屏障分别换账号、撤权和取消；换账号/撤权为collection_stale，取消为collection_cancelled；每次cancelScan、commitSync=0、缓冲不外露
 3. 健康主体和授权世代扫描完整M并通过提交守卫；commitSync恰一次；返回summary{callCount:1,inputTokens:100,outputTokens:10,totalTokens:110,scanIncomplete:false},diagnostics:[]，无私密哨兵/原生标识</x:v>
       </x:c>
-      <x:c r="H275" s="4" t="str">
+      <x:c r="H276" s="9" t="str">
         <x:v>准备：无产品DB；每子变体新建假端口与计数器
 变化：无SQLite；只观察假同步提交次数及数值
 核验：逐步断言扫描、取消、守卫、提交次数与返回白名单；无SQL</x:v>
       </x:c>
-      <x:c r="I275" s="4" t="str">
+      <x:c r="I276" s="9" t="str">
         <x:v>draft</x:v>
       </x:c>
-      <x:c r="J275" s="4" t="str">
+      <x:c r="J276" s="9" t="str">
         <x:v>未执行</x:v>
       </x:c>
-      <x:c r="K275" s="4" t="str">
+      <x:c r="K276" s="9" t="str">
         <x:v>细化用例</x:v>
       </x:c>
-      <x:c r="L275" s="4" t="str">
+      <x:c r="L276" s="9" t="str">
         <x:v>docs/testing/cases/04-TM-004-claude-collection.md:198</x:v>
       </x:c>
-      <x:c r="M275" s="4" t="str">
+      <x:c r="M276" s="9" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
-      <x:c r="N275" s="4" t="str">
+      <x:c r="N276" s="9" t="str">
         <x:v>v0.4.0-20261001T040433Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="276" ht="147" customHeight="1">
-      <x:c r="A276" s="9" t="str">
+    <x:row r="277" ht="147" customHeight="1">
+      <x:c r="A277" s="4" t="str">
         <x:v>TM-004</x:v>
       </x:c>
-      <x:c r="B276" s="9" t="str">
+      <x:c r="B277" s="4" t="str">
         <x:v>TC-TM004-CORE-05</x:v>
       </x:c>
-      <x:c r="C276" s="9" t="str">
+      <x:c r="C277" s="4" t="str">
         <x:v>多文件来源键与整代持久映射</x:v>
       </x:c>
-      <x:c r="D276" s="9" t="str">
+      <x:c r="D277" s="4" t="str">
         <x:v>TASK-TM004-INCREMENTAL
 TASK-TM004-LINEAGE</x:v>
       </x:c>
-      <x:c r="E276" s="9" t="str">
+      <x:c r="E277" s="4" t="str">
         <x:v>模块检查</x:v>
       </x:c>
-      <x:c r="F276" s="9" t="str">
+      <x:c r="F277" s="4" t="str">
         <x:v>tests/fixtures/tm004-storage-port-slice.json；合成M100/10、S200/20、Q50/5，三文件HMAC/游标/诊断与隔离SQLite；异常model_id哨兵与invalid_model_id诊断</x:v>
       </x:c>
-      <x:c r="G276" s="9" t="str">
+      <x:c r="G277" s="4" t="str">
         <x:v>1. 计算三个文件来源键、根键及换源/追加/替换向量；64hex键逐一等于fixture；普通追加键不变，换sourceId/文件摘要改变；数据库不收原摘要/相对名
 2. 构造完整三文件generation并核对文件归属与turnId代号；a/b/c各有自己的M/S/Q、游标和诊断；c异常model_id置null并增加invalid_model_id，SQLite/WAL无哨兵；turn代号仅进scope HMAC；未到末页/正文不稳零提交
 3. 分别在新库注入第二游标写失败与guard撤权；每次整代回滚或零开始，事件/游标/诊断/覆盖/密钥标记全空；取消并清缓冲
 4. 稳定末页通过guard后一次同步commitScanBatch并重扫；唯一3调用、input350/output35/total385、3游标/4诊断按文件归属、scan_incomplete=1；scope键匹配向量，重扫不增；SQLite/WAL无模型哨兵/原生标识</x:v>
       </x:c>
-      <x:c r="H276" s="9" t="str">
+      <x:c r="H277" s="4" t="str">
         <x:v>准备：每故障子场景新建本例空SQLite；故障注入只在本例库设置第二游标写入RAISE(ABORT)
 变化：成功一次事务新增三事件、三个游标、三诊断与根覆盖；失败和撤权零提交
 核验：只读查询usage_event、source_cursor、collection_diagnostic、coverage的数量/键/数值；核对源键和scope HMAC向量及无原生标识；关闭并核对SQLite/WAL无合成prompt/路径哨兵</x:v>
       </x:c>
-      <x:c r="I276" s="9" t="str">
+      <x:c r="I277" s="4" t="str">
         <x:v>draft</x:v>
       </x:c>
-      <x:c r="J276" s="9" t="str">
+      <x:c r="J277" s="4" t="str">
         <x:v>未执行</x:v>
       </x:c>
-      <x:c r="K276" s="9" t="str">
+      <x:c r="K277" s="4" t="str">
         <x:v>细化用例</x:v>
       </x:c>
-      <x:c r="L276" s="9" t="str">
+      <x:c r="L277" s="4" t="str">
         <x:v>docs/testing/cases/04-TM-004-claude-collection.md:206</x:v>
       </x:c>
-      <x:c r="M276" s="9" t="str">
+      <x:c r="M277" s="4" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
-      <x:c r="N276" s="9" t="str">
+      <x:c r="N277" s="4" t="str">
         <x:v>v0.4.0-20261001T040433Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="277" ht="87" customHeight="1">
-      <x:c r="A277" s="4" t="str">
+    <x:row r="278" ht="87" customHeight="1">
+      <x:c r="A278" s="9" t="str">
         <x:v>TM-005</x:v>
       </x:c>
-      <x:c r="B277" s="4" t="str">
+      <x:c r="B278" s="9" t="str">
         <x:v>TC-TM005-CORE-04</x:v>
       </x:c>
-      <x:c r="C277" s="4" t="str">
+      <x:c r="C278" s="9" t="str">
         <x:v>IANA当地日半开UTC界</x:v>
       </x:c>
-      <x:c r="D277" s="4" t="str">
+      <x:c r="D278" s="9" t="str">
         <x:v>TASK-TM005-RANGE-QUERY</x:v>
       </x:c>
-      <x:c r="E277" s="4" t="str">
+      <x:c r="E278" s="9" t="str">
         <x:v>模块检查</x:v>
       </x:c>
-      <x:c r="F277" s="4" t="str">
+      <x:c r="F278" s="9" t="str">
         <x:v>tests/fixtures/tm005-iana-core-slice.json；上海/UTC与纽约春秋四日、三种无效输入</x:v>
       </x:c>
-      <x:c r="G277" s="4" t="str">
+      <x:c r="G278" s="9" t="str">
         <x:v>1. 转换上海与UTC固定当地日；分别得到fixture固定24小时UTC半开界，传入事件UTC时刻不变
 2. 转换纽约春秋DST当地日及四类边界时刻；春23小时/秋25小时；before/at_end排除，at_start/before_end纳入
 3. 分别提交无效时区、无效日和非规范日期；invalid_timezone或invalid_local_day；无默认UTC范围/成功零</x:v>
       </x:c>
-      <x:c r="H277" s="4" t="str">
+      <x:c r="H278" s="9" t="str">
         <x:v>准备：无DB
 变化：无DB或系统时间变化
 核验：固定IANA各日UTC半开界、23/25小时、边界包含关系及错误码；无SQL</x:v>
       </x:c>
-      <x:c r="I277" s="4" t="str">
+      <x:c r="I278" s="9" t="str">
         <x:v>draft</x:v>
       </x:c>
-      <x:c r="J277" s="4" t="str">
+      <x:c r="J278" s="9" t="str">
         <x:v>未执行</x:v>
       </x:c>
-      <x:c r="K277" s="4" t="str">
+      <x:c r="K278" s="9" t="str">
         <x:v>细化用例</x:v>
       </x:c>
-      <x:c r="L277" s="4" t="str">
+      <x:c r="L278" s="9" t="str">
         <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:354</x:v>
       </x:c>
-      <x:c r="M277" s="4" t="str">
+      <x:c r="M278" s="9" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
-      <x:c r="N277" s="4" t="str">
+      <x:c r="N278" s="9" t="str">
         <x:v>v0.5.0-20261001T034729Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="278" ht="132" customHeight="1">
-      <x:c r="A278" s="9" t="str">
+    <x:row r="279" ht="132" customHeight="1">
+      <x:c r="A279" s="4" t="str">
         <x:v>TM-005</x:v>
       </x:c>
-      <x:c r="B278" s="9" t="str">
+      <x:c r="B279" s="4" t="str">
         <x:v>TC-TM005-CORE-05</x:v>
       </x:c>
-      <x:c r="C278" s="9" t="str">
+      <x:c r="C279" s="4" t="str">
         <x:v>双来源隔离SQLite同窗只读快照</x:v>
       </x:c>
-      <x:c r="D278" s="9" t="str">
+      <x:c r="D279" s="4" t="str">
         <x:v>TASK-TM005-EVENT-CONTRACT
 TASK-TM005-RANGE-QUERY</x:v>
       </x:c>
-      <x:c r="E278" s="9" t="str">
+      <x:c r="E279" s="4" t="str">
         <x:v>模块检查</x:v>
       </x:c>
-      <x:c r="F278" s="9" t="str">
+      <x:c r="F279" s="4" t="str">
         <x:v>tests/fixtures/tm005-sqlite-snapshot-slice.json；A/B双来源330、C异主体、D/E界外、F并发后新快照+55</x:v>
       </x:c>
-      <x:c r="G278" s="9" t="str">
+      <x:c r="G279" s="4" t="str">
         <x:v>1. 固定插入A–E并开启同一读事务；选A/B两调用，input300/output30/total330；C/D/E分别被主体或半开界排除，查询零写
 2. 在同一读事务取来源、模型、明细与逐日点；Codex110/Claude220；未知模型110/sonnet-test220；明细A/B和日点330；缓存读known20+unknown1，子项不加总
 3. 另一连接提交F后复查旧快照，再开新快照；旧事务各视图仍A/B和330；新事务A/B/F三调用、input350/output35/total385、Codex165/Claude220
 4. 查询空日及隐私边界；现有coverage不证明当地空日完整，不能报产品零；库/WAL/输出无原生ID、路径、正文或秘密</x:v>
       </x:c>
-      <x:c r="H278" s="9" t="str">
+      <x:c r="H279" s="4" t="str">
         <x:v>准备：固定准备程序仅在本例owner SQLite经UsageStore.commitBatch提交A–E；启用WAL并记录前态
 变化：查询零写入；另一连接固定提交F后旧读事务仍330，新读事务385
 核验：只读usage_event按主体/source/UTC半开界核对事件、来源/模型/明细/日点与子项未知数；coverage不能证明完整空日</x:v>
       </x:c>
-      <x:c r="I278" s="9" t="str">
+      <x:c r="I279" s="4" t="str">
         <x:v>draft</x:v>
       </x:c>
-      <x:c r="J278" s="9" t="str">
+      <x:c r="J279" s="4" t="str">
         <x:v>未执行</x:v>
       </x:c>
-      <x:c r="K278" s="9" t="str">
+      <x:c r="K279" s="4" t="str">
         <x:v>细化用例</x:v>
       </x:c>
-      <x:c r="L278" s="9" t="str">
+      <x:c r="L279" s="4" t="str">
         <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:362</x:v>
       </x:c>
-      <x:c r="M278" s="9" t="str">
+      <x:c r="M279" s="4" t="str">
         <x:v>尚未执行</x:v>
       </x:c>
-      <x:c r="N278" s="9" t="str">
+      <x:c r="N279" s="4" t="str">
         <x:v>v0.5.0-20261001T034729Z</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G5:G278">
+  <x:conditionalFormatting sqref="G5:G279">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="I5:I278">
+  <x:conditionalFormatting sqref="I5:I279">
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="16" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="17" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="J5:J278">
+  <x:conditionalFormatting sqref="J5:J279">
     <x:cfRule type="containsText" dxfId="18" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="19" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="20" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M278">
+  <x:conditionalFormatting sqref="M5:M279">
     <x:cfRule type="containsText" dxfId="21" priority="10" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="22" priority="11" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="23" priority="12" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc90cfc758c1542e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81f501feb0d642bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21625,7 +21676,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c8c0c3c927249f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc52d724d2194bf8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21939,7 +21990,7 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="72" customHeight="1">
+    <x:row r="9" ht="87" customHeight="1">
       <x:c r="A9" s="4" t="str">
         <x:v>v0.3.0-20261001T034652Z（续1）</x:v>
       </x:c>
@@ -21952,7 +22003,7 @@
       <x:c r="H9" s="4" t="str"/>
       <x:c r="I9" s="4" t="str"/>
       <x:c r="J9" s="4" t="str">
-        <x:v>source_check 1/1、四步与清理PASS，独立Excel回读PASS，第18批次；此前408ebf8红测失败保留。仅多文件模块，原27条产品TC与正式发行NOT_RUN。</x:v>
+        <x:v>source_check 1/1、四步与清理PASS，独立Excel回读PASS，第18批次；此前408ebf8红测失败保留。仅多文件模块，原27条产品TC与正式发行NOT_RUN。 CORE07主进程编排辅助TC已固定输入，程序/运行尚无。</x:v>
       </x:c>
       <x:c r="K9" s="4" t="str"/>
       <x:c r="L9" s="4" t="str"/>
@@ -22093,7 +22144,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ef5d7f22e44442b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf4f9079097f4817"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23258,7 +23309,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8347536de86f4d49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R442b04bb61294121"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.5.0-20261001T034729Z][TM-005] Index source checks and TM001 login probes
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R6859e9789eaa4df4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R4640075aba8a46ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R60a530bf23a54544"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R2359c002b9c04b97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R576e404900d24273"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R4abac05370484d31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R404411f10c8b4644"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R42b671ea6dee41d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Red5216beacbc41fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R980a7298878d4026"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R55e5b945aebc4eb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R5aecea853f344e4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rd27d59f669ab4628"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R006185a588df401c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rbfa8d23de5ca4a85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R031e61913cdb4f14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R814e04723aca453d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R55cace14a1724ac2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R0b6eb7aff5a040cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rf51350a9a644454b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Rc67567e977c24aa8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R6136b15bd3a141c4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -809,8 +809,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N24"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N28"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="运行批次"/>
     <x:tableColumn id="2" name="版本"/>
@@ -1146,8 +1146,8 @@
         <x:v>测试批次</x:v>
       </x:c>
       <x:c r="B9" s="10" t="n">
-        <x:f>COUNTA('06测试批次'!A5:A24)</x:f>
-        <x:v>20</x:v>
+        <x:f>COUNTA('06测试批次'!A5:A28)</x:f>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>06测试批次，每次运行一行，记录独立结果Excel位置</x:v>
@@ -1271,7 +1271,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>product_e2e · TASK-TM001-LOGIN-SESSION；仅LOGIN-10/11/12/13/14/15六条固定父TC，真实App定向回归：原始真实App定向run六条父TC、14步骤PASS，cleanup_completed=true；独立Excel/verification PASS。与LOGIN-AUTH为不同run，709d其余TM001父TC未运行；旧c291完整门禁FAIL及正式发行NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
+        <x:v>source_check · TM-005 CORE05合成双来源SQLite同窗快照固定辅助模块；非产品E2E：CORE05固定1/1、四步与owned_root清理PASS，独立Excel/verification回读PASS；原先两次红测失败原件保留，真实App/双来源原生日志产品TC仍未执行。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86fe8959df4e4996"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7713b6ac60884355"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8261aaa075b24b03"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R228a800dc39a4473"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6de93d56ad0c49f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf54ef2ef4ab8469b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc67abf79e706473f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5da135ac933f44c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14b7815ba70e4401"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24261c2e1b6a4d0b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc59ced9c7c9e4ae9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6d7bee66f884245"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7519,7 +7519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R417c62f167974b9f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafb3d6399e4a4a3e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7823,7 +7823,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:137</x:v>
       </x:c>
       <x:c r="M9" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-5e076fa3d05b4d949877333a3b5339e0</x:v>
       </x:c>
       <x:c r="N9" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -7870,7 +7870,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:152</x:v>
       </x:c>
       <x:c r="M10" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-5e076fa3d05b4d949877333a3b5339e0</x:v>
       </x:c>
       <x:c r="N10" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -7917,7 +7917,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:167</x:v>
       </x:c>
       <x:c r="M11" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-5e076fa3d05b4d949877333a3b5339e0</x:v>
       </x:c>
       <x:c r="N11" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -8011,7 +8011,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:197</x:v>
       </x:c>
       <x:c r="M13" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-5e076fa3d05b4d949877333a3b5339e0</x:v>
       </x:c>
       <x:c r="N13" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -8343,7 +8343,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:304</x:v>
       </x:c>
       <x:c r="M20" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-09f2c4fd672848a9a68ba851a5d7b3c9</x:v>
       </x:c>
       <x:c r="N20" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -8390,7 +8390,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:320</x:v>
       </x:c>
       <x:c r="M21" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-5e076fa3d05b4d949877333a3b5339e0</x:v>
       </x:c>
       <x:c r="N21" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -8437,7 +8437,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:341</x:v>
       </x:c>
       <x:c r="M22" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-5e076fa3d05b4d949877333a3b5339e0</x:v>
       </x:c>
       <x:c r="N22" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -8484,7 +8484,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:364</x:v>
       </x:c>
       <x:c r="M23" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-5e076fa3d05b4d949877333a3b5339e0</x:v>
       </x:c>
       <x:c r="N23" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -8531,7 +8531,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:386</x:v>
       </x:c>
       <x:c r="M24" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-5e076fa3d05b4d949877333a3b5339e0</x:v>
       </x:c>
       <x:c r="N24" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -8578,7 +8578,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:401</x:v>
       </x:c>
       <x:c r="M25" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-5e076fa3d05b4d949877333a3b5339e0</x:v>
       </x:c>
       <x:c r="N25" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -8625,7 +8625,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:416</x:v>
       </x:c>
       <x:c r="M26" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-5e076fa3d05b4d949877333a3b5339e0</x:v>
       </x:c>
       <x:c r="N26" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -20616,7 +20616,7 @@
         <x:v>draft</x:v>
       </x:c>
       <x:c r="J278" s="9" t="str">
-        <x:v>未执行</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="K278" s="9" t="str">
         <x:v>细化用例</x:v>
@@ -20625,7 +20625,7 @@
         <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:354</x:v>
       </x:c>
       <x:c r="M278" s="9" t="str">
-        <x:v>尚未执行</x:v>
+        <x:v>tm005-core04-20261001T193346Z</x:v>
       </x:c>
       <x:c r="N278" s="9" t="str">
         <x:v>v0.5.0-20261001T034729Z</x:v>
@@ -20666,7 +20666,7 @@
         <x:v>draft</x:v>
       </x:c>
       <x:c r="J279" s="4" t="str">
-        <x:v>未执行</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="K279" s="4" t="str">
         <x:v>细化用例</x:v>
@@ -20675,7 +20675,7 @@
         <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:362</x:v>
       </x:c>
       <x:c r="M279" s="4" t="str">
-        <x:v>尚未执行</x:v>
+        <x:v>tm005-core05-20261001T193346Z</x:v>
       </x:c>
       <x:c r="N279" s="4" t="str">
         <x:v>v0.5.0-20261001T034729Z</x:v>
@@ -20704,7 +20704,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81f501feb0d642bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re36cdc3eb98e42dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21658,25 +21658,201 @@
         <x:v>PASS</x:v>
       </x:c>
     </x:row>
+    <x:row r="25" ht="57" customHeight="1">
+      <x:c r="A25" s="4" t="str">
+        <x:v>local-5e076fa3d05b4d949877333a3b5339e0</x:v>
+      </x:c>
+      <x:c r="B25" s="4" t="str">
+        <x:v>v0.1.0-20260929T074814Z</x:v>
+      </x:c>
+      <x:c r="C25" s="4" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D25" s="4" t="str">
+        <x:v>TASK-TM001-LOGIN-VALIDATION；10父TC与12固定变体，18真实App执行加4父例派生</x:v>
+      </x:c>
+      <x:c r="E25" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F25" s="4" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G25" s="4" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H25" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I25" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J25" s="4" t="str">
+        <x:v>709d21253a0f88bc703a431cbf3adba3df17e508</x:v>
+      </x:c>
+      <x:c r="K25" s="4" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L25" s="4" t="str">
+        <x:v>10父TC与12固定变体共22/22报告行PASS、36步骤、cleanup=true；四父例由变体派生、18个真实App执行。仅709d LOGIN-VALIDATION定向，其他TM001功能未通过；旧c291完整门禁FAIL。</x:v>
+      </x:c>
+      <x:c r="M25" s="4" t="str">
+        <x:v>.local/test-results/local-5e076fa3d05b4d949877333a3b5339e0/TokenMeter测试结果-local-5e076fa3d05b4d949877333a3b5339e0.xlsx</x:v>
+      </x:c>
+      <x:c r="N25" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="42" customHeight="1">
+      <x:c r="A26" s="9" t="str">
+        <x:v>local-09f2c4fd672848a9a68ba851a5d7b3c9</x:v>
+      </x:c>
+      <x:c r="B26" s="9" t="str">
+        <x:v>v0.1.0-20260929T074814Z</x:v>
+      </x:c>
+      <x:c r="C26" s="9" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D26" s="9" t="str">
+        <x:v>TASK-TM001-LOGIN-RATE；仅LOGIN-16固定父TC</x:v>
+      </x:c>
+      <x:c r="E26" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F26" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G26" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H26" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I26" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J26" s="9" t="str">
+        <x:v>709d21253a0f88bc703a431cbf3adba3df17e508</x:v>
+      </x:c>
+      <x:c r="K26" s="9" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L26" s="9" t="str">
+        <x:v>LOGIN-16单例/3步真实App PASS、cleanup=true，独立Excel回读PASS；仅709d定向，其他TM001功能及完整发行门禁未通过。</x:v>
+      </x:c>
+      <x:c r="M26" s="9" t="str">
+        <x:v>.local/test-results/local-09f2c4fd672848a9a68ba851a5d7b3c9/TokenMeter测试结果-local-09f2c4fd672848a9a68ba851a5d7b3c9.xlsx</x:v>
+      </x:c>
+      <x:c r="N26" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="42" customHeight="1">
+      <x:c r="A27" s="4" t="str">
+        <x:v>tm005-core04-20261001T193346Z</x:v>
+      </x:c>
+      <x:c r="B27" s="4" t="str">
+        <x:v>v0.5.0-20261001T034729Z</x:v>
+      </x:c>
+      <x:c r="C27" s="4" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D27" s="4" t="str">
+        <x:v>TM-005 CORE04 IANA当地日/DST半开界固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E27" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F27" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G27" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H27" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I27" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J27" s="4" t="str">
+        <x:v>259cf7688691d472837d59a8c1ae50e14b591410</x:v>
+      </x:c>
+      <x:c r="K27" s="4" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L27" s="4" t="str">
+        <x:v>CORE04固定1/1、三步与memory_only清理PASS，独立Excel/verification回读PASS；纽约23/25小时与非法输入模块判据通过，安装App产品TC仍未执行。</x:v>
+      </x:c>
+      <x:c r="M27" s="4" t="str">
+        <x:v>.local/test-results/tm005-core04-20261001T193346Z/TokenMeter测试结果-tm005-core04-20261001T193346Z.xlsx</x:v>
+      </x:c>
+      <x:c r="N27" s="4" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="42" customHeight="1">
+      <x:c r="A28" s="9" t="str">
+        <x:v>tm005-core05-20261001T193346Z</x:v>
+      </x:c>
+      <x:c r="B28" s="9" t="str">
+        <x:v>v0.5.0-20261001T034729Z</x:v>
+      </x:c>
+      <x:c r="C28" s="9" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D28" s="9" t="str">
+        <x:v>TM-005 CORE05合成双来源SQLite同窗快照固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E28" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F28" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G28" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H28" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I28" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J28" s="9" t="str">
+        <x:v>259cf7688691d472837d59a8c1ae50e14b591410</x:v>
+      </x:c>
+      <x:c r="K28" s="9" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L28" s="9" t="str">
+        <x:v>CORE05固定1/1、四步与owned_root清理PASS，独立Excel/verification回读PASS；原先两次红测失败原件保留，真实App/双来源原生日志产品TC仍未执行。</x:v>
+      </x:c>
+      <x:c r="M28" s="9" t="str">
+        <x:v>.local/test-results/tm005-core05-20261001T193346Z/TokenMeter测试结果-tm005-core05-20261001T193346Z.xlsx</x:v>
+      </x:c>
+      <x:c r="N28" s="9" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E5:E24">
+  <x:conditionalFormatting sqref="E5:E28">
     <x:cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="26" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M24">
+  <x:conditionalFormatting sqref="M5:M28">
     <x:cfRule type="containsText" dxfId="27" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="29" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="N5:N24">
+  <x:conditionalFormatting sqref="N5:N28">
     <x:cfRule type="containsText" dxfId="30" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="32" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc52d724d2194bf8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac60af8e9db848b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21822,7 +21998,7 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="237" customHeight="1">
+    <x:row r="6" ht="282" customHeight="1">
       <x:c r="A6" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
@@ -21851,7 +22027,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J6" s="9" t="str">
-        <x:v>开发中，未发布。c291本地master最终包门禁FAIL：116项91 PASS/14 FAIL/11 BLOCKED；9f06cb1修复私有签名输入后开发检查PASS，但新定向App仍FAIL/BLOCKED并有ENOSPC，功能回归未完成。旧d2db551独立候选PASS不转用于新候选。正式发行完整门禁NOT_RUN，无稳定0.1原包。 709d UPDATE-05定向父1+变体13 PASS，后置de081a6导出Excel回读PASS；仅定向，77父TC范围外，旧c291完整门禁FAIL及未发行不变。 709d安装DMG的登录定向五父例/11步原始PASS，独立Excel回读PASS；仍非整版回归，旧c291完整门禁FAIL。 709d LOGIN-SESSION另六父例/14步原始PASS并单独导出Excel；未完成整版回归。</x:v>
+        <x:v>开发中，未发布。c291本地master最终包门禁FAIL：116项91 PASS/14 FAIL/11 BLOCKED；9f06cb1修复私有签名输入后开发检查PASS，但新定向App仍FAIL/BLOCKED并有ENOSPC，功能回归未完成。旧d2db551独立候选PASS不转用于新候选。正式发行完整门禁NOT_RUN，无稳定0.1原包。 709d UPDATE-05定向父1+变体13 PASS，后置de081a6导出Excel回读PASS；仅定向，77父TC范围外，旧c291完整门禁FAIL及未发行不变。 709d安装DMG的登录定向五父例/11步原始PASS，独立Excel回读PASS；仍非整版回归，旧c291完整门禁FAIL。 709d LOGIN-SESSION另六父例/14步原始PASS并单独导出Excel；未完成整版回归。 709d LOGIN-VALIDATION十父+十二变体及LOGIN-RATE一父另两次定向PASS/Excel；四批登录合计22父+12变体，但TM001其他功能未验收。</x:v>
       </x:c>
       <x:c r="K6" s="9" t="str">
         <x:v>旧SwiftUI PR #2 已合并、历史双平台六例PASS；不继承给Electron</x:v>
@@ -22070,7 +22246,7 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="327" customHeight="1">
+    <x:row r="11" ht="372" customHeight="1">
       <x:c r="A11" s="4" t="str">
         <x:v>v0.5.0-20261001T034729Z</x:v>
       </x:c>
@@ -22099,7 +22275,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J11" s="4" t="str">
-        <x:v>整版draft、未发布。原32条产品父TC、6稳定变体和两组摘要保留；纯统计CORE-01/02/03辅助TC在输入提交061c759后，经SOP-008内容核对及结构/治理457项PASS，独立切片development_slice_ready，程序绑定仍为空、模块实际运行unexecuted。静态oracle与切片就绪不证明真实双来源采集或产品E2E；固定产品数据、SQLite/IPC、安装App逐TC绑定未完成，正式发行完整门禁NOT_RUN。 独立代码提交6a0f6f的source_check CORE3/3、桌面29/29、build PASS，原件在TM005工作树.local/tm005-core-postcommit-20261001T162401Z；程序尚未进入本文档树、模块Excel导出/批次登记BLOCKED，产品E2E仍NOT_RUN。 CORE-01仅验证已给UTC半开界聚合，不验证IANA日期换算；该单独辅助TC待固定。 新增CORE04/05固定IANA当地日与合成双来源SQLite只读快照辅助TC，程序null/unexecuted；coverage表无连续空日证明，原32产品TC/6变体与发行仍BLOCKED/NOT_RUN。</x:v>
+        <x:v>整版draft、未发布。原32条产品父TC、6稳定变体和两组摘要保留；纯统计CORE-01/02/03辅助TC在输入提交061c759后，经SOP-008内容核对及结构/治理457项PASS，独立切片development_slice_ready，程序绑定仍为空、模块实际运行unexecuted。静态oracle与切片就绪不证明真实双来源采集或产品E2E；固定产品数据、SQLite/IPC、安装App逐TC绑定未完成，正式发行完整门禁NOT_RUN。 独立代码提交6a0f6f的source_check CORE3/3、桌面29/29、build PASS，原件在TM005工作树.local/tm005-core-postcommit-20261001T162401Z；程序尚未进入本文档树、模块Excel导出/批次登记BLOCKED，产品E2E仍NOT_RUN。 CORE-01仅验证已给UTC半开界聚合，不验证IANA日期换算；该单独辅助TC待固定。 新增CORE04/05固定IANA当地日与合成双来源SQLite只读快照辅助TC，程序null/unexecuted；coverage表无连续空日证明，原32产品TC/6变体与发行仍BLOCKED/NOT_RUN。 CORE04/05在259cf768候选固定模块分别1/1三/四步PASS且Excel回读；0.5产品E2E未运行。</x:v>
       </x:c>
       <x:c r="K11" s="4" t="str">
         <x:v>TM005语义oracle只验证规范化样例；0.4及此前稳定原包尚未形成，真实升级BLOCKED。</x:v>
@@ -22144,7 +22320,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf4f9079097f4817"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ac3655b89ed4f67"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23309,7 +23485,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R442b04bb61294121"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R114798d510fb437f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.1.0-20260929T074814Z][TM-001] Index password change probe
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R5aecea853f344e4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rd27d59f669ab4628"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R006185a588df401c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rbfa8d23de5ca4a85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R031e61913cdb4f14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R814e04723aca453d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R55cace14a1724ac2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R0b6eb7aff5a040cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rf51350a9a644454b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Rc67567e977c24aa8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R6136b15bd3a141c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Rfc64f14418c448ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rfd9f18be1749452c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R8ea424d0070c422f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R04abb273637d463a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rf5033cbd0f8a42de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R15c38db7c1904d7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R70ac51186f364251"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R212e9aaae0c54718"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Ra867a50951b247b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R71b5e166c51e4a5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R08bedfcee6524d9f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -809,8 +809,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N28"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N29"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="运行批次"/>
     <x:tableColumn id="2" name="版本"/>
@@ -1146,8 +1146,8 @@
         <x:v>测试批次</x:v>
       </x:c>
       <x:c r="B9" s="10" t="n">
-        <x:f>COUNTA('06测试批次'!A5:A28)</x:f>
-        <x:v>24</x:v>
+        <x:f>COUNTA('06测试批次'!A5:A29)</x:f>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>06测试批次，每次运行一行，记录独立结果Excel位置</x:v>
@@ -1263,7 +1263,7 @@
         <x:v>DMG及原始证据留本机；Git保存代码、文档和此工作簿</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="72" customHeight="1">
+    <x:row r="20" ht="87" customHeight="1">
       <x:c r="A20" s="9" t="str">
         <x:v>最近登记批次</x:v>
       </x:c>
@@ -1271,7 +1271,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>source_check · TM-005 CORE05合成双来源SQLite同窗快照固定辅助模块；非产品E2E：CORE05固定1/1、四步与owned_root清理PASS，独立Excel/verification回读PASS；原先两次红测失败原件保留，真实App/双来源原生日志产品TC仍未执行。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
+        <x:v>product_e2e · TASK-TM001-CHANGE-PASSWORD；PASSWORD-01..11十一父TC及09/11下六固定变体，15真实App执行加2父例派生：11父+6变体共17/17报告行PASS、32步、清理完成；15真实App执行/2父例派生。独立审计仅PASSWORD-05 PASS，不能称12项完整审计。仅709d改密功能定向，其他TM001功能、旧c291完整门禁FAIL及正式发行NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7713b6ac60884355"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0419773e35fb422f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R228a800dc39a4473"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8ca3cfe84354731"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf54ef2ef4ab8469b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R825253bf40594eae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5da135ac933f44c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4ecde44711a4d8b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24261c2e1b6a4d0b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd490caae6c264530"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6d7bee66f884245"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re39fae7d7d624a7f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7519,7 +7519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafb3d6399e4a4a3e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra394df7f4df24a47"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8672,7 +8672,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:431</x:v>
       </x:c>
       <x:c r="M27" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-64cdbd1050d84763928c0b6a7f30e2c3</x:v>
       </x:c>
       <x:c r="N27" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -8719,7 +8719,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:446</x:v>
       </x:c>
       <x:c r="M28" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-64cdbd1050d84763928c0b6a7f30e2c3</x:v>
       </x:c>
       <x:c r="N28" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -8766,7 +8766,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:461</x:v>
       </x:c>
       <x:c r="M29" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-64cdbd1050d84763928c0b6a7f30e2c3</x:v>
       </x:c>
       <x:c r="N29" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -8813,7 +8813,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:476</x:v>
       </x:c>
       <x:c r="M30" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-64cdbd1050d84763928c0b6a7f30e2c3</x:v>
       </x:c>
       <x:c r="N30" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -8862,7 +8862,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:491</x:v>
       </x:c>
       <x:c r="M31" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-64cdbd1050d84763928c0b6a7f30e2c3</x:v>
       </x:c>
       <x:c r="N31" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -8909,7 +8909,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:508</x:v>
       </x:c>
       <x:c r="M32" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-64cdbd1050d84763928c0b6a7f30e2c3</x:v>
       </x:c>
       <x:c r="N32" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -8956,7 +8956,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:523</x:v>
       </x:c>
       <x:c r="M33" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-64cdbd1050d84763928c0b6a7f30e2c3</x:v>
       </x:c>
       <x:c r="N33" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -9003,7 +9003,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:538</x:v>
       </x:c>
       <x:c r="M34" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-64cdbd1050d84763928c0b6a7f30e2c3</x:v>
       </x:c>
       <x:c r="N34" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -9050,7 +9050,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:553</x:v>
       </x:c>
       <x:c r="M35" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-64cdbd1050d84763928c0b6a7f30e2c3</x:v>
       </x:c>
       <x:c r="N35" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -9097,7 +9097,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:576</x:v>
       </x:c>
       <x:c r="M36" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-64cdbd1050d84763928c0b6a7f30e2c3</x:v>
       </x:c>
       <x:c r="N36" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -9144,7 +9144,7 @@
         <x:v>docs/testing/cases/01a-TM-001-login-scenarios.md:591</x:v>
       </x:c>
       <x:c r="M37" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-64cdbd1050d84763928c0b6a7f30e2c3</x:v>
       </x:c>
       <x:c r="N37" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -20704,7 +20704,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re36cdc3eb98e42dc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff907dc856434a68"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21834,25 +21834,69 @@
         <x:v>NOT_RUN</x:v>
       </x:c>
     </x:row>
+    <x:row r="29" ht="57" customHeight="1">
+      <x:c r="A29" s="4" t="str">
+        <x:v>local-64cdbd1050d84763928c0b6a7f30e2c3</x:v>
+      </x:c>
+      <x:c r="B29" s="4" t="str">
+        <x:v>v0.1.0-20260929T074814Z</x:v>
+      </x:c>
+      <x:c r="C29" s="4" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D29" s="4" t="str">
+        <x:v>TASK-TM001-CHANGE-PASSWORD；PASSWORD-01..11十一父TC及09/11下六固定变体，15真实App执行加2父例派生</x:v>
+      </x:c>
+      <x:c r="E29" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F29" s="4" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G29" s="4" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H29" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I29" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J29" s="4" t="str">
+        <x:v>709d21253a0f88bc703a431cbf3adba3df17e508</x:v>
+      </x:c>
+      <x:c r="K29" s="4" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L29" s="4" t="str">
+        <x:v>11父+6变体共17/17报告行PASS、32步、清理完成；15真实App执行/2父例派生。独立审计仅PASSWORD-05 PASS，不能称12项完整审计。仅709d改密功能定向，其他TM001功能、旧c291完整门禁FAIL及正式发行NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M29" s="4" t="str">
+        <x:v>.local/test-results/local-64cdbd1050d84763928c0b6a7f30e2c3/TokenMeter测试结果-local-64cdbd1050d84763928c0b6a7f30e2c3.xlsx</x:v>
+      </x:c>
+      <x:c r="N29" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E5:E28">
+  <x:conditionalFormatting sqref="E5:E29">
     <x:cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="26" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M28">
+  <x:conditionalFormatting sqref="M5:M29">
     <x:cfRule type="containsText" dxfId="27" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="29" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="N5:N28">
+  <x:conditionalFormatting sqref="N5:N29">
     <x:cfRule type="containsText" dxfId="30" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="32" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac60af8e9db848b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R174618c912c44748"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21998,7 +22042,7 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="282" customHeight="1">
+    <x:row r="6" ht="327" customHeight="1">
       <x:c r="A6" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
@@ -22027,7 +22071,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J6" s="9" t="str">
-        <x:v>开发中，未发布。c291本地master最终包门禁FAIL：116项91 PASS/14 FAIL/11 BLOCKED；9f06cb1修复私有签名输入后开发检查PASS，但新定向App仍FAIL/BLOCKED并有ENOSPC，功能回归未完成。旧d2db551独立候选PASS不转用于新候选。正式发行完整门禁NOT_RUN，无稳定0.1原包。 709d UPDATE-05定向父1+变体13 PASS，后置de081a6导出Excel回读PASS；仅定向，77父TC范围外，旧c291完整门禁FAIL及未发行不变。 709d安装DMG的登录定向五父例/11步原始PASS，独立Excel回读PASS；仍非整版回归，旧c291完整门禁FAIL。 709d LOGIN-SESSION另六父例/14步原始PASS并单独导出Excel；未完成整版回归。 709d LOGIN-VALIDATION十父+十二变体及LOGIN-RATE一父另两次定向PASS/Excel；四批登录合计22父+12变体，但TM001其他功能未验收。</x:v>
+        <x:v>开发中，未发布。c291本地master最终包门禁FAIL：116项91 PASS/14 FAIL/11 BLOCKED；9f06cb1修复私有签名输入后开发检查PASS，但新定向App仍FAIL/BLOCKED并有ENOSPC，功能回归未完成。旧d2db551独立候选PASS不转用于新候选。正式发行完整门禁NOT_RUN，无稳定0.1原包。 709d UPDATE-05定向父1+变体13 PASS，后置de081a6导出Excel回读PASS；仅定向，77父TC范围外，旧c291完整门禁FAIL及未发行不变。 709d安装DMG的登录定向五父例/11步原始PASS，独立Excel回读PASS；仍非整版回归，旧c291完整门禁FAIL。 709d LOGIN-SESSION另六父例/14步原始PASS并单独导出Excel；未完成整版回归。 709d LOGIN-VALIDATION十父+十二变体及LOGIN-RATE一父另两次定向PASS/Excel；四批登录合计22父+12变体，但TM001其他功能未验收。 709d CHANGE-PASSWORD十一父+六变体17行/32步另批定向PASS，PASSWORD-05单项独立审计PASS；未完成整版/12项审计。</x:v>
       </x:c>
       <x:c r="K6" s="9" t="str">
         <x:v>旧SwiftUI PR #2 已合并、历史双平台六例PASS；不继承给Electron</x:v>
@@ -22320,7 +22364,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ac3655b89ed4f67"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b6d80f555ee4313"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23485,7 +23529,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R114798d510fb437f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R432645b548d94627"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.1.0-20260929T074814Z][TM-001] Index session function probe
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Rfc64f14418c448ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rfd9f18be1749452c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R8ea424d0070c422f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R04abb273637d463a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rf5033cbd0f8a42de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R15c38db7c1904d7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R70ac51186f364251"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R212e9aaae0c54718"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Ra867a50951b247b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R71b5e166c51e4a5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R08bedfcee6524d9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R5b7e7fd9d8064136"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rca13714ea2eb4bd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R34fbcca2560341bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rbb59dd038c7e485d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R9304618290ec472c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Ra929ac29ea8c4312"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R1a21b4122a13461a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Rc4c3f614e89845c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R93d6c4490af544fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R1ea074624c644246"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R3a96156b72bc4508"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -809,8 +809,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N29"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N30"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="运行批次"/>
     <x:tableColumn id="2" name="版本"/>
@@ -1146,8 +1146,8 @@
         <x:v>测试批次</x:v>
       </x:c>
       <x:c r="B9" s="10" t="n">
-        <x:f>COUNTA('06测试批次'!A5:A29)</x:f>
-        <x:v>25</x:v>
+        <x:f>COUNTA('06测试批次'!A5:A30)</x:f>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>06测试批次，每次运行一行，记录独立结果Excel位置</x:v>
@@ -1271,7 +1271,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>product_e2e · TASK-TM001-CHANGE-PASSWORD；PASSWORD-01..11十一父TC及09/11下六固定变体，15真实App执行加2父例派生：11父+6变体共17/17报告行PASS、32步、清理完成；15真实App执行/2父例派生。独立审计仅PASSWORD-05 PASS，不能称12项完整审计。仅709d改密功能定向，其他TM001功能、旧c291完整门禁FAIL及正式发行NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
+        <x:v>product_e2e · TASK-TM001-SESSION；SESSION-01..10十父TC及SESSION-05#RESET/#DISABLE两变体，11真实App执行加1父例派生：10父+2变体共12/12报告行PASS、44步、清理完成；SESSION-05父例由两变体派生。独立审计仅SESSION-04 PASS，非12项完整审计。仅709d会话功能定向，其他TM001功能、旧c291完整门禁FAIL及正式发行NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0419773e35fb422f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0122596413d49e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8ca3cfe84354731"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b959ecddd074e70"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R825253bf40594eae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e5c7a429072496d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4ecde44711a4d8b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R978ff2256dcc47a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd490caae6c264530"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42d9cd88455e4cde"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re39fae7d7d624a7f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84934c925f564adf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7519,7 +7519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra394df7f4df24a47"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37f1853248c14e92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9193,7 +9193,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:76</x:v>
       </x:c>
       <x:c r="M38" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-ff24478631134a96bd7d40f2bbc5e254</x:v>
       </x:c>
       <x:c r="N38" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -9242,7 +9242,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:93</x:v>
       </x:c>
       <x:c r="M39" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-ff24478631134a96bd7d40f2bbc5e254</x:v>
       </x:c>
       <x:c r="N39" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -9291,7 +9291,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:110</x:v>
       </x:c>
       <x:c r="M40" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-ff24478631134a96bd7d40f2bbc5e254</x:v>
       </x:c>
       <x:c r="N40" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -9340,7 +9340,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:127</x:v>
       </x:c>
       <x:c r="M41" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-ff24478631134a96bd7d40f2bbc5e254</x:v>
       </x:c>
       <x:c r="N41" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -9389,7 +9389,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:149</x:v>
       </x:c>
       <x:c r="M42" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-ff24478631134a96bd7d40f2bbc5e254</x:v>
       </x:c>
       <x:c r="N42" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -9438,7 +9438,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:166</x:v>
       </x:c>
       <x:c r="M43" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-ff24478631134a96bd7d40f2bbc5e254</x:v>
       </x:c>
       <x:c r="N43" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -9487,7 +9487,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:183</x:v>
       </x:c>
       <x:c r="M44" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-ff24478631134a96bd7d40f2bbc5e254</x:v>
       </x:c>
       <x:c r="N44" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -9536,7 +9536,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:200</x:v>
       </x:c>
       <x:c r="M45" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-ff24478631134a96bd7d40f2bbc5e254</x:v>
       </x:c>
       <x:c r="N45" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -9586,7 +9586,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:217</x:v>
       </x:c>
       <x:c r="M46" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-ff24478631134a96bd7d40f2bbc5e254</x:v>
       </x:c>
       <x:c r="N46" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -9635,7 +9635,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:234</x:v>
       </x:c>
       <x:c r="M47" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-ff24478631134a96bd7d40f2bbc5e254</x:v>
       </x:c>
       <x:c r="N47" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -20704,7 +20704,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff907dc856434a68"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdb18eb57a8d40c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21878,25 +21878,69 @@
         <x:v>PASS</x:v>
       </x:c>
     </x:row>
+    <x:row r="30" ht="57" customHeight="1">
+      <x:c r="A30" s="9" t="str">
+        <x:v>local-ff24478631134a96bd7d40f2bbc5e254</x:v>
+      </x:c>
+      <x:c r="B30" s="9" t="str">
+        <x:v>v0.1.0-20260929T074814Z</x:v>
+      </x:c>
+      <x:c r="C30" s="9" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D30" s="9" t="str">
+        <x:v>TASK-TM001-SESSION；SESSION-01..10十父TC及SESSION-05#RESET/#DISABLE两变体，11真实App执行加1父例派生</x:v>
+      </x:c>
+      <x:c r="E30" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F30" s="9" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G30" s="9" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H30" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I30" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J30" s="9" t="str">
+        <x:v>709d21253a0f88bc703a431cbf3adba3df17e508</x:v>
+      </x:c>
+      <x:c r="K30" s="9" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L30" s="9" t="str">
+        <x:v>10父+2变体共12/12报告行PASS、44步、清理完成；SESSION-05父例由两变体派生。独立审计仅SESSION-04 PASS，非12项完整审计。仅709d会话功能定向，其他TM001功能、旧c291完整门禁FAIL及正式发行NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M30" s="9" t="str">
+        <x:v>.local/test-results/local-ff24478631134a96bd7d40f2bbc5e254/TokenMeter测试结果-local-ff24478631134a96bd7d40f2bbc5e254.xlsx</x:v>
+      </x:c>
+      <x:c r="N30" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E5:E29">
+  <x:conditionalFormatting sqref="E5:E30">
     <x:cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="26" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M29">
+  <x:conditionalFormatting sqref="M5:M30">
     <x:cfRule type="containsText" dxfId="27" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="29" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="N5:N29">
+  <x:conditionalFormatting sqref="N5:N30">
     <x:cfRule type="containsText" dxfId="30" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="32" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R174618c912c44748"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R464573aeb46c403f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22042,7 +22086,7 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="327" customHeight="1">
+    <x:row r="6" ht="372" customHeight="1">
       <x:c r="A6" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
@@ -22071,7 +22115,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J6" s="9" t="str">
-        <x:v>开发中，未发布。c291本地master最终包门禁FAIL：116项91 PASS/14 FAIL/11 BLOCKED；9f06cb1修复私有签名输入后开发检查PASS，但新定向App仍FAIL/BLOCKED并有ENOSPC，功能回归未完成。旧d2db551独立候选PASS不转用于新候选。正式发行完整门禁NOT_RUN，无稳定0.1原包。 709d UPDATE-05定向父1+变体13 PASS，后置de081a6导出Excel回读PASS；仅定向，77父TC范围外，旧c291完整门禁FAIL及未发行不变。 709d安装DMG的登录定向五父例/11步原始PASS，独立Excel回读PASS；仍非整版回归，旧c291完整门禁FAIL。 709d LOGIN-SESSION另六父例/14步原始PASS并单独导出Excel；未完成整版回归。 709d LOGIN-VALIDATION十父+十二变体及LOGIN-RATE一父另两次定向PASS/Excel；四批登录合计22父+12变体，但TM001其他功能未验收。 709d CHANGE-PASSWORD十一父+六变体17行/32步另批定向PASS，PASSWORD-05单项独立审计PASS；未完成整版/12项审计。</x:v>
+        <x:v>开发中，未发布。c291本地master最终包门禁FAIL：116项91 PASS/14 FAIL/11 BLOCKED；9f06cb1修复私有签名输入后开发检查PASS，但新定向App仍FAIL/BLOCKED并有ENOSPC，功能回归未完成。旧d2db551独立候选PASS不转用于新候选。正式发行完整门禁NOT_RUN，无稳定0.1原包。 709d UPDATE-05定向父1+变体13 PASS，后置de081a6导出Excel回读PASS；仅定向，77父TC范围外，旧c291完整门禁FAIL及未发行不变。 709d安装DMG的登录定向五父例/11步原始PASS，独立Excel回读PASS；仍非整版回归，旧c291完整门禁FAIL。 709d LOGIN-SESSION另六父例/14步原始PASS并单独导出Excel；未完成整版回归。 709d LOGIN-VALIDATION十父+十二变体及LOGIN-RATE一父另两次定向PASS/Excel；四批登录合计22父+12变体，但TM001其他功能未验收。 709d CHANGE-PASSWORD十一父+六变体17行/32步另批定向PASS，PASSWORD-05单项独立审计PASS；未完成整版/12项审计。 709d SESSION十父+两变体12行/44步另批定向PASS，SESSION-04单项审计PASS；整版/完整审计仍未完成。</x:v>
       </x:c>
       <x:c r="K6" s="9" t="str">
         <x:v>旧SwiftUI PR #2 已合并、历史双平台六例PASS；不继承给Electron</x:v>
@@ -22364,7 +22408,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b6d80f555ee4313"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8be3a10686445f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23529,7 +23573,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R432645b548d94627"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ae934e5fe044feb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.3.0-20261001T034652Z][TM-003] Index collector source check
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R5b7e7fd9d8064136"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rca13714ea2eb4bd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R34fbcca2560341bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rbb59dd038c7e485d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R9304618290ec472c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Ra929ac29ea8c4312"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R1a21b4122a13461a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Rc4c3f614e89845c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R93d6c4490af544fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R1ea074624c644246"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R3a96156b72bc4508"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R6f80327e98dd4abb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Re718f9c052b241ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R1917b91e169745b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rf2599f419df64a22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rf9517697bb1447f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rb18197dead8e41ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R1bd9d683b0d34ffc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R47fa7220a8814f42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rfa5f86ea44294dcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Recf318c6212c49e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R19e7cee4e06949b4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -809,8 +809,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N30"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N31"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="运行批次"/>
     <x:tableColumn id="2" name="版本"/>
@@ -1146,8 +1146,8 @@
         <x:v>测试批次</x:v>
       </x:c>
       <x:c r="B9" s="10" t="n">
-        <x:f>COUNTA('06测试批次'!A5:A30)</x:f>
-        <x:v>26</x:v>
+        <x:f>COUNTA('06测试批次'!A5:A31)</x:f>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>06测试批次，每次运行一行，记录独立结果Excel位置</x:v>
@@ -1271,7 +1271,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>product_e2e · TASK-TM001-SESSION；SESSION-01..10十父TC及SESSION-05#RESET/#DISABLE两变体，11真实App执行加1父例派生：10父+2变体共12/12报告行PASS、44步、清理完成；SESSION-05父例由两变体派生。独立审计仅SESSION-04 PASS，非12项完整审计。仅709d会话功能定向，其他TM001功能、旧c291完整门禁FAIL及正式发行NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
+        <x:v>source_check · TM-003 CORE07假TM002能力主进程编排与本例SQLite固定辅助模块；非产品E2E：CORE07固定1/1、五步与owner清理PASS；先前collector_not_implemented红测FAIL原件保留，独立Excel/verification回读PASS。仅fake能力+小文件/注入预算，真实App/IPC/Keychain、任意大文件及发行均NOT_RUN/BLOCKED。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0122596413d49e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R389a0173571c46e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b959ecddd074e70"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd76318df15e54cdf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e5c7a429072496d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3907da28b35f4cc3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R978ff2256dcc47a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2fb35876a9d49ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42d9cd88455e4cde"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3618c52efb834244"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84934c925f564adf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R283733861e4f4a78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7519,7 +7519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37f1853248c14e92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c1851f2b3e14ea7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20178,7 +20178,7 @@
         <x:v>draft</x:v>
       </x:c>
       <x:c r="J269" s="4" t="str">
-        <x:v>未执行</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="K269" s="4" t="str">
         <x:v>细化用例</x:v>
@@ -20187,7 +20187,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:243</x:v>
       </x:c>
       <x:c r="M269" s="4" t="str">
-        <x:v>尚未执行</x:v>
+        <x:v>tm003-core07-20261001T200438Z</x:v>
       </x:c>
       <x:c r="N269" s="4" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -20704,7 +20704,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdb18eb57a8d40c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7109505d2c164d93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21922,25 +21922,69 @@
         <x:v>PASS</x:v>
       </x:c>
     </x:row>
+    <x:row r="31" ht="57" customHeight="1">
+      <x:c r="A31" s="4" t="str">
+        <x:v>tm003-core07-20261001T200438Z</x:v>
+      </x:c>
+      <x:c r="B31" s="4" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="C31" s="4" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D31" s="4" t="str">
+        <x:v>TM-003 CORE07假TM002能力主进程编排与本例SQLite固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E31" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F31" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G31" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H31" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I31" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J31" s="4" t="str">
+        <x:v>33b1ee1636fc8e92ecba834856769df9f112c509</x:v>
+      </x:c>
+      <x:c r="K31" s="4" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L31" s="4" t="str">
+        <x:v>CORE07固定1/1、五步与owner清理PASS；先前collector_not_implemented红测FAIL原件保留，独立Excel/verification回读PASS。仅fake能力+小文件/注入预算，真实App/IPC/Keychain、任意大文件及发行均NOT_RUN/BLOCKED。</x:v>
+      </x:c>
+      <x:c r="M31" s="4" t="str">
+        <x:v>.local/test-results/tm003-core07-20261001T200438Z/TokenMeter测试结果-tm003-core07-20261001T200438Z.xlsx</x:v>
+      </x:c>
+      <x:c r="N31" s="4" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E5:E30">
+  <x:conditionalFormatting sqref="E5:E31">
     <x:cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="26" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M30">
+  <x:conditionalFormatting sqref="M5:M31">
     <x:cfRule type="containsText" dxfId="27" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="29" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="N5:N30">
+  <x:conditionalFormatting sqref="N5:N31">
     <x:cfRule type="containsText" dxfId="30" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="32" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R464573aeb46c403f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6d089132e2b4a94"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22254,7 +22298,7 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="87" customHeight="1">
+    <x:row r="9" ht="132" customHeight="1">
       <x:c r="A9" s="4" t="str">
         <x:v>v0.3.0-20261001T034652Z（续1）</x:v>
       </x:c>
@@ -22267,7 +22311,7 @@
       <x:c r="H9" s="4" t="str"/>
       <x:c r="I9" s="4" t="str"/>
       <x:c r="J9" s="4" t="str">
-        <x:v>source_check 1/1、四步与清理PASS，独立Excel回读PASS，第18批次；此前408ebf8红测失败保留。仅多文件模块，原27条产品TC与正式发行NOT_RUN。 CORE07主进程编排辅助TC已固定输入，程序/运行尚无。</x:v>
+        <x:v>source_check 1/1、四步与清理PASS，独立Excel回读PASS，第18批次；此前408ebf8红测失败保留。仅多文件模块，原27条产品TC与正式发行NOT_RUN。 CORE07主进程编排辅助TC已固定输入，程序/运行尚无。 CORE07在33b1ee1代码候选固定模块1/1五步PASS、Excel回读；真实App/大文件产品仍未验收。</x:v>
       </x:c>
       <x:c r="K9" s="4" t="str"/>
       <x:c r="L9" s="4" t="str"/>
@@ -22408,7 +22452,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8be3a10686445f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89616e7d2e0e4eb1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23573,7 +23617,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ae934e5fe044feb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra20c7708a25d4ed0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.1.0-20260929T074814Z][TM-001] Index admin function probe
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R6f80327e98dd4abb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Re718f9c052b241ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R1917b91e169745b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rf2599f419df64a22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rf9517697bb1447f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rb18197dead8e41ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R1bd9d683b0d34ffc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R47fa7220a8814f42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rfa5f86ea44294dcb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Recf318c6212c49e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R19e7cee4e06949b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R1f7ef9a4ca614d99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R62e780c2444344e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R60dae5e928114473"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R9308ab9f90f544f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Re62843944cd844b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R0ff9868f11644f92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R898bf95a4d9244fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Rea61de4a51cd48f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R1feb460eca984418"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Ra29fb61db43d4d85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R796669df95fa49cb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -809,8 +809,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N31"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N32"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="运行批次"/>
     <x:tableColumn id="2" name="版本"/>
@@ -832,8 +832,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="TMTable8" displayName="TMTable8" ref="A4:R11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:R11"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="TMTable8" displayName="TMTable8" ref="A4:R12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:R12"/>
   <x:tableColumns count="18">
     <x:tableColumn id="1" name="发布编号"/>
     <x:tableColumn id="2" name="版本"/>
@@ -1146,8 +1146,8 @@
         <x:v>测试批次</x:v>
       </x:c>
       <x:c r="B9" s="10" t="n">
-        <x:f>COUNTA('06测试批次'!A5:A31)</x:f>
-        <x:v>27</x:v>
+        <x:f>COUNTA('06测试批次'!A5:A32)</x:f>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>06测试批次，每次运行一行，记录独立结果Excel位置</x:v>
@@ -1271,7 +1271,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>source_check · TM-003 CORE07假TM002能力主进程编排与本例SQLite固定辅助模块；非产品E2E：CORE07固定1/1、五步与owner清理PASS；先前collector_not_implemented红测FAIL原件保留，独立Excel/verification回读PASS。仅fake能力+小文件/注入预算，真实App/IPC/Keychain、任意大文件及发行均NOT_RUN/BLOCKED。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
+        <x:v>product_e2e · TASK-TM001-ADMIN；ADMIN-01..06六父TC及ADMIN-02/05下五固定变体，九真实App执行加两父例派生：6父+5变体共11/11报告行PASS、33步、清理完成；ADMIN-02/05父例由变体派生。独立审计仅ADMIN-03 PASS，非12项完整审计。仅709d管理员功能定向，其他TM001功能、旧c291完整门禁FAIL及正式发行NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R389a0173571c46e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60d54a6ba0224a79"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd76318df15e54cdf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38fc160fbd0e4883"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3907da28b35f4cc3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R563a38c6851b4300"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2fb35876a9d49ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d53b72e0f624a4a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3618c52efb834244"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94b7439a0de84eb9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R283733861e4f4a78"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf81feecdfec4aec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7519,7 +7519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c1851f2b3e14ea7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra59ff02bbe264520"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9685,7 +9685,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:258</x:v>
       </x:c>
       <x:c r="M48" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-cd15a5fef2444f748088d1fcdd29fe0d</x:v>
       </x:c>
       <x:c r="N48" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -9734,7 +9734,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:276</x:v>
       </x:c>
       <x:c r="M49" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-cd15a5fef2444f748088d1fcdd29fe0d</x:v>
       </x:c>
       <x:c r="N49" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -9783,7 +9783,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:293</x:v>
       </x:c>
       <x:c r="M50" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-cd15a5fef2444f748088d1fcdd29fe0d</x:v>
       </x:c>
       <x:c r="N50" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -9832,7 +9832,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:310</x:v>
       </x:c>
       <x:c r="M51" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-cd15a5fef2444f748088d1fcdd29fe0d</x:v>
       </x:c>
       <x:c r="N51" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -9881,7 +9881,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:327</x:v>
       </x:c>
       <x:c r="M52" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-cd15a5fef2444f748088d1fcdd29fe0d</x:v>
       </x:c>
       <x:c r="N52" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -9930,7 +9930,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:344</x:v>
       </x:c>
       <x:c r="M53" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-cd15a5fef2444f748088d1fcdd29fe0d</x:v>
       </x:c>
       <x:c r="N53" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -20704,7 +20704,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7109505d2c164d93"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R295b2eb23bc04eaa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21966,25 +21966,69 @@
         <x:v>NOT_RUN</x:v>
       </x:c>
     </x:row>
+    <x:row r="32" ht="57" customHeight="1">
+      <x:c r="A32" s="9" t="str">
+        <x:v>local-cd15a5fef2444f748088d1fcdd29fe0d</x:v>
+      </x:c>
+      <x:c r="B32" s="9" t="str">
+        <x:v>v0.1.0-20260929T074814Z</x:v>
+      </x:c>
+      <x:c r="C32" s="9" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D32" s="9" t="str">
+        <x:v>TASK-TM001-ADMIN；ADMIN-01..06六父TC及ADMIN-02/05下五固定变体，九真实App执行加两父例派生</x:v>
+      </x:c>
+      <x:c r="E32" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F32" s="9" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G32" s="9" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H32" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I32" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J32" s="9" t="str">
+        <x:v>709d21253a0f88bc703a431cbf3adba3df17e508</x:v>
+      </x:c>
+      <x:c r="K32" s="9" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L32" s="9" t="str">
+        <x:v>6父+5变体共11/11报告行PASS、33步、清理完成；ADMIN-02/05父例由变体派生。独立审计仅ADMIN-03 PASS，非12项完整审计。仅709d管理员功能定向，其他TM001功能、旧c291完整门禁FAIL及正式发行NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M32" s="9" t="str">
+        <x:v>.local/test-results/local-cd15a5fef2444f748088d1fcdd29fe0d/TokenMeter测试结果-local-cd15a5fef2444f748088d1fcdd29fe0d.xlsx</x:v>
+      </x:c>
+      <x:c r="N32" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E5:E31">
+  <x:conditionalFormatting sqref="E5:E32">
     <x:cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="26" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M31">
+  <x:conditionalFormatting sqref="M5:M32">
     <x:cfRule type="containsText" dxfId="27" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="29" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="N5:N31">
+  <x:conditionalFormatting sqref="N5:N32">
     <x:cfRule type="containsText" dxfId="30" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="32" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6d089132e2b4a94"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfefa159669d54fe7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22130,7 +22174,7 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="372" customHeight="1">
+    <x:row r="6" ht="402" customHeight="1">
       <x:c r="A6" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
       </x:c>
@@ -22159,7 +22203,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J6" s="9" t="str">
-        <x:v>开发中，未发布。c291本地master最终包门禁FAIL：116项91 PASS/14 FAIL/11 BLOCKED；9f06cb1修复私有签名输入后开发检查PASS，但新定向App仍FAIL/BLOCKED并有ENOSPC，功能回归未完成。旧d2db551独立候选PASS不转用于新候选。正式发行完整门禁NOT_RUN，无稳定0.1原包。 709d UPDATE-05定向父1+变体13 PASS，后置de081a6导出Excel回读PASS；仅定向，77父TC范围外，旧c291完整门禁FAIL及未发行不变。 709d安装DMG的登录定向五父例/11步原始PASS，独立Excel回读PASS；仍非整版回归，旧c291完整门禁FAIL。 709d LOGIN-SESSION另六父例/14步原始PASS并单独导出Excel；未完成整版回归。 709d LOGIN-VALIDATION十父+十二变体及LOGIN-RATE一父另两次定向PASS/Excel；四批登录合计22父+12变体，但TM001其他功能未验收。 709d CHANGE-PASSWORD十一父+六变体17行/32步另批定向PASS，PASSWORD-05单项独立审计PASS；未完成整版/12项审计。 709d SESSION十父+两变体12行/44步另批定向PASS，SESSION-04单项审计PASS；整版/完整审计仍未完成。</x:v>
+        <x:v>开发中，未发布。c291本地master最终包门禁FAIL：116项91 PASS/14 FAIL/11 BLOCKED；9f06cb1修复私有签名输入后开发检查PASS，但新定向App仍FAIL/BLOCKED并有ENOSPC，功能回归未完成。旧d2db551独立候选PASS不转用于新候选。正式发行完整门禁NOT_RUN，无稳定0.1原包。 709d UPDATE-05定向父1+变体13 PASS，后置de081a6导出Excel回读PASS；仅定向，77父TC范围外，旧c291完整门禁FAIL及未发行不变。 709d安装DMG的登录定向五父例/11步原始PASS，独立Excel回读PASS；仍非整版回归，旧c291完整门禁FAIL。 709d LOGIN-SESSION另六父例/14步原始PASS并单独导出Excel；未完成整版回归。 709d LOGIN-VALIDATION十父+十二变体及LOGIN-RATE一父另两次定向PASS/Excel；四批登录合计22父+12变体，但TM001其他功能未验收。 709d CHANGE-PASSWORD十一父+六变体17行/32步另批定向PASS，PASSWORD-05单项独立审计PASS；未完成整版/12项审计。 709d SESSION十父+两变体12行/44步另批定向PASS，SESSION-04单项审计PASS；整版/完整审计仍未完成。 709d ADMIN六父+五变体11行/33步另批定向PASS，ADMIN-03单项审计</x:v>
       </x:c>
       <x:c r="K6" s="9" t="str">
         <x:v>旧SwiftUI PR #2 已合并、历史双平台六例PASS；不继承给Electron</x:v>
@@ -22186,77 +22230,45 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="342" customHeight="1">
+    <x:row r="7" ht="32" customHeight="1">
       <x:c r="A7" s="4" t="str">
+        <x:v>v0.1.0-20260929T074814Z（续1）</x:v>
+      </x:c>
+      <x:c r="B7" s="4" t="str"/>
+      <x:c r="C7" s="16" t="str"/>
+      <x:c r="D7" s="4" t="str"/>
+      <x:c r="E7" s="4" t="str"/>
+      <x:c r="F7" s="4" t="str"/>
+      <x:c r="G7" s="4" t="str"/>
+      <x:c r="H7" s="4" t="str"/>
+      <x:c r="I7" s="4" t="str"/>
+      <x:c r="J7" s="4" t="str">
+        <x:v>PASS；整版/完整审计仍未完成。</x:v>
+      </x:c>
+      <x:c r="K7" s="4" t="str"/>
+      <x:c r="L7" s="4" t="str"/>
+      <x:c r="M7" s="4" t="str"/>
+      <x:c r="N7" s="4" t="str"/>
+      <x:c r="O7" s="4" t="str"/>
+      <x:c r="P7" s="4" t="str"/>
+      <x:c r="Q7" s="4" t="str"/>
+      <x:c r="R7" s="4" t="str"/>
+    </x:row>
+    <x:row r="8" ht="342" customHeight="1">
+      <x:c r="A8" s="9" t="str">
         <x:v>v0.2.0-20261001T034118Z</x:v>
       </x:c>
-      <x:c r="B7" s="4" t="str">
+      <x:c r="B8" s="9" t="str">
         <x:v>0.2.0</x:v>
       </x:c>
-      <x:c r="C7" s="16" t="n">
+      <x:c r="C8" s="17" t="n">
         <x:v>46296.15368055556</x:v>
-      </x:c>
-      <x:c r="D7" s="4" t="str">
-        <x:v>产品功能</x:v>
-      </x:c>
-      <x:c r="E7" s="4" t="str">
-        <x:v>TM-002</x:v>
-      </x:c>
-      <x:c r="F7" s="4" t="str">
-        <x:v>未发布</x:v>
-      </x:c>
-      <x:c r="G7" s="4" t="str">
-        <x:v>internal</x:v>
-      </x:c>
-      <x:c r="H7" s="4" t="str">
-        <x:v>本机版本归档及 dmg/&lt;release_id&gt;/；当前无本版正式包</x:v>
-      </x:c>
-      <x:c r="I7" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J7" s="4" t="str">
-        <x:v>设计基线已完成：3功能点、9 TASK、28父TC、35变体。开发工作树已有原生目录面板、加密locator、根FD受限读取、React授权UI及33个固定E2E叶入口（28可执行、5场景摘要）；报告单元59/59、治理473/473、构建PASS。产品E2E因AX trusted=false及隔离标准测试账号不可用BLOCKED，Keychain最终包隔离未证实。本独立文档树未合该代码，机器绑定仍planned；正式发行完整门禁NOT_RUN、未发布。0.2公开配置为version0.2.0/build200及测试高版0.2.1/build201，实际0.2包尚未证明。 2026-10-02修订SECURITY-01三个恶意字串变体的固定IPC method/字段/错误码，产品状态不变；需在整合候选重核基线及固定程序。 EVIDENCE-01新增第七固定负例，本版36变体；SECURITY-01仅profile准备目录纠错。新输入未执行，产品E2E仍NOT_RUN。 0cc4f3e候选包预检33条全BLOCKED、零产品步骤；缺显式独立test/excluded账号，App未启动；固定结果Excel缺失，根总表批次待登记。</x:v>
-      </x:c>
-      <x:c r="K7" s="4" t="str">
-        <x:v>TM001独立候选d2门禁PASS只属历史；本地master c2911bc首次最终包门禁FAIL、无SOP-020稳定原包，不能作为0.2升级源；本版无实际产品运行。</x:v>
-      </x:c>
-      <x:c r="L7" s="4" t="str">
-        <x:v>releases/v0.2.0-20261001T034118Z/00-manifest.json</x:v>
-      </x:c>
-      <x:c r="M7" s="4" t="str">
-        <x:v>releases/v0.2.0-20261001T034118Z/06-iteration-record.md</x:v>
-      </x:c>
-      <x:c r="N7" s="4" t="str">
-        <x:v>未核实同名功能分支SHA/tree读回</x:v>
-      </x:c>
-      <x:c r="O7" s="4" t="str">
-        <x:v>产品E2E未执行；本机稳定包未归档</x:v>
-      </x:c>
-      <x:c r="P7" s="4" t="str">
-        <x:v>本轮五版稳定后一次受保护PR；待办</x:v>
-      </x:c>
-      <x:c r="Q7" s="4" t="str">
-        <x:v>本轮五版稳定及远端master读回后逐版登记；待办</x:v>
-      </x:c>
-      <x:c r="R7" s="4" t="str">
-        <x:v>releases/v0.2.0-20261001T034118Z/01-requirements.md:32</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="387" customHeight="1">
-      <x:c r="A8" s="9" t="str">
-        <x:v>v0.3.0-20261001T034652Z</x:v>
-      </x:c>
-      <x:c r="B8" s="9" t="str">
-        <x:v>0.3.0</x:v>
-      </x:c>
-      <x:c r="C8" s="17" t="n">
-        <x:v>46296.157546296294</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
         <x:v>产品功能</x:v>
       </x:c>
       <x:c r="E8" s="9" t="str">
-        <x:v>TM-003</x:v>
+        <x:v>TM-002</x:v>
       </x:c>
       <x:c r="F8" s="9" t="str">
         <x:v>未发布</x:v>
@@ -22265,28 +22277,28 @@
         <x:v>internal</x:v>
       </x:c>
       <x:c r="H8" s="9" t="str">
-        <x:v>dmg/&lt;release_id&gt;/：正式包仅在本机门禁 PASS 后保存</x:v>
+        <x:v>本机版本归档及 dmg/&lt;release_id&gt;/；当前无本版正式包</x:v>
       </x:c>
       <x:c r="I8" s="18" t="b">
         <x:v>0</x:v>
       </x:c>
       <x:c r="J8" s="9" t="str">
-        <x:v>整版draft、未发布。27条产品TC未执行；3条CORE辅助TC已在文档提交48ca089独立切片就绪，在开发分支311deedf运行模块3/3 PASS，原始receipt在该分支.local/ci/tm003-core-20261001/。代码尚未合入本文档树，机器绑定保持空；模块报告不能作为产品E2E或发行门禁，结果Excel规范待SOP修订。 2026-10-02新代码候选44379e6已有逐步模块3/3与桌面29/29/typecheck/build原件；source_check独立Excel导出程序仍缺，批次登记BLOCKED，产品E2E仍NOT_RUN。 固定导出器新run tm003-core-20261001T163807Z在ea6b187候选生成3/3/9步source_check独立Excel并回读PASS，现已按被测SHA登记模块批次；原27条产品TC与发行仍NOT_RUN。 新清理合同候选d7c3d39的独立run tm003-core-20261001T165439Z亦3/3/9步及Excel回读PASS，作为最新模块批次；旧ea6批次保留。 后续CORE-04/05的测试输入已编制，程序未绑定、未执行；独立SOP-008切片复核待文档干净提交。 CORE04/05基于9efc6fa独立source_check 2/2、9步和Excel回读PASS，第17批次；CORE06新输入未执行，产品E2E NOT_RUN。 CORE06在eef956b的固定</x:v>
+        <x:v>设计基线已完成：3功能点、9 TASK、28父TC、35变体。开发工作树已有原生目录面板、加密locator、根FD受限读取、React授权UI及33个固定E2E叶入口（28可执行、5场景摘要）；报告单元59/59、治理473/473、构建PASS。产品E2E因AX trusted=false及隔离标准测试账号不可用BLOCKED，Keychain最终包隔离未证实。本独立文档树未合该代码，机器绑定仍planned；正式发行完整门禁NOT_RUN、未发布。0.2公开配置为version0.2.0/build200及测试高版0.2.1/build201，实际0.2包尚未证明。 2026-10-02修订SECURITY-01三个恶意字串变体的固定IPC method/字段/错误码，产品状态不变；需在整合候选重核基线及固定程序。 EVIDENCE-01新增第七固定负例，本版36变体；SECURITY-01仅profile准备目录纠错。新输入未执行，产品E2E仍NOT_RUN。 0cc4f3e候选包预检33条全BLOCKED、零产品步骤；缺显式独立test/excluded账号，App未启动；固定结果Excel缺失，根总表批次待登记。</x:v>
       </x:c>
       <x:c r="K8" s="9" t="str">
-        <x:v>TM-001 干净源码候选为技术基底；其产品门禁不继承给TM-003</x:v>
+        <x:v>TM001独立候选d2门禁PASS只属历史；本地master c2911bc首次最终包门禁FAIL、无SOP-020稳定原包，不能作为0.2升级源；本版无实际产品运行。</x:v>
       </x:c>
       <x:c r="L8" s="9" t="str">
-        <x:v>releases/v0.3.0-20261001T034652Z/00-manifest.json</x:v>
+        <x:v>releases/v0.2.0-20261001T034118Z/00-manifest.json</x:v>
       </x:c>
       <x:c r="M8" s="9" t="str">
-        <x:v>releases/v0.3.0-20261001T034652Z/06-iteration-record.md</x:v>
+        <x:v>releases/v0.2.0-20261001T034118Z/06-iteration-record.md</x:v>
       </x:c>
       <x:c r="N8" s="9" t="str">
         <x:v>未核实同名功能分支SHA/tree读回</x:v>
       </x:c>
       <x:c r="O8" s="9" t="str">
-        <x:v>CORE模块3/3只在独立开发分支PASS；真实安装App产品E2E未运行；本机稳定包未归档</x:v>
+        <x:v>产品E2E未执行；本机稳定包未归档</x:v>
       </x:c>
       <x:c r="P8" s="9" t="str">
         <x:v>本轮五版稳定后一次受保护PR；待办</x:v>
@@ -22295,128 +22307,128 @@
         <x:v>本轮五版稳定及远端master读回后逐版登记；待办</x:v>
       </x:c>
       <x:c r="R8" s="9" t="str">
+        <x:v>releases/v0.2.0-20261001T034118Z/01-requirements.md:32</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="387" customHeight="1">
+      <x:c r="A9" s="4" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="B9" s="4" t="str">
+        <x:v>0.3.0</x:v>
+      </x:c>
+      <x:c r="C9" s="16" t="n">
+        <x:v>46296.157546296294</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="str">
+        <x:v>产品功能</x:v>
+      </x:c>
+      <x:c r="E9" s="4" t="str">
+        <x:v>TM-003</x:v>
+      </x:c>
+      <x:c r="F9" s="4" t="str">
+        <x:v>未发布</x:v>
+      </x:c>
+      <x:c r="G9" s="4" t="str">
+        <x:v>internal</x:v>
+      </x:c>
+      <x:c r="H9" s="4" t="str">
+        <x:v>dmg/&lt;release_id&gt;/：正式包仅在本机门禁 PASS 后保存</x:v>
+      </x:c>
+      <x:c r="I9" s="15" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J9" s="4" t="str">
+        <x:v>整版draft、未发布。27条产品TC未执行；3条CORE辅助TC已在文档提交48ca089独立切片就绪，在开发分支311deedf运行模块3/3 PASS，原始receipt在该分支.local/ci/tm003-core-20261001/。代码尚未合入本文档树，机器绑定保持空；模块报告不能作为产品E2E或发行门禁，结果Excel规范待SOP修订。 2026-10-02新代码候选44379e6已有逐步模块3/3与桌面29/29/typecheck/build原件；source_check独立Excel导出程序仍缺，批次登记BLOCKED，产品E2E仍NOT_RUN。 固定导出器新run tm003-core-20261001T163807Z在ea6b187候选生成3/3/9步source_check独立Excel并回读PASS，现已按被测SHA登记模块批次；原27条产品TC与发行仍NOT_RUN。 新清理合同候选d7c3d39的独立run tm003-core-20261001T165439Z亦3/3/9步及Excel回读PASS，作为最新模块批次；旧ea6批次保留。 后续CORE-04/05的测试输入已编制，程序未绑定、未执行；独立SOP-008切片复核待文档干净提交。 CORE04/05基于9efc6fa独立source_check 2/2、9步和Excel回读PASS，第17批次；CORE06新输入未执行，产品E2E NOT_RUN。 CORE06在eef956b的固定</x:v>
+      </x:c>
+      <x:c r="K9" s="4" t="str">
+        <x:v>TM-001 干净源码候选为技术基底；其产品门禁不继承给TM-003</x:v>
+      </x:c>
+      <x:c r="L9" s="4" t="str">
+        <x:v>releases/v0.3.0-20261001T034652Z/00-manifest.json</x:v>
+      </x:c>
+      <x:c r="M9" s="4" t="str">
+        <x:v>releases/v0.3.0-20261001T034652Z/06-iteration-record.md</x:v>
+      </x:c>
+      <x:c r="N9" s="4" t="str">
+        <x:v>未核实同名功能分支SHA/tree读回</x:v>
+      </x:c>
+      <x:c r="O9" s="4" t="str">
+        <x:v>CORE模块3/3只在独立开发分支PASS；真实安装App产品E2E未运行；本机稳定包未归档</x:v>
+      </x:c>
+      <x:c r="P9" s="4" t="str">
+        <x:v>本轮五版稳定后一次受保护PR；待办</x:v>
+      </x:c>
+      <x:c r="Q9" s="4" t="str">
+        <x:v>本轮五版稳定及远端master读回后逐版登记；待办</x:v>
+      </x:c>
+      <x:c r="R9" s="4" t="str">
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="132" customHeight="1">
-      <x:c r="A9" s="4" t="str">
+    <x:row r="10" ht="132" customHeight="1">
+      <x:c r="A10" s="9" t="str">
         <x:v>v0.3.0-20261001T034652Z（续1）</x:v>
       </x:c>
-      <x:c r="B9" s="4" t="str"/>
-      <x:c r="C9" s="16" t="str"/>
-      <x:c r="D9" s="4" t="str"/>
-      <x:c r="E9" s="4" t="str"/>
-      <x:c r="F9" s="4" t="str"/>
-      <x:c r="G9" s="4" t="str"/>
-      <x:c r="H9" s="4" t="str"/>
-      <x:c r="I9" s="4" t="str"/>
-      <x:c r="J9" s="4" t="str">
+      <x:c r="B10" s="9" t="str"/>
+      <x:c r="C10" s="17" t="str"/>
+      <x:c r="D10" s="9" t="str"/>
+      <x:c r="E10" s="9" t="str"/>
+      <x:c r="F10" s="9" t="str"/>
+      <x:c r="G10" s="9" t="str"/>
+      <x:c r="H10" s="9" t="str"/>
+      <x:c r="I10" s="9" t="str"/>
+      <x:c r="J10" s="9" t="str">
         <x:v>source_check 1/1、四步与清理PASS，独立Excel回读PASS，第18批次；此前408ebf8红测失败保留。仅多文件模块，原27条产品TC与正式发行NOT_RUN。 CORE07主进程编排辅助TC已固定输入，程序/运行尚无。 CORE07在33b1ee1代码候选固定模块1/1五步PASS、Excel回读；真实App/大文件产品仍未验收。</x:v>
       </x:c>
-      <x:c r="K9" s="4" t="str"/>
-      <x:c r="L9" s="4" t="str"/>
-      <x:c r="M9" s="4" t="str"/>
-      <x:c r="N9" s="4" t="str"/>
-      <x:c r="O9" s="4" t="str"/>
-      <x:c r="P9" s="4" t="str"/>
-      <x:c r="Q9" s="4" t="str"/>
-      <x:c r="R9" s="4" t="str"/>
-    </x:row>
-    <x:row r="10" ht="237" customHeight="1">
-      <x:c r="A10" s="9" t="str">
+      <x:c r="K10" s="9" t="str"/>
+      <x:c r="L10" s="9" t="str"/>
+      <x:c r="M10" s="9" t="str"/>
+      <x:c r="N10" s="9" t="str"/>
+      <x:c r="O10" s="9" t="str"/>
+      <x:c r="P10" s="9" t="str"/>
+      <x:c r="Q10" s="9" t="str"/>
+      <x:c r="R10" s="9" t="str"/>
+    </x:row>
+    <x:row r="11" ht="237" customHeight="1">
+      <x:c r="A11" s="4" t="str">
         <x:v>v0.4.0-20261001T040433Z</x:v>
       </x:c>
-      <x:c r="B10" s="9" t="str">
+      <x:c r="B11" s="4" t="str">
         <x:v>0.4.0</x:v>
       </x:c>
-      <x:c r="C10" s="17" t="n">
+      <x:c r="C11" s="16" t="n">
         <x:v>46296.16982638889</x:v>
-      </x:c>
-      <x:c r="D10" s="9" t="str">
-        <x:v>产品功能</x:v>
-      </x:c>
-      <x:c r="E10" s="9" t="str">
-        <x:v>TM-004</x:v>
-      </x:c>
-      <x:c r="F10" s="9" t="str">
-        <x:v>未发布</x:v>
-      </x:c>
-      <x:c r="G10" s="9" t="str">
-        <x:v>internal</x:v>
-      </x:c>
-      <x:c r="H10" s="9" t="str">
-        <x:v>dmg/&lt;release_id&gt;/：仅门禁PASS后放正式DMG</x:v>
-      </x:c>
-      <x:c r="I10" s="18" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J10" s="9" t="str">
-        <x:v>整版draft、未发布。原20产品细TC及四组摘要保留，3条reader CORE辅助TC在输入提交fea41fe/同步SOP后的干净候选ebbcfd0上按SOP-008独立判为development_slice_ready；程序绑定仍空。本版代码分支e52b62e报告reader目标9/9、桌面49/49和build PASS，仅为模块原件，Excel/总表批次尚无固定导出器。产品授权、稳定文件身份最终接口、SQLite原子事务、IPC/App E2E未验证，正式发行门禁NOT_RUN。 新增CORE04/05合成主进程触发及三文件存储辅助输入：拒绝码、提交守卫、来源/根分域HMAC、scope代号、modelId哨兵与整代事务；两例程序未绑定/未运行，原20条产品TC与正式发行NOT_RUN。</x:v>
-      </x:c>
-      <x:c r="K10" s="9" t="str">
-        <x:v>TM004源分支原生零/缺失与nested Agent定向探针仅为研究证据；0.3及此前稳定原包尚未形成，真实升级BLOCKED。</x:v>
-      </x:c>
-      <x:c r="L10" s="9" t="str">
-        <x:v>releases/v0.4.0-20261001T040433Z/00-manifest.json</x:v>
-      </x:c>
-      <x:c r="M10" s="9" t="str">
-        <x:v>releases/v0.4.0-20261001T040433Z/06-iteration-record.md</x:v>
-      </x:c>
-      <x:c r="N10" s="9" t="str">
-        <x:v>未核实同名远端功能分支SHA/tree</x:v>
-      </x:c>
-      <x:c r="O10" s="9" t="str">
-        <x:v>最终包产品E2E未执行；本机稳定包未归档</x:v>
-      </x:c>
-      <x:c r="P10" s="9" t="str">
-        <x:v>全部目标版本稳定后待办</x:v>
-      </x:c>
-      <x:c r="Q10" s="9" t="str">
-        <x:v>远端master读回后逐版待办</x:v>
-      </x:c>
-      <x:c r="R10" s="9" t="str">
-        <x:v>未提供</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="372" customHeight="1">
-      <x:c r="A11" s="4" t="str">
-        <x:v>v0.5.0-20261001T034729Z</x:v>
-      </x:c>
-      <x:c r="B11" s="4" t="str">
-        <x:v>0.5.0</x:v>
-      </x:c>
-      <x:c r="C11" s="16" t="n">
-        <x:v>46296.15797453704</x:v>
       </x:c>
       <x:c r="D11" s="4" t="str">
         <x:v>产品功能</x:v>
       </x:c>
       <x:c r="E11" s="4" t="str">
-        <x:v>TM-005</x:v>
+        <x:v>TM-004</x:v>
       </x:c>
       <x:c r="F11" s="4" t="str">
-        <x:v>draft</x:v>
+        <x:v>未发布</x:v>
       </x:c>
       <x:c r="G11" s="4" t="str">
         <x:v>internal</x:v>
       </x:c>
       <x:c r="H11" s="4" t="str">
-        <x:v>dmg/&lt;release_id&gt;/：仅门禁PASS后放正式原名包</x:v>
+        <x:v>dmg/&lt;release_id&gt;/：仅门禁PASS后放正式DMG</x:v>
       </x:c>
       <x:c r="I11" s="15" t="b">
         <x:v>0</x:v>
       </x:c>
       <x:c r="J11" s="4" t="str">
-        <x:v>整版draft、未发布。原32条产品父TC、6稳定变体和两组摘要保留；纯统计CORE-01/02/03辅助TC在输入提交061c759后，经SOP-008内容核对及结构/治理457项PASS，独立切片development_slice_ready，程序绑定仍为空、模块实际运行unexecuted。静态oracle与切片就绪不证明真实双来源采集或产品E2E；固定产品数据、SQLite/IPC、安装App逐TC绑定未完成，正式发行完整门禁NOT_RUN。 独立代码提交6a0f6f的source_check CORE3/3、桌面29/29、build PASS，原件在TM005工作树.local/tm005-core-postcommit-20261001T162401Z；程序尚未进入本文档树、模块Excel导出/批次登记BLOCKED，产品E2E仍NOT_RUN。 CORE-01仅验证已给UTC半开界聚合，不验证IANA日期换算；该单独辅助TC待固定。 新增CORE04/05固定IANA当地日与合成双来源SQLite只读快照辅助TC，程序null/unexecuted；coverage表无连续空日证明，原32产品TC/6变体与发行仍BLOCKED/NOT_RUN。 CORE04/05在259cf768候选固定模块分别1/1三/四步PASS且Excel回读；0.5产品E2E未运行。</x:v>
+        <x:v>整版draft、未发布。原20产品细TC及四组摘要保留，3条reader CORE辅助TC在输入提交fea41fe/同步SOP后的干净候选ebbcfd0上按SOP-008独立判为development_slice_ready；程序绑定仍空。本版代码分支e52b62e报告reader目标9/9、桌面49/49和build PASS，仅为模块原件，Excel/总表批次尚无固定导出器。产品授权、稳定文件身份最终接口、SQLite原子事务、IPC/App E2E未验证，正式发行门禁NOT_RUN。 新增CORE04/05合成主进程触发及三文件存储辅助输入：拒绝码、提交守卫、来源/根分域HMAC、scope代号、modelId哨兵与整代事务；两例程序未绑定/未运行，原20条产品TC与正式发行NOT_RUN。</x:v>
       </x:c>
       <x:c r="K11" s="4" t="str">
-        <x:v>TM005语义oracle只验证规范化样例；0.4及此前稳定原包尚未形成，真实升级BLOCKED。</x:v>
+        <x:v>TM004源分支原生零/缺失与nested Agent定向探针仅为研究证据；0.3及此前稳定原包尚未形成，真实升级BLOCKED。</x:v>
       </x:c>
       <x:c r="L11" s="4" t="str">
-        <x:v>releases/v0.5.0-20261001T034729Z/00-manifest.json</x:v>
+        <x:v>releases/v0.4.0-20261001T040433Z/00-manifest.json</x:v>
       </x:c>
       <x:c r="M11" s="4" t="str">
-        <x:v>releases/v0.5.0-20261001T034729Z/06-iteration-record.md</x:v>
+        <x:v>releases/v0.4.0-20261001T040433Z/06-iteration-record.md</x:v>
       </x:c>
       <x:c r="N11" s="4" t="str">
         <x:v>未核实同名远端功能分支SHA/tree</x:v>
@@ -22434,25 +22446,81 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
+    <x:row r="12" ht="372" customHeight="1">
+      <x:c r="A12" s="9" t="str">
+        <x:v>v0.5.0-20261001T034729Z</x:v>
+      </x:c>
+      <x:c r="B12" s="9" t="str">
+        <x:v>0.5.0</x:v>
+      </x:c>
+      <x:c r="C12" s="17" t="n">
+        <x:v>46296.15797453704</x:v>
+      </x:c>
+      <x:c r="D12" s="9" t="str">
+        <x:v>产品功能</x:v>
+      </x:c>
+      <x:c r="E12" s="9" t="str">
+        <x:v>TM-005</x:v>
+      </x:c>
+      <x:c r="F12" s="9" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="G12" s="9" t="str">
+        <x:v>internal</x:v>
+      </x:c>
+      <x:c r="H12" s="9" t="str">
+        <x:v>dmg/&lt;release_id&gt;/：仅门禁PASS后放正式原名包</x:v>
+      </x:c>
+      <x:c r="I12" s="18" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J12" s="9" t="str">
+        <x:v>整版draft、未发布。原32条产品父TC、6稳定变体和两组摘要保留；纯统计CORE-01/02/03辅助TC在输入提交061c759后，经SOP-008内容核对及结构/治理457项PASS，独立切片development_slice_ready，程序绑定仍为空、模块实际运行unexecuted。静态oracle与切片就绪不证明真实双来源采集或产品E2E；固定产品数据、SQLite/IPC、安装App逐TC绑定未完成，正式发行完整门禁NOT_RUN。 独立代码提交6a0f6f的source_check CORE3/3、桌面29/29、build PASS，原件在TM005工作树.local/tm005-core-postcommit-20261001T162401Z；程序尚未进入本文档树、模块Excel导出/批次登记BLOCKED，产品E2E仍NOT_RUN。 CORE-01仅验证已给UTC半开界聚合，不验证IANA日期换算；该单独辅助TC待固定。 新增CORE04/05固定IANA当地日与合成双来源SQLite只读快照辅助TC，程序null/unexecuted；coverage表无连续空日证明，原32产品TC/6变体与发行仍BLOCKED/NOT_RUN。 CORE04/05在259cf768候选固定模块分别1/1三/四步PASS且Excel回读；0.5产品E2E未运行。</x:v>
+      </x:c>
+      <x:c r="K12" s="9" t="str">
+        <x:v>TM005语义oracle只验证规范化样例；0.4及此前稳定原包尚未形成，真实升级BLOCKED。</x:v>
+      </x:c>
+      <x:c r="L12" s="9" t="str">
+        <x:v>releases/v0.5.0-20261001T034729Z/00-manifest.json</x:v>
+      </x:c>
+      <x:c r="M12" s="9" t="str">
+        <x:v>releases/v0.5.0-20261001T034729Z/06-iteration-record.md</x:v>
+      </x:c>
+      <x:c r="N12" s="9" t="str">
+        <x:v>未核实同名远端功能分支SHA/tree</x:v>
+      </x:c>
+      <x:c r="O12" s="9" t="str">
+        <x:v>最终包产品E2E未执行；本机稳定包未归档</x:v>
+      </x:c>
+      <x:c r="P12" s="9" t="str">
+        <x:v>全部目标版本稳定后待办</x:v>
+      </x:c>
+      <x:c r="Q12" s="9" t="str">
+        <x:v>远端master读回后逐版待办</x:v>
+      </x:c>
+      <x:c r="R12" s="9" t="str">
+        <x:v>未提供</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="F5:F11">
+  <x:conditionalFormatting sqref="F5:F12">
     <x:cfRule type="containsText" dxfId="33" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="34" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="35" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="J5:J11">
+  <x:conditionalFormatting sqref="J5:J12">
     <x:cfRule type="containsText" dxfId="36" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="37" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="38" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M11">
+  <x:conditionalFormatting sqref="M5:M12">
     <x:cfRule type="containsText" dxfId="39" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="40" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="41" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89616e7d2e0e4eb1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2089892258904863"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23617,7 +23685,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra20c7708a25d4ed0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R404a1b5e6b9340bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.3.0-20261001T034652Z][TM-003] Bind integrated core source checks
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R1f7ef9a4ca614d99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R62e780c2444344e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R60dae5e928114473"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R9308ab9f90f544f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Re62843944cd844b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R0ff9868f11644f92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R898bf95a4d9244fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Rea61de4a51cd48f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R1feb460eca984418"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Ra29fb61db43d4d85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R796669df95fa49cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R973aa54391a44687"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R4b282092e32c43aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Re5467380387b4478"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R1a9ed1474af742ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R818f478a06e9428b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R4eb2b9217f744629"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rbeb17a9fa52442f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Rb5b62cb9daf04f49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rfcecf67b1b7b400d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Rd322f63fd3ee45ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Re9b54c41d0cc48b8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60d54a6ba0224a79"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf48705fa661a4a3f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38fc160fbd0e4883"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61c84bf56a834a1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R563a38c6851b4300"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17a167dc21124505"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d53b72e0f624a4a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ddb6023d1a64466"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94b7439a0de84eb9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8099e739fb554904"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf81feecdfec4aec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8cdb253d7d7435b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7519,7 +7519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra59ff02bbe264520"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R304ed94fc7994fdf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18586,7 +18586,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L236" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:265</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:267</x:v>
       </x:c>
       <x:c r="M236" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18633,7 +18633,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L237" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:269</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:271</x:v>
       </x:c>
       <x:c r="M237" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18680,7 +18680,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L238" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:273</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:275</x:v>
       </x:c>
       <x:c r="M238" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18728,7 +18728,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L239" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:277</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:279</x:v>
       </x:c>
       <x:c r="M239" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18778,7 +18778,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L240" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:281</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:283</x:v>
       </x:c>
       <x:c r="M240" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18826,7 +18826,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L241" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:285</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:287</x:v>
       </x:c>
       <x:c r="M241" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18873,7 +18873,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L242" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:289</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:291</x:v>
       </x:c>
       <x:c r="M242" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18920,7 +18920,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L243" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:293</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:295</x:v>
       </x:c>
       <x:c r="M243" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18968,7 +18968,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L244" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:297</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:299</x:v>
       </x:c>
       <x:c r="M244" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19017,7 +19017,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L245" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:301</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:303</x:v>
       </x:c>
       <x:c r="M245" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19066,7 +19066,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L246" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:305</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:307</x:v>
       </x:c>
       <x:c r="M246" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19115,7 +19115,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L247" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:309</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:311</x:v>
       </x:c>
       <x:c r="M247" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19162,7 +19162,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L248" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:313</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:315</x:v>
       </x:c>
       <x:c r="M248" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19210,7 +19210,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L249" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:317</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:319</x:v>
       </x:c>
       <x:c r="M249" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19258,7 +19258,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L250" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:321</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:323</x:v>
       </x:c>
       <x:c r="M250" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19306,7 +19306,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L251" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:325</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:327</x:v>
       </x:c>
       <x:c r="M251" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19354,7 +19354,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L252" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:329</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:331</x:v>
       </x:c>
       <x:c r="M252" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19404,7 +19404,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L253" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:333</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:335</x:v>
       </x:c>
       <x:c r="M253" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19451,7 +19451,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L254" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:337</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:339</x:v>
       </x:c>
       <x:c r="M254" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19498,7 +19498,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L255" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:341</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:343</x:v>
       </x:c>
       <x:c r="M255" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19546,7 +19546,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L256" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:345</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:347</x:v>
       </x:c>
       <x:c r="M256" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19595,7 +19595,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L257" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:349</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:351</x:v>
       </x:c>
       <x:c r="M257" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19645,7 +19645,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L258" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:353</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:355</x:v>
       </x:c>
       <x:c r="M258" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19693,7 +19693,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L259" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:357</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:359</x:v>
       </x:c>
       <x:c r="M259" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19742,7 +19742,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L260" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:361</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:363</x:v>
       </x:c>
       <x:c r="M260" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19790,7 +19790,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L261" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:365</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:367</x:v>
       </x:c>
       <x:c r="M261" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19838,7 +19838,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L262" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:369</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:371</x:v>
       </x:c>
       <x:c r="M262" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19886,7 +19886,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L263" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:373</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:375</x:v>
       </x:c>
       <x:c r="M263" s="4" t="str">
         <x:v>tm003-core-20261001T165439Z (source_check；产品E2E未运行)</x:v>
@@ -19935,7 +19935,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L264" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:377</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:379</x:v>
       </x:c>
       <x:c r="M264" s="9" t="str">
         <x:v>tm003-core-20261001T165439Z (source_check；产品E2E未运行)</x:v>
@@ -19983,7 +19983,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L265" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:381</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:383</x:v>
       </x:c>
       <x:c r="M265" s="4" t="str">
         <x:v>tm003-core-20261001T165439Z (source_check；产品E2E未运行)</x:v>
@@ -20184,7 +20184,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L269" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:243</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:245</x:v>
       </x:c>
       <x:c r="M269" s="4" t="str">
         <x:v>tm003-core07-20261001T200438Z</x:v>
@@ -20704,7 +20704,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R295b2eb23bc04eaa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd02653cdd09d44aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22028,7 +22028,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfefa159669d54fe7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5886ec758ee247c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22520,7 +22520,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2089892258904863"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9107288e920e4826"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23685,7 +23685,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R404a1b5e6b9340bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R371e5cbd4c204476"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.3.0-20261001T034652Z][DOC] Index seven verified function and module runs
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R973aa54391a44687"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R4b282092e32c43aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Re5467380387b4478"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R1a9ed1474af742ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R818f478a06e9428b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R4eb2b9217f744629"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Rbeb17a9fa52442f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Rb5b62cb9daf04f49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rfcecf67b1b7b400d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Rd322f63fd3ee45ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Re9b54c41d0cc48b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R25c7ef4d21ef4fd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R5d7a18cf723244dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R845ee3a915ea440d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Red87944f69614163"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rcafe748a060048ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R1f583954536444c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R34eb875fe06146a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Ra5887627fa414360"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Re6430d6359494dd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Ra807e13620044663"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Rc40f3b57de954f70"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -809,8 +809,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N32"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N39" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N39"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="运行批次"/>
     <x:tableColumn id="2" name="版本"/>
@@ -1146,8 +1146,8 @@
         <x:v>测试批次</x:v>
       </x:c>
       <x:c r="B9" s="10" t="n">
-        <x:f>COUNTA('06测试批次'!A5:A32)</x:f>
-        <x:v>28</x:v>
+        <x:f>COUNTA('06测试批次'!A5:A39)</x:f>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>06测试批次，每次运行一行，记录独立结果Excel位置</x:v>
@@ -1263,7 +1263,7 @@
         <x:v>DMG及原始证据留本机；Git保存代码、文档和此工作簿</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="87" customHeight="1">
+    <x:row r="20" ht="72" customHeight="1">
       <x:c r="A20" s="9" t="str">
         <x:v>最近登记批次</x:v>
       </x:c>
@@ -1271,7 +1271,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>product_e2e · TASK-TM001-ADMIN；ADMIN-01..06六父TC及ADMIN-02/05下五固定变体，九真实App执行加两父例派生：6父+5变体共11/11报告行PASS、33步、清理完成；ADMIN-02/05父例由变体派生。独立审计仅ADMIN-03 PASS，非12项完整审计。仅709d管理员功能定向，其他TM001功能、旧c291完整门禁FAIL及正式发行NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
+        <x:v>source_check · TM-003 tm003-core07整合候选固定辅助模块；非产品E2E：1/1固定TC、5步与owner清理PASS；固定source_check导出及verification回读PASS。仅本整合候选的模块合同，产品App/授权/Keychain及发行均NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf48705fa661a4a3f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fb220f0980b4fa0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61c84bf56a834a1a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R946b9d11108544ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17a167dc21124505"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4f8eb3da8f543fb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ddb6023d1a64466"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R617d7812655a4209"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8099e739fb554904"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59b954f88c1d42a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8cdb253d7d7435b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8865092385ba41ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7519,7 +7519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R304ed94fc7994fdf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd10e713cd477473d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10177,7 +10177,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:435</x:v>
       </x:c>
       <x:c r="M58" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-a9e4d3d99b6f4997b2f5df32a8d95563</x:v>
       </x:c>
       <x:c r="N58" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -10226,7 +10226,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:452</x:v>
       </x:c>
       <x:c r="M59" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-a9e4d3d99b6f4997b2f5df32a8d95563</x:v>
       </x:c>
       <x:c r="N59" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -10276,7 +10276,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:469</x:v>
       </x:c>
       <x:c r="M60" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-a9e4d3d99b6f4997b2f5df32a8d95563</x:v>
       </x:c>
       <x:c r="N60" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -10325,7 +10325,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:487</x:v>
       </x:c>
       <x:c r="M61" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-a9e4d3d99b6f4997b2f5df32a8d95563</x:v>
       </x:c>
       <x:c r="N61" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -10375,7 +10375,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:504</x:v>
       </x:c>
       <x:c r="M62" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-a9e4d3d99b6f4997b2f5df32a8d95563</x:v>
       </x:c>
       <x:c r="N62" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -10425,7 +10425,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:522</x:v>
       </x:c>
       <x:c r="M63" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-a9e4d3d99b6f4997b2f5df32a8d95563</x:v>
       </x:c>
       <x:c r="N63" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -10474,7 +10474,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:542</x:v>
       </x:c>
       <x:c r="M64" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-6f929a978dc54f608824992e10d7ef1b</x:v>
       </x:c>
       <x:c r="N64" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -10522,7 +10522,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:559</x:v>
       </x:c>
       <x:c r="M65" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-6f929a978dc54f608824992e10d7ef1b</x:v>
       </x:c>
       <x:c r="N65" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -10571,7 +10571,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:575</x:v>
       </x:c>
       <x:c r="M66" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-6f929a978dc54f608824992e10d7ef1b</x:v>
       </x:c>
       <x:c r="N66" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -10620,7 +10620,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:592</x:v>
       </x:c>
       <x:c r="M67" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-6f929a978dc54f608824992e10d7ef1b</x:v>
       </x:c>
       <x:c r="N67" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -10720,7 +10720,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:632</x:v>
       </x:c>
       <x:c r="M69" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-8c8930fe7be44ef88bdf56a41b74900c</x:v>
       </x:c>
       <x:c r="N69" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -10770,7 +10770,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:650</x:v>
       </x:c>
       <x:c r="M70" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-8c8930fe7be44ef88bdf56a41b74900c</x:v>
       </x:c>
       <x:c r="N70" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -10820,7 +10820,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:668</x:v>
       </x:c>
       <x:c r="M71" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-8c8930fe7be44ef88bdf56a41b74900c</x:v>
       </x:c>
       <x:c r="N71" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -19889,7 +19889,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:375</x:v>
       </x:c>
       <x:c r="M263" s="4" t="str">
-        <x:v>tm003-core-20261001T165439Z (source_check；产品E2E未运行)</x:v>
+        <x:v>tm003-core-20261001T203711Z</x:v>
       </x:c>
       <x:c r="N263" s="4" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -19938,7 +19938,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:379</x:v>
       </x:c>
       <x:c r="M264" s="9" t="str">
-        <x:v>tm003-core-20261001T165439Z (source_check；产品E2E未运行)</x:v>
+        <x:v>tm003-core-20261001T203711Z</x:v>
       </x:c>
       <x:c r="N264" s="9" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -19986,7 +19986,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:383</x:v>
       </x:c>
       <x:c r="M265" s="4" t="str">
-        <x:v>tm003-core-20261001T165439Z (source_check；产品E2E未运行)</x:v>
+        <x:v>tm003-core-20261001T203711Z</x:v>
       </x:c>
       <x:c r="N265" s="4" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -20035,7 +20035,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:203</x:v>
       </x:c>
       <x:c r="M266" s="9" t="str">
-        <x:v>tm003-core45-20261001T175000Z (source_check；产品E2E未运行)</x:v>
+        <x:v>tm003-core45-20261001T203711Z</x:v>
       </x:c>
       <x:c r="N266" s="9" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -20086,7 +20086,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:216</x:v>
       </x:c>
       <x:c r="M267" s="4" t="str">
-        <x:v>tm003-core45-20261001T175000Z (source_check；产品E2E未运行)</x:v>
+        <x:v>tm003-core45-20261001T203711Z</x:v>
       </x:c>
       <x:c r="N267" s="4" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -20136,7 +20136,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:230</x:v>
       </x:c>
       <x:c r="M268" s="9" t="str">
-        <x:v>tm003-core06-20261001T182500Z (source_check；产品E2E未运行)</x:v>
+        <x:v>tm003-core06-20261001T203711Z</x:v>
       </x:c>
       <x:c r="N268" s="9" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -20187,7 +20187,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:245</x:v>
       </x:c>
       <x:c r="M269" s="4" t="str">
-        <x:v>tm003-core07-20261001T200438Z</x:v>
+        <x:v>tm003-core07-20261001T203711Z</x:v>
       </x:c>
       <x:c r="N269" s="4" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -20704,7 +20704,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd02653cdd09d44aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R159a1893198944d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22010,25 +22010,333 @@
         <x:v>PASS</x:v>
       </x:c>
     </x:row>
+    <x:row r="33" ht="42" customHeight="1">
+      <x:c r="A33" s="4" t="str">
+        <x:v>local-a9e4d3d99b6f4997b2f5df32a8d95563</x:v>
+      </x:c>
+      <x:c r="B33" s="4" t="str">
+        <x:v>v0.1.0-20260929T074814Z</x:v>
+      </x:c>
+      <x:c r="C33" s="4" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D33" s="4" t="str">
+        <x:v>TASK-TM001-CONFIG；CONFIG-01..06六父TC真实App定向</x:v>
+      </x:c>
+      <x:c r="E33" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F33" s="4" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G33" s="4" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H33" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I33" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J33" s="4" t="str">
+        <x:v>709d21253a0f88bc703a431cbf3adba3df17e508</x:v>
+      </x:c>
+      <x:c r="K33" s="4" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L33" s="4" t="str">
+        <x:v>6父6/6行、27步、清理PASS；六父例独立审计PASS。仅709d配置功能定向，其他TM001及正式门禁未通过。</x:v>
+      </x:c>
+      <x:c r="M33" s="4" t="str">
+        <x:v>.local/test-results/local-a9e4d3d99b6f4997b2f5df32a8d95563/TokenMeter测试结果-local-a9e4d3d99b6f4997b2f5df32a8d95563.xlsx</x:v>
+      </x:c>
+      <x:c r="N33" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="42" customHeight="1">
+      <x:c r="A34" s="9" t="str">
+        <x:v>local-6f929a978dc54f608824992e10d7ef1b</x:v>
+      </x:c>
+      <x:c r="B34" s="9" t="str">
+        <x:v>v0.1.0-20260929T074814Z</x:v>
+      </x:c>
+      <x:c r="C34" s="9" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D34" s="9" t="str">
+        <x:v>TASK-TM001-UPDATE；UPDATE-01..04四父TC真实App定向</x:v>
+      </x:c>
+      <x:c r="E34" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F34" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G34" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H34" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I34" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J34" s="9" t="str">
+        <x:v>709d21253a0f88bc703a431cbf3adba3df17e508</x:v>
+      </x:c>
+      <x:c r="K34" s="9" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L34" s="9" t="str">
+        <x:v>4父4/4行、15步、清理PASS；仅UPDATE-01/04两项独立审计PASS。UPDATE-05另见第16批次，UPDATE-06..08另测；旧完整门禁FAIL不变。</x:v>
+      </x:c>
+      <x:c r="M34" s="9" t="str">
+        <x:v>.local/test-results/local-6f929a978dc54f608824992e10d7ef1b/TokenMeter测试结果-local-6f929a978dc54f608824992e10d7ef1b.xlsx</x:v>
+      </x:c>
+      <x:c r="N34" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="42" customHeight="1">
+      <x:c r="A35" s="4" t="str">
+        <x:v>local-8c8930fe7be44ef88bdf56a41b74900c</x:v>
+      </x:c>
+      <x:c r="B35" s="4" t="str">
+        <x:v>v0.1.0-20260929T074814Z</x:v>
+      </x:c>
+      <x:c r="C35" s="4" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D35" s="4" t="str">
+        <x:v>TASK-TM001-UPDATE；UPDATE-06..08三父TC真实App定向</x:v>
+      </x:c>
+      <x:c r="E35" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F35" s="4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G35" s="4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H35" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I35" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J35" s="4" t="str">
+        <x:v>709d21253a0f88bc703a431cbf3adba3df17e508</x:v>
+      </x:c>
+      <x:c r="K35" s="4" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L35" s="4" t="str">
+        <x:v>3父3/3行、15步、清理PASS；仅UPDATE-07独立审计PASS。709d UPDATE父例及13变体分散于三个定向批次，不构成整体门禁。</x:v>
+      </x:c>
+      <x:c r="M35" s="4" t="str">
+        <x:v>.local/test-results/local-8c8930fe7be44ef88bdf56a41b74900c/TokenMeter测试结果-local-8c8930fe7be44ef88bdf56a41b74900c.xlsx</x:v>
+      </x:c>
+      <x:c r="N35" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="42" customHeight="1">
+      <x:c r="A36" s="9" t="str">
+        <x:v>tm003-core-20261001T203711Z</x:v>
+      </x:c>
+      <x:c r="B36" s="9" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="C36" s="9" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D36" s="9" t="str">
+        <x:v>TM-003 tm003-core整合候选固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E36" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F36" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G36" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H36" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I36" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J36" s="9" t="str">
+        <x:v>23241734f7821ee7664e3dae5104d68699d990a4</x:v>
+      </x:c>
+      <x:c r="K36" s="9" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L36" s="9" t="str">
+        <x:v>3/3固定TC、9步与owner清理PASS；固定source_check导出及verification回读PASS。仅本整合候选的模块合同，产品App/授权/Keychain及发行均NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M36" s="9" t="str">
+        <x:v>.local/test-results/tm003-core-20261001T203711Z/TokenMeter测试结果-tm003-core-20261001T203711Z.xlsx</x:v>
+      </x:c>
+      <x:c r="N36" s="9" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="42" customHeight="1">
+      <x:c r="A37" s="4" t="str">
+        <x:v>tm003-core45-20261001T203711Z</x:v>
+      </x:c>
+      <x:c r="B37" s="4" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="C37" s="4" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D37" s="4" t="str">
+        <x:v>TM-003 tm003-core45整合候选固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E37" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F37" s="4" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G37" s="4" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H37" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I37" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J37" s="4" t="str">
+        <x:v>23241734f7821ee7664e3dae5104d68699d990a4</x:v>
+      </x:c>
+      <x:c r="K37" s="4" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L37" s="4" t="str">
+        <x:v>2/2固定TC、9步与owner清理PASS；固定source_check导出及verification回读PASS。仅本整合候选的模块合同，产品App/授权/Keychain及发行均NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M37" s="4" t="str">
+        <x:v>.local/test-results/tm003-core45-20261001T203711Z/TokenMeter测试结果-tm003-core45-20261001T203711Z.xlsx</x:v>
+      </x:c>
+      <x:c r="N37" s="4" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="42" customHeight="1">
+      <x:c r="A38" s="9" t="str">
+        <x:v>tm003-core06-20261001T203711Z</x:v>
+      </x:c>
+      <x:c r="B38" s="9" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="C38" s="9" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D38" s="9" t="str">
+        <x:v>TM-003 tm003-core06整合候选固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E38" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F38" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G38" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H38" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I38" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J38" s="9" t="str">
+        <x:v>23241734f7821ee7664e3dae5104d68699d990a4</x:v>
+      </x:c>
+      <x:c r="K38" s="9" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L38" s="9" t="str">
+        <x:v>1/1固定TC、4步与owner清理PASS；固定source_check导出及verification回读PASS。仅本整合候选的模块合同，产品App/授权/Keychain及发行均NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M38" s="9" t="str">
+        <x:v>.local/test-results/tm003-core06-20261001T203711Z/TokenMeter测试结果-tm003-core06-20261001T203711Z.xlsx</x:v>
+      </x:c>
+      <x:c r="N38" s="9" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="42" customHeight="1">
+      <x:c r="A39" s="4" t="str">
+        <x:v>tm003-core07-20261001T203711Z</x:v>
+      </x:c>
+      <x:c r="B39" s="4" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="C39" s="4" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D39" s="4" t="str">
+        <x:v>TM-003 tm003-core07整合候选固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E39" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F39" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G39" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H39" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I39" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J39" s="4" t="str">
+        <x:v>23241734f7821ee7664e3dae5104d68699d990a4</x:v>
+      </x:c>
+      <x:c r="K39" s="4" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L39" s="4" t="str">
+        <x:v>1/1固定TC、5步与owner清理PASS；固定source_check导出及verification回读PASS。仅本整合候选的模块合同，产品App/授权/Keychain及发行均NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M39" s="4" t="str">
+        <x:v>.local/test-results/tm003-core07-20261001T203711Z/TokenMeter测试结果-tm003-core07-20261001T203711Z.xlsx</x:v>
+      </x:c>
+      <x:c r="N39" s="4" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E5:E32">
+  <x:conditionalFormatting sqref="E5:E39">
     <x:cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="26" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M32">
+  <x:conditionalFormatting sqref="M5:M39">
     <x:cfRule type="containsText" dxfId="27" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="29" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="N5:N32">
+  <x:conditionalFormatting sqref="N5:N39">
     <x:cfRule type="containsText" dxfId="30" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="32" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5886ec758ee247c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa546b87be274fd7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22520,7 +22828,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9107288e920e4826"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8172fa1e86d4ef5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23685,7 +23993,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R371e5cbd4c204476"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb53fa82bde54715"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.4.0-20261001T040433Z][TM-004] Bind fixed Claude source checks
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R25c7ef4d21ef4fd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R5d7a18cf723244dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R845ee3a915ea440d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Red87944f69614163"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rcafe748a060048ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R1f583954536444c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R34eb875fe06146a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Ra5887627fa414360"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Re6430d6359494dd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Ra807e13620044663"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Rc40f3b57de954f70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R4d5e79bc3cf34b82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rae8bfd785b544c9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R614371cc937644a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R95f19b7b2ae84d15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R12729d999cb247fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R7050cb4a43fc4fab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R0c70f567e13d4892"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R3d6767aa932b49ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rf52d0edfcbbb4473"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Raf81eb3f16d64d0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R1632fb0aa65e4b6c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fb220f0980b4fa0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd30e9130706149f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R946b9d11108544ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9cf139ab3904095"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4f8eb3da8f543fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30a108f2a98b4bed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R617d7812655a4209"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56e8401ed4aa4a36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59b954f88c1d42a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cfeb4e6c68e4845"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8865092385ba41ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41a2e8da96a2445a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7519,7 +7519,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd10e713cd477473d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25043e0a708f4375"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20704,7 +20704,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R159a1893198944d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3eb9cbcd99cc45a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22336,7 +22336,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa546b87be274fd7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b08fedd6fef434d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22828,7 +22828,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8172fa1e86d4ef5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0706c88ee02424c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23993,7 +23993,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb53fa82bde54715"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fa1ec01202f4d85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.3.0-20261001T034652Z][TM-003] Define private identity and product wiring slice
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R4d5e79bc3cf34b82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rae8bfd785b544c9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R614371cc937644a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R95f19b7b2ae84d15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R12729d999cb247fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R7050cb4a43fc4fab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R0c70f567e13d4892"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R3d6767aa932b49ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rf52d0edfcbbb4473"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Raf81eb3f16d64d0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R1632fb0aa65e4b6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R3cb0d6bcdf5b4d60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rc165cd0df46944a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rdd922679d5dc4e6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R200b34690b774c08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R803defdb9bef407a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rcc23deb0274f41c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R14ea53fc1d944102"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R79ce0cdc2a9b4f2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rc84140b5b6f04fdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R573be4995ee74c91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R61bd3827d3904eb5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -765,8 +765,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="TMTable5" displayName="TMTable5" ref="A4:L73" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:L73"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="TMTable5" displayName="TMTable5" ref="A4:L76" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:L76"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="任务编号"/>
     <x:tableColumn id="2" name="层级"/>
@@ -786,8 +786,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N279" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N279"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N282" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N282"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="功能编号"/>
     <x:tableColumn id="2" name="用例编号"/>
@@ -1134,8 +1134,8 @@
         <x:v>已登记用例</x:v>
       </x:c>
       <x:c r="B8" s="11" t="n">
-        <x:f>COUNTA('05测试用例'!B5:B279)</x:f>
-        <x:v>275</x:v>
+        <x:f>COUNTA('05测试用例'!B5:B282)</x:f>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>父用例与具有稳定 ID 的变体各占一行；含未来概要场景</x:v>
@@ -1169,7 +1169,7 @@
         <x:v>界面与治理检查</x:v>
       </x:c>
       <x:c r="B11" s="10" t="n">
-        <x:v>62</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="C11" s="4" t="str">
         <x:v>辅助检查不能替代产品E2E；稳定变体独立列出</x:v>
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd30e9130706149f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78890397488e4ca9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9cf139ab3904095"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59713f1f5768440e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30a108f2a98b4bed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64341a0fc6234bb4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56e8401ed4aa4a36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e47d71ac7c345b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cfeb4e6c68e4845"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd30a4ebacc7468f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41a2e8da96a2445a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0db642e62fc64cc4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6516,7 +6516,7 @@
         <x:v>规划中</x:v>
       </x:c>
       <x:c r="K48" s="9" t="str">
-        <x:v>releases/v0.3.0-20261001T034652Z/02-breakdown.md:26</x:v>
+        <x:v>releases/v0.3.0-20261001T034652Z/02-breakdown.md:29</x:v>
       </x:c>
       <x:c r="L48" s="9" t="str">
         <x:v>未提供</x:v>
@@ -6556,7 +6556,7 @@
         <x:v>规划中</x:v>
       </x:c>
       <x:c r="K49" s="4" t="str">
-        <x:v>releases/v0.3.0-20261001T034652Z/02-breakdown.md:27</x:v>
+        <x:v>releases/v0.3.0-20261001T034652Z/02-breakdown.md:30</x:v>
       </x:c>
       <x:c r="L49" s="4" t="str">
         <x:v>未提供</x:v>
@@ -6596,7 +6596,7 @@
         <x:v>规划中</x:v>
       </x:c>
       <x:c r="K50" s="9" t="str">
-        <x:v>releases/v0.3.0-20261001T034652Z/02-breakdown.md:28</x:v>
+        <x:v>releases/v0.3.0-20261001T034652Z/02-breakdown.md:31</x:v>
       </x:c>
       <x:c r="L50" s="9" t="str">
         <x:v>未提供</x:v>
@@ -6638,7 +6638,7 @@
         <x:v>规划中</x:v>
       </x:c>
       <x:c r="K51" s="4" t="str">
-        <x:v>releases/v0.3.0-20261001T034652Z/02-breakdown.md:29</x:v>
+        <x:v>releases/v0.3.0-20261001T034652Z/02-breakdown.md:32</x:v>
       </x:c>
       <x:c r="L51" s="4" t="str">
         <x:v>未提供</x:v>
@@ -6680,7 +6680,7 @@
         <x:v>规划中</x:v>
       </x:c>
       <x:c r="K52" s="9" t="str">
-        <x:v>releases/v0.3.0-20261001T034652Z/02-breakdown.md:30</x:v>
+        <x:v>releases/v0.3.0-20261001T034652Z/02-breakdown.md:33</x:v>
       </x:c>
       <x:c r="L52" s="9" t="str">
         <x:v>未提供</x:v>
@@ -7245,123 +7245,130 @@
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="67" ht="32" customHeight="1">
+    <x:row r="67" ht="87" customHeight="1">
       <x:c r="A67" s="4" t="str">
-        <x:v>TASK-TM001-PLAN</x:v>
+        <x:v>TASK-TM003-SECRET</x:v>
       </x:c>
       <x:c r="B67" s="4" t="str">
-        <x:v>历史分组</x:v>
+        <x:v>具体任务</x:v>
       </x:c>
       <x:c r="C67" s="4" t="str">
+        <x:v>FP-TM003-02</x:v>
+      </x:c>
+      <x:c r="D67" s="4" t="str">
+        <x:v>REQ-TM003</x:v>
+      </x:c>
+      <x:c r="E67" s="4" t="str">
+        <x:v>AC-TM003-002
+AC-TM003-004</x:v>
+      </x:c>
+      <x:c r="F67" s="4" t="str">
+        <x:v>IDENTITY/STORE已定合同；可替换加密端口及本例私有profile，独立于真实Keychain产品验证</x:v>
+      </x:c>
+      <x:c r="G67" s="4" t="str">
+        <x:v>产物：TM-003独占私有32字节密钥生命周期、origin+account.id 的 usage-principal-v1 HMAC、0600密文、缺失/损坏/错键停采集；产品默认系统随机源与macOS系统密钥保护，无明文回退
+完成条件：固定公开向量、重启同键、不同主体隔离；既有库缺/坏密文零重键零改库，安全失败；只在owner根测试</x:v>
+      </x:c>
+      <x:c r="H67" s="4" t="str">
+        <x:v>IDENTITY/STORE已定合同；可替换加密端口及本例私有profile，独立于真实Keychain产品验证</x:v>
+      </x:c>
+      <x:c r="I67" s="4" t="str">
         <x:v>不适用</x:v>
       </x:c>
-      <x:c r="D67" s="4" t="str">
-        <x:v>REQ-TM001</x:v>
-      </x:c>
-      <x:c r="E67" s="4" t="str">
-        <x:v>不适用</x:v>
-      </x:c>
-      <x:c r="F67" s="4" t="str">
-        <x:v>不适用</x:v>
-      </x:c>
-      <x:c r="G67" s="4" t="str">
-        <x:v>六文档、完整追踪、SOP 修正、基线通过</x:v>
-      </x:c>
-      <x:c r="H67" s="4" t="str">
-        <x:v>需求</x:v>
-      </x:c>
-      <x:c r="I67" s="4" t="str">
-        <x:v>TEST-TM001-GOVERNANCE</x:v>
-      </x:c>
       <x:c r="J67" s="4" t="str">
-        <x:v>historical_group_not_minimal_task</x:v>
+        <x:v>规划中</x:v>
       </x:c>
       <x:c r="K67" s="4" t="str">
-        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:9</x:v>
+        <x:v>releases/v0.3.0-20261001T034652Z/02-breakdown.md:26</x:v>
       </x:c>
       <x:c r="L67" s="4" t="str">
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="68" ht="42" customHeight="1">
+    <x:row r="68" ht="72" customHeight="1">
       <x:c r="A68" s="9" t="str">
-        <x:v>TASK-TM001-SERVER</x:v>
+        <x:v>TASK-TM003-WIRING</x:v>
       </x:c>
       <x:c r="B68" s="9" t="str">
-        <x:v>历史分组</x:v>
+        <x:v>具体任务</x:v>
       </x:c>
       <x:c r="C68" s="9" t="str">
+        <x:v>FP-TM003-02</x:v>
+      </x:c>
+      <x:c r="D68" s="9" t="str">
+        <x:v>REQ-TM003</x:v>
+      </x:c>
+      <x:c r="E68" s="9" t="str">
+        <x:v>AC-TM003-001
+AC-TM003-003
+AC-TM003-004</x:v>
+      </x:c>
+      <x:c r="F68" s="9" t="str">
+        <x:v>CORE-07主进程编排、SECRET、TM-002现有SourceAccess可替换端口；真实OS选择/Keychain产品验收仍BLOCKED</x:v>
+      </x:c>
+      <x:c r="G68" s="9" t="str">
+        <x:v>产物：TM-003独占主进程来源到Codex collector/UsageStore适配；renderer只传已确认sourceId，完整代际守卫后写库
+完成条件：真实SourceAccess类+本例helper/SQLite下确认前零读、A/B=330、撤销零新提交、换主体无串读</x:v>
+      </x:c>
+      <x:c r="H68" s="9" t="str">
+        <x:v>CORE-07主进程编排、SECRET、TM-002现有SourceAccess可替换端口；真实OS选择/Keychain产品验收仍BLOCKED</x:v>
+      </x:c>
+      <x:c r="I68" s="9" t="str">
         <x:v>不适用</x:v>
       </x:c>
-      <x:c r="D68" s="9" t="str">
-        <x:v>REQ-TM001</x:v>
-      </x:c>
-      <x:c r="E68" s="9" t="str">
-        <x:v>不适用</x:v>
-      </x:c>
-      <x:c r="F68" s="9" t="str">
-        <x:v>不适用</x:v>
-      </x:c>
-      <x:c r="G68" s="9" t="str">
-        <x:v>FastAPI/SQLAlchemy/Alembic 工程、真实认证/权限/审计 API；随机可撤销 token 固定30天到期、不滑动，改密/重置/停用撤销旧会话</x:v>
-      </x:c>
-      <x:c r="H68" s="9" t="str">
-        <x:v>计划、数据/测试</x:v>
-      </x:c>
-      <x:c r="I68" s="9" t="str">
-        <x:v>E2E-TM001-001、E2E-TM001-002、E2E-TM001-003</x:v>
-      </x:c>
       <x:c r="J68" s="9" t="str">
-        <x:v>historical_group_not_minimal_task</x:v>
+        <x:v>规划中</x:v>
       </x:c>
       <x:c r="K68" s="9" t="str">
-        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:10</x:v>
+        <x:v>releases/v0.3.0-20261001T034652Z/02-breakdown.md:27</x:v>
       </x:c>
       <x:c r="L68" s="9" t="str">
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="69" ht="42" customHeight="1">
+    <x:row r="69" ht="87" customHeight="1">
       <x:c r="A69" s="4" t="str">
-        <x:v>TASK-TM001-DATA</x:v>
+        <x:v>TASK-TM003-IPC</x:v>
       </x:c>
       <x:c r="B69" s="4" t="str">
-        <x:v>历史分组</x:v>
+        <x:v>具体任务</x:v>
       </x:c>
       <x:c r="C69" s="4" t="str">
+        <x:v>FP-TM003-03</x:v>
+      </x:c>
+      <x:c r="D69" s="4" t="str">
+        <x:v>REQ-TM003</x:v>
+      </x:c>
+      <x:c r="E69" s="4" t="str">
+        <x:v>AC-TM003-001
+AC-TM003-004</x:v>
+      </x:c>
+      <x:c r="F69" s="4" t="str">
+        <x:v>WIRING及TM-001现有单窗口sender检查；不依赖真实Keychain产品结论</x:v>
+      </x:c>
+      <x:c r="G69" s="4" t="str">
+        <x:v>产物：TM-003独占 index.ts、受限collection handler、preload/共享Snapshot的采集状态；collection:getState无参数、collection:refresh仅sourceId
+完成条件：非主sender/子frame/额外路径或身份字段拒绝；有效刷新/重复/停读/换主体只返回本主体白名单状态</x:v>
+      </x:c>
+      <x:c r="H69" s="4" t="str">
+        <x:v>WIRING及TM-001现有单窗口sender检查；不依赖真实Keychain产品结论</x:v>
+      </x:c>
+      <x:c r="I69" s="4" t="str">
         <x:v>不适用</x:v>
       </x:c>
-      <x:c r="D69" s="4" t="str">
-        <x:v>REQ-TM001</x:v>
-      </x:c>
-      <x:c r="E69" s="4" t="str">
-        <x:v>不适用</x:v>
-      </x:c>
-      <x:c r="F69" s="4" t="str">
-        <x:v>不适用</x:v>
-      </x:c>
-      <x:c r="G69" s="4" t="str">
-        <x:v>独立测试/生产 SQLite 文件、可执行造数 SQL、生产首建管理员、回归账号/独立预期及安全重置；已有生产密码不可被重建覆盖</x:v>
-      </x:c>
-      <x:c r="H69" s="4" t="str">
-        <x:v>计划、工程骨架</x:v>
-      </x:c>
-      <x:c r="I69" s="4" t="str">
-        <x:v>TEST-TM001-SERVER、E2E-TM001-001、E2E-TM001-005</x:v>
-      </x:c>
       <x:c r="J69" s="4" t="str">
-        <x:v>historical_group_not_minimal_task</x:v>
+        <x:v>规划中</x:v>
       </x:c>
       <x:c r="K69" s="4" t="str">
-        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:11</x:v>
+        <x:v>releases/v0.3.0-20261001T034652Z/02-breakdown.md:28</x:v>
       </x:c>
       <x:c r="L69" s="4" t="str">
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="70" ht="72" customHeight="1">
+    <x:row r="70" ht="32" customHeight="1">
       <x:c r="A70" s="9" t="str">
-        <x:v>TASK-TM001-MAC</x:v>
+        <x:v>TASK-TM001-PLAN</x:v>
       </x:c>
       <x:c r="B70" s="9" t="str">
         <x:v>历史分组</x:v>
@@ -7379,27 +7386,27 @@
         <x:v>不适用</x:v>
       </x:c>
       <x:c r="G70" s="9" t="str">
-        <x:v>Electron React/TypeScript 登录/改密/主页/管理、默认本机 API/更新源地址与配置管理页的用户覆盖持久化；默认开启可关闭的设备自动登录、按规范化 origin 隔离的受保护凭据文件与内存会话、稳定 UI 标识、Playwright Electron工程</x:v>
+        <x:v>六文档、完整追踪、SOP 修正、基线通过</x:v>
       </x:c>
       <x:c r="H70" s="9" t="str">
-        <x:v>API 合同、工程骨架</x:v>
+        <x:v>需求</x:v>
       </x:c>
       <x:c r="I70" s="9" t="str">
-        <x:v>E2E-TM001-001、E2E-TM001-002、E2E-TM001-003、E2E-TM001-004、E2E-TM001-005、E2E-TM001-006</x:v>
+        <x:v>TEST-TM001-GOVERNANCE</x:v>
       </x:c>
       <x:c r="J70" s="9" t="str">
         <x:v>historical_group_not_minimal_task</x:v>
       </x:c>
       <x:c r="K70" s="9" t="str">
-        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:12</x:v>
+        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:9</x:v>
       </x:c>
       <x:c r="L70" s="9" t="str">
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="71" ht="57" customHeight="1">
+    <x:row r="71" ht="42" customHeight="1">
       <x:c r="A71" s="4" t="str">
-        <x:v>TASK-TM001-UPDATE</x:v>
+        <x:v>TASK-TM001-SERVER</x:v>
       </x:c>
       <x:c r="B71" s="4" t="str">
         <x:v>历史分组</x:v>
@@ -7417,27 +7424,27 @@
         <x:v>不适用</x:v>
       </x:c>
       <x:c r="G71" s="4" t="str">
-        <x:v>固定 Ed25519 公钥、同机回环更新源/签名测试包/失败包及真实更新用例；默认49177配置、URL安全校验与升级时锁定更新设置；两构建沿用经校验的同一隔离profile，升级后服务验证自动登录</x:v>
+        <x:v>FastAPI/SQLAlchemy/Alembic 工程、真实认证/权限/审计 API；随机可撤销 token 固定30天到期、不滑动，改密/重置/停用撤销旧会话</x:v>
       </x:c>
       <x:c r="H71" s="4" t="str">
-        <x:v>Mac 工程</x:v>
+        <x:v>计划、数据/测试</x:v>
       </x:c>
       <x:c r="I71" s="4" t="str">
-        <x:v>E2E-TM001-004</x:v>
+        <x:v>E2E-TM001-001、E2E-TM001-002、E2E-TM001-003</x:v>
       </x:c>
       <x:c r="J71" s="4" t="str">
         <x:v>historical_group_not_minimal_task</x:v>
       </x:c>
       <x:c r="K71" s="4" t="str">
-        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:13</x:v>
+        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:10</x:v>
       </x:c>
       <x:c r="L71" s="4" t="str">
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="72" ht="57" customHeight="1">
+    <x:row r="72" ht="42" customHeight="1">
       <x:c r="A72" s="9" t="str">
-        <x:v>TASK-TM001-RUNNER</x:v>
+        <x:v>TASK-TM001-DATA</x:v>
       </x:c>
       <x:c r="B72" s="9" t="str">
         <x:v>历史分组</x:v>
@@ -7455,27 +7462,27 @@
         <x:v>不适用</x:v>
       </x:c>
       <x:c r="G72" s="9" t="str">
-        <x:v>本机Playwright从最终DMG安装App执行全部六例，原始JSON/trace/fixtureSQL/包摘要、父门禁复核；默认值与动态独占端口隔离测试；真实Squirrel自重启及profile、身份恢复</x:v>
+        <x:v>独立测试/生产 SQLite 文件、可执行造数 SQL、生产首建管理员、回归账号/独立预期及安全重置；已有生产密码不可被重建覆盖</x:v>
       </x:c>
       <x:c r="H72" s="9" t="str">
-        <x:v>数据/桌面工程</x:v>
+        <x:v>计划、工程骨架</x:v>
       </x:c>
       <x:c r="I72" s="9" t="str">
-        <x:v>E2E-TM001-001、E2E-TM001-002、E2E-TM001-003、E2E-TM001-004、E2E-TM001-005、E2E-TM001-006</x:v>
+        <x:v>TEST-TM001-SERVER、E2E-TM001-001、E2E-TM001-005</x:v>
       </x:c>
       <x:c r="J72" s="9" t="str">
         <x:v>historical_group_not_minimal_task</x:v>
       </x:c>
       <x:c r="K72" s="9" t="str">
-        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:14</x:v>
+        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:11</x:v>
       </x:c>
       <x:c r="L72" s="9" t="str">
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
-    <x:row r="73" ht="32" customHeight="1">
+    <x:row r="73" ht="72" customHeight="1">
       <x:c r="A73" s="4" t="str">
-        <x:v>TASK-TM001-REVIEW</x:v>
+        <x:v>TASK-TM001-MAC</x:v>
       </x:c>
       <x:c r="B73" s="4" t="str">
         <x:v>历史分组</x:v>
@@ -7493,33 +7500,147 @@
         <x:v>不适用</x:v>
       </x:c>
       <x:c r="G73" s="4" t="str">
-        <x:v>完整回归、流程复盘、PR 与合并判定、发布阻塞记录</x:v>
+        <x:v>Electron React/TypeScript 登录/改密/主页/管理、默认本机 API/更新源地址与配置管理页的用户覆盖持久化；默认开启可关闭的设备自动登录、按规范化 origin 隔离的受保护凭据文件与内存会话、稳定 UI 标识、Playwright Electron工程</x:v>
       </x:c>
       <x:c r="H73" s="4" t="str">
-        <x:v>全部实现任务</x:v>
+        <x:v>API 合同、工程骨架</x:v>
       </x:c>
       <x:c r="I73" s="4" t="str">
-        <x:v>TEST-TM001-GOVERNANCE</x:v>
+        <x:v>E2E-TM001-001、E2E-TM001-002、E2E-TM001-003、E2E-TM001-004、E2E-TM001-005、E2E-TM001-006</x:v>
       </x:c>
       <x:c r="J73" s="4" t="str">
         <x:v>historical_group_not_minimal_task</x:v>
       </x:c>
       <x:c r="K73" s="4" t="str">
-        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:15</x:v>
+        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:12</x:v>
       </x:c>
       <x:c r="L73" s="4" t="str">
         <x:v>未提供</x:v>
       </x:c>
     </x:row>
+    <x:row r="74" ht="57" customHeight="1">
+      <x:c r="A74" s="9" t="str">
+        <x:v>TASK-TM001-UPDATE</x:v>
+      </x:c>
+      <x:c r="B74" s="9" t="str">
+        <x:v>历史分组</x:v>
+      </x:c>
+      <x:c r="C74" s="9" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="D74" s="9" t="str">
+        <x:v>REQ-TM001</x:v>
+      </x:c>
+      <x:c r="E74" s="9" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="F74" s="9" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="G74" s="9" t="str">
+        <x:v>固定 Ed25519 公钥、同机回环更新源/签名测试包/失败包及真实更新用例；默认49177配置、URL安全校验与升级时锁定更新设置；两构建沿用经校验的同一隔离profile，升级后服务验证自动登录</x:v>
+      </x:c>
+      <x:c r="H74" s="9" t="str">
+        <x:v>Mac 工程</x:v>
+      </x:c>
+      <x:c r="I74" s="9" t="str">
+        <x:v>E2E-TM001-004</x:v>
+      </x:c>
+      <x:c r="J74" s="9" t="str">
+        <x:v>historical_group_not_minimal_task</x:v>
+      </x:c>
+      <x:c r="K74" s="9" t="str">
+        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:13</x:v>
+      </x:c>
+      <x:c r="L74" s="9" t="str">
+        <x:v>未提供</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="57" customHeight="1">
+      <x:c r="A75" s="4" t="str">
+        <x:v>TASK-TM001-RUNNER</x:v>
+      </x:c>
+      <x:c r="B75" s="4" t="str">
+        <x:v>历史分组</x:v>
+      </x:c>
+      <x:c r="C75" s="4" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="D75" s="4" t="str">
+        <x:v>REQ-TM001</x:v>
+      </x:c>
+      <x:c r="E75" s="4" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="F75" s="4" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="G75" s="4" t="str">
+        <x:v>本机Playwright从最终DMG安装App执行全部六例，原始JSON/trace/fixtureSQL/包摘要、父门禁复核；默认值与动态独占端口隔离测试；真实Squirrel自重启及profile、身份恢复</x:v>
+      </x:c>
+      <x:c r="H75" s="4" t="str">
+        <x:v>数据/桌面工程</x:v>
+      </x:c>
+      <x:c r="I75" s="4" t="str">
+        <x:v>E2E-TM001-001、E2E-TM001-002、E2E-TM001-003、E2E-TM001-004、E2E-TM001-005、E2E-TM001-006</x:v>
+      </x:c>
+      <x:c r="J75" s="4" t="str">
+        <x:v>historical_group_not_minimal_task</x:v>
+      </x:c>
+      <x:c r="K75" s="4" t="str">
+        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:14</x:v>
+      </x:c>
+      <x:c r="L75" s="4" t="str">
+        <x:v>未提供</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="32" customHeight="1">
+      <x:c r="A76" s="9" t="str">
+        <x:v>TASK-TM001-REVIEW</x:v>
+      </x:c>
+      <x:c r="B76" s="9" t="str">
+        <x:v>历史分组</x:v>
+      </x:c>
+      <x:c r="C76" s="9" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="D76" s="9" t="str">
+        <x:v>REQ-TM001</x:v>
+      </x:c>
+      <x:c r="E76" s="9" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="F76" s="9" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="G76" s="9" t="str">
+        <x:v>完整回归、流程复盘、PR 与合并判定、发布阻塞记录</x:v>
+      </x:c>
+      <x:c r="H76" s="9" t="str">
+        <x:v>全部实现任务</x:v>
+      </x:c>
+      <x:c r="I76" s="9" t="str">
+        <x:v>TEST-TM001-GOVERNANCE</x:v>
+      </x:c>
+      <x:c r="J76" s="9" t="str">
+        <x:v>historical_group_not_minimal_task</x:v>
+      </x:c>
+      <x:c r="K76" s="9" t="str">
+        <x:v>releases/v0.1.0-20260929T074814Z/02-breakdown.md:15</x:v>
+      </x:c>
+      <x:c r="L76" s="9" t="str">
+        <x:v>未提供</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="J5:J73">
+  <x:conditionalFormatting sqref="J5:J76">
     <x:cfRule type="containsText" dxfId="9" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="10" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="11" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25043e0a708f4375"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R982c2708ca2b4bbe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18586,7 +18707,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L236" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:267</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:312</x:v>
       </x:c>
       <x:c r="M236" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18633,7 +18754,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L237" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:271</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:316</x:v>
       </x:c>
       <x:c r="M237" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18680,7 +18801,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L238" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:275</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:320</x:v>
       </x:c>
       <x:c r="M238" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18728,7 +18849,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L239" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:279</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:324</x:v>
       </x:c>
       <x:c r="M239" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18778,7 +18899,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L240" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:283</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:328</x:v>
       </x:c>
       <x:c r="M240" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18826,7 +18947,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L241" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:287</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:332</x:v>
       </x:c>
       <x:c r="M241" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18873,7 +18994,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L242" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:291</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:336</x:v>
       </x:c>
       <x:c r="M242" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -18920,7 +19041,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L243" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:295</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:340</x:v>
       </x:c>
       <x:c r="M243" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -18968,7 +19089,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L244" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:299</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:344</x:v>
       </x:c>
       <x:c r="M244" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19017,7 +19138,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L245" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:303</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:348</x:v>
       </x:c>
       <x:c r="M245" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19066,7 +19187,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L246" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:307</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:352</x:v>
       </x:c>
       <x:c r="M246" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19115,7 +19236,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L247" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:311</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:356</x:v>
       </x:c>
       <x:c r="M247" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19162,7 +19283,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L248" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:315</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:360</x:v>
       </x:c>
       <x:c r="M248" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19210,7 +19331,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L249" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:319</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:364</x:v>
       </x:c>
       <x:c r="M249" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19258,7 +19379,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L250" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:323</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:368</x:v>
       </x:c>
       <x:c r="M250" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19306,7 +19427,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L251" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:327</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:372</x:v>
       </x:c>
       <x:c r="M251" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19354,7 +19475,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L252" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:331</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:376</x:v>
       </x:c>
       <x:c r="M252" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19404,7 +19525,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L253" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:335</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:380</x:v>
       </x:c>
       <x:c r="M253" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19451,7 +19572,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L254" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:339</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:384</x:v>
       </x:c>
       <x:c r="M254" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19498,7 +19619,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L255" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:343</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:388</x:v>
       </x:c>
       <x:c r="M255" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19546,7 +19667,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L256" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:347</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:392</x:v>
       </x:c>
       <x:c r="M256" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19595,7 +19716,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L257" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:351</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:396</x:v>
       </x:c>
       <x:c r="M257" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19645,7 +19766,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L258" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:355</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:400</x:v>
       </x:c>
       <x:c r="M258" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19693,7 +19814,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L259" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:359</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:404</x:v>
       </x:c>
       <x:c r="M259" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19742,7 +19863,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L260" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:363</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:408</x:v>
       </x:c>
       <x:c r="M260" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19790,7 +19911,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L261" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:367</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:412</x:v>
       </x:c>
       <x:c r="M261" s="4" t="str">
         <x:v>尚未执行</x:v>
@@ -19838,7 +19959,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L262" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:371</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:416</x:v>
       </x:c>
       <x:c r="M262" s="9" t="str">
         <x:v>尚未执行</x:v>
@@ -19886,7 +20007,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L263" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:375</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:420</x:v>
       </x:c>
       <x:c r="M263" s="4" t="str">
         <x:v>tm003-core-20261001T203711Z</x:v>
@@ -19935,7 +20056,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L264" s="9" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:379</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:424</x:v>
       </x:c>
       <x:c r="M264" s="9" t="str">
         <x:v>tm003-core-20261001T203711Z</x:v>
@@ -19983,7 +20104,7 @@
         <x:v>细化用例</x:v>
       </x:c>
       <x:c r="L265" s="4" t="str">
-        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:383</x:v>
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:428</x:v>
       </x:c>
       <x:c r="M265" s="4" t="str">
         <x:v>tm003-core-20261001T203711Z</x:v>
@@ -20681,30 +20802,177 @@
         <x:v>v0.5.0-20261001T034729Z</x:v>
       </x:c>
     </x:row>
+    <x:row r="280" ht="177" customHeight="1">
+      <x:c r="A280" s="9" t="str">
+        <x:v>TM-003</x:v>
+      </x:c>
+      <x:c r="B280" s="9" t="str">
+        <x:v>TC-TM003-CORE-08</x:v>
+      </x:c>
+      <x:c r="C280" s="9" t="str">
+        <x:v>私有身份密钥持久性与拒绝重键</x:v>
+      </x:c>
+      <x:c r="D280" s="9" t="str">
+        <x:v>TASK-TM003-SECRET</x:v>
+      </x:c>
+      <x:c r="E280" s="9" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F280" s="9" t="str">
+        <x:v>tests/fixtures/tm003-product-loop-slice.json；0700私有profile/0600库，公开32字节注入随机源，假系统密钥端口与三组principal向量；真实产品必须系统随机+系统密钥加密</x:v>
+      </x:c>
+      <x:c r="G280" s="9" t="str">
+        <x:v>1. 在空 owner profile 中以可用加密端口初始化密钥，求三组 principal 键。；随机源仅调用一次、32字节密钥仅在内存；密文记录0600/目录0700，无明文 key。三键逐字节等于 fixture；同账号不同 origin 和同 origin 不同账号各有不同键。尚无事件/游标/覆盖写入。
+2. 用第一主体经正式 UsageStore 提交 fixture A=110，关闭密钥端口与库，再用同 profile 重开并重放 A。；重开只解密原密文、不生成新密钥；第一 principal 键和 identity_key_state 标记不变；usage_event 始终一行、total110、游标不重计，第二/第三主体只读零行但状态为未核实而非产品已知零。
+3. 分别在独立复制的本例已有事件库中删除密文记录和损坏密文，再初始化。；两者均返回固定 identity_secret_unavailable/identity_secret_corrupt 停采集，随机源零调用，不创建新密文、不改事件、游标、覆盖或密钥标记；旧 A 仍可由只读库核对。
+4. 恢复原密文后让加密端口不可用，再换成另一有效32字节密钥尝试打开原库。；密钥不可用时停采集，不能明文回退；不同有效密钥被 marker 拒绝，A仍一行/110，记录和报告无密钥、密文、完整路径或原生日志正文。</x:v>
+      </x:c>
+      <x:c r="H280" s="9" t="str">
+        <x:v>准备：仅经UsageStore提交A；故障变体各复制owner库
+变化：重启重放及缺/坏/错键不改旧事件、游标或密钥标记
+核验：只读usage_event/source_cursor/coverage/identity_key_state；检查密文文件0600、无明文key</x:v>
+      </x:c>
+      <x:c r="I280" s="9" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J280" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K280" s="9" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L280" s="9" t="str">
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:263</x:v>
+      </x:c>
+      <x:c r="M280" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N280" s="9" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="281" ht="192" customHeight="1">
+      <x:c r="A281" s="4" t="str">
+        <x:v>TM-003</x:v>
+      </x:c>
+      <x:c r="B281" s="4" t="str">
+        <x:v>TC-TM003-CORE-09</x:v>
+      </x:c>
+      <x:c r="C281" s="4" t="str">
+        <x:v>已确认来源到本机库的主进程适配</x:v>
+      </x:c>
+      <x:c r="D281" s="4" t="str">
+        <x:v>TASK-TM003-WIRING</x:v>
+      </x:c>
+      <x:c r="E281" s="4" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F281" s="4" t="str">
+        <x:v>tests/fixtures/tm003-product-loop-slice.json；CORE08密钥、真实SourceAccess类/合成helper与CORE07两文件各410字节</x:v>
+      </x:c>
+      <x:c r="G281" s="4" t="str">
+        <x:v>1. 未经确认直接触发 Codex 采集，再通过 SourceAccess 的选择/预览/确认方法建立本例来源。；确认前 beginCandidateScan/readCandidateChunk/commitScanBatch 均0次、库空；确认记录只属第一主体，候选元数据不包含正文。
+2. 以已确认 sourceId 调用主进程适配器，读取两个完整文件并在末页守卫通过后落库；关闭重开库/来源后重扫。；完成前库空；完成后A/B两事件、input300/output30/cached60/total330、各游标410、覆盖仅在全代完成后标记；重启重扫仍两行/330，无原始路径/原生ID落库。
+3. 从独立成功库开始新代际，在 file-b 后由 SourceAccess 撤销来源再尝试提交。；旧代际被取消，守卫拒绝、提交0次；已提交A/B仍两行/330，原成功代际的coverage行保持原值，本次运行状态须标采集不可用/不完整且不能称新代际完成；旧 sourceId 不再可读。
+4. 切到 fixture 的第二主体后尝试旧 sourceId，再为第二主体确认独立来源并扫描。；旧 sourceId 在读取前拒绝、第一主体数据不出现在第二主体查询；第二主体成功扫描后各主体各两行/330，HMAC主体键不同，不能共享游标/来源能力。</x:v>
+      </x:c>
+      <x:c r="H281" s="4" t="str">
+        <x:v>准备：经正式SourceAccess和UsageStore操作；各故障路径新库
+变化：完整代际写A/B=330；撤销/换主体不增加旧主体事件
+核验：只读主体/来源唯一键、事件总量、游标、覆盖及提交次数</x:v>
+      </x:c>
+      <x:c r="I281" s="4" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J281" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K281" s="4" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L281" s="4" t="str">
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:276</x:v>
+      </x:c>
+      <x:c r="M281" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N281" s="4" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="282" ht="147" customHeight="1">
+      <x:c r="A282" s="9" t="str">
+        <x:v>TM-003</x:v>
+      </x:c>
+      <x:c r="B282" s="9" t="str">
+        <x:v>TC-TM003-CORE-10</x:v>
+      </x:c>
+      <x:c r="C282" s="9" t="str">
+        <x:v>主窗口 IPC 与刷新状态隔离</x:v>
+      </x:c>
+      <x:c r="D282" s="9" t="str">
+        <x:v>TASK-TM003-IPC</x:v>
+      </x:c>
+      <x:c r="E282" s="9" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F282" s="9" t="str">
+        <x:v>tests/fixtures/tm003-product-loop-slice.json；CORE09成功库、固定主窗口sender/frame端口及第二主体</x:v>
+      </x:c>
+      <x:c r="G282" s="9" t="str">
+        <x:v>1. 分别用非主窗口 sender、子 frame、路径/账号/密钥多余字段和未确认 sourceId 调用 handler。；全部拒绝，采集/DB调用0次；不接受任意路径或由 renderer 指定 principal/secret，不返回旧主体状态。
+2. 主窗口按固定 sourceId 刷新并取 state。；只触发第一主体 Codex 采集一次，返回两事件的 input300/output30/total330、cached已知60、覆盖与诊断代码/数量；库仍两行，序列化状态无密钥、密文、路径、原生ID或正文。
+3. 同主体再刷新并取 state，随后将来源暂停/撤销。；重扫仍两行/330；暂停/撤销后刷新拒绝、旧可信330只对第一主体保留可见且标采集不可用/覆盖不完整，不能报新已知零。
+4. 切换第二主体后由旧 sender/sourceId 取 state/刷新。；旧来源被拒绝，第二主体 state 为缺失/未核实且无第一主体330；第一主体持久事件不删除，按主体只读核对隔离。</x:v>
+      </x:c>
+      <x:c r="H282" s="9" t="str">
+        <x:v>准备：本例owner库只经handler/collector操作
+变化：合法刷新不重复；非法sender/输入/换主体零新写
+核验：只读usage_event/coverage与输出白名单、handler调用数</x:v>
+      </x:c>
+      <x:c r="I282" s="9" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J282" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K282" s="9" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L282" s="9" t="str">
+        <x:v>docs/testing/cases/03-TM-003-codex-collection.md:289</x:v>
+      </x:c>
+      <x:c r="M282" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N282" s="9" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G5:G279">
+  <x:conditionalFormatting sqref="G5:G282">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="I5:I279">
+  <x:conditionalFormatting sqref="I5:I282">
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="16" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="17" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="J5:J279">
+  <x:conditionalFormatting sqref="J5:J282">
     <x:cfRule type="containsText" dxfId="18" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="19" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="20" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M279">
+  <x:conditionalFormatting sqref="M5:M282">
     <x:cfRule type="containsText" dxfId="21" priority="10" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="22" priority="11" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="23" priority="12" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3eb9cbcd99cc45a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R661ea45b277542f6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22336,7 +22604,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b08fedd6fef434d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a44701823754209"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22828,7 +23096,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0706c88ee02424c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99c4afc143c44994"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23993,7 +24261,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fa1ec01202f4d85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R743c0e31b0624da0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.1.0-20260929T074814Z][TM-001] Index 709d bootstrap targeted run
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R3cb0d6bcdf5b4d60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rc165cd0df46944a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rdd922679d5dc4e6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R200b34690b774c08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R803defdb9bef407a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rcc23deb0274f41c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R14ea53fc1d944102"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R79ce0cdc2a9b4f2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rc84140b5b6f04fdb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R573be4995ee74c91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R61bd3827d3904eb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Re582a623448b4c2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R725aeafdf035426b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rdd8f5ee6505943d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R2bd640a59e9442de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R1d386a79530f40f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R3bae464479c54fff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R67ff4269af2f4ebd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R12deb8759fcb48c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R81c00dc18e6a4950"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R40b4fc7871cf4cf7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Rf143a7c129c94948"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -809,8 +809,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N39" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N39"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N40" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N40"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="运行批次"/>
     <x:tableColumn id="2" name="版本"/>
@@ -1146,8 +1146,8 @@
         <x:v>测试批次</x:v>
       </x:c>
       <x:c r="B9" s="10" t="n">
-        <x:f>COUNTA('06测试批次'!A5:A39)</x:f>
-        <x:v>35</x:v>
+        <x:f>COUNTA('06测试批次'!A5:A40)</x:f>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>06测试批次，每次运行一行，记录独立结果Excel位置</x:v>
@@ -1271,7 +1271,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>source_check · TM-003 tm003-core07整合候选固定辅助模块；非产品E2E：1/1固定TC、5步与owner清理PASS；固定source_check导出及verification回读PASS。仅本整合候选的模块合同，产品App/授权/Keychain及发行均NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
+        <x:v>product_e2e · TASK-TM001-BOOTSTRAP；BOOTSTRAP-01..04四父TC安装正式App定向：4父4/4、18步、清理PASS；12截图、独立Excel/verification回读PASS。仅709d首次建库/安装App定向，未做本批独立审计；其余TM001、完整门禁与发行未通过。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78890397488e4ca9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b2b58b21d51413d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59713f1f5768440e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc68078ec838b4b39"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64341a0fc6234bb4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8675b0726f440ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e47d71ac7c345b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b5b7dc9f1da48e5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd30a4ebacc7468f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18906c0dc8794e7b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0db642e62fc64cc4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbffd9f49b54c4a0f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7640,7 +7640,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R982c2708ca2b4bbe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b7d5ea1d8cf4cc7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10100,7 +10100,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:363</x:v>
       </x:c>
       <x:c r="M54" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-3d36f9cbe62a4c1e889e8ea2fa476281</x:v>
       </x:c>
       <x:c r="N54" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -10150,7 +10150,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:380</x:v>
       </x:c>
       <x:c r="M55" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-3d36f9cbe62a4c1e889e8ea2fa476281</x:v>
       </x:c>
       <x:c r="N55" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -10199,7 +10199,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:398</x:v>
       </x:c>
       <x:c r="M56" s="9" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-3d36f9cbe62a4c1e889e8ea2fa476281</x:v>
       </x:c>
       <x:c r="N56" s="9" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -10249,7 +10249,7 @@
         <x:v>docs/testing/cases/01b-TM-001-session-admin-release-scenarios.md:415</x:v>
       </x:c>
       <x:c r="M57" s="4" t="str">
-        <x:v>local-0512d4fc44544eba97f9d1ae79cbfc37</x:v>
+        <x:v>local-3d36f9cbe62a4c1e889e8ea2fa476281</x:v>
       </x:c>
       <x:c r="N57" s="4" t="str">
         <x:v>v0.1.0-20260929T074814Z</x:v>
@@ -20972,7 +20972,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R661ea45b277542f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cef30b7ec90422b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22586,25 +22586,69 @@
         <x:v>NOT_RUN</x:v>
       </x:c>
     </x:row>
+    <x:row r="40" ht="42" customHeight="1">
+      <x:c r="A40" s="9" t="str">
+        <x:v>local-3d36f9cbe62a4c1e889e8ea2fa476281</x:v>
+      </x:c>
+      <x:c r="B40" s="9" t="str">
+        <x:v>v0.1.0-20260929T074814Z</x:v>
+      </x:c>
+      <x:c r="C40" s="9" t="str">
+        <x:v>product_e2e</x:v>
+      </x:c>
+      <x:c r="D40" s="9" t="str">
+        <x:v>TASK-TM001-BOOTSTRAP；BOOTSTRAP-01..04四父TC安装正式App定向</x:v>
+      </x:c>
+      <x:c r="E40" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F40" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G40" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H40" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I40" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J40" s="9" t="str">
+        <x:v>709d21253a0f88bc703a431cbf3adba3df17e508</x:v>
+      </x:c>
+      <x:c r="K40" s="9" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L40" s="9" t="str">
+        <x:v>4父4/4、18步、清理PASS；12截图、独立Excel/verification回读PASS。仅709d首次建库/安装App定向，未做本批独立审计；其余TM001、完整门禁与发行未通过。</x:v>
+      </x:c>
+      <x:c r="M40" s="9" t="str">
+        <x:v>.local/test-results/local-3d36f9cbe62a4c1e889e8ea2fa476281/TokenMeter测试结果-local-3d36f9cbe62a4c1e889e8ea2fa476281.xlsx</x:v>
+      </x:c>
+      <x:c r="N40" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E5:E39">
+  <x:conditionalFormatting sqref="E5:E40">
     <x:cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="26" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M39">
+  <x:conditionalFormatting sqref="M5:M40">
     <x:cfRule type="containsText" dxfId="27" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="29" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="N5:N39">
+  <x:conditionalFormatting sqref="N5:N40">
     <x:cfRule type="containsText" dxfId="30" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="32" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a44701823754209"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea61f4ea009d4c73"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23096,7 +23140,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99c4afc143c44994"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb32f3e554b5241a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24261,7 +24305,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R743c0e31b0624da0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcea83dea6bf84594"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.4.0-20261001T040433Z][TM-004] Index integrated CORE01-05 source checks
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Re582a623448b4c2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R725aeafdf035426b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rdd8f5ee6505943d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R2bd640a59e9442de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R1d386a79530f40f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R3bae464479c54fff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R67ff4269af2f4ebd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R12deb8759fcb48c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R81c00dc18e6a4950"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R40b4fc7871cf4cf7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Rf143a7c129c94948"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Ra4f8d98df41041e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rbb8e251916d04868"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rc5f805f200d242d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rf4d8d5c4fe134d49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R6991c6c045a445d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R55615561eeb249bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R240979b2f1af4851"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R82efc12112f34203"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rbc131f664828428b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R1787dfe246cb409a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R3fd87e0127824051"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -809,8 +809,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N40" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N40"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N43" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N43"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="运行批次"/>
     <x:tableColumn id="2" name="版本"/>
@@ -1146,8 +1146,8 @@
         <x:v>测试批次</x:v>
       </x:c>
       <x:c r="B9" s="10" t="n">
-        <x:f>COUNTA('06测试批次'!A5:A40)</x:f>
-        <x:v>36</x:v>
+        <x:f>COUNTA('06测试批次'!A5:A43)</x:f>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>06测试批次，每次运行一行，记录独立结果Excel位置</x:v>
@@ -1271,7 +1271,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>product_e2e · TASK-TM001-BOOTSTRAP；BOOTSTRAP-01..04四父TC安装正式App定向：4父4/4、18步、清理PASS；12截图、独立Excel/verification回读PASS。仅709d首次建库/安装App定向，未做本批独立审计；其余TM001、完整门禁与发行未通过。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
+        <x:v>source_check · TM-004 CORE05三文件持久映射整合候选固定辅助模块；非产品E2E：1/1固定TC、4步与逐例清理PASS；固定source_check导出及verification回读PASS。仅同树辅助模块合同，原20产品TC、App/授权/服务及发行均NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b2b58b21d51413d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2829fb58b8e4e3b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc68078ec838b4b39"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a2cb8f825f94efe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8675b0726f440ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55e74f6419664647"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b5b7dc9f1da48e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e81fa3ce52243fe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18906c0dc8794e7b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc97a256db72846b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbffd9f49b54c4a0f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R123bd72d4ae64368"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7640,7 +7640,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b7d5ea1d8cf4cc7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cee48957f904f14"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20493,7 +20493,7 @@
         <x:v>draft</x:v>
       </x:c>
       <x:c r="J273" s="4" t="str">
-        <x:v>未执行</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="K273" s="4" t="str">
         <x:v>细化用例</x:v>
@@ -20502,7 +20502,7 @@
         <x:v>docs/testing/cases/04-TM-004-claude-collection.md:170</x:v>
       </x:c>
       <x:c r="M273" s="4" t="str">
-        <x:v>尚未执行</x:v>
+        <x:v>tm004-core-20261001T213019Z</x:v>
       </x:c>
       <x:c r="N273" s="4" t="str">
         <x:v>v0.4.0-20261001T040433Z</x:v>
@@ -20541,7 +20541,7 @@
         <x:v>draft</x:v>
       </x:c>
       <x:c r="J274" s="9" t="str">
-        <x:v>未执行</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="K274" s="9" t="str">
         <x:v>细化用例</x:v>
@@ -20550,7 +20550,7 @@
         <x:v>docs/testing/cases/04-TM-004-claude-collection.md:178</x:v>
       </x:c>
       <x:c r="M274" s="9" t="str">
-        <x:v>尚未执行</x:v>
+        <x:v>tm004-core-20261001T213019Z</x:v>
       </x:c>
       <x:c r="N274" s="9" t="str">
         <x:v>v0.4.0-20261001T040433Z</x:v>
@@ -20590,7 +20590,7 @@
         <x:v>draft</x:v>
       </x:c>
       <x:c r="J275" s="4" t="str">
-        <x:v>未执行</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="K275" s="4" t="str">
         <x:v>细化用例</x:v>
@@ -20599,7 +20599,7 @@
         <x:v>docs/testing/cases/04-TM-004-claude-collection.md:186</x:v>
       </x:c>
       <x:c r="M275" s="4" t="str">
-        <x:v>尚未执行</x:v>
+        <x:v>tm004-core-20261001T213019Z</x:v>
       </x:c>
       <x:c r="N275" s="4" t="str">
         <x:v>v0.4.0-20261001T040433Z</x:v>
@@ -20639,7 +20639,7 @@
         <x:v>draft</x:v>
       </x:c>
       <x:c r="J276" s="9" t="str">
-        <x:v>未执行</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="K276" s="9" t="str">
         <x:v>细化用例</x:v>
@@ -20648,7 +20648,7 @@
         <x:v>docs/testing/cases/04-TM-004-claude-collection.md:198</x:v>
       </x:c>
       <x:c r="M276" s="9" t="str">
-        <x:v>尚未执行</x:v>
+        <x:v>tm004-core04-20261001T213019Z</x:v>
       </x:c>
       <x:c r="N276" s="9" t="str">
         <x:v>v0.4.0-20261001T040433Z</x:v>
@@ -20689,7 +20689,7 @@
         <x:v>draft</x:v>
       </x:c>
       <x:c r="J277" s="4" t="str">
-        <x:v>未执行</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="K277" s="4" t="str">
         <x:v>细化用例</x:v>
@@ -20698,7 +20698,7 @@
         <x:v>docs/testing/cases/04-TM-004-claude-collection.md:206</x:v>
       </x:c>
       <x:c r="M277" s="4" t="str">
-        <x:v>尚未执行</x:v>
+        <x:v>tm004-core05-20261001T213019Z</x:v>
       </x:c>
       <x:c r="N277" s="4" t="str">
         <x:v>v0.4.0-20261001T040433Z</x:v>
@@ -20972,7 +20972,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cef30b7ec90422b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49a48a6b66b24ce7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22630,25 +22630,157 @@
         <x:v>PASS</x:v>
       </x:c>
     </x:row>
+    <x:row r="41" ht="42" customHeight="1">
+      <x:c r="A41" s="4" t="str">
+        <x:v>tm004-core-20261001T213019Z</x:v>
+      </x:c>
+      <x:c r="B41" s="4" t="str">
+        <x:v>v0.4.0-20261001T040433Z</x:v>
+      </x:c>
+      <x:c r="C41" s="4" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D41" s="4" t="str">
+        <x:v>TM-004 CORE01–03解析器整合候选固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E41" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F41" s="4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G41" s="4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H41" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I41" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J41" s="4" t="str">
+        <x:v>08463b31c5eef5e6c90978cb8d6cd79e4aa76e1a</x:v>
+      </x:c>
+      <x:c r="K41" s="4" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L41" s="4" t="str">
+        <x:v>3/3固定TC、9步与逐例清理PASS；固定source_check导出及verification回读PASS。仅同树辅助模块合同，原20产品TC、App/授权/服务及发行均NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M41" s="4" t="str">
+        <x:v>.local/test-results/tm004-core-20261001T213019Z/TokenMeter测试结果-tm004-core-20261001T213019Z.xlsx</x:v>
+      </x:c>
+      <x:c r="N41" s="4" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="42" customHeight="1">
+      <x:c r="A42" s="9" t="str">
+        <x:v>tm004-core04-20261001T213019Z</x:v>
+      </x:c>
+      <x:c r="B42" s="9" t="str">
+        <x:v>v0.4.0-20261001T040433Z</x:v>
+      </x:c>
+      <x:c r="C42" s="9" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D42" s="9" t="str">
+        <x:v>TM-004 CORE04主进程触发整合候选固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E42" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F42" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G42" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H42" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I42" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J42" s="9" t="str">
+        <x:v>08463b31c5eef5e6c90978cb8d6cd79e4aa76e1a</x:v>
+      </x:c>
+      <x:c r="K42" s="9" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L42" s="9" t="str">
+        <x:v>1/1固定TC、3步与逐例清理PASS；固定source_check导出及verification回读PASS。仅同树辅助模块合同，原20产品TC、App/授权/服务及发行均NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M42" s="9" t="str">
+        <x:v>.local/test-results/tm004-core04-20261001T213019Z/TokenMeter测试结果-tm004-core04-20261001T213019Z.xlsx</x:v>
+      </x:c>
+      <x:c r="N42" s="9" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="42" customHeight="1">
+      <x:c r="A43" s="4" t="str">
+        <x:v>tm004-core05-20261001T213019Z</x:v>
+      </x:c>
+      <x:c r="B43" s="4" t="str">
+        <x:v>v0.4.0-20261001T040433Z</x:v>
+      </x:c>
+      <x:c r="C43" s="4" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D43" s="4" t="str">
+        <x:v>TM-004 CORE05三文件持久映射整合候选固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E43" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F43" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G43" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H43" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I43" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J43" s="4" t="str">
+        <x:v>08463b31c5eef5e6c90978cb8d6cd79e4aa76e1a</x:v>
+      </x:c>
+      <x:c r="K43" s="4" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L43" s="4" t="str">
+        <x:v>1/1固定TC、4步与逐例清理PASS；固定source_check导出及verification回读PASS。仅同树辅助模块合同，原20产品TC、App/授权/服务及发行均NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M43" s="4" t="str">
+        <x:v>.local/test-results/tm004-core05-20261001T213019Z/TokenMeter测试结果-tm004-core05-20261001T213019Z.xlsx</x:v>
+      </x:c>
+      <x:c r="N43" s="4" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E5:E40">
+  <x:conditionalFormatting sqref="E5:E43">
     <x:cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="26" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M40">
+  <x:conditionalFormatting sqref="M5:M43">
     <x:cfRule type="containsText" dxfId="27" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="29" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="N5:N40">
+  <x:conditionalFormatting sqref="N5:N43">
     <x:cfRule type="containsText" dxfId="30" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="32" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea61f4ea009d4c73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4da937c8421542c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23140,7 +23272,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb32f3e554b5241a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd8c59834cad4a65"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24305,7 +24437,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcea83dea6bf84594"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5602c13daa24499e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.2.0-20261001T034118Z][TM-002] Bind 25 fixed auxiliary test IDs
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Ra4f8d98df41041e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rbb8e251916d04868"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rc5f805f200d242d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rf4d8d5c4fe134d49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R6991c6c045a445d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R55615561eeb249bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R240979b2f1af4851"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R82efc12112f34203"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rbc131f664828428b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R1787dfe246cb409a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R3fd87e0127824051"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R979e864ed88a421e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rcf160d41b5c64d6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rb478feb582a44898"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R62f96965f18b4165"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rcaecb9c5edff4271"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R8d8137e30b4b4cff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Re6bf7c7d10df4df3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R4c6c81e9f3c9435b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rff99ac9c8ed14746"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R576c8065402c49d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R45024f3ea21449c5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2829fb58b8e4e3b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R167b8999760f4471"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a2cb8f825f94efe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e93a1ee773b42f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55e74f6419664647"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08b8bec042dd4560"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e81fa3ce52243fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bbe512b04b747bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc97a256db72846b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64d2a756b88843b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R123bd72d4ae64368"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dc7ec0418ba4063"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7640,7 +7640,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cee48957f904f14"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re852f6b6070746ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20972,7 +20972,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49a48a6b66b24ce7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re068c2a390c849cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22780,7 +22780,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4da937c8421542c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racb0587e60b74444"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23272,7 +23272,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd8c59834cad4a65"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3a5c29434f44e40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24437,7 +24437,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5602c13daa24499e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0473e66b4554171"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.3.0-20261001T034652Z][TM-003] Index CORE08 source check and governance runtime
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R979e864ed88a421e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rcf160d41b5c64d6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rb478feb582a44898"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R62f96965f18b4165"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rcaecb9c5edff4271"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R8d8137e30b4b4cff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Re6bf7c7d10df4df3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R4c6c81e9f3c9435b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rff99ac9c8ed14746"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R576c8065402c49d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R45024f3ea21449c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Re60ad307bc624cba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R869b52894da64148"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R276fb5c257d8442e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Red79df0315d947c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Re40804555259416f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rdff2e0925ebe44f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R2b84aff271f243dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Rfcba6c88d3d44a78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R8116b1164695443b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R9ce622b3025e476d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Rce6d1578b4ad4f27"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -809,8 +809,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N43" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N43"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N44"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="运行批次"/>
     <x:tableColumn id="2" name="版本"/>
@@ -1146,8 +1146,8 @@
         <x:v>测试批次</x:v>
       </x:c>
       <x:c r="B9" s="10" t="n">
-        <x:f>COUNTA('06测试批次'!A5:A43)</x:f>
-        <x:v>39</x:v>
+        <x:f>COUNTA('06测试批次'!A5:A44)</x:f>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>06测试批次，每次运行一行，记录独立结果Excel位置</x:v>
@@ -1271,7 +1271,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>source_check · TM-004 CORE05三文件持久映射整合候选固定辅助模块；非产品E2E：1/1固定TC、4步与逐例清理PASS；固定source_check导出及verification回读PASS。仅同树辅助模块合同，原20产品TC、App/授权/服务及发行均NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
+        <x:v>source_check · TM-003 CORE08开发候选私有密钥生命周期固定辅助模块；非产品E2E：CORE08固定四步1/1与owner清理PASS；独立Excel/verification回读PASS。先前红测FAIL原件保留；仅代码候选辅助合同，产品App/真实Keychain及发行NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R167b8999760f4471"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree166958d99d40c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e93a1ee773b42f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R258567ac30514228"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08b8bec042dd4560"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55c259f9a3eb4581"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bbe512b04b747bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd095365c43504e07"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64d2a756b88843b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0856a692cdb04fcd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dc7ec0418ba4063"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf41b0f5f112d4c4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7640,7 +7640,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re852f6b6070746ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a8319a5ae234689"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20836,7 +20836,7 @@
         <x:v>draft</x:v>
       </x:c>
       <x:c r="J280" s="9" t="str">
-        <x:v>未执行</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="K280" s="9" t="str">
         <x:v>细化用例</x:v>
@@ -20845,7 +20845,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:263</x:v>
       </x:c>
       <x:c r="M280" s="9" t="str">
-        <x:v>尚未执行</x:v>
+        <x:v>tm003-core08-20261001T215000Z</x:v>
       </x:c>
       <x:c r="N280" s="9" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -20972,7 +20972,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re068c2a390c849cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0901ff8db43b43d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22762,25 +22762,69 @@
         <x:v>NOT_RUN</x:v>
       </x:c>
     </x:row>
+    <x:row r="44" ht="42" customHeight="1">
+      <x:c r="A44" s="9" t="str">
+        <x:v>tm003-core08-20261001T215000Z</x:v>
+      </x:c>
+      <x:c r="B44" s="9" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="C44" s="9" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D44" s="9" t="str">
+        <x:v>TM-003 CORE08开发候选私有密钥生命周期固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E44" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F44" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G44" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H44" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I44" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J44" s="9" t="str">
+        <x:v>724732d77e2ff26dc8db8bd5607c7eec1ae1b800</x:v>
+      </x:c>
+      <x:c r="K44" s="9" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L44" s="9" t="str">
+        <x:v>CORE08固定四步1/1与owner清理PASS；独立Excel/verification回读PASS。先前红测FAIL原件保留；仅代码候选辅助合同，产品App/真实Keychain及发行NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M44" s="9" t="str">
+        <x:v>.local/test-results/tm003-core08-20261001T215000Z/TokenMeter测试结果-tm003-core08-20261001T215000Z.xlsx</x:v>
+      </x:c>
+      <x:c r="N44" s="9" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E5:E43">
+  <x:conditionalFormatting sqref="E5:E44">
     <x:cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="26" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M43">
+  <x:conditionalFormatting sqref="M5:M44">
     <x:cfRule type="containsText" dxfId="27" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="29" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="N5:N43">
+  <x:conditionalFormatting sqref="N5:N44">
     <x:cfRule type="containsText" dxfId="30" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="32" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racb0587e60b74444"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ddc967f20134f20"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23272,7 +23316,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3a5c29434f44e40"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13f38179e5df46b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24437,7 +24481,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0473e66b4554171"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5dc7f339cf84d85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.4.0-20261001T040433Z][TM-004] Define SourceAccess to UsageStore slice
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="Re60ad307bc624cba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R869b52894da64148"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R276fb5c257d8442e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Red79df0315d947c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Re40804555259416f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rdff2e0925ebe44f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R2b84aff271f243dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Rfcba6c88d3d44a78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R8116b1164695443b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R9ce622b3025e476d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="Rce6d1578b4ad4f27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R11c75e7501aa4a66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rcd3395bbe05047c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R97521633a63f4ee4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rf3827660e9d147a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R7263d892a32a4ea1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R5f8da0600f4e4c6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R7eb3784ad5c347e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Ra7afe048b4874971"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rf1d918338b9f4722"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Ra71b3e2eb1d143a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R8d8da5cb8ed14905"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -786,8 +786,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N282" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N282"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N283" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N283"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="功能编号"/>
     <x:tableColumn id="2" name="用例编号"/>
@@ -1134,8 +1134,8 @@
         <x:v>已登记用例</x:v>
       </x:c>
       <x:c r="B8" s="11" t="n">
-        <x:f>COUNTA('05测试用例'!B5:B282)</x:f>
-        <x:v>278</x:v>
+        <x:f>COUNTA('05测试用例'!B5:B283)</x:f>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>父用例与具有稳定 ID 的变体各占一行；含未来概要场景</x:v>
@@ -1169,7 +1169,7 @@
         <x:v>界面与治理检查</x:v>
       </x:c>
       <x:c r="B11" s="10" t="n">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C11" s="4" t="str">
         <x:v>辅助检查不能替代产品E2E；稳定变体独立列出</x:v>
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree166958d99d40c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0051db329a5045c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R258567ac30514228"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbed2d8d073d4d9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55c259f9a3eb4581"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0d713258afa4f66"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd095365c43504e07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8cb2580f5bb4754"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0856a692cdb04fcd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb66f75821784020"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf41b0f5f112d4c4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R815db8d424fd485f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7640,7 +7640,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a8319a5ae234689"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R431c2d98733447a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20949,30 +20949,81 @@
         <x:v>v0.3.0-20261001T034652Z</x:v>
       </x:c>
     </x:row>
+    <x:row r="283" ht="177" customHeight="1">
+      <x:c r="A283" s="4" t="str">
+        <x:v>TM-004</x:v>
+      </x:c>
+      <x:c r="B283" s="4" t="str">
+        <x:v>TC-TM004-CORE-06</x:v>
+      </x:c>
+      <x:c r="C283" s="4" t="str">
+        <x:v>真实SourceAccess到私有库的多文件贯通</x:v>
+      </x:c>
+      <x:c r="D283" s="4" t="str">
+        <x:v>TASK-TM004-SOURCE
+TASK-TM004-INCREMENTAL</x:v>
+      </x:c>
+      <x:c r="E283" s="4" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F283" s="4" t="str">
+        <x:v>tests/fixtures/tm004-sourceaccess-store-slice.json；四个2.1.126原生来源去敏投影文件、独立合成追加行；两页2+2/97字节分块与固定HMAC向量</x:v>
+      </x:c>
+      <x:c r="G283" s="4" t="str">
+        <x:v>1. 未确认时扫描，再经真实SourceAccess选择/预览/确认并核对四文件/root键；确认前扫描/读取/库提交均0、库空；确认仅绑定第一主体和sourceId，四文件/root键等于fixture，不把路径/原摘要当库键
+2. 真实主进程采集按两页2+2及97字节片段读完四文件，末页守卫后提交；只一次同步commitScanBatch；M+fork新+Agent父/子共5唯一调用、input85/output32/total117，四游标到LF末、coverage.scan_incomplete=0，复制fork不重计、子父归属已核验，DB/WAL无原生标识或正文
+3. 关闭重开owner来源/库/helper，重扫相同四文件；主体/root/文件键不变、事件5行/117，四游标和覆盖稳定，零新增调用；不自动读取未经确认来源
+4. 向主文件仅追加固定合成50/5完整LF行，续扫并重扫；只新增一调用，6行、input135/output37/total172，主游标推进追加字节数，其余三游标不变，无cursor_reset，复制fork不重计
+5. 从成功库独立副本分别在第一页后撤权、换主体、子文件提前EOF；每次取消scan、commitScanBatch=0；旧6行/172、四游标/覆盖原值不变，新主体无旧事件，本轮不可用/不完整而非已知零；SQLite/WAL与owner清理核对</x:v>
+      </x:c>
+      <x:c r="H283" s="4" t="str">
+        <x:v>准备：每故障从本例成功owner库复制；无生产库；只经UsageStore写入
+变化：成功首次5行/117、追加后6行/172、四游标及覆盖；故障零新写
+核验：只读usage_event/source_cursor/coverage/identity_key_state与SQLite/WAL隐私扫描；逐代际表摘要比较</x:v>
+      </x:c>
+      <x:c r="I283" s="4" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J283" s="4" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K283" s="4" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L283" s="4" t="str">
+        <x:v>docs/testing/cases/04-TM-004-claude-collection.md:221</x:v>
+      </x:c>
+      <x:c r="M283" s="4" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N283" s="4" t="str">
+        <x:v>v0.4.0-20261001T040433Z</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G5:G282">
+  <x:conditionalFormatting sqref="G5:G283">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="I5:I282">
+  <x:conditionalFormatting sqref="I5:I283">
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="16" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="17" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="J5:J282">
+  <x:conditionalFormatting sqref="J5:J283">
     <x:cfRule type="containsText" dxfId="18" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="19" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="20" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M282">
+  <x:conditionalFormatting sqref="M5:M283">
     <x:cfRule type="containsText" dxfId="21" priority="10" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="22" priority="11" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="23" priority="12" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0901ff8db43b43d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9ed34bc6b194032"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22824,7 +22875,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ddc967f20134f20"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb1d38cc0b164ee5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23316,7 +23367,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13f38179e5df46b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd349354a00ac4a68"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24481,7 +24532,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5dc7f339cf84d85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R114ad88e1a934f07"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.4.0-20261001T040433Z][TM-004] Match generated source IDs in CORE06
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R11c75e7501aa4a66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rcd3395bbe05047c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R97521633a63f4ee4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="Rf3827660e9d147a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="R7263d892a32a4ea1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R5f8da0600f4e4c6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R7eb3784ad5c347e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="Ra7afe048b4874971"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rf1d918338b9f4722"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="Ra71b3e2eb1d143a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R8d8da5cb8ed14905"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R77a41ceb7e1d4eb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Re90e5233cf324df1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rb3dba04077c2466f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R23c0a48c7a024d2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rd1467ec4d93f475f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R8b8439e4b95c43b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Redcd7efcc1be4df9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R87136a7531ae4a7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rd7591be5ae5a472b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R4aa101cd0367474c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R1fbdb36192e64380"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0051db329a5045c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9529159d9c8449b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbed2d8d073d4d9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85e279ca487f4777"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0d713258afa4f66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e3d5e78a6bb4298"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8cb2580f5bb4754"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R522391434b6d4376"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb66f75821784020"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf314f7705274a05"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R815db8d424fd485f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6414fd99d1e45fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7640,7 +7640,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R431c2d98733447a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd84c01bca41647ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20949,7 +20949,7 @@
         <x:v>v0.3.0-20261001T034652Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="283" ht="177" customHeight="1">
+    <x:row r="283" ht="192" customHeight="1">
       <x:c r="A283" s="4" t="str">
         <x:v>TM-004</x:v>
       </x:c>
@@ -20967,12 +20967,12 @@
         <x:v>模块检查</x:v>
       </x:c>
       <x:c r="F283" s="4" t="str">
-        <x:v>tests/fixtures/tm004-sourceaccess-store-slice.json；四个2.1.126原生来源去敏投影文件、独立合成追加行；两页2+2/97字节分块与固定HMAC向量</x:v>
+        <x:v>tests/fixtures/tm004-sourceaccess-store-slice.json；四个2.1.126原生来源去敏投影文件、独立合成追加行；两页2+2/97字节分块与固定UUID参考向量及真实确认随机UUID的独立参考HMAC判据</x:v>
       </x:c>
       <x:c r="G283" s="4" t="str">
-        <x:v>1. 未确认时扫描，再经真实SourceAccess选择/预览/确认并核对四文件/root键；确认前扫描/读取/库提交均0、库空；确认仅绑定第一主体和sourceId，四文件/root键等于fixture，不把路径/原摘要当库键
+        <x:v>1. 未确认时扫描，再经真实SourceAccess选择/预览/确认并核对四文件/root键；确认前扫描/读取/库提交均0、库空；真实确认只绑定第一主体并生成随机UUID，不注入固定sourceId；fixture固定UUID的四文件/root向量核参考算法，实际UUID的键等于独立参考HMAC输出；不把路径/原摘要当库键
 2. 真实主进程采集按两页2+2及97字节片段读完四文件，末页守卫后提交；只一次同步commitScanBatch；M+fork新+Agent父/子共5唯一调用、input85/output32/total117，四游标到LF末、coverage.scan_incomplete=0，复制fork不重计、子父归属已核验，DB/WAL无原生标识或正文
-3. 关闭重开owner来源/库/helper，重扫相同四文件；主体/root/文件键不变、事件5行/117，四游标和覆盖稳定，零新增调用；不自动读取未经确认来源
+3. 关闭重开owner来源/库/helper，重扫相同四文件；本轮随机sourceId与主体/root/文件键不变、事件5行/117，四游标和覆盖稳定，零新增调用；不自动读取未经确认来源
 4. 向主文件仅追加固定合成50/5完整LF行，续扫并重扫；只新增一调用，6行、input135/output37/total172，主游标推进追加字节数，其余三游标不变，无cursor_reset，复制fork不重计
 5. 从成功库独立副本分别在第一页后撤权、换主体、子文件提前EOF；每次取消scan、commitScanBatch=0；旧6行/172、四游标/覆盖原值不变，新主体无旧事件，本轮不可用/不完整而非已知零；SQLite/WAL与owner清理核对</x:v>
       </x:c>
@@ -21023,7 +21023,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9ed34bc6b194032"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fa96ea4ab404d84"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22875,7 +22875,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb1d38cc0b164ee5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6601eb6dd0b94b41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23367,7 +23367,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd349354a00ac4a68"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c41e605622d4d2e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24532,7 +24532,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R114ad88e1a934f07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ca33cc787ed485f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.5.0-20261001T034729Z][TM-005] Define dual source query view slice
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R77a41ceb7e1d4eb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Re90e5233cf324df1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rb3dba04077c2466f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R23c0a48c7a024d2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rd1467ec4d93f475f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="R8b8439e4b95c43b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Redcd7efcc1be4df9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R87136a7531ae4a7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rd7591be5ae5a472b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R4aa101cd0367474c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R1fbdb36192e64380"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R4b8a303160f5400f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R3dbd15b232e04066"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R46efc5047b764b33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R8dd1972c7c3e4d01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rf8394c7616484a88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rf6317604a1364bbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Ra5a8cac4b33a4931"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R40d4e4b74585463b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R4f58192d49164ab6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R050217ba2a5c4ec5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R5d42d572a2814a72"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -786,8 +786,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N283" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N283"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TMTable6" displayName="TMTable6" ref="A4:N284" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N284"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="功能编号"/>
     <x:tableColumn id="2" name="用例编号"/>
@@ -1134,8 +1134,8 @@
         <x:v>已登记用例</x:v>
       </x:c>
       <x:c r="B8" s="11" t="n">
-        <x:f>COUNTA('05测试用例'!B5:B283)</x:f>
-        <x:v>279</x:v>
+        <x:f>COUNTA('05测试用例'!B5:B284)</x:f>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>父用例与具有稳定 ID 的变体各占一行；含未来概要场景</x:v>
@@ -1169,7 +1169,7 @@
         <x:v>界面与治理检查</x:v>
       </x:c>
       <x:c r="B11" s="10" t="n">
-        <x:v>66</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C11" s="4" t="str">
         <x:v>辅助检查不能替代产品E2E；稳定变体独立列出</x:v>
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9529159d9c8449b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fed29b5aa264417"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85e279ca487f4777"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c3d33699d2c4545"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e3d5e78a6bb4298"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbb5786e72754e88"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R522391434b6d4376"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R901e345719de4d1f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf314f7705274a05"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80f007a5ff5c43f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6414fd99d1e45fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb10df9d3590b4d26"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7640,7 +7640,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd84c01bca41647ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R096d115e78054a86"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21000,30 +21000,80 @@
         <x:v>v0.4.0-20261001T040433Z</x:v>
       </x:c>
     </x:row>
+    <x:row r="284" ht="207" customHeight="1">
+      <x:c r="A284" s="9" t="str">
+        <x:v>TM-005</x:v>
+      </x:c>
+      <x:c r="B284" s="9" t="str">
+        <x:v>TC-TM005-CORE-06</x:v>
+      </x:c>
+      <x:c r="C284" s="9" t="str">
+        <x:v>同快照双来源查询视图与模型身份</x:v>
+      </x:c>
+      <x:c r="D284" s="9" t="str">
+        <x:v>TASK-TM005-RANGE-QUERY</x:v>
+      </x:c>
+      <x:c r="E284" s="9" t="str">
+        <x:v>模块检查</x:v>
+      </x:c>
+      <x:c r="F284" s="9" t="str">
+        <x:v>tests/fixtures/tm005-query-view-slice.json引用CORE05物理库种子；上海当地09-29半开UTC、A–H合成事件、字面unknown_model及99字符含冒号模型</x:v>
+      </x:c>
+      <x:c r="G284" s="9" t="str">
+        <x:v>1. A–E仅经真实UsageStore提交到owner库，再在上海09-29 UTC半开窗开启同一只读查询事务；仅A/B两行、calls2、input300/output30、known330；Codex110/Claude220；state partial、total null；C异主体、D界前、E上界排除，查询零写
+2. 同一事务读模型/明细/当地日趋势及三类未知子项；模型null110与sonnet-test220分离，明细A/B，趋势partial/known330/total null；cached read20/未知1、cache write0/未知2、reasoning2/未知1，不加总；输出白名单无原生标识或秘密
+3. 第一事务保持时另一连接写F50/5，再分别查旧事务与新事务；旧事务仍A/B330；新事务A/B/F三调用input350/output35/known385、Codex165/Claude220且partial/total null；WAL不可用则BLOCKED
+4. 独立A–E库经UsageStore增加字面unknown_model的G及99字符含冒号模型H，重查同一日；A/B/G/H四行input370/output37/known407、Codex110/Claude297；modelId null110、sonnet-test220、字面unknown_model33、长冒号模型44互异且原值保留；仍partial/total null
+5. 查询当地10-01无事件日并核对隐私、只读与owner清理；missing/known0/total null，绝不成功完整零；库/WAL与输出无原生ID/路径/正文/secret/密文，仅清理本例拥有目录</x:v>
+      </x:c>
+      <x:c r="H284" s="9" t="str">
+        <x:v>准备：真实UsageStore.commitBatch只写本例owner空库；并发、模型补充与空日各独立副本
+变化：查询零写；基础A/B已知330，F后新事务385，G/H独立分支407
+核验：只读usage_event集合/模型原值/来源/时间及SQLite/WAL隐私；事务前后表摘要与owner清理</x:v>
+      </x:c>
+      <x:c r="I284" s="9" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="J284" s="9" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K284" s="9" t="str">
+        <x:v>细化用例</x:v>
+      </x:c>
+      <x:c r="L284" s="9" t="str">
+        <x:v>releases/v0.5.0-20261001T034729Z/04a-test-cases.md:375</x:v>
+      </x:c>
+      <x:c r="M284" s="9" t="str">
+        <x:v>尚未执行</x:v>
+      </x:c>
+      <x:c r="N284" s="9" t="str">
+        <x:v>v0.5.0-20261001T034729Z</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G5:G283">
+  <x:conditionalFormatting sqref="G5:G284">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="I5:I283">
+  <x:conditionalFormatting sqref="I5:I284">
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="16" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="17" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="J5:J283">
+  <x:conditionalFormatting sqref="J5:J284">
     <x:cfRule type="containsText" dxfId="18" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="19" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="20" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M283">
+  <x:conditionalFormatting sqref="M5:M284">
     <x:cfRule type="containsText" dxfId="21" priority="10" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="22" priority="11" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="23" priority="12" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fa96ea4ab404d84"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5e37fd6971d4f24"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22875,7 +22925,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6601eb6dd0b94b41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red69b6cf9ea349bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23367,7 +23417,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c41e605622d4d2e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1c06ea376e14a32"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24532,7 +24582,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ca33cc787ed485f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92d89f73c8be4cab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[v0.3.0-20261001T034652Z][TM-003] Bind final core suites and register nine source checks
</commit_message>
<xml_diff>
--- a/TokenMeter项目总表.xlsx
+++ b/TokenMeter项目总表.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R4b8a303160f5400f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="R3dbd15b232e04066"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="R46efc5047b764b33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R8dd1972c7c3e4d01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rf8394c7616484a88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rf6317604a1364bbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="Ra5a8cac4b33a4931"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R40d4e4b74585463b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="R4f58192d49164ab6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R050217ba2a5c4ec5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R5d42d572a2814a72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00项目总览" sheetId="1" r:id="R9a0aa274d76c4726"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01需求清单" sheetId="2" r:id="Rfdb325963c5945ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02验收条件" sheetId="3" r:id="Rb144adf4e7fc4b29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03功能点" sheetId="4" r:id="R5e7a0981a3e345ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04开发任务" sheetId="5" r:id="Rc388648c81fd4ccf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05测试用例" sheetId="6" r:id="Rb407bb5e288743e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06测试批次" sheetId="7" r:id="R617128a7b85d4040"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07发布版本" sheetId="8" r:id="R25c324dfd5a4437a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08问题复盘" sheetId="9" r:id="Rc8ec9f5767e849e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09执行SOP" sheetId="10" r:id="R87c6e3652fa249dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10项目约定" sheetId="11" r:id="R1918838afdf44649"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -809,8 +809,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N44"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TMTable7" displayName="TMTable7" ref="A4:N53" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N53"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="运行批次"/>
     <x:tableColumn id="2" name="版本"/>
@@ -1146,8 +1146,8 @@
         <x:v>测试批次</x:v>
       </x:c>
       <x:c r="B9" s="10" t="n">
-        <x:f>COUNTA('06测试批次'!A5:A44)</x:f>
-        <x:v>40</x:v>
+        <x:f>COUNTA('06测试批次'!A5:A53)</x:f>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>06测试批次，每次运行一行，记录独立结果Excel位置</x:v>
@@ -1271,7 +1271,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>source_check · TM-003 CORE08开发候选私有密钥生命周期固定辅助模块；非产品E2E：CORE08固定四步1/1与owner清理PASS；独立Excel/verification回读PASS。先前红测FAIL原件保留；仅代码候选辅助合同，产品App/真实Keychain及发行NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
+        <x:v>source_check · TM-003 tm003-core09旧代码候选固定辅助模块；非产品E2E：1/1固定TC、4步与逐例清理PASS；原始报告及独立Excel/verification回读一致。只属于所列旧代码候选；本次文档绑定后未据此声称当前候选PASS，产品App E2E及发行NOT_RUN。；是否覆盖完整产品回归以批次范围和原始证据为准。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
@@ -1288,7 +1288,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fed29b5aa264417"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd57e4d1c608d430a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1996,7 +1996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c3d33699d2c4545"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3eb98c4c3e8249ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2145,7 +2145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbb5786e72754e88"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde09c7aff4b64aef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2580,7 +2580,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R901e345719de4d1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R296ffe6bd6b64c7f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3627,7 +3627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80f007a5ff5c43f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c82bc0790c141fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4734,7 +4734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb10df9d3590b4d26"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe158d460f334dcd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7640,7 +7640,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R096d115e78054a86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ca7d295c1f24741"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20010,7 +20010,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:420</x:v>
       </x:c>
       <x:c r="M263" s="4" t="str">
-        <x:v>tm003-core-20261001T203711Z</x:v>
+        <x:v>tm003-final-20261001T215242Z-tm003-core</x:v>
       </x:c>
       <x:c r="N263" s="4" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -20059,7 +20059,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:424</x:v>
       </x:c>
       <x:c r="M264" s="9" t="str">
-        <x:v>tm003-core-20261001T203711Z</x:v>
+        <x:v>tm003-final-20261001T215242Z-tm003-core</x:v>
       </x:c>
       <x:c r="N264" s="9" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -20107,7 +20107,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:428</x:v>
       </x:c>
       <x:c r="M265" s="4" t="str">
-        <x:v>tm003-core-20261001T203711Z</x:v>
+        <x:v>tm003-final-20261001T215242Z-tm003-core</x:v>
       </x:c>
       <x:c r="N265" s="4" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -20156,7 +20156,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:203</x:v>
       </x:c>
       <x:c r="M266" s="9" t="str">
-        <x:v>tm003-core45-20261001T203711Z</x:v>
+        <x:v>tm003-final-20261001T215242Z-tm003-core45</x:v>
       </x:c>
       <x:c r="N266" s="9" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -20207,7 +20207,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:216</x:v>
       </x:c>
       <x:c r="M267" s="4" t="str">
-        <x:v>tm003-core45-20261001T203711Z</x:v>
+        <x:v>tm003-final-20261001T215242Z-tm003-core45</x:v>
       </x:c>
       <x:c r="N267" s="4" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -20257,7 +20257,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:230</x:v>
       </x:c>
       <x:c r="M268" s="9" t="str">
-        <x:v>tm003-core06-20261001T203711Z</x:v>
+        <x:v>tm003-final-20261001T215242Z-tm003-core06</x:v>
       </x:c>
       <x:c r="N268" s="9" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -20308,7 +20308,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:245</x:v>
       </x:c>
       <x:c r="M269" s="4" t="str">
-        <x:v>tm003-core07-20261001T203711Z</x:v>
+        <x:v>tm003-final-20261001T215242Z-tm003-core07</x:v>
       </x:c>
       <x:c r="N269" s="4" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -20845,7 +20845,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:263</x:v>
       </x:c>
       <x:c r="M280" s="9" t="str">
-        <x:v>tm003-core08-20261001T215000Z</x:v>
+        <x:v>tm003-core08-20261001T220500Z</x:v>
       </x:c>
       <x:c r="N280" s="9" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -20885,7 +20885,7 @@
         <x:v>draft</x:v>
       </x:c>
       <x:c r="J281" s="4" t="str">
-        <x:v>未执行</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="K281" s="4" t="str">
         <x:v>细化用例</x:v>
@@ -20894,7 +20894,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:276</x:v>
       </x:c>
       <x:c r="M281" s="4" t="str">
-        <x:v>尚未执行</x:v>
+        <x:v>tm003-core09-20261001T220500Z</x:v>
       </x:c>
       <x:c r="N281" s="4" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -20934,7 +20934,7 @@
         <x:v>draft</x:v>
       </x:c>
       <x:c r="J282" s="9" t="str">
-        <x:v>未执行</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="K282" s="9" t="str">
         <x:v>细化用例</x:v>
@@ -20943,7 +20943,7 @@
         <x:v>docs/testing/cases/03-TM-003-codex-collection.md:289</x:v>
       </x:c>
       <x:c r="M282" s="9" t="str">
-        <x:v>尚未执行</x:v>
+        <x:v>tm003-final-20261001T215242Z-tm003-core10</x:v>
       </x:c>
       <x:c r="N282" s="9" t="str">
         <x:v>v0.3.0-20261001T034652Z</x:v>
@@ -21073,7 +21073,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5e37fd6971d4f24"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d69bda786a64f8e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22907,25 +22907,421 @@
         <x:v>NOT_RUN</x:v>
       </x:c>
     </x:row>
+    <x:row r="45" ht="57" customHeight="1">
+      <x:c r="A45" s="4" t="str">
+        <x:v>tm003-final-20261001T215242Z-tm003-core</x:v>
+      </x:c>
+      <x:c r="B45" s="4" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="C45" s="4" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D45" s="4" t="str">
+        <x:v>TM-003 tm003-core旧代码候选固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E45" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F45" s="4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G45" s="4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H45" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I45" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J45" s="4" t="str">
+        <x:v>2d2f70d056c32f3f207b0c966092b8fa0754ecfc</x:v>
+      </x:c>
+      <x:c r="K45" s="4" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L45" s="4" t="str">
+        <x:v>3/3固定TC、9步与逐例清理PASS；原始报告及独立Excel/verification回读一致。只属于所列旧代码候选；本次文档绑定后未据此声称当前候选PASS，产品App E2E及发行NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M45" s="4" t="str">
+        <x:v>.local/test-results/tm003-final-20261001T215242Z-tm003-core/TokenMeter测试结果-tm003-final-20261001T215242Z-tm003-core.xlsx</x:v>
+      </x:c>
+      <x:c r="N45" s="4" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="57" customHeight="1">
+      <x:c r="A46" s="9" t="str">
+        <x:v>tm003-final-20261001T215242Z-tm003-core45</x:v>
+      </x:c>
+      <x:c r="B46" s="9" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="C46" s="9" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D46" s="9" t="str">
+        <x:v>TM-003 tm003-core45旧代码候选固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E46" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F46" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G46" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H46" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I46" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J46" s="9" t="str">
+        <x:v>2d2f70d056c32f3f207b0c966092b8fa0754ecfc</x:v>
+      </x:c>
+      <x:c r="K46" s="9" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L46" s="9" t="str">
+        <x:v>2/2固定TC、9步与逐例清理PASS；原始报告及独立Excel/verification回读一致。只属于所列旧代码候选；本次文档绑定后未据此声称当前候选PASS，产品App E2E及发行NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M46" s="9" t="str">
+        <x:v>.local/test-results/tm003-final-20261001T215242Z-tm003-core45/TokenMeter测试结果-tm003-final-20261001T215242Z-tm003-core45.xlsx</x:v>
+      </x:c>
+      <x:c r="N46" s="9" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="57" customHeight="1">
+      <x:c r="A47" s="4" t="str">
+        <x:v>tm003-final-20261001T215242Z-tm003-core06</x:v>
+      </x:c>
+      <x:c r="B47" s="4" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="C47" s="4" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D47" s="4" t="str">
+        <x:v>TM-003 tm003-core06旧代码候选固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E47" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F47" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G47" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H47" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I47" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J47" s="4" t="str">
+        <x:v>2d2f70d056c32f3f207b0c966092b8fa0754ecfc</x:v>
+      </x:c>
+      <x:c r="K47" s="4" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L47" s="4" t="str">
+        <x:v>1/1固定TC、4步与逐例清理PASS；原始报告及独立Excel/verification回读一致。只属于所列旧代码候选；本次文档绑定后未据此声称当前候选PASS，产品App E2E及发行NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M47" s="4" t="str">
+        <x:v>.local/test-results/tm003-final-20261001T215242Z-tm003-core06/TokenMeter测试结果-tm003-final-20261001T215242Z-tm003-core06.xlsx</x:v>
+      </x:c>
+      <x:c r="N47" s="4" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="57" customHeight="1">
+      <x:c r="A48" s="9" t="str">
+        <x:v>tm003-final-20261001T215242Z-tm003-core07</x:v>
+      </x:c>
+      <x:c r="B48" s="9" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="C48" s="9" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D48" s="9" t="str">
+        <x:v>TM-003 tm003-core07旧代码候选固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E48" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F48" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G48" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H48" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I48" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J48" s="9" t="str">
+        <x:v>2d2f70d056c32f3f207b0c966092b8fa0754ecfc</x:v>
+      </x:c>
+      <x:c r="K48" s="9" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L48" s="9" t="str">
+        <x:v>1/1固定TC、5步与逐例清理PASS；原始报告及独立Excel/verification回读一致。只属于所列旧代码候选；本次文档绑定后未据此声称当前候选PASS，产品App E2E及发行NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M48" s="9" t="str">
+        <x:v>.local/test-results/tm003-final-20261001T215242Z-tm003-core07/TokenMeter测试结果-tm003-final-20261001T215242Z-tm003-core07.xlsx</x:v>
+      </x:c>
+      <x:c r="N48" s="9" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="57" customHeight="1">
+      <x:c r="A49" s="4" t="str">
+        <x:v>tm003-final-20261001T215242Z-tm003-core08</x:v>
+      </x:c>
+      <x:c r="B49" s="4" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="C49" s="4" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D49" s="4" t="str">
+        <x:v>TM-003 tm003-core08旧代码候选固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E49" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F49" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G49" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H49" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I49" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J49" s="4" t="str">
+        <x:v>2d2f70d056c32f3f207b0c966092b8fa0754ecfc</x:v>
+      </x:c>
+      <x:c r="K49" s="4" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L49" s="4" t="str">
+        <x:v>1/1固定TC、4步与逐例清理PASS；原始报告及独立Excel/verification回读一致。只属于所列旧代码候选；本次文档绑定后未据此声称当前候选PASS，产品App E2E及发行NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M49" s="4" t="str">
+        <x:v>.local/test-results/tm003-final-20261001T215242Z-tm003-core08/TokenMeter测试结果-tm003-final-20261001T215242Z-tm003-core08.xlsx</x:v>
+      </x:c>
+      <x:c r="N49" s="4" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="57" customHeight="1">
+      <x:c r="A50" s="9" t="str">
+        <x:v>tm003-final-20261001T215242Z-tm003-core09</x:v>
+      </x:c>
+      <x:c r="B50" s="9" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="C50" s="9" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D50" s="9" t="str">
+        <x:v>TM-003 tm003-core09旧代码候选固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E50" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F50" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G50" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H50" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I50" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J50" s="9" t="str">
+        <x:v>2d2f70d056c32f3f207b0c966092b8fa0754ecfc</x:v>
+      </x:c>
+      <x:c r="K50" s="9" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L50" s="9" t="str">
+        <x:v>1/1固定TC、4步与逐例清理PASS；原始报告及独立Excel/verification回读一致。只属于所列旧代码候选；本次文档绑定后未据此声称当前候选PASS，产品App E2E及发行NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M50" s="9" t="str">
+        <x:v>.local/test-results/tm003-final-20261001T215242Z-tm003-core09/TokenMeter测试结果-tm003-final-20261001T215242Z-tm003-core09.xlsx</x:v>
+      </x:c>
+      <x:c r="N50" s="9" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="57" customHeight="1">
+      <x:c r="A51" s="4" t="str">
+        <x:v>tm003-final-20261001T215242Z-tm003-core10</x:v>
+      </x:c>
+      <x:c r="B51" s="4" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="C51" s="4" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D51" s="4" t="str">
+        <x:v>TM-003 tm003-core10旧代码候选固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E51" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F51" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G51" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H51" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I51" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J51" s="4" t="str">
+        <x:v>2d2f70d056c32f3f207b0c966092b8fa0754ecfc</x:v>
+      </x:c>
+      <x:c r="K51" s="4" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L51" s="4" t="str">
+        <x:v>1/1固定TC、4步与逐例清理PASS；原始报告及独立Excel/verification回读一致。只属于所列旧代码候选；本次文档绑定后未据此声称当前候选PASS，产品App E2E及发行NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M51" s="4" t="str">
+        <x:v>.local/test-results/tm003-final-20261001T215242Z-tm003-core10/TokenMeter测试结果-tm003-final-20261001T215242Z-tm003-core10.xlsx</x:v>
+      </x:c>
+      <x:c r="N51" s="4" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="57" customHeight="1">
+      <x:c r="A52" s="9" t="str">
+        <x:v>tm003-core08-20261001T220500Z</x:v>
+      </x:c>
+      <x:c r="B52" s="9" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="C52" s="9" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D52" s="9" t="str">
+        <x:v>TM-003 tm003-core08旧代码候选固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E52" s="9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F52" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G52" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H52" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I52" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J52" s="9" t="str">
+        <x:v>3c07fe7fa6b3049707f10a86df4afc0f6399d0f0</x:v>
+      </x:c>
+      <x:c r="K52" s="9" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L52" s="9" t="str">
+        <x:v>1/1固定TC、4步与逐例清理PASS；原始报告及独立Excel/verification回读一致。只属于所列旧代码候选；本次文档绑定后未据此声称当前候选PASS，产品App E2E及发行NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M52" s="9" t="str">
+        <x:v>.local/test-results/tm003-core08-20261001T220500Z/TokenMeter测试结果-tm003-core08-20261001T220500Z.xlsx</x:v>
+      </x:c>
+      <x:c r="N52" s="9" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="57" customHeight="1">
+      <x:c r="A53" s="4" t="str">
+        <x:v>tm003-core09-20261001T220500Z</x:v>
+      </x:c>
+      <x:c r="B53" s="4" t="str">
+        <x:v>v0.3.0-20261001T034652Z</x:v>
+      </x:c>
+      <x:c r="C53" s="4" t="str">
+        <x:v>source_check</x:v>
+      </x:c>
+      <x:c r="D53" s="4" t="str">
+        <x:v>TM-003 tm003-core09旧代码候选固定辅助模块；非产品E2E</x:v>
+      </x:c>
+      <x:c r="E53" s="4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F53" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G53" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H53" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I53" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J53" s="4" t="str">
+        <x:v>3c07fe7fa6b3049707f10a86df4afc0f6399d0f0</x:v>
+      </x:c>
+      <x:c r="K53" s="4" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L53" s="4" t="str">
+        <x:v>1/1固定TC、4步与逐例清理PASS；原始报告及独立Excel/verification回读一致。只属于所列旧代码候选；本次文档绑定后未据此声称当前候选PASS，产品App E2E及发行NOT_RUN。</x:v>
+      </x:c>
+      <x:c r="M53" s="4" t="str">
+        <x:v>.local/test-results/tm003-core09-20261001T220500Z/TokenMeter测试结果-tm003-core09-20261001T220500Z.xlsx</x:v>
+      </x:c>
+      <x:c r="N53" s="4" t="str">
+        <x:v>NOT_RUN</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E5:E44">
+  <x:conditionalFormatting sqref="E5:E53">
     <x:cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="26" priority="3" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M44">
+  <x:conditionalFormatting sqref="M5:M53">
     <x:cfRule type="containsText" dxfId="27" priority="4" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="29" priority="6" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="N5:N44">
+  <x:conditionalFormatting sqref="N5:N53">
     <x:cfRule type="containsText" dxfId="30" priority="7" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="预期待明确"/>
     <x:cfRule type="containsText" dxfId="32" priority="9" operator="containsText" text="未执行"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red69b6cf9ea349bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e1fd508037243f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23417,7 +23813,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1c06ea376e14a32"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9517e8a26d74eb6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24582,7 +24978,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92d89f73c8be4cab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc82639d811b84a4a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>